<commit_message>
added addinitonal test cases
</commit_message>
<xml_diff>
--- a/testdata.xlsx
+++ b/testdata.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29231"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sshiwani\workspace\find-information-products-services-tests\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{55804917-92F1-4B7D-BF36-02503B3D2E86}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{65523A05-6494-4F6F-9A24-032AF18B86CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="22780" windowHeight="14540" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -500,7 +500,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
@@ -508,7 +508,6 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -3987,10 +3986,10 @@
       <c r="HU3"/>
     </row>
     <row r="4" spans="1:229" x14ac:dyDescent="0.35">
-      <c r="A4" s="7" t="s">
+      <c r="A4" s="3" t="s">
         <v>123</v>
       </c>
-      <c r="B4" s="7" t="s">
+      <c r="B4" s="3" t="s">
         <v>124</v>
       </c>
       <c r="C4" s="3" t="s">
@@ -4007,10 +4006,10 @@
       </c>
     </row>
     <row r="5" spans="1:229" x14ac:dyDescent="0.35">
-      <c r="A5" s="7" t="s">
+      <c r="A5" s="3" t="s">
         <v>127</v>
       </c>
-      <c r="B5" s="7" t="s">
+      <c r="B5" s="3" t="s">
         <v>128</v>
       </c>
       <c r="C5" s="3" t="s">

</xml_diff>

<commit_message>
verifying user group subcategory pages
</commit_message>
<xml_diff>
--- a/testdata.xlsx
+++ b/testdata.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sshiwani\workspace\find-information-products-services-tests\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{84601013-AC13-48B6-BBD5-5C3C5F01E49F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4F43993A-715F-4D1C-B894-7EEE8875F979}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="22780" windowHeight="14540" firstSheet="2" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="22780" windowHeight="14540" firstSheet="21" activeTab="23" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="category_phase" sheetId="1" r:id="rId1"/>
@@ -35,6 +35,8 @@
     <sheet name="UGSubcategory_Employer" sheetId="20" r:id="rId20"/>
     <sheet name="UGSubcategory_LAWorkforce" sheetId="21" r:id="rId21"/>
     <sheet name="UGSubcategory_NEETOrCareerSeek" sheetId="22" r:id="rId22"/>
+    <sheet name="UGSubcategory_ParentOrCarer" sheetId="23" r:id="rId23"/>
+    <sheet name="UGSubcateg_ProfExtUserofDfEData" sheetId="24" r:id="rId24"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -46,7 +48,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="861" uniqueCount="395">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="877" uniqueCount="442">
   <si>
     <t>Search and filter products and services</t>
   </si>
@@ -435,9 +437,6 @@
     <t>Col3</t>
   </si>
   <si>
-    <t>View products in this category</t>
-  </si>
-  <si>
     <t>categories/user-group/adult-learner-18</t>
   </si>
   <si>
@@ -450,9 +449,6 @@
     <t>Adult learner (18+)</t>
   </si>
   <si>
-    <t>//*[@id="main-content"]/div/div/div/ul[1]/li/div/p</t>
-  </si>
-  <si>
     <t>Adult in work based learning or training</t>
   </si>
   <si>
@@ -465,18 +461,6 @@
     <t>Student (higher education)</t>
   </si>
   <si>
-    <t>//*[@id="main-content"]/div/div/div/ul[2]/li[1]/div/p</t>
-  </si>
-  <si>
-    <t>//*[@id="main-content"]/div/div/div/ul[2]/li[2]/div/p</t>
-  </si>
-  <si>
-    <t>//*[@id="main-content"]/div/div/div/ul[2]/li[3]/div/p</t>
-  </si>
-  <si>
-    <t>//*[@id="main-content"]/div/div/div/ul[2]/li[4]/div/p</t>
-  </si>
-  <si>
     <t>//*[@id="main-content"]/div/div/div/p[2]</t>
   </si>
   <si>
@@ -528,9 +512,6 @@
     <t>Young person (16-18)</t>
   </si>
   <si>
-    <t>//*[@id="main-content"]/div/div/div/ul[2]/li[5]/div/p</t>
-  </si>
-  <si>
     <t>Young person with SEND (16-25)</t>
   </si>
   <si>
@@ -579,30 +560,9 @@
     <t>Higher education workforce</t>
   </si>
   <si>
-    <t>//*[@id="main-content"]/div/div/div/ul[2]/li[6]/div/p</t>
-  </si>
-  <si>
     <t>School workforce</t>
   </si>
   <si>
-    <t>9 sub-categories</t>
-  </si>
-  <si>
-    <t>3 sub-categories</t>
-  </si>
-  <si>
-    <t>1 sub-categories</t>
-  </si>
-  <si>
-    <t>10 sub-categories</t>
-  </si>
-  <si>
-    <t>5 sub-categories</t>
-  </si>
-  <si>
-    <t>//*[@id="main-content"]/div/div/div/ul[2]/li[7]/div/p</t>
-  </si>
-  <si>
     <t>SEND professional</t>
   </si>
   <si>
@@ -705,9 +665,6 @@
     <t>Parent or carer of young person (16-18)</t>
   </si>
   <si>
-    <t>//*[@id="main-content"]/div/div/div/ul[2]/li[8]/div/p</t>
-  </si>
-  <si>
     <t>categories/user-group/professional-external-user-of-dfe-data</t>
   </si>
   <si>
@@ -1231,6 +1188,192 @@
   </si>
   <si>
     <t>#type-data-collection-and-reporting</t>
+  </si>
+  <si>
+    <t>products?userGroup=parent-or-carer</t>
+  </si>
+  <si>
+    <t>ul.moj-filter-tags li a:has-text(' Parent or carer')</t>
+  </si>
+  <si>
+    <t>Remove this filter Parent or carer</t>
+  </si>
+  <si>
+    <t>products?userGroup=expectant-parent</t>
+  </si>
+  <si>
+    <t>ul.moj-filter-tags li a:has-text(' Expectant parent ')</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Remove this filter Expectant parent </t>
+  </si>
+  <si>
+    <t>Expectant parent  (Parent or carer)</t>
+  </si>
+  <si>
+    <t>products?userGroup=parent-or-carer-of-adult-learner</t>
+  </si>
+  <si>
+    <t>ul.moj-filter-tags li a:has-text(' Parent or carer of adult learner  (Parent or carer)')</t>
+  </si>
+  <si>
+    <t>Remove this filter Parent or carer of adult learner  (Parent or carer)</t>
+  </si>
+  <si>
+    <t>Parent or carer of adult learner  (Parent or carer)</t>
+  </si>
+  <si>
+    <t>products?userGroup=parent-or-carer-of-career-seeker</t>
+  </si>
+  <si>
+    <t>ul.moj-filter-tags li a:has-text(' Parent or carer of career seeker  (Parent or carer)')</t>
+  </si>
+  <si>
+    <t>Remove this filter Parent or carer of career seeker  (Parent or carer)</t>
+  </si>
+  <si>
+    <t>Parent or carer of career seeker  (Parent or carer)</t>
+  </si>
+  <si>
+    <t>products?userGroup=parent-or-carer-of-child-early-years-age</t>
+  </si>
+  <si>
+    <t>ul.moj-filter-tags li a:has-text(' Parent or carer of child (early years age) ')</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Remove this filter Parent or carer of child (early years age) </t>
+  </si>
+  <si>
+    <t>Parent or carer of child (early years age)  (Parent or carer)</t>
+  </si>
+  <si>
+    <t>products?userGroup=parent-or-carer-of-child-primary-age</t>
+  </si>
+  <si>
+    <t>ul.moj-filter-tags li a:has-text(' Parent or carer of child (primary age) ')</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Remove this filter Parent or carer of child (primary age) </t>
+  </si>
+  <si>
+    <t>Parent or carer of child (primary age)  (Parent or carer)</t>
+  </si>
+  <si>
+    <t>products?userGroup=parent-or-carer-of-child-secondary-age</t>
+  </si>
+  <si>
+    <t>ul.moj-filter-tags li a:has-text(' Parent or carer of child (secondary age) ')</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Remove this filter Parent or carer of child (secondary age) </t>
+  </si>
+  <si>
+    <t>Parent or carer of child (secondary age)  (Parent or carer)</t>
+  </si>
+  <si>
+    <t>products?userGroup=parent-or-carer-of-child-send</t>
+  </si>
+  <si>
+    <t>ul.moj-filter-tags li a:has-text(' Parent or carer of child (SEND) ')</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Remove this filter Parent or carer of child (SEND) </t>
+  </si>
+  <si>
+    <t>Parent or carer of child (SEND)  (Parent or carer)</t>
+  </si>
+  <si>
+    <t>products?userGroup=parent-or-carer-of-young-person-16-18</t>
+  </si>
+  <si>
+    <t>ul.moj-filter-tags li a:has-text(' Parent or carer of young person (16-18)  (Parent or carer)')</t>
+  </si>
+  <si>
+    <t>Remove this filter Parent or carer of young person (16-18)  (Parent or carer)</t>
+  </si>
+  <si>
+    <t>Parent or carer of young person (16-18)  (Parent or carer)</t>
+  </si>
+  <si>
+    <t>products?userGroup=professional-external-user-of-dfe-data</t>
+  </si>
+  <si>
+    <t>ul.moj-filter-tags li a:has-text(' Professional external user of DfE data')</t>
+  </si>
+  <si>
+    <t>Remove this filter Professional external user of DfE data</t>
+  </si>
+  <si>
+    <t>products?userGroup=colleague-in-another-part-of-government-data-user</t>
+  </si>
+  <si>
+    <t>ul.moj-filter-tags li a:has-text(' Colleague in another part of government (data user)  (Professional external user of DfE data)')</t>
+  </si>
+  <si>
+    <t>Remove this filter Colleague in another part of government (data user)  (Professional external user of DfE data)</t>
+  </si>
+  <si>
+    <t>Colleague in another part of government (data user)  (Professional external user of DfE data)</t>
+  </si>
+  <si>
+    <t>products?userGroup=journalist-data-user</t>
+  </si>
+  <si>
+    <t>ul.moj-filter-tags li a:has-text(' Journalist (data user)  (Professional external user of DfE data)')</t>
+  </si>
+  <si>
+    <t>Remove this filter Journalist (data user)  (Professional external user of DfE data)</t>
+  </si>
+  <si>
+    <t>Journalist (data user)  (Professional external user of DfE data)</t>
+  </si>
+  <si>
+    <t>products?userGroup=member-of-a-professional-network-data-user</t>
+  </si>
+  <si>
+    <t>ul.moj-filter-tags li a:has-text(' Member of a professional network (data user)  (Professional external user of DfE data)')</t>
+  </si>
+  <si>
+    <t>Remove this filter Member of a professional network (data user)  (Professional external user of DfE data)</t>
+  </si>
+  <si>
+    <t>Member of a professional network (data user)  (Professional external user of DfE data)</t>
+  </si>
+  <si>
+    <t>products?userGroup=professional-representative-bodies-workforce-data-user</t>
+  </si>
+  <si>
+    <t>ul.moj-filter-tags li a:has-text(' Professional representative bodies workforce (data user)  (Professional external user of DfE data)')</t>
+  </si>
+  <si>
+    <t>Remove this filter Professional representative bodies workforce (data user)  (Professional external user of DfE data)</t>
+  </si>
+  <si>
+    <t>Professional representative bodies workforce (data user)  (Professional external user of DfE data)</t>
+  </si>
+  <si>
+    <t>products?userGroup=researcher-data-user</t>
+  </si>
+  <si>
+    <t>ul.moj-filter-tags li a:has-text(' Researcher (data user)  (Professional external user of DfE data)')</t>
+  </si>
+  <si>
+    <t>Remove this filter Researcher (data user)  (Professional external user of DfE data)</t>
+  </si>
+  <si>
+    <t>Researcher (data user)  (Professional external user of DfE data)</t>
+  </si>
+  <si>
+    <t>products?userGroup=trade-union-bodies-workforce-data-user</t>
+  </si>
+  <si>
+    <t>ul.moj-filter-tags li a:has-text(' Trade union bodies workforce (data user)  (Professional external user of DfE data)')</t>
+  </si>
+  <si>
+    <t>Remove this filter Trade union bodies workforce (data user)  (Professional external user of DfE data)</t>
+  </si>
+  <si>
+    <t>Trade union bodies workforce (data user)  (Professional external user of DfE data)</t>
   </si>
 </sst>
 </file>
@@ -1284,7 +1427,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="5">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -1344,11 +1487,22 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
@@ -1358,6 +1512,7 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -9838,75 +9993,53 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" s="3" t="s">
-        <v>186</v>
+        <v>172</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>187</v>
+        <v>173</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="14" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="3" t="s">
-        <v>188</v>
-      </c>
       <c r="B3" s="3" t="s">
-        <v>134</v>
+        <v>139</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>129</v>
+        <v>140</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A4" s="3" t="s">
-        <v>189</v>
-      </c>
       <c r="B4" s="3" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>129</v>
+        <v>138</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A5" s="3" t="s">
-        <v>190</v>
-      </c>
-      <c r="B5" s="3" t="s">
-        <v>140</v>
-      </c>
-      <c r="C5" s="3" t="s">
-        <v>129</v>
-      </c>
+        <v>174</v>
+      </c>
+      <c r="B5" s="3"/>
+      <c r="C5" s="3"/>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A6" s="3" t="s">
-        <v>191</v>
-      </c>
-      <c r="B6" s="3" t="s">
-        <v>141</v>
-      </c>
-      <c r="C6" s="3" t="s">
-        <v>129</v>
-      </c>
+        <v>175</v>
+      </c>
+      <c r="B6" s="3"/>
+      <c r="C6" s="3"/>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A7" s="3"/>
-      <c r="B7" s="3" t="s">
-        <v>145</v>
-      </c>
-      <c r="C7" s="3" t="s">
-        <v>146</v>
+      <c r="A7" s="3" t="s">
+        <v>176</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A8" s="3"/>
-      <c r="B8" s="3" t="s">
-        <v>143</v>
-      </c>
-      <c r="C8" s="3" t="s">
-        <v>144</v>
+      <c r="A8" s="3" t="s">
+        <v>177</v>
       </c>
     </row>
   </sheetData>
@@ -9937,97 +10070,67 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" s="3" t="s">
-        <v>192</v>
+        <v>178</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>193</v>
+        <v>179</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="14" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="3" t="s">
-        <v>194</v>
-      </c>
       <c r="B3" s="3" t="s">
-        <v>134</v>
+        <v>139</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>129</v>
+        <v>140</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A4" s="3" t="s">
-        <v>195</v>
-      </c>
       <c r="B4" s="3" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>129</v>
+        <v>138</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A5" s="3" t="s">
-        <v>196</v>
-      </c>
-      <c r="B5" s="3" t="s">
-        <v>140</v>
-      </c>
-      <c r="C5" s="3" t="s">
-        <v>129</v>
-      </c>
+        <v>180</v>
+      </c>
+      <c r="B5" s="3"/>
+      <c r="C5" s="3"/>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A6" s="3" t="s">
-        <v>197</v>
-      </c>
-      <c r="B6" s="3" t="s">
-        <v>141</v>
-      </c>
-      <c r="C6" s="3" t="s">
-        <v>129</v>
-      </c>
+        <v>181</v>
+      </c>
+      <c r="B6" s="3"/>
+      <c r="C6" s="3"/>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A7" s="3" t="s">
-        <v>198</v>
-      </c>
-      <c r="B7" s="3" t="s">
-        <v>142</v>
-      </c>
-      <c r="C7" s="3" t="s">
-        <v>129</v>
-      </c>
+        <v>182</v>
+      </c>
+      <c r="B7" s="3"/>
+      <c r="C7" s="3"/>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A8" s="3" t="s">
-        <v>199</v>
-      </c>
-      <c r="B8" s="3" t="s">
-        <v>160</v>
-      </c>
-      <c r="C8" s="3" t="s">
-        <v>129</v>
-      </c>
+        <v>183</v>
+      </c>
+      <c r="B8" s="3"/>
+      <c r="C8" s="3"/>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A9" s="3"/>
-      <c r="B9" s="3" t="s">
-        <v>145</v>
-      </c>
-      <c r="C9" s="3" t="s">
-        <v>146</v>
+      <c r="A9" s="3" t="s">
+        <v>184</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A10" s="3"/>
-      <c r="B10" s="3" t="s">
-        <v>143</v>
-      </c>
-      <c r="C10" s="3" t="s">
-        <v>144</v>
+      <c r="A10" s="3" t="s">
+        <v>185</v>
       </c>
     </row>
   </sheetData>
@@ -10059,97 +10162,67 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" s="3" t="s">
-        <v>200</v>
+        <v>186</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>201</v>
+        <v>187</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="14" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="3" t="s">
-        <v>202</v>
-      </c>
       <c r="B3" s="3" t="s">
-        <v>134</v>
+        <v>139</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>129</v>
+        <v>140</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A4" s="3" t="s">
-        <v>203</v>
-      </c>
       <c r="B4" s="3" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>129</v>
+        <v>138</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A5" s="3" t="s">
-        <v>204</v>
-      </c>
-      <c r="B5" s="3" t="s">
-        <v>140</v>
-      </c>
-      <c r="C5" s="3" t="s">
-        <v>129</v>
-      </c>
+        <v>188</v>
+      </c>
+      <c r="B5" s="3"/>
+      <c r="C5" s="3"/>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A6" s="3" t="s">
-        <v>205</v>
-      </c>
-      <c r="B6" s="3" t="s">
-        <v>141</v>
-      </c>
-      <c r="C6" s="3" t="s">
-        <v>129</v>
-      </c>
+        <v>189</v>
+      </c>
+      <c r="B6" s="3"/>
+      <c r="C6" s="3"/>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A7" s="3" t="s">
-        <v>206</v>
-      </c>
-      <c r="B7" s="3" t="s">
-        <v>142</v>
-      </c>
-      <c r="C7" s="3" t="s">
-        <v>129</v>
-      </c>
+        <v>190</v>
+      </c>
+      <c r="B7" s="3"/>
+      <c r="C7" s="3"/>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A8" s="3" t="s">
-        <v>207</v>
-      </c>
-      <c r="B8" s="3" t="s">
-        <v>160</v>
-      </c>
-      <c r="C8" s="3" t="s">
-        <v>129</v>
-      </c>
+        <v>191</v>
+      </c>
+      <c r="B8" s="3"/>
+      <c r="C8" s="3"/>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A9" s="3"/>
-      <c r="B9" s="3" t="s">
-        <v>145</v>
-      </c>
-      <c r="C9" s="3" t="s">
-        <v>146</v>
+      <c r="A9" s="3" t="s">
+        <v>192</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A10" s="3"/>
-      <c r="B10" s="3" t="s">
-        <v>143</v>
-      </c>
-      <c r="C10" s="3" t="s">
-        <v>144</v>
+      <c r="A10" s="3" t="s">
+        <v>193</v>
       </c>
     </row>
   </sheetData>
@@ -10180,130 +10253,88 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" s="3" t="s">
-        <v>208</v>
+        <v>194</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>209</v>
+        <v>195</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="14" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="3" t="s">
-        <v>210</v>
-      </c>
       <c r="B3" s="3" t="s">
-        <v>134</v>
+        <v>139</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>129</v>
+        <v>140</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A4" s="3" t="s">
-        <v>211</v>
-      </c>
       <c r="B4" s="3" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>129</v>
+        <v>138</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A5" s="3" t="s">
-        <v>212</v>
-      </c>
-      <c r="B5" s="3" t="s">
-        <v>140</v>
-      </c>
-      <c r="C5" s="3" t="s">
-        <v>129</v>
-      </c>
+        <v>196</v>
+      </c>
+      <c r="B5" s="3"/>
+      <c r="C5" s="3"/>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A6" s="3" t="s">
-        <v>213</v>
-      </c>
-      <c r="B6" s="3" t="s">
-        <v>141</v>
-      </c>
-      <c r="C6" s="3" t="s">
-        <v>129</v>
-      </c>
+        <v>197</v>
+      </c>
+      <c r="B6" s="3"/>
+      <c r="C6" s="3"/>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A7" s="3" t="s">
-        <v>214</v>
-      </c>
-      <c r="B7" s="3" t="s">
-        <v>142</v>
-      </c>
-      <c r="C7" s="3" t="s">
-        <v>129</v>
-      </c>
+        <v>198</v>
+      </c>
+      <c r="B7" s="3"/>
+      <c r="C7" s="3"/>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A8" s="3" t="s">
-        <v>215</v>
-      </c>
-      <c r="B8" s="3" t="s">
-        <v>160</v>
-      </c>
-      <c r="C8" s="3" t="s">
-        <v>129</v>
-      </c>
+        <v>199</v>
+      </c>
+      <c r="B8" s="3"/>
+      <c r="C8" s="3"/>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A9" s="3" t="s">
-        <v>216</v>
-      </c>
-      <c r="B9" s="3" t="s">
-        <v>177</v>
-      </c>
-      <c r="C9" s="3" t="s">
-        <v>129</v>
-      </c>
+        <v>200</v>
+      </c>
+      <c r="B9" s="3"/>
+      <c r="C9" s="3"/>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A10" s="3" t="s">
-        <v>217</v>
-      </c>
-      <c r="B10" s="3" t="s">
-        <v>184</v>
-      </c>
-      <c r="C10" s="3" t="s">
-        <v>129</v>
-      </c>
+        <v>201</v>
+      </c>
+      <c r="B10" s="3"/>
+      <c r="C10" s="3"/>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A11" s="3" t="s">
-        <v>218</v>
-      </c>
-      <c r="B11" s="3" t="s">
-        <v>219</v>
-      </c>
-      <c r="C11" s="3" t="s">
-        <v>129</v>
-      </c>
+        <v>202</v>
+      </c>
+      <c r="B11" s="3"/>
+      <c r="C11" s="3"/>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A12" s="3"/>
-      <c r="B12" s="3" t="s">
-        <v>145</v>
-      </c>
-      <c r="C12" s="3" t="s">
-        <v>146</v>
+      <c r="A12" s="3" t="s">
+        <v>203</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A13" s="3"/>
-      <c r="B13" s="3" t="s">
-        <v>143</v>
-      </c>
-      <c r="C13" s="3" t="s">
-        <v>144</v>
+      <c r="A13" s="3" t="s">
+        <v>204</v>
       </c>
     </row>
   </sheetData>
@@ -10334,108 +10365,74 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" s="3" t="s">
-        <v>220</v>
+        <v>205</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>221</v>
+        <v>206</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="14" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="3" t="s">
-        <v>222</v>
-      </c>
       <c r="B3" s="3" t="s">
-        <v>134</v>
+        <v>139</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>129</v>
+        <v>140</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A4" s="3" t="s">
-        <v>223</v>
-      </c>
       <c r="B4" s="3" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>129</v>
+        <v>138</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A5" s="3" t="s">
-        <v>224</v>
-      </c>
-      <c r="B5" s="3" t="s">
-        <v>140</v>
-      </c>
-      <c r="C5" s="3" t="s">
-        <v>129</v>
-      </c>
+        <v>207</v>
+      </c>
+      <c r="B5" s="3"/>
+      <c r="C5" s="3"/>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A6" s="3" t="s">
-        <v>225</v>
-      </c>
-      <c r="B6" s="3" t="s">
-        <v>141</v>
-      </c>
-      <c r="C6" s="3" t="s">
-        <v>129</v>
-      </c>
+        <v>208</v>
+      </c>
+      <c r="B6" s="3"/>
+      <c r="C6" s="3"/>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A7" s="3" t="s">
-        <v>226</v>
-      </c>
-      <c r="B7" s="3" t="s">
-        <v>142</v>
-      </c>
-      <c r="C7" s="3" t="s">
-        <v>129</v>
-      </c>
+        <v>209</v>
+      </c>
+      <c r="B7" s="3"/>
+      <c r="C7" s="3"/>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A8" s="3" t="s">
-        <v>227</v>
-      </c>
-      <c r="B8" s="3" t="s">
-        <v>160</v>
-      </c>
-      <c r="C8" s="3" t="s">
-        <v>129</v>
-      </c>
+        <v>210</v>
+      </c>
+      <c r="B8" s="3"/>
+      <c r="C8" s="3"/>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A9" s="3" t="s">
-        <v>228</v>
-      </c>
-      <c r="B9" s="3" t="s">
-        <v>177</v>
-      </c>
-      <c r="C9" s="3" t="s">
-        <v>129</v>
-      </c>
+        <v>211</v>
+      </c>
+      <c r="B9" s="3"/>
+      <c r="C9" s="3"/>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A10" s="3"/>
-      <c r="B10" s="3" t="s">
-        <v>145</v>
-      </c>
-      <c r="C10" s="3" t="s">
-        <v>146</v>
+      <c r="A10" s="3" t="s">
+        <v>212</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A11" s="3"/>
-      <c r="B11" s="3" t="s">
-        <v>143</v>
-      </c>
-      <c r="C11" s="3" t="s">
-        <v>144</v>
+      <c r="A11" s="3" t="s">
+        <v>213</v>
       </c>
     </row>
   </sheetData>
@@ -10466,130 +10463,88 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" s="3" t="s">
-        <v>229</v>
+        <v>214</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>230</v>
+        <v>215</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="14" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="3" t="s">
-        <v>231</v>
-      </c>
       <c r="B3" s="3" t="s">
-        <v>134</v>
+        <v>139</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>129</v>
+        <v>140</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A4" s="3" t="s">
-        <v>232</v>
-      </c>
       <c r="B4" s="3" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>129</v>
+        <v>138</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A5" s="3" t="s">
-        <v>233</v>
-      </c>
-      <c r="B5" s="3" t="s">
-        <v>140</v>
-      </c>
-      <c r="C5" s="3" t="s">
-        <v>129</v>
-      </c>
+        <v>216</v>
+      </c>
+      <c r="B5" s="3"/>
+      <c r="C5" s="3"/>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A6" s="3" t="s">
-        <v>234</v>
-      </c>
-      <c r="B6" s="3" t="s">
-        <v>141</v>
-      </c>
-      <c r="C6" s="3" t="s">
-        <v>129</v>
-      </c>
+        <v>217</v>
+      </c>
+      <c r="B6" s="3"/>
+      <c r="C6" s="3"/>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A7" s="3" t="s">
-        <v>235</v>
-      </c>
-      <c r="B7" s="3" t="s">
-        <v>142</v>
-      </c>
-      <c r="C7" s="3" t="s">
-        <v>129</v>
-      </c>
+        <v>218</v>
+      </c>
+      <c r="B7" s="3"/>
+      <c r="C7" s="3"/>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A8" s="3" t="s">
-        <v>236</v>
-      </c>
-      <c r="B8" s="3" t="s">
-        <v>160</v>
-      </c>
-      <c r="C8" s="3" t="s">
-        <v>129</v>
-      </c>
+        <v>219</v>
+      </c>
+      <c r="B8" s="3"/>
+      <c r="C8" s="3"/>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A9" s="3" t="s">
-        <v>237</v>
-      </c>
-      <c r="B9" s="3" t="s">
-        <v>177</v>
-      </c>
-      <c r="C9" s="3" t="s">
-        <v>129</v>
-      </c>
+        <v>220</v>
+      </c>
+      <c r="B9" s="3"/>
+      <c r="C9" s="3"/>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A10" s="3" t="s">
-        <v>238</v>
-      </c>
-      <c r="B10" s="3" t="s">
-        <v>184</v>
-      </c>
-      <c r="C10" s="3" t="s">
-        <v>129</v>
-      </c>
+        <v>221</v>
+      </c>
+      <c r="B10" s="3"/>
+      <c r="C10" s="3"/>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A11" s="3" t="s">
-        <v>239</v>
-      </c>
-      <c r="B11" s="3" t="s">
-        <v>219</v>
-      </c>
-      <c r="C11" s="3" t="s">
-        <v>183</v>
-      </c>
+        <v>222</v>
+      </c>
+      <c r="B11" s="3"/>
+      <c r="C11" s="3"/>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A12" s="3"/>
-      <c r="B12" s="3" t="s">
-        <v>145</v>
-      </c>
-      <c r="C12" s="3" t="s">
-        <v>146</v>
+      <c r="A12" s="3" t="s">
+        <v>223</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A13" s="3"/>
-      <c r="B13" s="3" t="s">
-        <v>143</v>
-      </c>
-      <c r="C13" s="3" t="s">
-        <v>144</v>
+      <c r="A13" s="3" t="s">
+        <v>224</v>
       </c>
     </row>
   </sheetData>
@@ -10632,36 +10587,36 @@
         <v>35</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>249</v>
+        <v>234</v>
       </c>
       <c r="H1" s="2" t="s">
-        <v>250</v>
+        <v>235</v>
       </c>
     </row>
     <row r="2" spans="1:229" s="4" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A2" s="3" t="s">
-        <v>244</v>
+        <v>229</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>243</v>
+        <v>228</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>240</v>
+        <v>225</v>
       </c>
       <c r="D2" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>241</v>
+        <v>226</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>242</v>
+        <v>227</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>251</v>
+        <v>236</v>
       </c>
       <c r="H2" s="3" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="I2"/>
       <c r="J2"/>
@@ -10887,106 +10842,106 @@
     </row>
     <row r="3" spans="1:229" x14ac:dyDescent="0.35">
       <c r="A3" s="3" t="s">
-        <v>245</v>
+        <v>230</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>247</v>
+        <v>232</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>248</v>
+        <v>233</v>
       </c>
       <c r="D3" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>241</v>
+        <v>226</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>242</v>
+        <v>227</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>252</v>
+        <v>237</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>253</v>
+        <v>238</v>
       </c>
     </row>
     <row r="4" spans="1:229" x14ac:dyDescent="0.35">
       <c r="A4" s="3" t="s">
-        <v>246</v>
+        <v>231</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>254</v>
+        <v>239</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>255</v>
+        <v>240</v>
       </c>
       <c r="D4" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E4" s="3" t="s">
+        <v>226</v>
+      </c>
+      <c r="F4" s="3" t="s">
+        <v>227</v>
+      </c>
+      <c r="G4" s="3" t="s">
         <v>241</v>
       </c>
-      <c r="F4" s="3" t="s">
+      <c r="H4" s="3" t="s">
         <v>242</v>
-      </c>
-      <c r="G4" s="3" t="s">
-        <v>256</v>
-      </c>
-      <c r="H4" s="3" t="s">
-        <v>257</v>
       </c>
     </row>
     <row r="5" spans="1:229" x14ac:dyDescent="0.35">
       <c r="A5" s="3" t="s">
-        <v>258</v>
+        <v>243</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>259</v>
+        <v>244</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>260</v>
+        <v>245</v>
       </c>
       <c r="D5" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>241</v>
+        <v>226</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>242</v>
+        <v>227</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>261</v>
+        <v>246</v>
       </c>
       <c r="H5" s="3" t="s">
-        <v>262</v>
+        <v>247</v>
       </c>
     </row>
     <row r="6" spans="1:229" x14ac:dyDescent="0.35">
       <c r="A6" s="3" t="s">
-        <v>263</v>
+        <v>248</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>264</v>
+        <v>249</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>265</v>
+        <v>250</v>
       </c>
       <c r="D6" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>241</v>
+        <v>226</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>242</v>
+        <v>227</v>
       </c>
       <c r="G6" s="3" t="s">
-        <v>266</v>
+        <v>251</v>
       </c>
       <c r="H6" s="3" t="s">
-        <v>267</v>
+        <v>252</v>
       </c>
     </row>
   </sheetData>
@@ -11030,36 +10985,36 @@
         <v>35</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>249</v>
+        <v>234</v>
       </c>
       <c r="H1" s="2" t="s">
-        <v>250</v>
+        <v>235</v>
       </c>
     </row>
     <row r="2" spans="1:229" s="4" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A2" s="3" t="s">
-        <v>268</v>
+        <v>253</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>269</v>
+        <v>254</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>270</v>
+        <v>255</v>
       </c>
       <c r="D2" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>241</v>
+        <v>226</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>242</v>
+        <v>227</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>251</v>
+        <v>236</v>
       </c>
       <c r="H2" s="3" t="s">
-        <v>149</v>
+        <v>143</v>
       </c>
       <c r="I2"/>
       <c r="J2"/>
@@ -11285,80 +11240,80 @@
     </row>
     <row r="3" spans="1:229" x14ac:dyDescent="0.35">
       <c r="A3" s="3" t="s">
-        <v>271</v>
+        <v>256</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>272</v>
+        <v>257</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>273</v>
+        <v>258</v>
       </c>
       <c r="D3" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>241</v>
+        <v>226</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>242</v>
+        <v>227</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>251</v>
+        <v>236</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>274</v>
+        <v>259</v>
       </c>
     </row>
     <row r="4" spans="1:229" x14ac:dyDescent="0.35">
       <c r="A4" s="3" t="s">
-        <v>275</v>
+        <v>260</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>276</v>
+        <v>261</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>277</v>
+        <v>262</v>
       </c>
       <c r="D4" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>241</v>
+        <v>226</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>242</v>
+        <v>227</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>251</v>
+        <v>236</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>278</v>
+        <v>263</v>
       </c>
     </row>
     <row r="5" spans="1:229" x14ac:dyDescent="0.35">
       <c r="A5" s="3" t="s">
-        <v>279</v>
+        <v>264</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>280</v>
+        <v>265</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>281</v>
+        <v>266</v>
       </c>
       <c r="D5" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>241</v>
+        <v>226</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>242</v>
+        <v>227</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>251</v>
+        <v>236</v>
       </c>
       <c r="H5" s="3" t="s">
-        <v>282</v>
+        <v>267</v>
       </c>
     </row>
   </sheetData>
@@ -11401,36 +11356,36 @@
         <v>35</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>249</v>
+        <v>234</v>
       </c>
       <c r="H1" s="2" t="s">
-        <v>250</v>
+        <v>235</v>
       </c>
     </row>
     <row r="2" spans="1:229" s="4" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A2" s="3" t="s">
-        <v>283</v>
+        <v>268</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>284</v>
+        <v>269</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>285</v>
+        <v>270</v>
       </c>
       <c r="D2" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>241</v>
+        <v>226</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>242</v>
+        <v>227</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>251</v>
+        <v>236</v>
       </c>
       <c r="H2" s="3" t="s">
-        <v>158</v>
+        <v>152</v>
       </c>
       <c r="I2"/>
       <c r="J2"/>
@@ -11656,132 +11611,132 @@
     </row>
     <row r="3" spans="1:229" x14ac:dyDescent="0.35">
       <c r="A3" s="3" t="s">
-        <v>286</v>
+        <v>271</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>287</v>
+        <v>272</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>288</v>
+        <v>273</v>
       </c>
       <c r="D3" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>241</v>
+        <v>226</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>242</v>
+        <v>227</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>251</v>
+        <v>236</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>289</v>
+        <v>274</v>
       </c>
     </row>
     <row r="4" spans="1:229" x14ac:dyDescent="0.35">
       <c r="A4" s="3" t="s">
-        <v>290</v>
+        <v>275</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>292</v>
+        <v>277</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>291</v>
+        <v>276</v>
       </c>
       <c r="D4" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>241</v>
+        <v>226</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>242</v>
+        <v>227</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>251</v>
+        <v>236</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>293</v>
+        <v>278</v>
       </c>
     </row>
     <row r="5" spans="1:229" x14ac:dyDescent="0.35">
       <c r="A5" s="8" t="s">
-        <v>294</v>
+        <v>279</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>295</v>
+        <v>280</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>296</v>
+        <v>281</v>
       </c>
       <c r="D5" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>241</v>
+        <v>226</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>242</v>
+        <v>227</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>251</v>
+        <v>236</v>
       </c>
       <c r="H5" s="3" t="s">
-        <v>297</v>
+        <v>282</v>
       </c>
     </row>
     <row r="6" spans="1:229" x14ac:dyDescent="0.35">
       <c r="A6" s="3" t="s">
-        <v>298</v>
+        <v>283</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>299</v>
+        <v>284</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>300</v>
+        <v>285</v>
       </c>
       <c r="D6" s="7" t="s">
         <v>0</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>241</v>
+        <v>226</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>242</v>
+        <v>227</v>
       </c>
       <c r="G6" s="3" t="s">
-        <v>251</v>
+        <v>236</v>
       </c>
       <c r="H6" s="3" t="s">
-        <v>301</v>
+        <v>286</v>
       </c>
     </row>
     <row r="7" spans="1:229" x14ac:dyDescent="0.35">
       <c r="A7" s="3" t="s">
-        <v>302</v>
+        <v>287</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>304</v>
+        <v>289</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>303</v>
+        <v>288</v>
       </c>
       <c r="D7" s="7" t="s">
         <v>0</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>241</v>
+        <v>226</v>
       </c>
       <c r="F7" s="3" t="s">
-        <v>242</v>
+        <v>227</v>
       </c>
       <c r="G7" s="3" t="s">
-        <v>251</v>
+        <v>236</v>
       </c>
       <c r="H7" s="3" t="s">
-        <v>305</v>
+        <v>290</v>
       </c>
     </row>
   </sheetData>
@@ -11825,36 +11780,36 @@
         <v>35</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>249</v>
+        <v>234</v>
       </c>
       <c r="H1" s="2" t="s">
-        <v>250</v>
+        <v>235</v>
       </c>
     </row>
     <row r="2" spans="1:229" s="4" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A2" s="3" t="s">
-        <v>306</v>
+        <v>291</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>307</v>
+        <v>292</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>308</v>
+        <v>293</v>
       </c>
       <c r="D2" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>241</v>
+        <v>226</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>242</v>
+        <v>227</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>251</v>
+        <v>236</v>
       </c>
       <c r="H2" s="3" t="s">
-        <v>164</v>
+        <v>157</v>
       </c>
       <c r="I2"/>
       <c r="J2"/>
@@ -12080,106 +12035,106 @@
     </row>
     <row r="3" spans="1:229" x14ac:dyDescent="0.35">
       <c r="A3" s="3" t="s">
-        <v>309</v>
+        <v>294</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>310</v>
+        <v>295</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>311</v>
+        <v>296</v>
       </c>
       <c r="D3" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>241</v>
+        <v>226</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>242</v>
+        <v>227</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>251</v>
+        <v>236</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>312</v>
+        <v>297</v>
       </c>
     </row>
     <row r="4" spans="1:229" x14ac:dyDescent="0.35">
       <c r="A4" s="3" t="s">
-        <v>313</v>
+        <v>298</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>314</v>
+        <v>299</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>315</v>
+        <v>300</v>
       </c>
       <c r="D4" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>241</v>
+        <v>226</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>242</v>
+        <v>227</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>251</v>
+        <v>236</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>316</v>
+        <v>301</v>
       </c>
     </row>
     <row r="5" spans="1:229" x14ac:dyDescent="0.35">
       <c r="A5" s="8" t="s">
-        <v>317</v>
+        <v>302</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>318</v>
+        <v>303</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>319</v>
+        <v>304</v>
       </c>
       <c r="D5" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>241</v>
+        <v>226</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>242</v>
+        <v>227</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>251</v>
+        <v>236</v>
       </c>
       <c r="H5" s="3" t="s">
-        <v>320</v>
+        <v>305</v>
       </c>
     </row>
     <row r="6" spans="1:229" x14ac:dyDescent="0.35">
       <c r="A6" s="3" t="s">
-        <v>321</v>
+        <v>306</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>322</v>
+        <v>307</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>323</v>
+        <v>308</v>
       </c>
       <c r="D6" s="7" t="s">
         <v>0</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>241</v>
+        <v>226</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>242</v>
+        <v>227</v>
       </c>
       <c r="G6" s="3" t="s">
-        <v>251</v>
+        <v>236</v>
       </c>
       <c r="H6" s="3" t="s">
-        <v>324</v>
+        <v>309</v>
       </c>
     </row>
   </sheetData>
@@ -12440,36 +12395,36 @@
         <v>35</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>249</v>
+        <v>234</v>
       </c>
       <c r="H1" s="2" t="s">
-        <v>250</v>
+        <v>235</v>
       </c>
     </row>
     <row r="2" spans="1:229" s="4" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A2" s="3" t="s">
-        <v>325</v>
+        <v>310</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>326</v>
+        <v>311</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>327</v>
+        <v>312</v>
       </c>
       <c r="D2" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>241</v>
+        <v>226</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>242</v>
+        <v>227</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>251</v>
+        <v>236</v>
       </c>
       <c r="H2" s="3" t="s">
-        <v>188</v>
+        <v>174</v>
       </c>
       <c r="I2"/>
       <c r="J2"/>
@@ -12695,80 +12650,80 @@
     </row>
     <row r="3" spans="1:229" x14ac:dyDescent="0.35">
       <c r="A3" s="3" t="s">
-        <v>328</v>
+        <v>313</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>329</v>
+        <v>314</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>330</v>
+        <v>315</v>
       </c>
       <c r="D3" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>241</v>
+        <v>226</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>242</v>
+        <v>227</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>251</v>
+        <v>236</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>331</v>
+        <v>316</v>
       </c>
     </row>
     <row r="4" spans="1:229" x14ac:dyDescent="0.35">
       <c r="A4" s="3" t="s">
-        <v>332</v>
+        <v>317</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>333</v>
+        <v>318</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>334</v>
+        <v>319</v>
       </c>
       <c r="D4" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>241</v>
+        <v>226</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>242</v>
+        <v>227</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>251</v>
+        <v>236</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>335</v>
+        <v>320</v>
       </c>
     </row>
     <row r="5" spans="1:229" x14ac:dyDescent="0.35">
       <c r="A5" s="3" t="s">
-        <v>336</v>
+        <v>321</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>337</v>
+        <v>322</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>338</v>
+        <v>323</v>
       </c>
       <c r="D5" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>241</v>
+        <v>226</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>242</v>
+        <v>227</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>251</v>
+        <v>236</v>
       </c>
       <c r="H5" s="3" t="s">
-        <v>339</v>
+        <v>324</v>
       </c>
     </row>
   </sheetData>
@@ -12811,36 +12766,36 @@
         <v>35</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>249</v>
+        <v>234</v>
       </c>
       <c r="H1" s="2" t="s">
-        <v>250</v>
+        <v>235</v>
       </c>
     </row>
     <row r="2" spans="1:229" s="4" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A2" s="3" t="s">
-        <v>340</v>
+        <v>325</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>341</v>
+        <v>326</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>342</v>
+        <v>327</v>
       </c>
       <c r="D2" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>241</v>
+        <v>226</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>242</v>
+        <v>227</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>251</v>
+        <v>236</v>
       </c>
       <c r="H2" s="3" t="s">
-        <v>194</v>
+        <v>180</v>
       </c>
       <c r="I2"/>
       <c r="J2"/>
@@ -13066,132 +13021,132 @@
     </row>
     <row r="3" spans="1:229" x14ac:dyDescent="0.35">
       <c r="A3" s="3" t="s">
-        <v>343</v>
+        <v>328</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>344</v>
+        <v>329</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>345</v>
+        <v>330</v>
       </c>
       <c r="D3" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>241</v>
+        <v>226</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>242</v>
+        <v>227</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>251</v>
+        <v>236</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>346</v>
+        <v>331</v>
       </c>
     </row>
     <row r="4" spans="1:229" x14ac:dyDescent="0.35">
       <c r="A4" s="3" t="s">
-        <v>347</v>
+        <v>332</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>348</v>
+        <v>333</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>349</v>
+        <v>334</v>
       </c>
       <c r="D4" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>241</v>
+        <v>226</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>242</v>
+        <v>227</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>251</v>
+        <v>236</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>350</v>
+        <v>335</v>
       </c>
     </row>
     <row r="5" spans="1:229" x14ac:dyDescent="0.35">
       <c r="A5" s="8" t="s">
-        <v>351</v>
+        <v>336</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>352</v>
+        <v>337</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>353</v>
+        <v>338</v>
       </c>
       <c r="D5" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>241</v>
+        <v>226</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>242</v>
+        <v>227</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>251</v>
+        <v>236</v>
       </c>
       <c r="H5" s="3" t="s">
-        <v>354</v>
+        <v>339</v>
       </c>
     </row>
     <row r="6" spans="1:229" x14ac:dyDescent="0.35">
       <c r="A6" s="3" t="s">
-        <v>355</v>
+        <v>340</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>357</v>
+        <v>342</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>356</v>
+        <v>341</v>
       </c>
       <c r="D6" s="7" t="s">
         <v>0</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>241</v>
+        <v>226</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>242</v>
+        <v>227</v>
       </c>
       <c r="G6" s="3" t="s">
-        <v>251</v>
+        <v>236</v>
       </c>
       <c r="H6" s="3" t="s">
-        <v>358</v>
+        <v>343</v>
       </c>
     </row>
     <row r="7" spans="1:229" x14ac:dyDescent="0.35">
       <c r="A7" s="3" t="s">
-        <v>359</v>
+        <v>344</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>360</v>
+        <v>345</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>361</v>
+        <v>346</v>
       </c>
       <c r="D7" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>241</v>
+        <v>226</v>
       </c>
       <c r="F7" s="3" t="s">
-        <v>242</v>
+        <v>227</v>
       </c>
       <c r="G7" s="3" t="s">
-        <v>251</v>
+        <v>236</v>
       </c>
       <c r="H7" s="3" t="s">
-        <v>362</v>
+        <v>347</v>
       </c>
     </row>
   </sheetData>
@@ -13234,36 +13189,36 @@
         <v>35</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>249</v>
+        <v>234</v>
       </c>
       <c r="H1" s="2" t="s">
-        <v>250</v>
+        <v>235</v>
       </c>
     </row>
     <row r="2" spans="1:229" s="4" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A2" s="3" t="s">
-        <v>363</v>
+        <v>348</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>364</v>
+        <v>349</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>365</v>
+        <v>350</v>
       </c>
       <c r="D2" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>241</v>
+        <v>226</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>242</v>
+        <v>227</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>251</v>
+        <v>236</v>
       </c>
       <c r="H2" s="3" t="s">
-        <v>202</v>
+        <v>188</v>
       </c>
       <c r="I2"/>
       <c r="J2"/>
@@ -13489,135 +13444,1087 @@
     </row>
     <row r="3" spans="1:229" x14ac:dyDescent="0.35">
       <c r="A3" s="3" t="s">
-        <v>366</v>
+        <v>351</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>367</v>
+        <v>352</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>368</v>
+        <v>353</v>
       </c>
       <c r="D3" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>241</v>
+        <v>226</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>242</v>
+        <v>227</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>251</v>
+        <v>236</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>369</v>
+        <v>354</v>
       </c>
     </row>
     <row r="4" spans="1:229" x14ac:dyDescent="0.35">
       <c r="A4" s="3" t="s">
-        <v>370</v>
+        <v>355</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>372</v>
+        <v>357</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>371</v>
+        <v>356</v>
       </c>
       <c r="D4" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>241</v>
+        <v>226</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>242</v>
+        <v>227</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>251</v>
+        <v>236</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>373</v>
+        <v>358</v>
       </c>
     </row>
     <row r="5" spans="1:229" x14ac:dyDescent="0.35">
       <c r="A5" s="8" t="s">
-        <v>374</v>
+        <v>359</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>375</v>
+        <v>360</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>376</v>
+        <v>361</v>
       </c>
       <c r="D5" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>241</v>
+        <v>226</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>242</v>
+        <v>227</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>251</v>
+        <v>236</v>
       </c>
       <c r="H5" s="3" t="s">
-        <v>377</v>
+        <v>362</v>
       </c>
     </row>
     <row r="6" spans="1:229" x14ac:dyDescent="0.35">
       <c r="A6" s="3" t="s">
-        <v>378</v>
+        <v>363</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>380</v>
+        <v>365</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>379</v>
+        <v>364</v>
       </c>
       <c r="D6" s="7" t="s">
         <v>0</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>241</v>
+        <v>226</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>242</v>
+        <v>227</v>
       </c>
       <c r="G6" s="3" t="s">
-        <v>251</v>
+        <v>236</v>
       </c>
       <c r="H6" s="3" t="s">
-        <v>381</v>
+        <v>366</v>
       </c>
     </row>
     <row r="7" spans="1:229" x14ac:dyDescent="0.35">
       <c r="A7" s="3" t="s">
-        <v>382</v>
+        <v>367</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>383</v>
+        <v>368</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>384</v>
+        <v>369</v>
       </c>
       <c r="D7" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>241</v>
+        <v>226</v>
       </c>
       <c r="F7" s="3" t="s">
-        <v>242</v>
+        <v>227</v>
       </c>
       <c r="G7" s="3" t="s">
-        <v>251</v>
+        <v>236</v>
       </c>
       <c r="H7" s="3" t="s">
+        <v>370</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{20DD36AA-F163-4AAB-BD30-4AE6290CCAE7}">
+  <dimension ref="A1:HU10"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="50.90625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="52.26953125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="42.453125" customWidth="1"/>
+    <col min="4" max="4" width="33.36328125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="33.08984375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="17.08984375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="40.81640625" customWidth="1"/>
+    <col min="8" max="8" width="62.54296875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:229" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>234</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="2" spans="1:229" s="4" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A2" s="3" t="s">
+        <v>380</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>381</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>382</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>226</v>
+      </c>
+      <c r="F2" s="3" t="s">
+        <v>227</v>
+      </c>
+      <c r="G2" s="3" t="s">
+        <v>236</v>
+      </c>
+      <c r="H2" s="3" t="s">
+        <v>196</v>
+      </c>
+      <c r="I2"/>
+      <c r="J2"/>
+      <c r="K2"/>
+      <c r="L2"/>
+      <c r="M2"/>
+      <c r="N2"/>
+      <c r="O2"/>
+      <c r="P2"/>
+      <c r="Q2"/>
+      <c r="R2"/>
+      <c r="S2"/>
+      <c r="T2"/>
+      <c r="U2"/>
+      <c r="V2"/>
+      <c r="W2"/>
+      <c r="X2"/>
+      <c r="Y2"/>
+      <c r="Z2"/>
+      <c r="AA2"/>
+      <c r="AB2"/>
+      <c r="AC2"/>
+      <c r="AD2"/>
+      <c r="AE2"/>
+      <c r="AF2"/>
+      <c r="AG2"/>
+      <c r="AH2"/>
+      <c r="AI2"/>
+      <c r="AJ2"/>
+      <c r="AK2"/>
+      <c r="AL2"/>
+      <c r="AM2"/>
+      <c r="AN2"/>
+      <c r="AO2"/>
+      <c r="AP2"/>
+      <c r="AQ2"/>
+      <c r="AR2"/>
+      <c r="AS2"/>
+      <c r="AT2"/>
+      <c r="AU2"/>
+      <c r="AV2"/>
+      <c r="AW2"/>
+      <c r="AX2"/>
+      <c r="AY2"/>
+      <c r="AZ2"/>
+      <c r="BA2"/>
+      <c r="BB2"/>
+      <c r="BC2"/>
+      <c r="BD2"/>
+      <c r="BE2"/>
+      <c r="BF2"/>
+      <c r="BG2"/>
+      <c r="BH2"/>
+      <c r="BI2"/>
+      <c r="BJ2"/>
+      <c r="BK2"/>
+      <c r="BL2"/>
+      <c r="BM2"/>
+      <c r="BN2"/>
+      <c r="BO2"/>
+      <c r="BP2"/>
+      <c r="BQ2"/>
+      <c r="BR2"/>
+      <c r="BS2"/>
+      <c r="BT2"/>
+      <c r="BU2"/>
+      <c r="BV2"/>
+      <c r="BW2"/>
+      <c r="BX2"/>
+      <c r="BY2"/>
+      <c r="BZ2"/>
+      <c r="CA2"/>
+      <c r="CB2"/>
+      <c r="CC2"/>
+      <c r="CD2"/>
+      <c r="CE2"/>
+      <c r="CF2"/>
+      <c r="CG2"/>
+      <c r="CH2"/>
+      <c r="CI2"/>
+      <c r="CJ2"/>
+      <c r="CK2"/>
+      <c r="CL2"/>
+      <c r="CM2"/>
+      <c r="CN2"/>
+      <c r="CO2"/>
+      <c r="CP2"/>
+      <c r="CQ2"/>
+      <c r="CR2"/>
+      <c r="CS2"/>
+      <c r="CT2"/>
+      <c r="CU2"/>
+      <c r="CV2"/>
+      <c r="CW2"/>
+      <c r="CX2"/>
+      <c r="CY2"/>
+      <c r="CZ2"/>
+      <c r="DA2"/>
+      <c r="DB2"/>
+      <c r="DC2"/>
+      <c r="DD2"/>
+      <c r="DE2"/>
+      <c r="DF2"/>
+      <c r="DG2"/>
+      <c r="DH2"/>
+      <c r="DI2"/>
+      <c r="DJ2"/>
+      <c r="DK2"/>
+      <c r="DL2"/>
+      <c r="DM2"/>
+      <c r="DN2"/>
+      <c r="DO2"/>
+      <c r="DP2"/>
+      <c r="DQ2"/>
+      <c r="DR2"/>
+      <c r="DS2"/>
+      <c r="DT2"/>
+      <c r="DU2"/>
+      <c r="DV2"/>
+      <c r="DW2"/>
+      <c r="DX2"/>
+      <c r="DY2"/>
+      <c r="DZ2"/>
+      <c r="EA2"/>
+      <c r="EB2"/>
+      <c r="EC2"/>
+      <c r="ED2"/>
+      <c r="EE2"/>
+      <c r="EF2"/>
+      <c r="EG2"/>
+      <c r="EH2"/>
+      <c r="EI2"/>
+      <c r="EJ2"/>
+      <c r="EK2"/>
+      <c r="EL2"/>
+      <c r="EM2"/>
+      <c r="EN2"/>
+      <c r="EO2"/>
+      <c r="EP2"/>
+      <c r="EQ2"/>
+      <c r="ER2"/>
+      <c r="ES2"/>
+      <c r="ET2"/>
+      <c r="EU2"/>
+      <c r="EV2"/>
+      <c r="EW2"/>
+      <c r="EX2"/>
+      <c r="EY2"/>
+      <c r="EZ2"/>
+      <c r="FA2"/>
+      <c r="FB2"/>
+      <c r="FC2"/>
+      <c r="FD2"/>
+      <c r="FE2"/>
+      <c r="FF2"/>
+      <c r="FG2"/>
+      <c r="FH2"/>
+      <c r="FI2"/>
+      <c r="FJ2"/>
+      <c r="FK2"/>
+      <c r="FL2"/>
+      <c r="FM2"/>
+      <c r="FN2"/>
+      <c r="FO2"/>
+      <c r="FP2"/>
+      <c r="FQ2"/>
+      <c r="FR2"/>
+      <c r="FS2"/>
+      <c r="FT2"/>
+      <c r="FU2"/>
+      <c r="FV2"/>
+      <c r="FW2"/>
+      <c r="FX2"/>
+      <c r="FY2"/>
+      <c r="FZ2"/>
+      <c r="GA2"/>
+      <c r="GB2"/>
+      <c r="GC2"/>
+      <c r="GD2"/>
+      <c r="GE2"/>
+      <c r="GF2"/>
+      <c r="GG2"/>
+      <c r="GH2"/>
+      <c r="GI2"/>
+      <c r="GJ2"/>
+      <c r="GK2"/>
+      <c r="GL2"/>
+      <c r="GM2"/>
+      <c r="GN2"/>
+      <c r="GO2"/>
+      <c r="GP2"/>
+      <c r="GQ2"/>
+      <c r="GR2"/>
+      <c r="GS2"/>
+      <c r="GT2"/>
+      <c r="GU2"/>
+      <c r="GV2"/>
+      <c r="GW2"/>
+      <c r="GX2"/>
+      <c r="GY2"/>
+      <c r="GZ2"/>
+      <c r="HA2"/>
+      <c r="HB2"/>
+      <c r="HC2"/>
+      <c r="HD2"/>
+      <c r="HE2"/>
+      <c r="HF2"/>
+      <c r="HG2"/>
+      <c r="HH2"/>
+      <c r="HI2"/>
+      <c r="HJ2"/>
+      <c r="HK2"/>
+      <c r="HL2"/>
+      <c r="HM2"/>
+      <c r="HN2"/>
+      <c r="HO2"/>
+      <c r="HP2"/>
+      <c r="HQ2"/>
+      <c r="HR2"/>
+      <c r="HS2"/>
+      <c r="HT2"/>
+      <c r="HU2"/>
+    </row>
+    <row r="3" spans="1:229" x14ac:dyDescent="0.35">
+      <c r="A3" s="3" t="s">
+        <v>383</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>384</v>
+      </c>
+      <c r="C3" s="3" t="s">
         <v>385</v>
       </c>
+      <c r="D3" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>226</v>
+      </c>
+      <c r="F3" s="3" t="s">
+        <v>227</v>
+      </c>
+      <c r="G3" s="3" t="s">
+        <v>236</v>
+      </c>
+      <c r="H3" s="3" t="s">
+        <v>386</v>
+      </c>
+    </row>
+    <row r="4" spans="1:229" x14ac:dyDescent="0.35">
+      <c r="A4" s="3" t="s">
+        <v>387</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>388</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>389</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>226</v>
+      </c>
+      <c r="F4" s="3" t="s">
+        <v>227</v>
+      </c>
+      <c r="G4" s="3" t="s">
+        <v>236</v>
+      </c>
+      <c r="H4" s="3" t="s">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="5" spans="1:229" x14ac:dyDescent="0.35">
+      <c r="A5" s="8" t="s">
+        <v>391</v>
+      </c>
+      <c r="B5" s="8" t="s">
+        <v>392</v>
+      </c>
+      <c r="C5" s="8" t="s">
+        <v>393</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>226</v>
+      </c>
+      <c r="F5" s="3" t="s">
+        <v>227</v>
+      </c>
+      <c r="G5" s="3" t="s">
+        <v>236</v>
+      </c>
+      <c r="H5" s="3" t="s">
+        <v>394</v>
+      </c>
+    </row>
+    <row r="6" spans="1:229" x14ac:dyDescent="0.35">
+      <c r="A6" s="3" t="s">
+        <v>395</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>396</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>397</v>
+      </c>
+      <c r="D6" s="7" t="s">
+        <v>0</v>
+      </c>
+      <c r="E6" s="3" t="s">
+        <v>226</v>
+      </c>
+      <c r="F6" s="3" t="s">
+        <v>227</v>
+      </c>
+      <c r="G6" s="3" t="s">
+        <v>236</v>
+      </c>
+      <c r="H6" s="3" t="s">
+        <v>398</v>
+      </c>
+    </row>
+    <row r="7" spans="1:229" x14ac:dyDescent="0.35">
+      <c r="A7" s="3" t="s">
+        <v>399</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>400</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>401</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="E7" s="3" t="s">
+        <v>226</v>
+      </c>
+      <c r="F7" s="3" t="s">
+        <v>227</v>
+      </c>
+      <c r="G7" s="3" t="s">
+        <v>236</v>
+      </c>
+      <c r="H7" s="3" t="s">
+        <v>402</v>
+      </c>
+    </row>
+    <row r="8" spans="1:229" x14ac:dyDescent="0.35">
+      <c r="A8" s="3" t="s">
+        <v>403</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>404</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>405</v>
+      </c>
+      <c r="D8" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="E8" s="3" t="s">
+        <v>226</v>
+      </c>
+      <c r="F8" s="3" t="s">
+        <v>227</v>
+      </c>
+      <c r="G8" s="3" t="s">
+        <v>236</v>
+      </c>
+      <c r="H8" s="3" t="s">
+        <v>406</v>
+      </c>
+    </row>
+    <row r="9" spans="1:229" x14ac:dyDescent="0.35">
+      <c r="A9" s="3" t="s">
+        <v>407</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>408</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>409</v>
+      </c>
+      <c r="D9" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="E9" s="3" t="s">
+        <v>226</v>
+      </c>
+      <c r="F9" s="3" t="s">
+        <v>227</v>
+      </c>
+      <c r="G9" s="3" t="s">
+        <v>236</v>
+      </c>
+      <c r="H9" s="3" t="s">
+        <v>410</v>
+      </c>
+    </row>
+    <row r="10" spans="1:229" x14ac:dyDescent="0.35">
+      <c r="A10" s="3" t="s">
+        <v>411</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>412</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>413</v>
+      </c>
+      <c r="D10" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="E10" s="3" t="s">
+        <v>226</v>
+      </c>
+      <c r="F10" s="3" t="s">
+        <v>227</v>
+      </c>
+      <c r="G10" s="3" t="s">
+        <v>236</v>
+      </c>
+      <c r="H10" s="3" t="s">
+        <v>414</v>
+      </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C6EE6111-FDB3-4B43-8820-BBF68AAFCD6D}">
+  <dimension ref="A1:HU8"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="50.90625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="52.26953125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="42.453125" customWidth="1"/>
+    <col min="4" max="4" width="33.36328125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="33.08984375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="17.08984375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="40.81640625" customWidth="1"/>
+    <col min="8" max="8" width="62.54296875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:229" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>234</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="2" spans="1:229" s="4" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A2" s="3" t="s">
+        <v>415</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>416</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>417</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>226</v>
+      </c>
+      <c r="F2" s="3" t="s">
+        <v>227</v>
+      </c>
+      <c r="G2" s="3" t="s">
+        <v>236</v>
+      </c>
+      <c r="H2" s="3" t="s">
+        <v>207</v>
+      </c>
+      <c r="I2"/>
+      <c r="J2"/>
+      <c r="K2"/>
+      <c r="L2"/>
+      <c r="M2"/>
+      <c r="N2"/>
+      <c r="O2"/>
+      <c r="P2"/>
+      <c r="Q2"/>
+      <c r="R2"/>
+      <c r="S2"/>
+      <c r="T2"/>
+      <c r="U2"/>
+      <c r="V2"/>
+      <c r="W2"/>
+      <c r="X2"/>
+      <c r="Y2"/>
+      <c r="Z2"/>
+      <c r="AA2"/>
+      <c r="AB2"/>
+      <c r="AC2"/>
+      <c r="AD2"/>
+      <c r="AE2"/>
+      <c r="AF2"/>
+      <c r="AG2"/>
+      <c r="AH2"/>
+      <c r="AI2"/>
+      <c r="AJ2"/>
+      <c r="AK2"/>
+      <c r="AL2"/>
+      <c r="AM2"/>
+      <c r="AN2"/>
+      <c r="AO2"/>
+      <c r="AP2"/>
+      <c r="AQ2"/>
+      <c r="AR2"/>
+      <c r="AS2"/>
+      <c r="AT2"/>
+      <c r="AU2"/>
+      <c r="AV2"/>
+      <c r="AW2"/>
+      <c r="AX2"/>
+      <c r="AY2"/>
+      <c r="AZ2"/>
+      <c r="BA2"/>
+      <c r="BB2"/>
+      <c r="BC2"/>
+      <c r="BD2"/>
+      <c r="BE2"/>
+      <c r="BF2"/>
+      <c r="BG2"/>
+      <c r="BH2"/>
+      <c r="BI2"/>
+      <c r="BJ2"/>
+      <c r="BK2"/>
+      <c r="BL2"/>
+      <c r="BM2"/>
+      <c r="BN2"/>
+      <c r="BO2"/>
+      <c r="BP2"/>
+      <c r="BQ2"/>
+      <c r="BR2"/>
+      <c r="BS2"/>
+      <c r="BT2"/>
+      <c r="BU2"/>
+      <c r="BV2"/>
+      <c r="BW2"/>
+      <c r="BX2"/>
+      <c r="BY2"/>
+      <c r="BZ2"/>
+      <c r="CA2"/>
+      <c r="CB2"/>
+      <c r="CC2"/>
+      <c r="CD2"/>
+      <c r="CE2"/>
+      <c r="CF2"/>
+      <c r="CG2"/>
+      <c r="CH2"/>
+      <c r="CI2"/>
+      <c r="CJ2"/>
+      <c r="CK2"/>
+      <c r="CL2"/>
+      <c r="CM2"/>
+      <c r="CN2"/>
+      <c r="CO2"/>
+      <c r="CP2"/>
+      <c r="CQ2"/>
+      <c r="CR2"/>
+      <c r="CS2"/>
+      <c r="CT2"/>
+      <c r="CU2"/>
+      <c r="CV2"/>
+      <c r="CW2"/>
+      <c r="CX2"/>
+      <c r="CY2"/>
+      <c r="CZ2"/>
+      <c r="DA2"/>
+      <c r="DB2"/>
+      <c r="DC2"/>
+      <c r="DD2"/>
+      <c r="DE2"/>
+      <c r="DF2"/>
+      <c r="DG2"/>
+      <c r="DH2"/>
+      <c r="DI2"/>
+      <c r="DJ2"/>
+      <c r="DK2"/>
+      <c r="DL2"/>
+      <c r="DM2"/>
+      <c r="DN2"/>
+      <c r="DO2"/>
+      <c r="DP2"/>
+      <c r="DQ2"/>
+      <c r="DR2"/>
+      <c r="DS2"/>
+      <c r="DT2"/>
+      <c r="DU2"/>
+      <c r="DV2"/>
+      <c r="DW2"/>
+      <c r="DX2"/>
+      <c r="DY2"/>
+      <c r="DZ2"/>
+      <c r="EA2"/>
+      <c r="EB2"/>
+      <c r="EC2"/>
+      <c r="ED2"/>
+      <c r="EE2"/>
+      <c r="EF2"/>
+      <c r="EG2"/>
+      <c r="EH2"/>
+      <c r="EI2"/>
+      <c r="EJ2"/>
+      <c r="EK2"/>
+      <c r="EL2"/>
+      <c r="EM2"/>
+      <c r="EN2"/>
+      <c r="EO2"/>
+      <c r="EP2"/>
+      <c r="EQ2"/>
+      <c r="ER2"/>
+      <c r="ES2"/>
+      <c r="ET2"/>
+      <c r="EU2"/>
+      <c r="EV2"/>
+      <c r="EW2"/>
+      <c r="EX2"/>
+      <c r="EY2"/>
+      <c r="EZ2"/>
+      <c r="FA2"/>
+      <c r="FB2"/>
+      <c r="FC2"/>
+      <c r="FD2"/>
+      <c r="FE2"/>
+      <c r="FF2"/>
+      <c r="FG2"/>
+      <c r="FH2"/>
+      <c r="FI2"/>
+      <c r="FJ2"/>
+      <c r="FK2"/>
+      <c r="FL2"/>
+      <c r="FM2"/>
+      <c r="FN2"/>
+      <c r="FO2"/>
+      <c r="FP2"/>
+      <c r="FQ2"/>
+      <c r="FR2"/>
+      <c r="FS2"/>
+      <c r="FT2"/>
+      <c r="FU2"/>
+      <c r="FV2"/>
+      <c r="FW2"/>
+      <c r="FX2"/>
+      <c r="FY2"/>
+      <c r="FZ2"/>
+      <c r="GA2"/>
+      <c r="GB2"/>
+      <c r="GC2"/>
+      <c r="GD2"/>
+      <c r="GE2"/>
+      <c r="GF2"/>
+      <c r="GG2"/>
+      <c r="GH2"/>
+      <c r="GI2"/>
+      <c r="GJ2"/>
+      <c r="GK2"/>
+      <c r="GL2"/>
+      <c r="GM2"/>
+      <c r="GN2"/>
+      <c r="GO2"/>
+      <c r="GP2"/>
+      <c r="GQ2"/>
+      <c r="GR2"/>
+      <c r="GS2"/>
+      <c r="GT2"/>
+      <c r="GU2"/>
+      <c r="GV2"/>
+      <c r="GW2"/>
+      <c r="GX2"/>
+      <c r="GY2"/>
+      <c r="GZ2"/>
+      <c r="HA2"/>
+      <c r="HB2"/>
+      <c r="HC2"/>
+      <c r="HD2"/>
+      <c r="HE2"/>
+      <c r="HF2"/>
+      <c r="HG2"/>
+      <c r="HH2"/>
+      <c r="HI2"/>
+      <c r="HJ2"/>
+      <c r="HK2"/>
+      <c r="HL2"/>
+      <c r="HM2"/>
+      <c r="HN2"/>
+      <c r="HO2"/>
+      <c r="HP2"/>
+      <c r="HQ2"/>
+      <c r="HR2"/>
+      <c r="HS2"/>
+      <c r="HT2"/>
+      <c r="HU2"/>
+    </row>
+    <row r="3" spans="1:229" x14ac:dyDescent="0.35">
+      <c r="A3" s="3" t="s">
+        <v>418</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>419</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>420</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>226</v>
+      </c>
+      <c r="F3" s="3" t="s">
+        <v>227</v>
+      </c>
+      <c r="G3" s="3" t="s">
+        <v>236</v>
+      </c>
+      <c r="H3" s="3" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="4" spans="1:229" x14ac:dyDescent="0.35">
+      <c r="A4" s="3" t="s">
+        <v>422</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>423</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>424</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>226</v>
+      </c>
+      <c r="F4" s="3" t="s">
+        <v>227</v>
+      </c>
+      <c r="G4" s="3" t="s">
+        <v>236</v>
+      </c>
+      <c r="H4" s="3" t="s">
+        <v>425</v>
+      </c>
+    </row>
+    <row r="5" spans="1:229" x14ac:dyDescent="0.35">
+      <c r="A5" s="8" t="s">
+        <v>426</v>
+      </c>
+      <c r="B5" s="8" t="s">
+        <v>427</v>
+      </c>
+      <c r="C5" s="8" t="s">
+        <v>428</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>226</v>
+      </c>
+      <c r="F5" s="3" t="s">
+        <v>227</v>
+      </c>
+      <c r="G5" s="3" t="s">
+        <v>236</v>
+      </c>
+      <c r="H5" s="3" t="s">
+        <v>429</v>
+      </c>
+    </row>
+    <row r="6" spans="1:229" x14ac:dyDescent="0.35">
+      <c r="A6" s="3" t="s">
+        <v>430</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>431</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>432</v>
+      </c>
+      <c r="D6" s="7" t="s">
+        <v>0</v>
+      </c>
+      <c r="E6" s="3" t="s">
+        <v>226</v>
+      </c>
+      <c r="F6" s="3" t="s">
+        <v>227</v>
+      </c>
+      <c r="G6" s="3" t="s">
+        <v>236</v>
+      </c>
+      <c r="H6" s="3" t="s">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="7" spans="1:229" x14ac:dyDescent="0.35">
+      <c r="A7" s="3" t="s">
+        <v>434</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>435</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>436</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="E7" s="3" t="s">
+        <v>226</v>
+      </c>
+      <c r="F7" s="3" t="s">
+        <v>227</v>
+      </c>
+      <c r="G7" s="3" t="s">
+        <v>236</v>
+      </c>
+      <c r="H7" s="3" t="s">
+        <v>437</v>
+      </c>
+    </row>
+    <row r="8" spans="1:229" x14ac:dyDescent="0.35">
+      <c r="A8" s="9" t="s">
+        <v>438</v>
+      </c>
+      <c r="B8" s="9" t="s">
+        <v>439</v>
+      </c>
+      <c r="C8" s="9" t="s">
+        <v>440</v>
+      </c>
+      <c r="D8" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="E8" s="3" t="s">
+        <v>226</v>
+      </c>
+      <c r="F8" s="3" t="s">
+        <v>227</v>
+      </c>
+      <c r="G8" s="3" t="s">
+        <v>236</v>
+      </c>
+      <c r="H8" s="9" t="s">
+        <v>441</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -13657,22 +14564,22 @@
     </row>
     <row r="2" spans="1:1029" x14ac:dyDescent="0.35">
       <c r="A2" s="3" t="s">
-        <v>387</v>
+        <v>372</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>388</v>
+        <v>373</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>389</v>
+        <v>374</v>
       </c>
       <c r="D2" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>386</v>
+        <v>371</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>390</v>
+        <v>375</v>
       </c>
     </row>
     <row r="3" spans="1:1029" x14ac:dyDescent="0.35">
@@ -13689,7 +14596,7 @@
         <v>0</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>386</v>
+        <v>371</v>
       </c>
       <c r="F3" s="3" t="s">
         <v>93</v>
@@ -13709,7 +14616,7 @@
         <v>0</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>386</v>
+        <v>371</v>
       </c>
       <c r="F4" s="3" t="s">
         <v>124</v>
@@ -13729,7 +14636,7 @@
         <v>0</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>386</v>
+        <v>371</v>
       </c>
       <c r="F5" s="3" t="s">
         <v>73</v>
@@ -14772,7 +15679,7 @@
         <v>0</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>386</v>
+        <v>371</v>
       </c>
       <c r="F6" s="3" t="s">
         <v>97</v>
@@ -14792,7 +15699,7 @@
         <v>0</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>386</v>
+        <v>371</v>
       </c>
       <c r="F7" s="3" t="s">
         <v>89</v>
@@ -14812,7 +15719,7 @@
         <v>0</v>
       </c>
       <c r="E8" s="3" t="s">
-        <v>386</v>
+        <v>371</v>
       </c>
       <c r="F8" s="3" t="s">
         <v>76</v>
@@ -15855,7 +16762,7 @@
         <v>0</v>
       </c>
       <c r="E9" s="3" t="s">
-        <v>386</v>
+        <v>371</v>
       </c>
       <c r="F9" s="3" t="s">
         <v>79</v>
@@ -15875,7 +16782,7 @@
         <v>0</v>
       </c>
       <c r="E10" s="3" t="s">
-        <v>386</v>
+        <v>371</v>
       </c>
       <c r="F10" s="3" t="s">
         <v>85</v>
@@ -15895,7 +16802,7 @@
         <v>0</v>
       </c>
       <c r="E11" s="3" t="s">
-        <v>386</v>
+        <v>371</v>
       </c>
       <c r="F11" s="3" t="s">
         <v>120</v>
@@ -16427,13 +17334,13 @@
     </row>
     <row r="4" spans="1:229" s="4" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A4" s="3" t="s">
-        <v>391</v>
+        <v>376</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>392</v>
+        <v>377</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>393</v>
+        <v>378</v>
       </c>
       <c r="D4" s="3" t="s">
         <v>0</v>
@@ -16442,7 +17349,7 @@
         <v>101</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>394</v>
+        <v>379</v>
       </c>
       <c r="G4"/>
       <c r="H4"/>
@@ -16736,60 +17643,60 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" s="3" t="s">
+        <v>129</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>131</v>
+      </c>
+      <c r="C2" s="3" t="s">
         <v>130</v>
-      </c>
-      <c r="B2" s="3" t="s">
-        <v>132</v>
-      </c>
-      <c r="C2" s="3" t="s">
-        <v>131</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="14" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B3" s="3" t="s">
-        <v>145</v>
+        <v>139</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>146</v>
+        <v>140</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.35">
       <c r="B4" s="3" t="s">
-        <v>143</v>
+        <v>137</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>144</v>
+        <v>138</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A5" s="3" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="B5" s="3"/>
       <c r="C5" s="3"/>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A6" s="3" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="B6" s="3"/>
       <c r="C6" s="3"/>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A7" s="3" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="B7" s="3"/>
       <c r="C7" s="3"/>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A8" s="3" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A9" s="3" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
     </row>
   </sheetData>
@@ -16819,75 +17726,53 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" s="3" t="s">
-        <v>147</v>
+        <v>141</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>148</v>
+        <v>142</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="14" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="3" t="s">
-        <v>149</v>
-      </c>
       <c r="B3" s="3" t="s">
-        <v>134</v>
+        <v>139</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>129</v>
+        <v>140</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A4" s="3" t="s">
-        <v>150</v>
-      </c>
       <c r="B4" s="3" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>129</v>
+        <v>138</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A5" s="3" t="s">
-        <v>151</v>
-      </c>
-      <c r="B5" s="3" t="s">
-        <v>140</v>
-      </c>
-      <c r="C5" s="3" t="s">
-        <v>129</v>
-      </c>
+        <v>143</v>
+      </c>
+      <c r="B5" s="3"/>
+      <c r="C5" s="3"/>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A6" s="3" t="s">
-        <v>152</v>
-      </c>
-      <c r="B6" s="3" t="s">
-        <v>141</v>
-      </c>
-      <c r="C6" s="3" t="s">
-        <v>129</v>
-      </c>
+        <v>144</v>
+      </c>
+      <c r="B6" s="3"/>
+      <c r="C6" s="3"/>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A7" s="3"/>
-      <c r="B7" s="3" t="s">
+      <c r="A7" s="3" t="s">
         <v>145</v>
       </c>
-      <c r="C7" s="3" t="s">
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A8" s="3" t="s">
         <v>146</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A8" s="3"/>
-      <c r="B8" s="3" t="s">
-        <v>143</v>
-      </c>
-      <c r="C8" s="3" t="s">
-        <v>144</v>
       </c>
     </row>
   </sheetData>
@@ -16917,97 +17802,67 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" s="3" t="s">
-        <v>153</v>
+        <v>147</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>154</v>
+        <v>148</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="14" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="3" t="s">
-        <v>158</v>
-      </c>
       <c r="B3" s="3" t="s">
-        <v>134</v>
+        <v>139</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>129</v>
+        <v>140</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A4" s="3" t="s">
-        <v>157</v>
-      </c>
       <c r="B4" s="3" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>129</v>
+        <v>138</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A5" s="3" t="s">
-        <v>156</v>
-      </c>
-      <c r="B5" s="3" t="s">
-        <v>140</v>
-      </c>
-      <c r="C5" s="3" t="s">
-        <v>129</v>
-      </c>
+        <v>152</v>
+      </c>
+      <c r="B5" s="3"/>
+      <c r="C5" s="3"/>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A6" s="3" t="s">
-        <v>155</v>
-      </c>
-      <c r="B6" s="3" t="s">
-        <v>141</v>
-      </c>
-      <c r="C6" s="3" t="s">
-        <v>129</v>
-      </c>
+        <v>151</v>
+      </c>
+      <c r="B6" s="3"/>
+      <c r="C6" s="3"/>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A7" s="3" t="s">
-        <v>159</v>
-      </c>
-      <c r="B7" s="3" t="s">
-        <v>142</v>
-      </c>
-      <c r="C7" s="3" t="s">
-        <v>129</v>
-      </c>
+        <v>150</v>
+      </c>
+      <c r="B7" s="3"/>
+      <c r="C7" s="3"/>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A8" s="3" t="s">
-        <v>161</v>
-      </c>
-      <c r="B8" s="3" t="s">
-        <v>160</v>
-      </c>
-      <c r="C8" s="3" t="s">
-        <v>129</v>
-      </c>
+        <v>149</v>
+      </c>
+      <c r="B8" s="3"/>
+      <c r="C8" s="3"/>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A9" s="3"/>
-      <c r="B9" s="3" t="s">
-        <v>145</v>
-      </c>
-      <c r="C9" s="3" t="s">
-        <v>146</v>
+      <c r="A9" s="3" t="s">
+        <v>153</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A10" s="3"/>
-      <c r="B10" s="3" t="s">
-        <v>143</v>
-      </c>
-      <c r="C10" s="3" t="s">
-        <v>144</v>
+      <c r="A10" s="3" t="s">
+        <v>154</v>
       </c>
     </row>
   </sheetData>
@@ -17038,86 +17893,60 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" s="3" t="s">
-        <v>162</v>
+        <v>155</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>163</v>
+        <v>156</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="14" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="3" t="s">
-        <v>164</v>
-      </c>
       <c r="B3" s="3" t="s">
-        <v>134</v>
+        <v>139</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>129</v>
+        <v>140</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A4" s="3" t="s">
-        <v>165</v>
-      </c>
       <c r="B4" s="3" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>129</v>
+        <v>138</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A5" s="3" t="s">
-        <v>166</v>
-      </c>
-      <c r="B5" s="3" t="s">
-        <v>140</v>
-      </c>
-      <c r="C5" s="3" t="s">
-        <v>129</v>
-      </c>
+        <v>157</v>
+      </c>
+      <c r="B5" s="3"/>
+      <c r="C5" s="3"/>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A6" s="3" t="s">
-        <v>167</v>
-      </c>
-      <c r="B6" s="3" t="s">
-        <v>141</v>
-      </c>
-      <c r="C6" s="3" t="s">
-        <v>129</v>
-      </c>
+        <v>158</v>
+      </c>
+      <c r="B6" s="3"/>
+      <c r="C6" s="3"/>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A7" s="3" t="s">
-        <v>168</v>
-      </c>
-      <c r="B7" s="3" t="s">
-        <v>142</v>
-      </c>
-      <c r="C7" s="3" t="s">
-        <v>129</v>
-      </c>
+        <v>159</v>
+      </c>
+      <c r="B7" s="3"/>
+      <c r="C7" s="3"/>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A8" s="3"/>
-      <c r="B8" s="3" t="s">
-        <v>145</v>
-      </c>
-      <c r="C8" s="3" t="s">
-        <v>146</v>
+      <c r="A8" s="3" t="s">
+        <v>160</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A9" s="3"/>
-      <c r="B9" s="3" t="s">
-        <v>143</v>
-      </c>
-      <c r="C9" s="3" t="s">
-        <v>144</v>
+      <c r="A9" s="3" t="s">
+        <v>161</v>
       </c>
     </row>
   </sheetData>
@@ -17148,119 +17977,81 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" s="3" t="s">
-        <v>169</v>
+        <v>162</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>170</v>
+        <v>163</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="14" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="3" t="s">
-        <v>171</v>
-      </c>
       <c r="B3" s="3" t="s">
-        <v>134</v>
+        <v>139</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>129</v>
+        <v>140</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A4" s="3" t="s">
-        <v>172</v>
-      </c>
       <c r="B4" s="3" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>182</v>
+        <v>138</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A5" s="3" t="s">
-        <v>173</v>
-      </c>
-      <c r="B5" s="3" t="s">
-        <v>140</v>
-      </c>
-      <c r="C5" s="3" t="s">
-        <v>180</v>
-      </c>
+        <v>164</v>
+      </c>
+      <c r="B5" s="3"/>
+      <c r="C5" s="3"/>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A6" s="3" t="s">
-        <v>174</v>
-      </c>
-      <c r="B6" s="3" t="s">
-        <v>141</v>
-      </c>
-      <c r="C6" s="3" t="s">
-        <v>181</v>
-      </c>
+        <v>165</v>
+      </c>
+      <c r="B6" s="3"/>
+      <c r="C6" s="3"/>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A7" s="3" t="s">
-        <v>175</v>
-      </c>
-      <c r="B7" s="3" t="s">
-        <v>142</v>
-      </c>
-      <c r="C7" s="3" t="s">
-        <v>180</v>
-      </c>
+        <v>166</v>
+      </c>
+      <c r="B7" s="3"/>
+      <c r="C7" s="3"/>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A8" s="3" t="s">
-        <v>176</v>
-      </c>
-      <c r="B8" s="3" t="s">
-        <v>160</v>
-      </c>
-      <c r="C8" s="3" t="s">
-        <v>180</v>
-      </c>
+        <v>167</v>
+      </c>
+      <c r="B8" s="3"/>
+      <c r="C8" s="3"/>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A9" s="3" t="s">
-        <v>178</v>
-      </c>
-      <c r="B9" s="3" t="s">
-        <v>177</v>
-      </c>
-      <c r="C9" s="3" t="s">
-        <v>179</v>
-      </c>
+        <v>168</v>
+      </c>
+      <c r="B9" s="3"/>
+      <c r="C9" s="3"/>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A10" s="3" t="s">
-        <v>185</v>
-      </c>
-      <c r="B10" s="3" t="s">
-        <v>184</v>
-      </c>
-      <c r="C10" s="3" t="s">
-        <v>183</v>
-      </c>
+        <v>169</v>
+      </c>
+      <c r="B10" s="3"/>
+      <c r="C10" s="3"/>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A11" s="3"/>
-      <c r="B11" s="3" t="s">
-        <v>145</v>
-      </c>
-      <c r="C11" s="3" t="s">
-        <v>146</v>
+      <c r="A11" s="3" t="s">
+        <v>170</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A12" s="3"/>
-      <c r="B12" s="3" t="s">
-        <v>143</v>
-      </c>
-      <c r="C12" s="3" t="s">
-        <v>144</v>
+      <c r="A12" s="3" t="s">
+        <v>171</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
content update in phase and home page
</commit_message>
<xml_diff>
--- a/testdata.xlsx
+++ b/testdata.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29328"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sshiwani\workspace\find-information-products-services-tests\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4F43993A-715F-4D1C-B894-7EEE8875F979}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F9D47F77-FF77-46CE-ACAE-C8E70E8090EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="22780" windowHeight="14540" firstSheet="21" activeTab="23" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="22780" windowHeight="14540" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="category_phase" sheetId="1" r:id="rId1"/>
@@ -48,7 +48,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="877" uniqueCount="442">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="883" uniqueCount="446">
   <si>
     <t>Search and filter products and services</t>
   </si>
@@ -1374,6 +1374,18 @@
   </si>
   <si>
     <t>Trade union bodies workforce (data user)  (Professional external user of DfE data)</t>
+  </si>
+  <si>
+    <t>products?phase=did-not-progress</t>
+  </si>
+  <si>
+    <t>ul.moj-filter-tags li a:has-text(' Did not progress')</t>
+  </si>
+  <si>
+    <t>Remove this filter Did not progress</t>
+  </si>
+  <si>
+    <t>#phase-did-not-progress</t>
   </si>
 </sst>
 </file>
@@ -1793,7 +1805,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:ARE8"/>
+  <dimension ref="A1:ARE9"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="30" bestFit="1" customWidth="1"/>
@@ -4152,13 +4164,13 @@
     </row>
     <row r="4" spans="1:1149" s="5" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A4" s="3" t="s">
-        <v>10</v>
+        <v>442</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>11</v>
+        <v>443</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>12</v>
+        <v>444</v>
       </c>
       <c r="D4" s="3" t="s">
         <v>0</v>
@@ -4167,7 +4179,7 @@
         <v>1</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>13</v>
+        <v>445</v>
       </c>
       <c r="G4"/>
       <c r="H4"/>
@@ -5315,13 +5327,13 @@
     </row>
     <row r="5" spans="1:1149" s="5" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A5" s="3" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="D5" s="3" t="s">
         <v>0</v>
@@ -5330,7 +5342,7 @@
         <v>1</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="G5"/>
       <c r="H5"/>
@@ -6478,13 +6490,13 @@
     </row>
     <row r="6" spans="1:1149" s="5" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A6" s="3" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="D6" s="3" t="s">
         <v>0</v>
@@ -6493,7 +6505,7 @@
         <v>1</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="G6"/>
       <c r="H6"/>
@@ -7641,13 +7653,13 @@
     </row>
     <row r="7" spans="1:1149" s="5" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A7" s="3" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="D7" s="3" t="s">
         <v>0</v>
@@ -7656,7 +7668,7 @@
         <v>1</v>
       </c>
       <c r="F7" s="3" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="G7"/>
       <c r="H7"/>
@@ -8804,13 +8816,13 @@
     </row>
     <row r="8" spans="1:1149" s="5" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A8" s="3" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="D8" s="3" t="s">
         <v>0</v>
@@ -8819,7 +8831,7 @@
         <v>1</v>
       </c>
       <c r="F8" s="3" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="G8"/>
       <c r="H8"/>
@@ -9965,6 +9977,1169 @@
       <c r="ARD8"/>
       <c r="ARE8"/>
     </row>
+    <row r="9" spans="1:1149" s="5" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A9" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="D9" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="E9" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="F9" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="G9"/>
+      <c r="H9"/>
+      <c r="I9"/>
+      <c r="J9"/>
+      <c r="K9"/>
+      <c r="L9"/>
+      <c r="M9"/>
+      <c r="N9"/>
+      <c r="O9"/>
+      <c r="P9"/>
+      <c r="Q9"/>
+      <c r="R9"/>
+      <c r="S9"/>
+      <c r="T9"/>
+      <c r="U9"/>
+      <c r="V9"/>
+      <c r="W9"/>
+      <c r="X9"/>
+      <c r="Y9"/>
+      <c r="Z9"/>
+      <c r="AA9"/>
+      <c r="AB9"/>
+      <c r="AC9"/>
+      <c r="AD9"/>
+      <c r="AE9"/>
+      <c r="AF9"/>
+      <c r="AG9"/>
+      <c r="AH9"/>
+      <c r="AI9"/>
+      <c r="AJ9"/>
+      <c r="AK9"/>
+      <c r="AL9"/>
+      <c r="AM9"/>
+      <c r="AN9"/>
+      <c r="AO9"/>
+      <c r="AP9"/>
+      <c r="AQ9"/>
+      <c r="AR9"/>
+      <c r="AS9"/>
+      <c r="AT9"/>
+      <c r="AU9"/>
+      <c r="AV9"/>
+      <c r="AW9"/>
+      <c r="AX9"/>
+      <c r="AY9"/>
+      <c r="AZ9"/>
+      <c r="BA9"/>
+      <c r="BB9"/>
+      <c r="BC9"/>
+      <c r="BD9"/>
+      <c r="BE9"/>
+      <c r="BF9"/>
+      <c r="BG9"/>
+      <c r="BH9"/>
+      <c r="BI9"/>
+      <c r="BJ9"/>
+      <c r="BK9"/>
+      <c r="BL9"/>
+      <c r="BM9"/>
+      <c r="BN9"/>
+      <c r="BO9"/>
+      <c r="BP9"/>
+      <c r="BQ9"/>
+      <c r="BR9"/>
+      <c r="BS9"/>
+      <c r="BT9"/>
+      <c r="BU9"/>
+      <c r="BV9"/>
+      <c r="BW9"/>
+      <c r="BX9"/>
+      <c r="BY9"/>
+      <c r="BZ9"/>
+      <c r="CA9"/>
+      <c r="CB9"/>
+      <c r="CC9"/>
+      <c r="CD9"/>
+      <c r="CE9"/>
+      <c r="CF9"/>
+      <c r="CG9"/>
+      <c r="CH9"/>
+      <c r="CI9"/>
+      <c r="CJ9"/>
+      <c r="CK9"/>
+      <c r="CL9"/>
+      <c r="CM9"/>
+      <c r="CN9"/>
+      <c r="CO9"/>
+      <c r="CP9"/>
+      <c r="CQ9"/>
+      <c r="CR9"/>
+      <c r="CS9"/>
+      <c r="CT9"/>
+      <c r="CU9"/>
+      <c r="CV9"/>
+      <c r="CW9"/>
+      <c r="CX9"/>
+      <c r="CY9"/>
+      <c r="CZ9"/>
+      <c r="DA9"/>
+      <c r="DB9"/>
+      <c r="DC9"/>
+      <c r="DD9"/>
+      <c r="DE9"/>
+      <c r="DF9"/>
+      <c r="DG9"/>
+      <c r="DH9"/>
+      <c r="DI9"/>
+      <c r="DJ9"/>
+      <c r="DK9"/>
+      <c r="DL9"/>
+      <c r="DM9"/>
+      <c r="DN9"/>
+      <c r="DO9"/>
+      <c r="DP9"/>
+      <c r="DQ9"/>
+      <c r="DR9"/>
+      <c r="DS9"/>
+      <c r="DT9"/>
+      <c r="DU9"/>
+      <c r="DV9"/>
+      <c r="DW9"/>
+      <c r="DX9"/>
+      <c r="DY9"/>
+      <c r="DZ9"/>
+      <c r="EA9"/>
+      <c r="EB9"/>
+      <c r="EC9"/>
+      <c r="ED9"/>
+      <c r="EE9"/>
+      <c r="EF9"/>
+      <c r="EG9"/>
+      <c r="EH9"/>
+      <c r="EI9"/>
+      <c r="EJ9"/>
+      <c r="EK9"/>
+      <c r="EL9"/>
+      <c r="EM9"/>
+      <c r="EN9"/>
+      <c r="EO9"/>
+      <c r="EP9"/>
+      <c r="EQ9"/>
+      <c r="ER9"/>
+      <c r="ES9"/>
+      <c r="ET9"/>
+      <c r="EU9"/>
+      <c r="EV9"/>
+      <c r="EW9"/>
+      <c r="EX9"/>
+      <c r="EY9"/>
+      <c r="EZ9"/>
+      <c r="FA9"/>
+      <c r="FB9"/>
+      <c r="FC9"/>
+      <c r="FD9"/>
+      <c r="FE9"/>
+      <c r="FF9"/>
+      <c r="FG9"/>
+      <c r="FH9"/>
+      <c r="FI9"/>
+      <c r="FJ9"/>
+      <c r="FK9"/>
+      <c r="FL9"/>
+      <c r="FM9"/>
+      <c r="FN9"/>
+      <c r="FO9"/>
+      <c r="FP9"/>
+      <c r="FQ9"/>
+      <c r="FR9"/>
+      <c r="FS9"/>
+      <c r="FT9"/>
+      <c r="FU9"/>
+      <c r="FV9"/>
+      <c r="FW9"/>
+      <c r="FX9"/>
+      <c r="FY9"/>
+      <c r="FZ9"/>
+      <c r="GA9"/>
+      <c r="GB9"/>
+      <c r="GC9"/>
+      <c r="GD9"/>
+      <c r="GE9"/>
+      <c r="GF9"/>
+      <c r="GG9"/>
+      <c r="GH9"/>
+      <c r="GI9"/>
+      <c r="GJ9"/>
+      <c r="GK9"/>
+      <c r="GL9"/>
+      <c r="GM9"/>
+      <c r="GN9"/>
+      <c r="GO9"/>
+      <c r="GP9"/>
+      <c r="GQ9"/>
+      <c r="GR9"/>
+      <c r="GS9"/>
+      <c r="GT9"/>
+      <c r="GU9"/>
+      <c r="GV9"/>
+      <c r="GW9"/>
+      <c r="GX9"/>
+      <c r="GY9"/>
+      <c r="GZ9"/>
+      <c r="HA9"/>
+      <c r="HB9"/>
+      <c r="HC9"/>
+      <c r="HD9"/>
+      <c r="HE9"/>
+      <c r="HF9"/>
+      <c r="HG9"/>
+      <c r="HH9"/>
+      <c r="HI9"/>
+      <c r="HJ9"/>
+      <c r="HK9"/>
+      <c r="HL9"/>
+      <c r="HM9"/>
+      <c r="HN9"/>
+      <c r="HO9"/>
+      <c r="HP9"/>
+      <c r="HQ9"/>
+      <c r="HR9"/>
+      <c r="HS9"/>
+      <c r="HT9"/>
+      <c r="HU9"/>
+      <c r="HV9"/>
+      <c r="HW9"/>
+      <c r="HX9"/>
+      <c r="HY9"/>
+      <c r="HZ9"/>
+      <c r="IA9"/>
+      <c r="IB9"/>
+      <c r="IC9"/>
+      <c r="ID9"/>
+      <c r="IE9"/>
+      <c r="IF9"/>
+      <c r="IG9"/>
+      <c r="IH9"/>
+      <c r="II9"/>
+      <c r="IJ9"/>
+      <c r="IK9"/>
+      <c r="IL9"/>
+      <c r="IM9"/>
+      <c r="IN9"/>
+      <c r="IO9"/>
+      <c r="IP9"/>
+      <c r="IQ9"/>
+      <c r="IR9"/>
+      <c r="IS9"/>
+      <c r="IT9"/>
+      <c r="IU9"/>
+      <c r="IV9"/>
+      <c r="IW9"/>
+      <c r="IX9"/>
+      <c r="IY9"/>
+      <c r="IZ9"/>
+      <c r="JA9"/>
+      <c r="JB9"/>
+      <c r="JC9"/>
+      <c r="JD9"/>
+      <c r="JE9"/>
+      <c r="JF9"/>
+      <c r="JG9"/>
+      <c r="JH9"/>
+      <c r="JI9"/>
+      <c r="JJ9"/>
+      <c r="JK9"/>
+      <c r="JL9"/>
+      <c r="JM9"/>
+      <c r="JN9"/>
+      <c r="JO9"/>
+      <c r="JP9"/>
+      <c r="JQ9"/>
+      <c r="JR9"/>
+      <c r="JS9"/>
+      <c r="JT9"/>
+      <c r="JU9"/>
+      <c r="JV9"/>
+      <c r="JW9"/>
+      <c r="JX9"/>
+      <c r="JY9"/>
+      <c r="JZ9"/>
+      <c r="KA9"/>
+      <c r="KB9"/>
+      <c r="KC9"/>
+      <c r="KD9"/>
+      <c r="KE9"/>
+      <c r="KF9"/>
+      <c r="KG9"/>
+      <c r="KH9"/>
+      <c r="KI9"/>
+      <c r="KJ9"/>
+      <c r="KK9"/>
+      <c r="KL9"/>
+      <c r="KM9"/>
+      <c r="KN9"/>
+      <c r="KO9"/>
+      <c r="KP9"/>
+      <c r="KQ9"/>
+      <c r="KR9"/>
+      <c r="KS9"/>
+      <c r="KT9"/>
+      <c r="KU9"/>
+      <c r="KV9"/>
+      <c r="KW9"/>
+      <c r="KX9"/>
+      <c r="KY9"/>
+      <c r="KZ9"/>
+      <c r="LA9"/>
+      <c r="LB9"/>
+      <c r="LC9"/>
+      <c r="LD9"/>
+      <c r="LE9"/>
+      <c r="LF9"/>
+      <c r="LG9"/>
+      <c r="LH9"/>
+      <c r="LI9"/>
+      <c r="LJ9"/>
+      <c r="LK9"/>
+      <c r="LL9"/>
+      <c r="LM9"/>
+      <c r="LN9"/>
+      <c r="LO9"/>
+      <c r="LP9"/>
+      <c r="LQ9"/>
+      <c r="LR9"/>
+      <c r="LS9"/>
+      <c r="LT9"/>
+      <c r="LU9"/>
+      <c r="LV9"/>
+      <c r="LW9"/>
+      <c r="LX9"/>
+      <c r="LY9"/>
+      <c r="LZ9"/>
+      <c r="MA9"/>
+      <c r="MB9"/>
+      <c r="MC9"/>
+      <c r="MD9"/>
+      <c r="ME9"/>
+      <c r="MF9"/>
+      <c r="MG9"/>
+      <c r="MH9"/>
+      <c r="MI9"/>
+      <c r="MJ9"/>
+      <c r="MK9"/>
+      <c r="ML9"/>
+      <c r="MM9"/>
+      <c r="MN9"/>
+      <c r="MO9"/>
+      <c r="MP9"/>
+      <c r="MQ9"/>
+      <c r="MR9"/>
+      <c r="MS9"/>
+      <c r="MT9"/>
+      <c r="MU9"/>
+      <c r="MV9"/>
+      <c r="MW9"/>
+      <c r="MX9"/>
+      <c r="MY9"/>
+      <c r="MZ9"/>
+      <c r="NA9"/>
+      <c r="NB9"/>
+      <c r="NC9"/>
+      <c r="ND9"/>
+      <c r="NE9"/>
+      <c r="NF9"/>
+      <c r="NG9"/>
+      <c r="NH9"/>
+      <c r="NI9"/>
+      <c r="NJ9"/>
+      <c r="NK9"/>
+      <c r="NL9"/>
+      <c r="NM9"/>
+      <c r="NN9"/>
+      <c r="NO9"/>
+      <c r="NP9"/>
+      <c r="NQ9"/>
+      <c r="NR9"/>
+      <c r="NS9"/>
+      <c r="NT9"/>
+      <c r="NU9"/>
+      <c r="NV9"/>
+      <c r="NW9"/>
+      <c r="NX9"/>
+      <c r="NY9"/>
+      <c r="NZ9"/>
+      <c r="OA9"/>
+      <c r="OB9"/>
+      <c r="OC9"/>
+      <c r="OD9"/>
+      <c r="OE9"/>
+      <c r="OF9"/>
+      <c r="OG9"/>
+      <c r="OH9"/>
+      <c r="OI9"/>
+      <c r="OJ9"/>
+      <c r="OK9"/>
+      <c r="OL9"/>
+      <c r="OM9"/>
+      <c r="ON9"/>
+      <c r="OO9"/>
+      <c r="OP9"/>
+      <c r="OQ9"/>
+      <c r="OR9"/>
+      <c r="OS9"/>
+      <c r="OT9"/>
+      <c r="OU9"/>
+      <c r="OV9"/>
+      <c r="OW9"/>
+      <c r="OX9"/>
+      <c r="OY9"/>
+      <c r="OZ9"/>
+      <c r="PA9"/>
+      <c r="PB9"/>
+      <c r="PC9"/>
+      <c r="PD9"/>
+      <c r="PE9"/>
+      <c r="PF9"/>
+      <c r="PG9"/>
+      <c r="PH9"/>
+      <c r="PI9"/>
+      <c r="PJ9"/>
+      <c r="PK9"/>
+      <c r="PL9"/>
+      <c r="PM9"/>
+      <c r="PN9"/>
+      <c r="PO9"/>
+      <c r="PP9"/>
+      <c r="PQ9"/>
+      <c r="PR9"/>
+      <c r="PS9"/>
+      <c r="PT9"/>
+      <c r="PU9"/>
+      <c r="PV9"/>
+      <c r="PW9"/>
+      <c r="PX9"/>
+      <c r="PY9"/>
+      <c r="PZ9"/>
+      <c r="QA9"/>
+      <c r="QB9"/>
+      <c r="QC9"/>
+      <c r="QD9"/>
+      <c r="QE9"/>
+      <c r="QF9"/>
+      <c r="QG9"/>
+      <c r="QH9"/>
+      <c r="QI9"/>
+      <c r="QJ9"/>
+      <c r="QK9"/>
+      <c r="QL9"/>
+      <c r="QM9"/>
+      <c r="QN9"/>
+      <c r="QO9"/>
+      <c r="QP9"/>
+      <c r="QQ9"/>
+      <c r="QR9"/>
+      <c r="QS9"/>
+      <c r="QT9"/>
+      <c r="QU9"/>
+      <c r="QV9"/>
+      <c r="QW9"/>
+      <c r="QX9"/>
+      <c r="QY9"/>
+      <c r="QZ9"/>
+      <c r="RA9"/>
+      <c r="RB9"/>
+      <c r="RC9"/>
+      <c r="RD9"/>
+      <c r="RE9"/>
+      <c r="RF9"/>
+      <c r="RG9"/>
+      <c r="RH9"/>
+      <c r="RI9"/>
+      <c r="RJ9"/>
+      <c r="RK9"/>
+      <c r="RL9"/>
+      <c r="RM9"/>
+      <c r="RN9"/>
+      <c r="RO9"/>
+      <c r="RP9"/>
+      <c r="RQ9"/>
+      <c r="RR9"/>
+      <c r="RS9"/>
+      <c r="RT9"/>
+      <c r="RU9"/>
+      <c r="RV9"/>
+      <c r="RW9"/>
+      <c r="RX9"/>
+      <c r="RY9"/>
+      <c r="RZ9"/>
+      <c r="SA9"/>
+      <c r="SB9"/>
+      <c r="SC9"/>
+      <c r="SD9"/>
+      <c r="SE9"/>
+      <c r="SF9"/>
+      <c r="SG9"/>
+      <c r="SH9"/>
+      <c r="SI9"/>
+      <c r="SJ9"/>
+      <c r="SK9"/>
+      <c r="SL9"/>
+      <c r="SM9"/>
+      <c r="SN9"/>
+      <c r="SO9"/>
+      <c r="SP9"/>
+      <c r="SQ9"/>
+      <c r="SR9"/>
+      <c r="SS9"/>
+      <c r="ST9"/>
+      <c r="SU9"/>
+      <c r="SV9"/>
+      <c r="SW9"/>
+      <c r="SX9"/>
+      <c r="SY9"/>
+      <c r="SZ9"/>
+      <c r="TA9"/>
+      <c r="TB9"/>
+      <c r="TC9"/>
+      <c r="TD9"/>
+      <c r="TE9"/>
+      <c r="TF9"/>
+      <c r="TG9"/>
+      <c r="TH9"/>
+      <c r="TI9"/>
+      <c r="TJ9"/>
+      <c r="TK9"/>
+      <c r="TL9"/>
+      <c r="TM9"/>
+      <c r="TN9"/>
+      <c r="TO9"/>
+      <c r="TP9"/>
+      <c r="TQ9"/>
+      <c r="TR9"/>
+      <c r="TS9"/>
+      <c r="TT9"/>
+      <c r="TU9"/>
+      <c r="TV9"/>
+      <c r="TW9"/>
+      <c r="TX9"/>
+      <c r="TY9"/>
+      <c r="TZ9"/>
+      <c r="UA9"/>
+      <c r="UB9"/>
+      <c r="UC9"/>
+      <c r="UD9"/>
+      <c r="UE9"/>
+      <c r="UF9"/>
+      <c r="UG9"/>
+      <c r="UH9"/>
+      <c r="UI9"/>
+      <c r="UJ9"/>
+      <c r="UK9"/>
+      <c r="UL9"/>
+      <c r="UM9"/>
+      <c r="UN9"/>
+      <c r="UO9"/>
+      <c r="UP9"/>
+      <c r="UQ9"/>
+      <c r="UR9"/>
+      <c r="US9"/>
+      <c r="UT9"/>
+      <c r="UU9"/>
+      <c r="UV9"/>
+      <c r="UW9"/>
+      <c r="UX9"/>
+      <c r="UY9"/>
+      <c r="UZ9"/>
+      <c r="VA9"/>
+      <c r="VB9"/>
+      <c r="VC9"/>
+      <c r="VD9"/>
+      <c r="VE9"/>
+      <c r="VF9"/>
+      <c r="VG9"/>
+      <c r="VH9"/>
+      <c r="VI9"/>
+      <c r="VJ9"/>
+      <c r="VK9"/>
+      <c r="VL9"/>
+      <c r="VM9"/>
+      <c r="VN9"/>
+      <c r="VO9"/>
+      <c r="VP9"/>
+      <c r="VQ9"/>
+      <c r="VR9"/>
+      <c r="VS9"/>
+      <c r="VT9"/>
+      <c r="VU9"/>
+      <c r="VV9"/>
+      <c r="VW9"/>
+      <c r="VX9"/>
+      <c r="VY9"/>
+      <c r="VZ9"/>
+      <c r="WA9"/>
+      <c r="WB9"/>
+      <c r="WC9"/>
+      <c r="WD9"/>
+      <c r="WE9"/>
+      <c r="WF9"/>
+      <c r="WG9"/>
+      <c r="WH9"/>
+      <c r="WI9"/>
+      <c r="WJ9"/>
+      <c r="WK9"/>
+      <c r="WL9"/>
+      <c r="WM9"/>
+      <c r="WN9"/>
+      <c r="WO9"/>
+      <c r="WP9"/>
+      <c r="WQ9"/>
+      <c r="WR9"/>
+      <c r="WS9"/>
+      <c r="WT9"/>
+      <c r="WU9"/>
+      <c r="WV9"/>
+      <c r="WW9"/>
+      <c r="WX9"/>
+      <c r="WY9"/>
+      <c r="WZ9"/>
+      <c r="XA9"/>
+      <c r="XB9"/>
+      <c r="XC9"/>
+      <c r="XD9"/>
+      <c r="XE9"/>
+      <c r="XF9"/>
+      <c r="XG9"/>
+      <c r="XH9"/>
+      <c r="XI9"/>
+      <c r="XJ9"/>
+      <c r="XK9"/>
+      <c r="XL9"/>
+      <c r="XM9"/>
+      <c r="XN9"/>
+      <c r="XO9"/>
+      <c r="XP9"/>
+      <c r="XQ9"/>
+      <c r="XR9"/>
+      <c r="XS9"/>
+      <c r="XT9"/>
+      <c r="XU9"/>
+      <c r="XV9"/>
+      <c r="XW9"/>
+      <c r="XX9"/>
+      <c r="XY9"/>
+      <c r="XZ9"/>
+      <c r="YA9"/>
+      <c r="YB9"/>
+      <c r="YC9"/>
+      <c r="YD9"/>
+      <c r="YE9"/>
+      <c r="YF9"/>
+      <c r="YG9"/>
+      <c r="YH9"/>
+      <c r="YI9"/>
+      <c r="YJ9"/>
+      <c r="YK9"/>
+      <c r="YL9"/>
+      <c r="YM9"/>
+      <c r="YN9"/>
+      <c r="YO9"/>
+      <c r="YP9"/>
+      <c r="YQ9"/>
+      <c r="YR9"/>
+      <c r="YS9"/>
+      <c r="YT9"/>
+      <c r="YU9"/>
+      <c r="YV9"/>
+      <c r="YW9"/>
+      <c r="YX9"/>
+      <c r="YY9"/>
+      <c r="YZ9"/>
+      <c r="ZA9"/>
+      <c r="ZB9"/>
+      <c r="ZC9"/>
+      <c r="ZD9"/>
+      <c r="ZE9"/>
+      <c r="ZF9"/>
+      <c r="ZG9"/>
+      <c r="ZH9"/>
+      <c r="ZI9"/>
+      <c r="ZJ9"/>
+      <c r="ZK9"/>
+      <c r="ZL9"/>
+      <c r="ZM9"/>
+      <c r="ZN9"/>
+      <c r="ZO9"/>
+      <c r="ZP9"/>
+      <c r="ZQ9"/>
+      <c r="ZR9"/>
+      <c r="ZS9"/>
+      <c r="ZT9"/>
+      <c r="ZU9"/>
+      <c r="ZV9"/>
+      <c r="ZW9"/>
+      <c r="ZX9"/>
+      <c r="ZY9"/>
+      <c r="ZZ9"/>
+      <c r="AAA9"/>
+      <c r="AAB9"/>
+      <c r="AAC9"/>
+      <c r="AAD9"/>
+      <c r="AAE9"/>
+      <c r="AAF9"/>
+      <c r="AAG9"/>
+      <c r="AAH9"/>
+      <c r="AAI9"/>
+      <c r="AAJ9"/>
+      <c r="AAK9"/>
+      <c r="AAL9"/>
+      <c r="AAM9"/>
+      <c r="AAN9"/>
+      <c r="AAO9"/>
+      <c r="AAP9"/>
+      <c r="AAQ9"/>
+      <c r="AAR9"/>
+      <c r="AAS9"/>
+      <c r="AAT9"/>
+      <c r="AAU9"/>
+      <c r="AAV9"/>
+      <c r="AAW9"/>
+      <c r="AAX9"/>
+      <c r="AAY9"/>
+      <c r="AAZ9"/>
+      <c r="ABA9"/>
+      <c r="ABB9"/>
+      <c r="ABC9"/>
+      <c r="ABD9"/>
+      <c r="ABE9"/>
+      <c r="ABF9"/>
+      <c r="ABG9"/>
+      <c r="ABH9"/>
+      <c r="ABI9"/>
+      <c r="ABJ9"/>
+      <c r="ABK9"/>
+      <c r="ABL9"/>
+      <c r="ABM9"/>
+      <c r="ABN9"/>
+      <c r="ABO9"/>
+      <c r="ABP9"/>
+      <c r="ABQ9"/>
+      <c r="ABR9"/>
+      <c r="ABS9"/>
+      <c r="ABT9"/>
+      <c r="ABU9"/>
+      <c r="ABV9"/>
+      <c r="ABW9"/>
+      <c r="ABX9"/>
+      <c r="ABY9"/>
+      <c r="ABZ9"/>
+      <c r="ACA9"/>
+      <c r="ACB9"/>
+      <c r="ACC9"/>
+      <c r="ACD9"/>
+      <c r="ACE9"/>
+      <c r="ACF9"/>
+      <c r="ACG9"/>
+      <c r="ACH9"/>
+      <c r="ACI9"/>
+      <c r="ACJ9"/>
+      <c r="ACK9"/>
+      <c r="ACL9"/>
+      <c r="ACM9"/>
+      <c r="ACN9"/>
+      <c r="ACO9"/>
+      <c r="ACP9"/>
+      <c r="ACQ9"/>
+      <c r="ACR9"/>
+      <c r="ACS9"/>
+      <c r="ACT9"/>
+      <c r="ACU9"/>
+      <c r="ACV9"/>
+      <c r="ACW9"/>
+      <c r="ACX9"/>
+      <c r="ACY9"/>
+      <c r="ACZ9"/>
+      <c r="ADA9"/>
+      <c r="ADB9"/>
+      <c r="ADC9"/>
+      <c r="ADD9"/>
+      <c r="ADE9"/>
+      <c r="ADF9"/>
+      <c r="ADG9"/>
+      <c r="ADH9"/>
+      <c r="ADI9"/>
+      <c r="ADJ9"/>
+      <c r="ADK9"/>
+      <c r="ADL9"/>
+      <c r="ADM9"/>
+      <c r="ADN9"/>
+      <c r="ADO9"/>
+      <c r="ADP9"/>
+      <c r="ADQ9"/>
+      <c r="ADR9"/>
+      <c r="ADS9"/>
+      <c r="ADT9"/>
+      <c r="ADU9"/>
+      <c r="ADV9"/>
+      <c r="ADW9"/>
+      <c r="ADX9"/>
+      <c r="ADY9"/>
+      <c r="ADZ9"/>
+      <c r="AEA9"/>
+      <c r="AEB9"/>
+      <c r="AEC9"/>
+      <c r="AED9"/>
+      <c r="AEE9"/>
+      <c r="AEF9"/>
+      <c r="AEG9"/>
+      <c r="AEH9"/>
+      <c r="AEI9"/>
+      <c r="AEJ9"/>
+      <c r="AEK9"/>
+      <c r="AEL9"/>
+      <c r="AEM9"/>
+      <c r="AEN9"/>
+      <c r="AEO9"/>
+      <c r="AEP9"/>
+      <c r="AEQ9"/>
+      <c r="AER9"/>
+      <c r="AES9"/>
+      <c r="AET9"/>
+      <c r="AEU9"/>
+      <c r="AEV9"/>
+      <c r="AEW9"/>
+      <c r="AEX9"/>
+      <c r="AEY9"/>
+      <c r="AEZ9"/>
+      <c r="AFA9"/>
+      <c r="AFB9"/>
+      <c r="AFC9"/>
+      <c r="AFD9"/>
+      <c r="AFE9"/>
+      <c r="AFF9"/>
+      <c r="AFG9"/>
+      <c r="AFH9"/>
+      <c r="AFI9"/>
+      <c r="AFJ9"/>
+      <c r="AFK9"/>
+      <c r="AFL9"/>
+      <c r="AFM9"/>
+      <c r="AFN9"/>
+      <c r="AFO9"/>
+      <c r="AFP9"/>
+      <c r="AFQ9"/>
+      <c r="AFR9"/>
+      <c r="AFS9"/>
+      <c r="AFT9"/>
+      <c r="AFU9"/>
+      <c r="AFV9"/>
+      <c r="AFW9"/>
+      <c r="AFX9"/>
+      <c r="AFY9"/>
+      <c r="AFZ9"/>
+      <c r="AGA9"/>
+      <c r="AGB9"/>
+      <c r="AGC9"/>
+      <c r="AGD9"/>
+      <c r="AGE9"/>
+      <c r="AGF9"/>
+      <c r="AGG9"/>
+      <c r="AGH9"/>
+      <c r="AGI9"/>
+      <c r="AGJ9"/>
+      <c r="AGK9"/>
+      <c r="AGL9"/>
+      <c r="AGM9"/>
+      <c r="AGN9"/>
+      <c r="AGO9"/>
+      <c r="AGP9"/>
+      <c r="AGQ9"/>
+      <c r="AGR9"/>
+      <c r="AGS9"/>
+      <c r="AGT9"/>
+      <c r="AGU9"/>
+      <c r="AGV9"/>
+      <c r="AGW9"/>
+      <c r="AGX9"/>
+      <c r="AGY9"/>
+      <c r="AGZ9"/>
+      <c r="AHA9"/>
+      <c r="AHB9"/>
+      <c r="AHC9"/>
+      <c r="AHD9"/>
+      <c r="AHE9"/>
+      <c r="AHF9"/>
+      <c r="AHG9"/>
+      <c r="AHH9"/>
+      <c r="AHI9"/>
+      <c r="AHJ9"/>
+      <c r="AHK9"/>
+      <c r="AHL9"/>
+      <c r="AHM9"/>
+      <c r="AHN9"/>
+      <c r="AHO9"/>
+      <c r="AHP9"/>
+      <c r="AHQ9"/>
+      <c r="AHR9"/>
+      <c r="AHS9"/>
+      <c r="AHT9"/>
+      <c r="AHU9"/>
+      <c r="AHV9"/>
+      <c r="AHW9"/>
+      <c r="AHX9"/>
+      <c r="AHY9"/>
+      <c r="AHZ9"/>
+      <c r="AIA9"/>
+      <c r="AIB9"/>
+      <c r="AIC9"/>
+      <c r="AID9"/>
+      <c r="AIE9"/>
+      <c r="AIF9"/>
+      <c r="AIG9"/>
+      <c r="AIH9"/>
+      <c r="AII9"/>
+      <c r="AIJ9"/>
+      <c r="AIK9"/>
+      <c r="AIL9"/>
+      <c r="AIM9"/>
+      <c r="AIN9"/>
+      <c r="AIO9"/>
+      <c r="AIP9"/>
+      <c r="AIQ9"/>
+      <c r="AIR9"/>
+      <c r="AIS9"/>
+      <c r="AIT9"/>
+      <c r="AIU9"/>
+      <c r="AIV9"/>
+      <c r="AIW9"/>
+      <c r="AIX9"/>
+      <c r="AIY9"/>
+      <c r="AIZ9"/>
+      <c r="AJA9"/>
+      <c r="AJB9"/>
+      <c r="AJC9"/>
+      <c r="AJD9"/>
+      <c r="AJE9"/>
+      <c r="AJF9"/>
+      <c r="AJG9"/>
+      <c r="AJH9"/>
+      <c r="AJI9"/>
+      <c r="AJJ9"/>
+      <c r="AJK9"/>
+      <c r="AJL9"/>
+      <c r="AJM9"/>
+      <c r="AJN9"/>
+      <c r="AJO9"/>
+      <c r="AJP9"/>
+      <c r="AJQ9"/>
+      <c r="AJR9"/>
+      <c r="AJS9"/>
+      <c r="AJT9"/>
+      <c r="AJU9"/>
+      <c r="AJV9"/>
+      <c r="AJW9"/>
+      <c r="AJX9"/>
+      <c r="AJY9"/>
+      <c r="AJZ9"/>
+      <c r="AKA9"/>
+      <c r="AKB9"/>
+      <c r="AKC9"/>
+      <c r="AKD9"/>
+      <c r="AKE9"/>
+      <c r="AKF9"/>
+      <c r="AKG9"/>
+      <c r="AKH9"/>
+      <c r="AKI9"/>
+      <c r="AKJ9"/>
+      <c r="AKK9"/>
+      <c r="AKL9"/>
+      <c r="AKM9"/>
+      <c r="AKN9"/>
+      <c r="AKO9"/>
+      <c r="AKP9"/>
+      <c r="AKQ9"/>
+      <c r="AKR9"/>
+      <c r="AKS9"/>
+      <c r="AKT9"/>
+      <c r="AKU9"/>
+      <c r="AKV9"/>
+      <c r="AKW9"/>
+      <c r="AKX9"/>
+      <c r="AKY9"/>
+      <c r="AKZ9"/>
+      <c r="ALA9"/>
+      <c r="ALB9"/>
+      <c r="ALC9"/>
+      <c r="ALD9"/>
+      <c r="ALE9"/>
+      <c r="ALF9"/>
+      <c r="ALG9"/>
+      <c r="ALH9"/>
+      <c r="ALI9"/>
+      <c r="ALJ9"/>
+      <c r="ALK9"/>
+      <c r="ALL9"/>
+      <c r="ALM9"/>
+      <c r="ALN9"/>
+      <c r="ALO9"/>
+      <c r="ALP9"/>
+      <c r="ALQ9"/>
+      <c r="ALR9"/>
+      <c r="ALS9"/>
+      <c r="ALT9"/>
+      <c r="ALU9"/>
+      <c r="ALV9"/>
+      <c r="ALW9"/>
+      <c r="ALX9"/>
+      <c r="ALY9"/>
+      <c r="ALZ9"/>
+      <c r="AMA9"/>
+      <c r="AMB9"/>
+      <c r="AMC9"/>
+      <c r="AMD9"/>
+      <c r="AME9"/>
+      <c r="AMF9"/>
+      <c r="AMG9"/>
+      <c r="AMH9"/>
+      <c r="AMI9"/>
+      <c r="AMJ9"/>
+      <c r="AMK9"/>
+      <c r="AML9"/>
+      <c r="AMM9"/>
+      <c r="AMN9"/>
+      <c r="AMO9"/>
+      <c r="AMP9"/>
+      <c r="AMQ9"/>
+      <c r="AMR9"/>
+      <c r="AMS9"/>
+      <c r="AMT9"/>
+      <c r="AMU9"/>
+      <c r="AMV9"/>
+      <c r="AMW9"/>
+      <c r="AMX9"/>
+      <c r="AMY9"/>
+      <c r="AMZ9"/>
+      <c r="ANA9"/>
+      <c r="ANB9"/>
+      <c r="ANC9"/>
+      <c r="AND9"/>
+      <c r="ANE9"/>
+      <c r="ANF9"/>
+      <c r="ANG9"/>
+      <c r="ANH9"/>
+      <c r="ANI9"/>
+      <c r="ANJ9"/>
+      <c r="ANK9"/>
+      <c r="ANL9"/>
+      <c r="ANM9"/>
+      <c r="ANN9"/>
+      <c r="ANO9"/>
+      <c r="ANP9"/>
+      <c r="ANQ9"/>
+      <c r="ANR9"/>
+      <c r="ANS9"/>
+      <c r="ANT9"/>
+      <c r="ANU9"/>
+      <c r="ANV9"/>
+      <c r="ANW9"/>
+      <c r="ANX9"/>
+      <c r="ANY9"/>
+      <c r="ANZ9"/>
+      <c r="AOA9"/>
+      <c r="AOB9"/>
+      <c r="AOC9"/>
+      <c r="AOD9"/>
+      <c r="AOE9"/>
+      <c r="AOF9"/>
+      <c r="AOG9"/>
+      <c r="AOH9"/>
+      <c r="AOI9"/>
+      <c r="AOJ9"/>
+      <c r="AOK9"/>
+      <c r="AOL9"/>
+      <c r="AOM9"/>
+      <c r="AON9"/>
+      <c r="AOO9"/>
+      <c r="AOP9"/>
+      <c r="AOQ9"/>
+      <c r="AOR9"/>
+      <c r="AOS9"/>
+      <c r="AOT9"/>
+      <c r="AOU9"/>
+      <c r="AOV9"/>
+      <c r="AOW9"/>
+      <c r="AOX9"/>
+      <c r="AOY9"/>
+      <c r="AOZ9"/>
+      <c r="APA9"/>
+      <c r="APB9"/>
+      <c r="APC9"/>
+      <c r="APD9"/>
+      <c r="APE9"/>
+      <c r="APF9"/>
+      <c r="APG9"/>
+      <c r="APH9"/>
+      <c r="API9"/>
+      <c r="APJ9"/>
+      <c r="APK9"/>
+      <c r="APL9"/>
+      <c r="APM9"/>
+      <c r="APN9"/>
+      <c r="APO9"/>
+      <c r="APP9"/>
+      <c r="APQ9"/>
+      <c r="APR9"/>
+      <c r="APS9"/>
+      <c r="APT9"/>
+      <c r="APU9"/>
+      <c r="APV9"/>
+      <c r="APW9"/>
+      <c r="APX9"/>
+      <c r="APY9"/>
+      <c r="APZ9"/>
+      <c r="AQA9"/>
+      <c r="AQB9"/>
+      <c r="AQC9"/>
+      <c r="AQD9"/>
+      <c r="AQE9"/>
+      <c r="AQF9"/>
+      <c r="AQG9"/>
+      <c r="AQH9"/>
+      <c r="AQI9"/>
+      <c r="AQJ9"/>
+      <c r="AQK9"/>
+      <c r="AQL9"/>
+      <c r="AQM9"/>
+      <c r="AQN9"/>
+      <c r="AQO9"/>
+      <c r="AQP9"/>
+      <c r="AQQ9"/>
+      <c r="AQR9"/>
+      <c r="AQS9"/>
+      <c r="AQT9"/>
+      <c r="AQU9"/>
+      <c r="AQV9"/>
+      <c r="AQW9"/>
+      <c r="AQX9"/>
+      <c r="AQY9"/>
+      <c r="AQZ9"/>
+      <c r="ARA9"/>
+      <c r="ARB9"/>
+      <c r="ARC9"/>
+      <c r="ARD9"/>
+      <c r="ARE9"/>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
updated business area test cases based on story#171 and #194
</commit_message>
<xml_diff>
--- a/testdata.xlsx
+++ b/testdata.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sshiwani\workspace\find-information-products-services-tests\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CF52F74F-C8C7-4680-9CCB-7A8939371F03}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A7442755-0F79-49B6-9FA8-E67CA91AD833}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="22780" windowHeight="14540" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="22780" windowHeight="14540" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="category_phase" sheetId="1" r:id="rId1"/>
@@ -48,7 +48,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="883" uniqueCount="446">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="889" uniqueCount="450">
   <si>
     <t>Search and filter products and services</t>
   </si>
@@ -260,42 +260,6 @@
     <t>#channel-web</t>
   </si>
   <si>
-    <t>products?group=families</t>
-  </si>
-  <si>
-    <t>ul.moj-filter-tags li a:has-text('families')</t>
-  </si>
-  <si>
-    <t>Remove this filter families</t>
-  </si>
-  <si>
-    <t>#group-families</t>
-  </si>
-  <si>
-    <t>ul.moj-filter-tags li a:has-text('regions')</t>
-  </si>
-  <si>
-    <t>Remove this filter regions</t>
-  </si>
-  <si>
-    <t>#group-regions</t>
-  </si>
-  <si>
-    <t>ul.moj-filter-tags li a:has-text('schools')</t>
-  </si>
-  <si>
-    <t>Remove this filter schools</t>
-  </si>
-  <si>
-    <t>#group-schools</t>
-  </si>
-  <si>
-    <t>products?group=schools</t>
-  </si>
-  <si>
-    <t>products?group=regions</t>
-  </si>
-  <si>
     <t>products?group=skills</t>
   </si>
   <si>
@@ -1386,6 +1350,54 @@
   </si>
   <si>
     <t>#phase-did-not-progress</t>
+  </si>
+  <si>
+    <t>products?group=children-and-families</t>
+  </si>
+  <si>
+    <t>ul.moj-filter-tags li a:has-text(' children-and-families')</t>
+  </si>
+  <si>
+    <t>Remove this filter children-and-families</t>
+  </si>
+  <si>
+    <t>#group-children-and-families</t>
+  </si>
+  <si>
+    <t>products?group=regional-digital-services</t>
+  </si>
+  <si>
+    <t>Remove this filter regional-digital-services</t>
+  </si>
+  <si>
+    <t>ul.moj-filter-tags li a:has-text(' regional-digital-services')</t>
+  </si>
+  <si>
+    <t>products?group=schools-digital</t>
+  </si>
+  <si>
+    <t>ul.moj-filter-tags li a:has-text(' schools-digital')</t>
+  </si>
+  <si>
+    <t>Remove this filter schools-digital</t>
+  </si>
+  <si>
+    <t>#group-schools-digital</t>
+  </si>
+  <si>
+    <t>products?group=sector-facing-services</t>
+  </si>
+  <si>
+    <t>ul.moj-filter-tags li a:has-text(' sector-facing-services')</t>
+  </si>
+  <si>
+    <t>Remove this filter sector-facing-services</t>
+  </si>
+  <si>
+    <t>#group-sector-facing-services</t>
+  </si>
+  <si>
+    <t>#group-regional-digital-services</t>
   </si>
 </sst>
 </file>
@@ -1407,7 +1419,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1435,6 +1447,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="6"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.59999389629810485"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1514,7 +1532,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
@@ -1525,6 +1543,7 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -4164,13 +4183,13 @@
     </row>
     <row r="4" spans="1:1149" s="5" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A4" s="3" t="s">
-        <v>442</v>
+        <v>430</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>443</v>
+        <v>431</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>444</v>
+        <v>432</v>
       </c>
       <c r="D4" s="3" t="s">
         <v>0</v>
@@ -4179,7 +4198,7 @@
         <v>1</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>445</v>
+        <v>433</v>
       </c>
       <c r="G4"/>
       <c r="H4"/>
@@ -11157,64 +11176,64 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" s="6" t="s">
-        <v>126</v>
+        <v>114</v>
       </c>
       <c r="B1" s="6" t="s">
-        <v>127</v>
+        <v>115</v>
       </c>
       <c r="C1" s="6" t="s">
-        <v>128</v>
+        <v>116</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" s="3" t="s">
-        <v>172</v>
+        <v>160</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>131</v>
+        <v>119</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>173</v>
+        <v>161</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="14" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B3" s="3" t="s">
-        <v>139</v>
+        <v>127</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>140</v>
+        <v>128</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.35">
       <c r="B4" s="3" t="s">
-        <v>137</v>
+        <v>125</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>138</v>
+        <v>126</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A5" s="3" t="s">
-        <v>174</v>
+        <v>162</v>
       </c>
       <c r="B5" s="3"/>
       <c r="C5" s="3"/>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A6" s="3" t="s">
-        <v>175</v>
+        <v>163</v>
       </c>
       <c r="B6" s="3"/>
       <c r="C6" s="3"/>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A7" s="3" t="s">
-        <v>176</v>
+        <v>164</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A8" s="3" t="s">
-        <v>177</v>
+        <v>165</v>
       </c>
     </row>
   </sheetData>
@@ -11234,78 +11253,78 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" s="6" t="s">
-        <v>126</v>
+        <v>114</v>
       </c>
       <c r="B1" s="6" t="s">
-        <v>127</v>
+        <v>115</v>
       </c>
       <c r="C1" s="6" t="s">
-        <v>128</v>
+        <v>116</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" s="3" t="s">
-        <v>178</v>
+        <v>166</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>131</v>
+        <v>119</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>179</v>
+        <v>167</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="14" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B3" s="3" t="s">
-        <v>139</v>
+        <v>127</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>140</v>
+        <v>128</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.35">
       <c r="B4" s="3" t="s">
-        <v>137</v>
+        <v>125</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>138</v>
+        <v>126</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A5" s="3" t="s">
-        <v>180</v>
+        <v>168</v>
       </c>
       <c r="B5" s="3"/>
       <c r="C5" s="3"/>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A6" s="3" t="s">
-        <v>181</v>
+        <v>169</v>
       </c>
       <c r="B6" s="3"/>
       <c r="C6" s="3"/>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A7" s="3" t="s">
-        <v>182</v>
+        <v>170</v>
       </c>
       <c r="B7" s="3"/>
       <c r="C7" s="3"/>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A8" s="3" t="s">
-        <v>183</v>
+        <v>171</v>
       </c>
       <c r="B8" s="3"/>
       <c r="C8" s="3"/>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A9" s="3" t="s">
-        <v>184</v>
+        <v>172</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A10" s="3" t="s">
-        <v>185</v>
+        <v>173</v>
       </c>
     </row>
   </sheetData>
@@ -11326,78 +11345,78 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" s="6" t="s">
-        <v>126</v>
+        <v>114</v>
       </c>
       <c r="B1" s="6" t="s">
-        <v>127</v>
+        <v>115</v>
       </c>
       <c r="C1" s="6" t="s">
-        <v>128</v>
+        <v>116</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" s="3" t="s">
-        <v>186</v>
+        <v>174</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>131</v>
+        <v>119</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>187</v>
+        <v>175</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="14" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B3" s="3" t="s">
-        <v>139</v>
+        <v>127</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>140</v>
+        <v>128</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.35">
       <c r="B4" s="3" t="s">
-        <v>137</v>
+        <v>125</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>138</v>
+        <v>126</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A5" s="3" t="s">
-        <v>188</v>
+        <v>176</v>
       </c>
       <c r="B5" s="3"/>
       <c r="C5" s="3"/>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A6" s="3" t="s">
-        <v>189</v>
+        <v>177</v>
       </c>
       <c r="B6" s="3"/>
       <c r="C6" s="3"/>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A7" s="3" t="s">
-        <v>190</v>
+        <v>178</v>
       </c>
       <c r="B7" s="3"/>
       <c r="C7" s="3"/>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A8" s="3" t="s">
-        <v>191</v>
+        <v>179</v>
       </c>
       <c r="B8" s="3"/>
       <c r="C8" s="3"/>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A9" s="3" t="s">
-        <v>192</v>
+        <v>180</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A10" s="3" t="s">
-        <v>193</v>
+        <v>181</v>
       </c>
     </row>
   </sheetData>
@@ -11417,99 +11436,99 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" s="6" t="s">
-        <v>126</v>
+        <v>114</v>
       </c>
       <c r="B1" s="6" t="s">
-        <v>127</v>
+        <v>115</v>
       </c>
       <c r="C1" s="6" t="s">
-        <v>128</v>
+        <v>116</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" s="3" t="s">
-        <v>194</v>
+        <v>182</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>131</v>
+        <v>119</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>195</v>
+        <v>183</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="14" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B3" s="3" t="s">
-        <v>139</v>
+        <v>127</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>140</v>
+        <v>128</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.35">
       <c r="B4" s="3" t="s">
-        <v>137</v>
+        <v>125</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>138</v>
+        <v>126</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A5" s="3" t="s">
-        <v>196</v>
+        <v>184</v>
       </c>
       <c r="B5" s="3"/>
       <c r="C5" s="3"/>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A6" s="3" t="s">
-        <v>197</v>
+        <v>185</v>
       </c>
       <c r="B6" s="3"/>
       <c r="C6" s="3"/>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A7" s="3" t="s">
-        <v>198</v>
+        <v>186</v>
       </c>
       <c r="B7" s="3"/>
       <c r="C7" s="3"/>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A8" s="3" t="s">
-        <v>199</v>
+        <v>187</v>
       </c>
       <c r="B8" s="3"/>
       <c r="C8" s="3"/>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A9" s="3" t="s">
-        <v>200</v>
+        <v>188</v>
       </c>
       <c r="B9" s="3"/>
       <c r="C9" s="3"/>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A10" s="3" t="s">
-        <v>201</v>
+        <v>189</v>
       </c>
       <c r="B10" s="3"/>
       <c r="C10" s="3"/>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A11" s="3" t="s">
-        <v>202</v>
+        <v>190</v>
       </c>
       <c r="B11" s="3"/>
       <c r="C11" s="3"/>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A12" s="3" t="s">
-        <v>203</v>
+        <v>191</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A13" s="3" t="s">
-        <v>204</v>
+        <v>192</v>
       </c>
     </row>
   </sheetData>
@@ -11529,85 +11548,85 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" s="6" t="s">
-        <v>126</v>
+        <v>114</v>
       </c>
       <c r="B1" s="6" t="s">
-        <v>127</v>
+        <v>115</v>
       </c>
       <c r="C1" s="6" t="s">
-        <v>128</v>
+        <v>116</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" s="3" t="s">
-        <v>205</v>
+        <v>193</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>131</v>
+        <v>119</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>206</v>
+        <v>194</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="14" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B3" s="3" t="s">
-        <v>139</v>
+        <v>127</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>140</v>
+        <v>128</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.35">
       <c r="B4" s="3" t="s">
-        <v>137</v>
+        <v>125</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>138</v>
+        <v>126</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A5" s="3" t="s">
-        <v>207</v>
+        <v>195</v>
       </c>
       <c r="B5" s="3"/>
       <c r="C5" s="3"/>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A6" s="3" t="s">
-        <v>208</v>
+        <v>196</v>
       </c>
       <c r="B6" s="3"/>
       <c r="C6" s="3"/>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A7" s="3" t="s">
-        <v>209</v>
+        <v>197</v>
       </c>
       <c r="B7" s="3"/>
       <c r="C7" s="3"/>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A8" s="3" t="s">
-        <v>210</v>
+        <v>198</v>
       </c>
       <c r="B8" s="3"/>
       <c r="C8" s="3"/>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A9" s="3" t="s">
-        <v>211</v>
+        <v>199</v>
       </c>
       <c r="B9" s="3"/>
       <c r="C9" s="3"/>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A10" s="3" t="s">
-        <v>212</v>
+        <v>200</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A11" s="3" t="s">
-        <v>213</v>
+        <v>201</v>
       </c>
     </row>
   </sheetData>
@@ -11627,99 +11646,99 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" s="6" t="s">
-        <v>126</v>
+        <v>114</v>
       </c>
       <c r="B1" s="6" t="s">
-        <v>127</v>
+        <v>115</v>
       </c>
       <c r="C1" s="6" t="s">
-        <v>128</v>
+        <v>116</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" s="3" t="s">
-        <v>214</v>
+        <v>202</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>131</v>
+        <v>119</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>215</v>
+        <v>203</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="14" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B3" s="3" t="s">
-        <v>139</v>
+        <v>127</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>140</v>
+        <v>128</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.35">
       <c r="B4" s="3" t="s">
-        <v>137</v>
+        <v>125</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>138</v>
+        <v>126</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A5" s="3" t="s">
-        <v>216</v>
+        <v>204</v>
       </c>
       <c r="B5" s="3"/>
       <c r="C5" s="3"/>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A6" s="3" t="s">
-        <v>217</v>
+        <v>205</v>
       </c>
       <c r="B6" s="3"/>
       <c r="C6" s="3"/>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A7" s="3" t="s">
-        <v>218</v>
+        <v>206</v>
       </c>
       <c r="B7" s="3"/>
       <c r="C7" s="3"/>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A8" s="3" t="s">
-        <v>219</v>
+        <v>207</v>
       </c>
       <c r="B8" s="3"/>
       <c r="C8" s="3"/>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A9" s="3" t="s">
-        <v>220</v>
+        <v>208</v>
       </c>
       <c r="B9" s="3"/>
       <c r="C9" s="3"/>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A10" s="3" t="s">
-        <v>221</v>
+        <v>209</v>
       </c>
       <c r="B10" s="3"/>
       <c r="C10" s="3"/>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A11" s="3" t="s">
-        <v>222</v>
+        <v>210</v>
       </c>
       <c r="B11" s="3"/>
       <c r="C11" s="3"/>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A12" s="3" t="s">
-        <v>223</v>
+        <v>211</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A13" s="3" t="s">
-        <v>224</v>
+        <v>212</v>
       </c>
     </row>
   </sheetData>
@@ -11762,36 +11781,36 @@
         <v>35</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>234</v>
+        <v>222</v>
       </c>
       <c r="H1" s="2" t="s">
-        <v>235</v>
+        <v>223</v>
       </c>
     </row>
     <row r="2" spans="1:229" s="4" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A2" s="3" t="s">
-        <v>229</v>
+        <v>217</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>228</v>
+        <v>216</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>225</v>
+        <v>213</v>
       </c>
       <c r="D2" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>226</v>
+        <v>214</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>227</v>
+        <v>215</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>236</v>
+        <v>224</v>
       </c>
       <c r="H2" s="3" t="s">
-        <v>132</v>
+        <v>120</v>
       </c>
       <c r="I2"/>
       <c r="J2"/>
@@ -12017,106 +12036,106 @@
     </row>
     <row r="3" spans="1:229" x14ac:dyDescent="0.35">
       <c r="A3" s="3" t="s">
-        <v>230</v>
+        <v>218</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>232</v>
+        <v>220</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>233</v>
+        <v>221</v>
       </c>
       <c r="D3" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E3" s="3" t="s">
+        <v>214</v>
+      </c>
+      <c r="F3" s="3" t="s">
+        <v>215</v>
+      </c>
+      <c r="G3" s="3" t="s">
+        <v>225</v>
+      </c>
+      <c r="H3" s="3" t="s">
         <v>226</v>
-      </c>
-      <c r="F3" s="3" t="s">
-        <v>227</v>
-      </c>
-      <c r="G3" s="3" t="s">
-        <v>237</v>
-      </c>
-      <c r="H3" s="3" t="s">
-        <v>238</v>
       </c>
     </row>
     <row r="4" spans="1:229" x14ac:dyDescent="0.35">
       <c r="A4" s="3" t="s">
-        <v>231</v>
+        <v>219</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>239</v>
+        <v>227</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>240</v>
+        <v>228</v>
       </c>
       <c r="D4" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>226</v>
+        <v>214</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>227</v>
+        <v>215</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>241</v>
+        <v>229</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>242</v>
+        <v>230</v>
       </c>
     </row>
     <row r="5" spans="1:229" x14ac:dyDescent="0.35">
       <c r="A5" s="3" t="s">
-        <v>243</v>
+        <v>231</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>244</v>
+        <v>232</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>245</v>
+        <v>233</v>
       </c>
       <c r="D5" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>226</v>
+        <v>214</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>227</v>
+        <v>215</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>246</v>
+        <v>234</v>
       </c>
       <c r="H5" s="3" t="s">
-        <v>247</v>
+        <v>235</v>
       </c>
     </row>
     <row r="6" spans="1:229" x14ac:dyDescent="0.35">
       <c r="A6" s="3" t="s">
-        <v>248</v>
+        <v>236</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>249</v>
+        <v>237</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>250</v>
+        <v>238</v>
       </c>
       <c r="D6" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>226</v>
+        <v>214</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>227</v>
+        <v>215</v>
       </c>
       <c r="G6" s="3" t="s">
-        <v>251</v>
+        <v>239</v>
       </c>
       <c r="H6" s="3" t="s">
-        <v>252</v>
+        <v>240</v>
       </c>
     </row>
   </sheetData>
@@ -12160,36 +12179,36 @@
         <v>35</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>234</v>
+        <v>222</v>
       </c>
       <c r="H1" s="2" t="s">
-        <v>235</v>
+        <v>223</v>
       </c>
     </row>
     <row r="2" spans="1:229" s="4" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A2" s="3" t="s">
-        <v>253</v>
+        <v>241</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>254</v>
+        <v>242</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>255</v>
+        <v>243</v>
       </c>
       <c r="D2" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>226</v>
+        <v>214</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>227</v>
+        <v>215</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>236</v>
+        <v>224</v>
       </c>
       <c r="H2" s="3" t="s">
-        <v>143</v>
+        <v>131</v>
       </c>
       <c r="I2"/>
       <c r="J2"/>
@@ -12415,80 +12434,80 @@
     </row>
     <row r="3" spans="1:229" x14ac:dyDescent="0.35">
       <c r="A3" s="3" t="s">
-        <v>256</v>
+        <v>244</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>257</v>
+        <v>245</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>258</v>
+        <v>246</v>
       </c>
       <c r="D3" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>226</v>
+        <v>214</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>227</v>
+        <v>215</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>236</v>
+        <v>224</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>259</v>
+        <v>247</v>
       </c>
     </row>
     <row r="4" spans="1:229" x14ac:dyDescent="0.35">
       <c r="A4" s="3" t="s">
-        <v>260</v>
+        <v>248</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>261</v>
+        <v>249</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>262</v>
+        <v>250</v>
       </c>
       <c r="D4" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>226</v>
+        <v>214</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>227</v>
+        <v>215</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>236</v>
+        <v>224</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>263</v>
+        <v>251</v>
       </c>
     </row>
     <row r="5" spans="1:229" x14ac:dyDescent="0.35">
       <c r="A5" s="3" t="s">
-        <v>264</v>
+        <v>252</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>265</v>
+        <v>253</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>266</v>
+        <v>254</v>
       </c>
       <c r="D5" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>226</v>
+        <v>214</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>227</v>
+        <v>215</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>236</v>
+        <v>224</v>
       </c>
       <c r="H5" s="3" t="s">
-        <v>267</v>
+        <v>255</v>
       </c>
     </row>
   </sheetData>
@@ -12531,36 +12550,36 @@
         <v>35</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>234</v>
+        <v>222</v>
       </c>
       <c r="H1" s="2" t="s">
-        <v>235</v>
+        <v>223</v>
       </c>
     </row>
     <row r="2" spans="1:229" s="4" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A2" s="3" t="s">
-        <v>268</v>
+        <v>256</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>269</v>
+        <v>257</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>270</v>
+        <v>258</v>
       </c>
       <c r="D2" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>226</v>
+        <v>214</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>227</v>
+        <v>215</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>236</v>
+        <v>224</v>
       </c>
       <c r="H2" s="3" t="s">
-        <v>152</v>
+        <v>140</v>
       </c>
       <c r="I2"/>
       <c r="J2"/>
@@ -12786,132 +12805,132 @@
     </row>
     <row r="3" spans="1:229" x14ac:dyDescent="0.35">
       <c r="A3" s="3" t="s">
-        <v>271</v>
+        <v>259</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>272</v>
+        <v>260</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>273</v>
+        <v>261</v>
       </c>
       <c r="D3" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>226</v>
+        <v>214</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>227</v>
+        <v>215</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>236</v>
+        <v>224</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>274</v>
+        <v>262</v>
       </c>
     </row>
     <row r="4" spans="1:229" x14ac:dyDescent="0.35">
       <c r="A4" s="3" t="s">
-        <v>275</v>
+        <v>263</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>277</v>
+        <v>265</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>276</v>
+        <v>264</v>
       </c>
       <c r="D4" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>226</v>
+        <v>214</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>227</v>
+        <v>215</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>236</v>
+        <v>224</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>278</v>
+        <v>266</v>
       </c>
     </row>
     <row r="5" spans="1:229" x14ac:dyDescent="0.35">
       <c r="A5" s="8" t="s">
-        <v>279</v>
+        <v>267</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>280</v>
+        <v>268</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>281</v>
+        <v>269</v>
       </c>
       <c r="D5" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>226</v>
+        <v>214</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>227</v>
+        <v>215</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>236</v>
+        <v>224</v>
       </c>
       <c r="H5" s="3" t="s">
-        <v>282</v>
+        <v>270</v>
       </c>
     </row>
     <row r="6" spans="1:229" x14ac:dyDescent="0.35">
       <c r="A6" s="3" t="s">
-        <v>283</v>
+        <v>271</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>284</v>
+        <v>272</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>285</v>
+        <v>273</v>
       </c>
       <c r="D6" s="7" t="s">
         <v>0</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>226</v>
+        <v>214</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>227</v>
+        <v>215</v>
       </c>
       <c r="G6" s="3" t="s">
-        <v>236</v>
+        <v>224</v>
       </c>
       <c r="H6" s="3" t="s">
-        <v>286</v>
+        <v>274</v>
       </c>
     </row>
     <row r="7" spans="1:229" x14ac:dyDescent="0.35">
       <c r="A7" s="3" t="s">
-        <v>287</v>
+        <v>275</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>289</v>
+        <v>277</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>288</v>
+        <v>276</v>
       </c>
       <c r="D7" s="7" t="s">
         <v>0</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>226</v>
+        <v>214</v>
       </c>
       <c r="F7" s="3" t="s">
-        <v>227</v>
+        <v>215</v>
       </c>
       <c r="G7" s="3" t="s">
-        <v>236</v>
+        <v>224</v>
       </c>
       <c r="H7" s="3" t="s">
-        <v>290</v>
+        <v>278</v>
       </c>
     </row>
   </sheetData>
@@ -12955,36 +12974,36 @@
         <v>35</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>234</v>
+        <v>222</v>
       </c>
       <c r="H1" s="2" t="s">
-        <v>235</v>
+        <v>223</v>
       </c>
     </row>
     <row r="2" spans="1:229" s="4" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A2" s="3" t="s">
-        <v>291</v>
+        <v>279</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>292</v>
+        <v>280</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>293</v>
+        <v>281</v>
       </c>
       <c r="D2" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>226</v>
+        <v>214</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>227</v>
+        <v>215</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>236</v>
+        <v>224</v>
       </c>
       <c r="H2" s="3" t="s">
-        <v>157</v>
+        <v>145</v>
       </c>
       <c r="I2"/>
       <c r="J2"/>
@@ -13210,106 +13229,106 @@
     </row>
     <row r="3" spans="1:229" x14ac:dyDescent="0.35">
       <c r="A3" s="3" t="s">
-        <v>294</v>
+        <v>282</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>295</v>
+        <v>283</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>296</v>
+        <v>284</v>
       </c>
       <c r="D3" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>226</v>
+        <v>214</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>227</v>
+        <v>215</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>236</v>
+        <v>224</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>297</v>
+        <v>285</v>
       </c>
     </row>
     <row r="4" spans="1:229" x14ac:dyDescent="0.35">
       <c r="A4" s="3" t="s">
-        <v>298</v>
+        <v>286</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>299</v>
+        <v>287</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>300</v>
+        <v>288</v>
       </c>
       <c r="D4" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>226</v>
+        <v>214</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>227</v>
+        <v>215</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>236</v>
+        <v>224</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>301</v>
+        <v>289</v>
       </c>
     </row>
     <row r="5" spans="1:229" x14ac:dyDescent="0.35">
       <c r="A5" s="8" t="s">
-        <v>302</v>
+        <v>290</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>303</v>
+        <v>291</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>304</v>
+        <v>292</v>
       </c>
       <c r="D5" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>226</v>
+        <v>214</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>227</v>
+        <v>215</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>236</v>
+        <v>224</v>
       </c>
       <c r="H5" s="3" t="s">
-        <v>305</v>
+        <v>293</v>
       </c>
     </row>
     <row r="6" spans="1:229" x14ac:dyDescent="0.35">
       <c r="A6" s="3" t="s">
-        <v>306</v>
+        <v>294</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>307</v>
+        <v>295</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>308</v>
+        <v>296</v>
       </c>
       <c r="D6" s="7" t="s">
         <v>0</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>226</v>
+        <v>214</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>227</v>
+        <v>215</v>
       </c>
       <c r="G6" s="3" t="s">
-        <v>236</v>
+        <v>224</v>
       </c>
       <c r="H6" s="3" t="s">
-        <v>309</v>
+        <v>297</v>
       </c>
     </row>
   </sheetData>
@@ -13375,7 +13394,7 @@
         <v>41</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>125</v>
+        <v>113</v>
       </c>
       <c r="C3" s="3" t="s">
         <v>42</v>
@@ -13415,10 +13434,10 @@
         <v>48</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>115</v>
+        <v>103</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>116</v>
+        <v>104</v>
       </c>
       <c r="D5" s="3" t="s">
         <v>0</v>
@@ -13570,36 +13589,36 @@
         <v>35</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>234</v>
+        <v>222</v>
       </c>
       <c r="H1" s="2" t="s">
-        <v>235</v>
+        <v>223</v>
       </c>
     </row>
     <row r="2" spans="1:229" s="4" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A2" s="3" t="s">
-        <v>310</v>
+        <v>298</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>311</v>
+        <v>299</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>312</v>
+        <v>300</v>
       </c>
       <c r="D2" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>226</v>
+        <v>214</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>227</v>
+        <v>215</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>236</v>
+        <v>224</v>
       </c>
       <c r="H2" s="3" t="s">
-        <v>174</v>
+        <v>162</v>
       </c>
       <c r="I2"/>
       <c r="J2"/>
@@ -13825,80 +13844,80 @@
     </row>
     <row r="3" spans="1:229" x14ac:dyDescent="0.35">
       <c r="A3" s="3" t="s">
-        <v>313</v>
+        <v>301</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>314</v>
+        <v>302</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>315</v>
+        <v>303</v>
       </c>
       <c r="D3" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>226</v>
+        <v>214</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>227</v>
+        <v>215</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>236</v>
+        <v>224</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>316</v>
+        <v>304</v>
       </c>
     </row>
     <row r="4" spans="1:229" x14ac:dyDescent="0.35">
       <c r="A4" s="3" t="s">
-        <v>317</v>
+        <v>305</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>318</v>
+        <v>306</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>319</v>
+        <v>307</v>
       </c>
       <c r="D4" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>226</v>
+        <v>214</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>227</v>
+        <v>215</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>236</v>
+        <v>224</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>320</v>
+        <v>308</v>
       </c>
     </row>
     <row r="5" spans="1:229" x14ac:dyDescent="0.35">
       <c r="A5" s="3" t="s">
-        <v>321</v>
+        <v>309</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>322</v>
+        <v>310</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>323</v>
+        <v>311</v>
       </c>
       <c r="D5" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>226</v>
+        <v>214</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>227</v>
+        <v>215</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>236</v>
+        <v>224</v>
       </c>
       <c r="H5" s="3" t="s">
-        <v>324</v>
+        <v>312</v>
       </c>
     </row>
   </sheetData>
@@ -13941,36 +13960,36 @@
         <v>35</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>234</v>
+        <v>222</v>
       </c>
       <c r="H1" s="2" t="s">
-        <v>235</v>
+        <v>223</v>
       </c>
     </row>
     <row r="2" spans="1:229" s="4" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A2" s="3" t="s">
-        <v>325</v>
+        <v>313</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>326</v>
+        <v>314</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>327</v>
+        <v>315</v>
       </c>
       <c r="D2" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>226</v>
+        <v>214</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>227</v>
+        <v>215</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>236</v>
+        <v>224</v>
       </c>
       <c r="H2" s="3" t="s">
-        <v>180</v>
+        <v>168</v>
       </c>
       <c r="I2"/>
       <c r="J2"/>
@@ -14196,132 +14215,132 @@
     </row>
     <row r="3" spans="1:229" x14ac:dyDescent="0.35">
       <c r="A3" s="3" t="s">
-        <v>328</v>
+        <v>316</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>329</v>
+        <v>317</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>330</v>
+        <v>318</v>
       </c>
       <c r="D3" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>226</v>
+        <v>214</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>227</v>
+        <v>215</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>236</v>
+        <v>224</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>331</v>
+        <v>319</v>
       </c>
     </row>
     <row r="4" spans="1:229" x14ac:dyDescent="0.35">
       <c r="A4" s="3" t="s">
-        <v>332</v>
+        <v>320</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>333</v>
+        <v>321</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>334</v>
+        <v>322</v>
       </c>
       <c r="D4" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>226</v>
+        <v>214</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>227</v>
+        <v>215</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>236</v>
+        <v>224</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>335</v>
+        <v>323</v>
       </c>
     </row>
     <row r="5" spans="1:229" x14ac:dyDescent="0.35">
       <c r="A5" s="8" t="s">
-        <v>336</v>
+        <v>324</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>337</v>
+        <v>325</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>338</v>
+        <v>326</v>
       </c>
       <c r="D5" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>226</v>
+        <v>214</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>227</v>
+        <v>215</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>236</v>
+        <v>224</v>
       </c>
       <c r="H5" s="3" t="s">
-        <v>339</v>
+        <v>327</v>
       </c>
     </row>
     <row r="6" spans="1:229" x14ac:dyDescent="0.35">
       <c r="A6" s="3" t="s">
-        <v>340</v>
+        <v>328</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>342</v>
+        <v>330</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>341</v>
+        <v>329</v>
       </c>
       <c r="D6" s="7" t="s">
         <v>0</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>226</v>
+        <v>214</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>227</v>
+        <v>215</v>
       </c>
       <c r="G6" s="3" t="s">
-        <v>236</v>
+        <v>224</v>
       </c>
       <c r="H6" s="3" t="s">
-        <v>343</v>
+        <v>331</v>
       </c>
     </row>
     <row r="7" spans="1:229" x14ac:dyDescent="0.35">
       <c r="A7" s="3" t="s">
-        <v>344</v>
+        <v>332</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>345</v>
+        <v>333</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>346</v>
+        <v>334</v>
       </c>
       <c r="D7" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>226</v>
+        <v>214</v>
       </c>
       <c r="F7" s="3" t="s">
-        <v>227</v>
+        <v>215</v>
       </c>
       <c r="G7" s="3" t="s">
-        <v>236</v>
+        <v>224</v>
       </c>
       <c r="H7" s="3" t="s">
-        <v>347</v>
+        <v>335</v>
       </c>
     </row>
   </sheetData>
@@ -14364,36 +14383,36 @@
         <v>35</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>234</v>
+        <v>222</v>
       </c>
       <c r="H1" s="2" t="s">
-        <v>235</v>
+        <v>223</v>
       </c>
     </row>
     <row r="2" spans="1:229" s="4" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A2" s="3" t="s">
-        <v>348</v>
+        <v>336</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>349</v>
+        <v>337</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>350</v>
+        <v>338</v>
       </c>
       <c r="D2" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>226</v>
+        <v>214</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>227</v>
+        <v>215</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>236</v>
+        <v>224</v>
       </c>
       <c r="H2" s="3" t="s">
-        <v>188</v>
+        <v>176</v>
       </c>
       <c r="I2"/>
       <c r="J2"/>
@@ -14619,132 +14638,132 @@
     </row>
     <row r="3" spans="1:229" x14ac:dyDescent="0.35">
       <c r="A3" s="3" t="s">
-        <v>351</v>
+        <v>339</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>352</v>
+        <v>340</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>353</v>
+        <v>341</v>
       </c>
       <c r="D3" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>226</v>
+        <v>214</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>227</v>
+        <v>215</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>236</v>
+        <v>224</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>354</v>
+        <v>342</v>
       </c>
     </row>
     <row r="4" spans="1:229" x14ac:dyDescent="0.35">
       <c r="A4" s="3" t="s">
-        <v>355</v>
+        <v>343</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>357</v>
+        <v>345</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>356</v>
+        <v>344</v>
       </c>
       <c r="D4" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>226</v>
+        <v>214</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>227</v>
+        <v>215</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>236</v>
+        <v>224</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>358</v>
+        <v>346</v>
       </c>
     </row>
     <row r="5" spans="1:229" x14ac:dyDescent="0.35">
       <c r="A5" s="8" t="s">
-        <v>359</v>
+        <v>347</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>360</v>
+        <v>348</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>361</v>
+        <v>349</v>
       </c>
       <c r="D5" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>226</v>
+        <v>214</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>227</v>
+        <v>215</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>236</v>
+        <v>224</v>
       </c>
       <c r="H5" s="3" t="s">
-        <v>362</v>
+        <v>350</v>
       </c>
     </row>
     <row r="6" spans="1:229" x14ac:dyDescent="0.35">
       <c r="A6" s="3" t="s">
-        <v>363</v>
+        <v>351</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>365</v>
+        <v>353</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>364</v>
+        <v>352</v>
       </c>
       <c r="D6" s="7" t="s">
         <v>0</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>226</v>
+        <v>214</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>227</v>
+        <v>215</v>
       </c>
       <c r="G6" s="3" t="s">
-        <v>236</v>
+        <v>224</v>
       </c>
       <c r="H6" s="3" t="s">
-        <v>366</v>
+        <v>354</v>
       </c>
     </row>
     <row r="7" spans="1:229" x14ac:dyDescent="0.35">
       <c r="A7" s="3" t="s">
-        <v>367</v>
+        <v>355</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>368</v>
+        <v>356</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>369</v>
+        <v>357</v>
       </c>
       <c r="D7" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>226</v>
+        <v>214</v>
       </c>
       <c r="F7" s="3" t="s">
-        <v>227</v>
+        <v>215</v>
       </c>
       <c r="G7" s="3" t="s">
-        <v>236</v>
+        <v>224</v>
       </c>
       <c r="H7" s="3" t="s">
-        <v>370</v>
+        <v>358</v>
       </c>
     </row>
   </sheetData>
@@ -14787,36 +14806,36 @@
         <v>35</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>234</v>
+        <v>222</v>
       </c>
       <c r="H1" s="2" t="s">
-        <v>235</v>
+        <v>223</v>
       </c>
     </row>
     <row r="2" spans="1:229" s="4" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A2" s="3" t="s">
-        <v>380</v>
+        <v>368</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>381</v>
+        <v>369</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>382</v>
+        <v>370</v>
       </c>
       <c r="D2" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>226</v>
+        <v>214</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>227</v>
+        <v>215</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>236</v>
+        <v>224</v>
       </c>
       <c r="H2" s="3" t="s">
-        <v>196</v>
+        <v>184</v>
       </c>
       <c r="I2"/>
       <c r="J2"/>
@@ -15042,210 +15061,210 @@
     </row>
     <row r="3" spans="1:229" x14ac:dyDescent="0.35">
       <c r="A3" s="3" t="s">
-        <v>383</v>
+        <v>371</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>384</v>
+        <v>372</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>385</v>
+        <v>373</v>
       </c>
       <c r="D3" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>226</v>
+        <v>214</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>227</v>
+        <v>215</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>236</v>
+        <v>224</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>386</v>
+        <v>374</v>
       </c>
     </row>
     <row r="4" spans="1:229" x14ac:dyDescent="0.35">
       <c r="A4" s="3" t="s">
-        <v>387</v>
+        <v>375</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>388</v>
+        <v>376</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>389</v>
+        <v>377</v>
       </c>
       <c r="D4" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>226</v>
+        <v>214</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>227</v>
+        <v>215</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>236</v>
+        <v>224</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>390</v>
+        <v>378</v>
       </c>
     </row>
     <row r="5" spans="1:229" x14ac:dyDescent="0.35">
       <c r="A5" s="8" t="s">
-        <v>391</v>
+        <v>379</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>392</v>
+        <v>380</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>393</v>
+        <v>381</v>
       </c>
       <c r="D5" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>226</v>
+        <v>214</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>227</v>
+        <v>215</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>236</v>
+        <v>224</v>
       </c>
       <c r="H5" s="3" t="s">
-        <v>394</v>
+        <v>382</v>
       </c>
     </row>
     <row r="6" spans="1:229" x14ac:dyDescent="0.35">
       <c r="A6" s="3" t="s">
-        <v>395</v>
+        <v>383</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>396</v>
+        <v>384</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>397</v>
+        <v>385</v>
       </c>
       <c r="D6" s="7" t="s">
         <v>0</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>226</v>
+        <v>214</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>227</v>
+        <v>215</v>
       </c>
       <c r="G6" s="3" t="s">
-        <v>236</v>
+        <v>224</v>
       </c>
       <c r="H6" s="3" t="s">
-        <v>398</v>
+        <v>386</v>
       </c>
     </row>
     <row r="7" spans="1:229" x14ac:dyDescent="0.35">
       <c r="A7" s="3" t="s">
-        <v>399</v>
+        <v>387</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>400</v>
+        <v>388</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>401</v>
+        <v>389</v>
       </c>
       <c r="D7" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>226</v>
+        <v>214</v>
       </c>
       <c r="F7" s="3" t="s">
-        <v>227</v>
+        <v>215</v>
       </c>
       <c r="G7" s="3" t="s">
-        <v>236</v>
+        <v>224</v>
       </c>
       <c r="H7" s="3" t="s">
-        <v>402</v>
+        <v>390</v>
       </c>
     </row>
     <row r="8" spans="1:229" x14ac:dyDescent="0.35">
       <c r="A8" s="3" t="s">
-        <v>403</v>
+        <v>391</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>404</v>
+        <v>392</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>405</v>
+        <v>393</v>
       </c>
       <c r="D8" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E8" s="3" t="s">
-        <v>226</v>
+        <v>214</v>
       </c>
       <c r="F8" s="3" t="s">
-        <v>227</v>
+        <v>215</v>
       </c>
       <c r="G8" s="3" t="s">
-        <v>236</v>
+        <v>224</v>
       </c>
       <c r="H8" s="3" t="s">
-        <v>406</v>
+        <v>394</v>
       </c>
     </row>
     <row r="9" spans="1:229" x14ac:dyDescent="0.35">
       <c r="A9" s="3" t="s">
-        <v>407</v>
+        <v>395</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>408</v>
+        <v>396</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>409</v>
+        <v>397</v>
       </c>
       <c r="D9" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E9" s="3" t="s">
-        <v>226</v>
+        <v>214</v>
       </c>
       <c r="F9" s="3" t="s">
-        <v>227</v>
+        <v>215</v>
       </c>
       <c r="G9" s="3" t="s">
-        <v>236</v>
+        <v>224</v>
       </c>
       <c r="H9" s="3" t="s">
-        <v>410</v>
+        <v>398</v>
       </c>
     </row>
     <row r="10" spans="1:229" x14ac:dyDescent="0.35">
       <c r="A10" s="3" t="s">
-        <v>411</v>
+        <v>399</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>412</v>
+        <v>400</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>413</v>
+        <v>401</v>
       </c>
       <c r="D10" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E10" s="3" t="s">
-        <v>226</v>
+        <v>214</v>
       </c>
       <c r="F10" s="3" t="s">
-        <v>227</v>
+        <v>215</v>
       </c>
       <c r="G10" s="3" t="s">
-        <v>236</v>
+        <v>224</v>
       </c>
       <c r="H10" s="3" t="s">
-        <v>414</v>
+        <v>402</v>
       </c>
     </row>
   </sheetData>
@@ -15289,36 +15308,36 @@
         <v>35</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>234</v>
+        <v>222</v>
       </c>
       <c r="H1" s="2" t="s">
-        <v>235</v>
+        <v>223</v>
       </c>
     </row>
     <row r="2" spans="1:229" s="4" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A2" s="3" t="s">
-        <v>415</v>
+        <v>403</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>416</v>
+        <v>404</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>417</v>
+        <v>405</v>
       </c>
       <c r="D2" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>226</v>
+        <v>214</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>227</v>
+        <v>215</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>236</v>
+        <v>224</v>
       </c>
       <c r="H2" s="3" t="s">
-        <v>207</v>
+        <v>195</v>
       </c>
       <c r="I2"/>
       <c r="J2"/>
@@ -15544,158 +15563,158 @@
     </row>
     <row r="3" spans="1:229" x14ac:dyDescent="0.35">
       <c r="A3" s="3" t="s">
-        <v>418</v>
+        <v>406</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>419</v>
+        <v>407</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>420</v>
+        <v>408</v>
       </c>
       <c r="D3" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>226</v>
+        <v>214</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>227</v>
+        <v>215</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>236</v>
+        <v>224</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>421</v>
+        <v>409</v>
       </c>
     </row>
     <row r="4" spans="1:229" x14ac:dyDescent="0.35">
       <c r="A4" s="3" t="s">
-        <v>422</v>
+        <v>410</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>423</v>
+        <v>411</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>424</v>
+        <v>412</v>
       </c>
       <c r="D4" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>226</v>
+        <v>214</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>227</v>
+        <v>215</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>236</v>
+        <v>224</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>425</v>
+        <v>413</v>
       </c>
     </row>
     <row r="5" spans="1:229" x14ac:dyDescent="0.35">
       <c r="A5" s="8" t="s">
-        <v>426</v>
+        <v>414</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>427</v>
+        <v>415</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>428</v>
+        <v>416</v>
       </c>
       <c r="D5" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>226</v>
+        <v>214</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>227</v>
+        <v>215</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>236</v>
+        <v>224</v>
       </c>
       <c r="H5" s="3" t="s">
-        <v>429</v>
+        <v>417</v>
       </c>
     </row>
     <row r="6" spans="1:229" x14ac:dyDescent="0.35">
       <c r="A6" s="3" t="s">
-        <v>430</v>
+        <v>418</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>431</v>
+        <v>419</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>432</v>
+        <v>420</v>
       </c>
       <c r="D6" s="7" t="s">
         <v>0</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>226</v>
+        <v>214</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>227</v>
+        <v>215</v>
       </c>
       <c r="G6" s="3" t="s">
-        <v>236</v>
+        <v>224</v>
       </c>
       <c r="H6" s="3" t="s">
-        <v>433</v>
+        <v>421</v>
       </c>
     </row>
     <row r="7" spans="1:229" x14ac:dyDescent="0.35">
       <c r="A7" s="3" t="s">
-        <v>434</v>
+        <v>422</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>435</v>
+        <v>423</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>436</v>
+        <v>424</v>
       </c>
       <c r="D7" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>226</v>
+        <v>214</v>
       </c>
       <c r="F7" s="3" t="s">
-        <v>227</v>
+        <v>215</v>
       </c>
       <c r="G7" s="3" t="s">
-        <v>236</v>
+        <v>224</v>
       </c>
       <c r="H7" s="3" t="s">
-        <v>437</v>
+        <v>425</v>
       </c>
     </row>
     <row r="8" spans="1:229" x14ac:dyDescent="0.35">
       <c r="A8" s="9" t="s">
-        <v>438</v>
+        <v>426</v>
       </c>
       <c r="B8" s="9" t="s">
-        <v>439</v>
+        <v>427</v>
       </c>
       <c r="C8" s="9" t="s">
-        <v>440</v>
+        <v>428</v>
       </c>
       <c r="D8" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E8" s="3" t="s">
-        <v>226</v>
+        <v>214</v>
       </c>
       <c r="F8" s="3" t="s">
-        <v>227</v>
+        <v>215</v>
       </c>
       <c r="G8" s="3" t="s">
-        <v>236</v>
+        <v>224</v>
       </c>
       <c r="H8" s="9" t="s">
-        <v>441</v>
+        <v>429</v>
       </c>
     </row>
   </sheetData>
@@ -15706,7 +15725,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F9169CA5-09CB-4ADC-8EEE-AB383FD3DBB7}">
-  <dimension ref="A1:AMO11"/>
+  <dimension ref="A1:AMO12"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="40.54296875" bestFit="1" customWidth="1"/>
@@ -15739,82 +15758,82 @@
     </row>
     <row r="2" spans="1:1029" x14ac:dyDescent="0.35">
       <c r="A2" s="3" t="s">
-        <v>372</v>
+        <v>360</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>373</v>
+        <v>361</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>374</v>
+        <v>362</v>
       </c>
       <c r="D2" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>371</v>
+        <v>359</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>375</v>
+        <v>363</v>
       </c>
     </row>
     <row r="3" spans="1:1029" x14ac:dyDescent="0.35">
-      <c r="A3" s="3" t="s">
-        <v>90</v>
-      </c>
-      <c r="B3" s="3" t="s">
-        <v>91</v>
-      </c>
-      <c r="C3" s="3" t="s">
-        <v>92</v>
+      <c r="A3" s="10" t="s">
+        <v>78</v>
+      </c>
+      <c r="B3" s="10" t="s">
+        <v>79</v>
+      </c>
+      <c r="C3" s="10" t="s">
+        <v>80</v>
       </c>
       <c r="D3" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>371</v>
-      </c>
-      <c r="F3" s="3" t="s">
-        <v>93</v>
+        <v>359</v>
+      </c>
+      <c r="F3" s="10" t="s">
+        <v>81</v>
       </c>
     </row>
     <row r="4" spans="1:1029" x14ac:dyDescent="0.35">
       <c r="A4" s="3" t="s">
-        <v>121</v>
+        <v>109</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>122</v>
+        <v>110</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>123</v>
+        <v>111</v>
       </c>
       <c r="D4" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>371</v>
+        <v>359</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>124</v>
+        <v>112</v>
       </c>
     </row>
     <row r="5" spans="1:1029" s="4" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A5" s="3" t="s">
-        <v>70</v>
+        <v>434</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>71</v>
+        <v>435</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>72</v>
+        <v>436</v>
       </c>
       <c r="D5" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>371</v>
+        <v>359</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>73</v>
+        <v>437</v>
       </c>
       <c r="G5"/>
       <c r="H5"/>
@@ -16841,63 +16860,63 @@
       <c r="AMO5"/>
     </row>
     <row r="6" spans="1:1029" x14ac:dyDescent="0.35">
-      <c r="A6" s="3" t="s">
-        <v>94</v>
-      </c>
-      <c r="B6" s="3" t="s">
-        <v>95</v>
-      </c>
-      <c r="C6" s="3" t="s">
-        <v>96</v>
+      <c r="A6" s="10" t="s">
+        <v>82</v>
+      </c>
+      <c r="B6" s="10" t="s">
+        <v>83</v>
+      </c>
+      <c r="C6" s="10" t="s">
+        <v>84</v>
       </c>
       <c r="D6" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>371</v>
-      </c>
-      <c r="F6" s="3" t="s">
-        <v>97</v>
+        <v>359</v>
+      </c>
+      <c r="F6" s="10" t="s">
+        <v>85</v>
       </c>
     </row>
     <row r="7" spans="1:1029" x14ac:dyDescent="0.35">
       <c r="A7" s="3" t="s">
-        <v>86</v>
+        <v>74</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>87</v>
+        <v>75</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>88</v>
+        <v>76</v>
       </c>
       <c r="D7" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>371</v>
+        <v>359</v>
       </c>
       <c r="F7" s="3" t="s">
-        <v>89</v>
+        <v>77</v>
       </c>
     </row>
     <row r="8" spans="1:1029" s="4" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A8" s="3" t="s">
-        <v>81</v>
+        <v>438</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>74</v>
+        <v>440</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>75</v>
+        <v>439</v>
       </c>
       <c r="D8" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E8" s="3" t="s">
-        <v>371</v>
+        <v>359</v>
       </c>
       <c r="F8" s="3" t="s">
-        <v>76</v>
+        <v>449</v>
       </c>
       <c r="G8"/>
       <c r="H8"/>
@@ -17925,62 +17944,82 @@
     </row>
     <row r="9" spans="1:1029" x14ac:dyDescent="0.35">
       <c r="A9" s="3" t="s">
-        <v>80</v>
+        <v>441</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>77</v>
+        <v>442</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>78</v>
+        <v>443</v>
       </c>
       <c r="D9" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E9" s="3" t="s">
-        <v>371</v>
+        <v>359</v>
       </c>
       <c r="F9" s="3" t="s">
-        <v>79</v>
+        <v>444</v>
       </c>
     </row>
     <row r="10" spans="1:1029" x14ac:dyDescent="0.35">
       <c r="A10" s="3" t="s">
-        <v>82</v>
+        <v>445</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>83</v>
+        <v>446</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>84</v>
+        <v>447</v>
       </c>
       <c r="D10" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E10" s="3" t="s">
-        <v>371</v>
+        <v>359</v>
       </c>
       <c r="F10" s="3" t="s">
-        <v>85</v>
+        <v>448</v>
       </c>
     </row>
     <row r="11" spans="1:1029" x14ac:dyDescent="0.35">
-      <c r="A11" s="3" t="s">
-        <v>117</v>
-      </c>
-      <c r="B11" s="3" t="s">
-        <v>118</v>
-      </c>
-      <c r="C11" s="3" t="s">
-        <v>119</v>
+      <c r="A11" s="10" t="s">
+        <v>70</v>
+      </c>
+      <c r="B11" s="10" t="s">
+        <v>71</v>
+      </c>
+      <c r="C11" s="10" t="s">
+        <v>72</v>
       </c>
       <c r="D11" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E11" s="3" t="s">
-        <v>371</v>
-      </c>
-      <c r="F11" s="3" t="s">
-        <v>120</v>
+        <v>359</v>
+      </c>
+      <c r="F11" s="10" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="12" spans="1:1029" x14ac:dyDescent="0.35">
+      <c r="A12" s="3" t="s">
+        <v>105</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>106</v>
+      </c>
+      <c r="C12" s="3" t="s">
+        <v>107</v>
+      </c>
+      <c r="D12" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="E12" s="3" t="s">
+        <v>359</v>
+      </c>
+      <c r="F12" s="3" t="s">
+        <v>108</v>
       </c>
     </row>
   </sheetData>
@@ -18023,22 +18062,22 @@
     </row>
     <row r="2" spans="1:229" s="4" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A2" s="3" t="s">
-        <v>98</v>
+        <v>86</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>99</v>
+        <v>87</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>100</v>
+        <v>88</v>
       </c>
       <c r="D2" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>101</v>
+        <v>89</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>102</v>
+        <v>90</v>
       </c>
       <c r="G2"/>
       <c r="H2"/>
@@ -18266,22 +18305,22 @@
     </row>
     <row r="3" spans="1:229" s="4" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A3" s="3" t="s">
-        <v>103</v>
+        <v>91</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>104</v>
+        <v>92</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>105</v>
+        <v>93</v>
       </c>
       <c r="D3" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>101</v>
+        <v>89</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>106</v>
+        <v>94</v>
       </c>
       <c r="G3"/>
       <c r="H3"/>
@@ -18509,22 +18548,22 @@
     </row>
     <row r="4" spans="1:229" s="4" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A4" s="3" t="s">
-        <v>376</v>
+        <v>364</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>377</v>
+        <v>365</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>378</v>
+        <v>366</v>
       </c>
       <c r="D4" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>101</v>
+        <v>89</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>379</v>
+        <v>367</v>
       </c>
       <c r="G4"/>
       <c r="H4"/>
@@ -18752,42 +18791,42 @@
     </row>
     <row r="5" spans="1:229" x14ac:dyDescent="0.35">
       <c r="A5" s="3" t="s">
-        <v>107</v>
+        <v>95</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>108</v>
+        <v>96</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>109</v>
+        <v>97</v>
       </c>
       <c r="D5" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>101</v>
+        <v>89</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>110</v>
+        <v>98</v>
       </c>
     </row>
     <row r="6" spans="1:229" x14ac:dyDescent="0.35">
       <c r="A6" s="3" t="s">
-        <v>111</v>
+        <v>99</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>112</v>
+        <v>100</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>113</v>
+        <v>101</v>
       </c>
       <c r="D6" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>101</v>
+        <v>89</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>114</v>
+        <v>102</v>
       </c>
     </row>
   </sheetData>
@@ -18807,71 +18846,71 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" s="6" t="s">
-        <v>126</v>
+        <v>114</v>
       </c>
       <c r="B1" s="6" t="s">
-        <v>127</v>
+        <v>115</v>
       </c>
       <c r="C1" s="6" t="s">
-        <v>128</v>
+        <v>116</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" s="3" t="s">
-        <v>129</v>
+        <v>117</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>131</v>
+        <v>119</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>130</v>
+        <v>118</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="14" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B3" s="3" t="s">
-        <v>139</v>
+        <v>127</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>140</v>
+        <v>128</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.35">
       <c r="B4" s="3" t="s">
-        <v>137</v>
+        <v>125</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>138</v>
+        <v>126</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A5" s="3" t="s">
-        <v>132</v>
+        <v>120</v>
       </c>
       <c r="B5" s="3"/>
       <c r="C5" s="3"/>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A6" s="3" t="s">
-        <v>133</v>
+        <v>121</v>
       </c>
       <c r="B6" s="3"/>
       <c r="C6" s="3"/>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A7" s="3" t="s">
-        <v>134</v>
+        <v>122</v>
       </c>
       <c r="B7" s="3"/>
       <c r="C7" s="3"/>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A8" s="3" t="s">
-        <v>135</v>
+        <v>123</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A9" s="3" t="s">
-        <v>136</v>
+        <v>124</v>
       </c>
     </row>
   </sheetData>
@@ -18890,64 +18929,64 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" s="6" t="s">
-        <v>126</v>
+        <v>114</v>
       </c>
       <c r="B1" s="6" t="s">
-        <v>127</v>
+        <v>115</v>
       </c>
       <c r="C1" s="6" t="s">
-        <v>128</v>
+        <v>116</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" s="3" t="s">
-        <v>141</v>
+        <v>129</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>131</v>
+        <v>119</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>142</v>
+        <v>130</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="14" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B3" s="3" t="s">
-        <v>139</v>
+        <v>127</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>140</v>
+        <v>128</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.35">
       <c r="B4" s="3" t="s">
-        <v>137</v>
+        <v>125</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>138</v>
+        <v>126</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A5" s="3" t="s">
-        <v>143</v>
+        <v>131</v>
       </c>
       <c r="B5" s="3"/>
       <c r="C5" s="3"/>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A6" s="3" t="s">
-        <v>144</v>
+        <v>132</v>
       </c>
       <c r="B6" s="3"/>
       <c r="C6" s="3"/>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A7" s="3" t="s">
-        <v>145</v>
+        <v>133</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A8" s="3" t="s">
-        <v>146</v>
+        <v>134</v>
       </c>
     </row>
   </sheetData>
@@ -18966,78 +19005,78 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" s="6" t="s">
-        <v>126</v>
+        <v>114</v>
       </c>
       <c r="B1" s="6" t="s">
-        <v>127</v>
+        <v>115</v>
       </c>
       <c r="C1" s="6" t="s">
-        <v>128</v>
+        <v>116</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" s="3" t="s">
-        <v>147</v>
+        <v>135</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>131</v>
+        <v>119</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>148</v>
+        <v>136</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="14" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B3" s="3" t="s">
-        <v>139</v>
+        <v>127</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>140</v>
+        <v>128</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.35">
       <c r="B4" s="3" t="s">
-        <v>137</v>
+        <v>125</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>138</v>
+        <v>126</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A5" s="3" t="s">
-        <v>152</v>
+        <v>140</v>
       </c>
       <c r="B5" s="3"/>
       <c r="C5" s="3"/>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A6" s="3" t="s">
-        <v>151</v>
+        <v>139</v>
       </c>
       <c r="B6" s="3"/>
       <c r="C6" s="3"/>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A7" s="3" t="s">
-        <v>150</v>
+        <v>138</v>
       </c>
       <c r="B7" s="3"/>
       <c r="C7" s="3"/>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A8" s="3" t="s">
-        <v>149</v>
+        <v>137</v>
       </c>
       <c r="B8" s="3"/>
       <c r="C8" s="3"/>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A9" s="3" t="s">
-        <v>153</v>
+        <v>141</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A10" s="3" t="s">
-        <v>154</v>
+        <v>142</v>
       </c>
     </row>
   </sheetData>
@@ -19057,71 +19096,71 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" s="6" t="s">
-        <v>126</v>
+        <v>114</v>
       </c>
       <c r="B1" s="6" t="s">
-        <v>127</v>
+        <v>115</v>
       </c>
       <c r="C1" s="6" t="s">
-        <v>128</v>
+        <v>116</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" s="3" t="s">
-        <v>155</v>
+        <v>143</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>131</v>
+        <v>119</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>156</v>
+        <v>144</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="14" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B3" s="3" t="s">
-        <v>139</v>
+        <v>127</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>140</v>
+        <v>128</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.35">
       <c r="B4" s="3" t="s">
-        <v>137</v>
+        <v>125</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>138</v>
+        <v>126</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A5" s="3" t="s">
-        <v>157</v>
+        <v>145</v>
       </c>
       <c r="B5" s="3"/>
       <c r="C5" s="3"/>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A6" s="3" t="s">
-        <v>158</v>
+        <v>146</v>
       </c>
       <c r="B6" s="3"/>
       <c r="C6" s="3"/>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A7" s="3" t="s">
-        <v>159</v>
+        <v>147</v>
       </c>
       <c r="B7" s="3"/>
       <c r="C7" s="3"/>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A8" s="3" t="s">
-        <v>160</v>
+        <v>148</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A9" s="3" t="s">
-        <v>161</v>
+        <v>149</v>
       </c>
     </row>
   </sheetData>
@@ -19141,92 +19180,92 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" s="6" t="s">
-        <v>126</v>
+        <v>114</v>
       </c>
       <c r="B1" s="6" t="s">
-        <v>127</v>
+        <v>115</v>
       </c>
       <c r="C1" s="6" t="s">
-        <v>128</v>
+        <v>116</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" s="3" t="s">
-        <v>162</v>
+        <v>150</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>131</v>
+        <v>119</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>163</v>
+        <v>151</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="14" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B3" s="3" t="s">
-        <v>139</v>
+        <v>127</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>140</v>
+        <v>128</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.35">
       <c r="B4" s="3" t="s">
-        <v>137</v>
+        <v>125</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>138</v>
+        <v>126</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A5" s="3" t="s">
-        <v>164</v>
+        <v>152</v>
       </c>
       <c r="B5" s="3"/>
       <c r="C5" s="3"/>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A6" s="3" t="s">
-        <v>165</v>
+        <v>153</v>
       </c>
       <c r="B6" s="3"/>
       <c r="C6" s="3"/>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A7" s="3" t="s">
-        <v>166</v>
+        <v>154</v>
       </c>
       <c r="B7" s="3"/>
       <c r="C7" s="3"/>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A8" s="3" t="s">
-        <v>167</v>
+        <v>155</v>
       </c>
       <c r="B8" s="3"/>
       <c r="C8" s="3"/>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A9" s="3" t="s">
-        <v>168</v>
+        <v>156</v>
       </c>
       <c r="B9" s="3"/>
       <c r="C9" s="3"/>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A10" s="3" t="s">
-        <v>169</v>
+        <v>157</v>
       </c>
       <c r="B10" s="3"/>
       <c r="C10" s="3"/>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A11" s="3" t="s">
-        <v>170</v>
+        <v>158</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A12" s="3" t="s">
-        <v>171</v>
+        <v>159</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Product overview, categories page and Propose a change form
</commit_message>
<xml_diff>
--- a/testdata.xlsx
+++ b/testdata.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sshiwani\workspace\find-information-products-services-tests\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A7442755-0F79-49B6-9FA8-E67CA91AD833}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{24635E98-D493-4C20-BE24-573CC1FCB0CA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="22780" windowHeight="14540" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="22780" windowHeight="14540" firstSheet="14" activeTab="15" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="category_phase" sheetId="1" r:id="rId1"/>
@@ -689,9 +689,6 @@
     <t>Social worker</t>
   </si>
   <si>
-    <t>Remove this filter Adult learner</t>
-  </si>
-  <si>
     <t>//h3[normalize-space()='User groups']</t>
   </si>
   <si>
@@ -1398,6 +1395,9 @@
   </si>
   <si>
     <t>#group-regional-digital-services</t>
+  </si>
+  <si>
+    <t>Remove this filter Adult learner (18+)</t>
   </si>
 </sst>
 </file>
@@ -4183,13 +4183,13 @@
     </row>
     <row r="4" spans="1:1149" s="5" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A4" s="3" t="s">
+        <v>429</v>
+      </c>
+      <c r="B4" s="3" t="s">
         <v>430</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="C4" s="3" t="s">
         <v>431</v>
-      </c>
-      <c r="C4" s="3" t="s">
-        <v>432</v>
       </c>
       <c r="D4" s="3" t="s">
         <v>0</v>
@@ -4198,7 +4198,7 @@
         <v>1</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>433</v>
+        <v>432</v>
       </c>
       <c r="G4"/>
       <c r="H4"/>
@@ -11781,33 +11781,33 @@
         <v>35</v>
       </c>
       <c r="G1" s="2" t="s">
+        <v>221</v>
+      </c>
+      <c r="H1" s="2" t="s">
         <v>222</v>
-      </c>
-      <c r="H1" s="2" t="s">
-        <v>223</v>
       </c>
     </row>
     <row r="2" spans="1:229" s="4" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A2" s="3" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>213</v>
+        <v>449</v>
       </c>
       <c r="D2" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E2" s="3" t="s">
+        <v>213</v>
+      </c>
+      <c r="F2" s="3" t="s">
         <v>214</v>
       </c>
-      <c r="F2" s="3" t="s">
-        <v>215</v>
-      </c>
       <c r="G2" s="3" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="H2" s="3" t="s">
         <v>120</v>
@@ -12036,106 +12036,106 @@
     </row>
     <row r="3" spans="1:229" x14ac:dyDescent="0.35">
       <c r="A3" s="3" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="B3" s="3" t="s">
+        <v>219</v>
+      </c>
+      <c r="C3" s="3" t="s">
         <v>220</v>
-      </c>
-      <c r="C3" s="3" t="s">
-        <v>221</v>
       </c>
       <c r="D3" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E3" s="3" t="s">
+        <v>213</v>
+      </c>
+      <c r="F3" s="3" t="s">
         <v>214</v>
       </c>
-      <c r="F3" s="3" t="s">
-        <v>215</v>
-      </c>
       <c r="G3" s="3" t="s">
+        <v>224</v>
+      </c>
+      <c r="H3" s="3" t="s">
         <v>225</v>
-      </c>
-      <c r="H3" s="3" t="s">
-        <v>226</v>
       </c>
     </row>
     <row r="4" spans="1:229" x14ac:dyDescent="0.35">
       <c r="A4" s="3" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="B4" s="3" t="s">
+        <v>226</v>
+      </c>
+      <c r="C4" s="3" t="s">
         <v>227</v>
-      </c>
-      <c r="C4" s="3" t="s">
-        <v>228</v>
       </c>
       <c r="D4" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E4" s="3" t="s">
+        <v>213</v>
+      </c>
+      <c r="F4" s="3" t="s">
         <v>214</v>
       </c>
-      <c r="F4" s="3" t="s">
-        <v>215</v>
-      </c>
       <c r="G4" s="3" t="s">
+        <v>228</v>
+      </c>
+      <c r="H4" s="3" t="s">
         <v>229</v>
-      </c>
-      <c r="H4" s="3" t="s">
-        <v>230</v>
       </c>
     </row>
     <row r="5" spans="1:229" x14ac:dyDescent="0.35">
       <c r="A5" s="3" t="s">
+        <v>230</v>
+      </c>
+      <c r="B5" s="3" t="s">
         <v>231</v>
       </c>
-      <c r="B5" s="3" t="s">
+      <c r="C5" s="3" t="s">
         <v>232</v>
-      </c>
-      <c r="C5" s="3" t="s">
-        <v>233</v>
       </c>
       <c r="D5" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E5" s="3" t="s">
+        <v>213</v>
+      </c>
+      <c r="F5" s="3" t="s">
         <v>214</v>
       </c>
-      <c r="F5" s="3" t="s">
-        <v>215</v>
-      </c>
       <c r="G5" s="3" t="s">
+        <v>233</v>
+      </c>
+      <c r="H5" s="3" t="s">
         <v>234</v>
-      </c>
-      <c r="H5" s="3" t="s">
-        <v>235</v>
       </c>
     </row>
     <row r="6" spans="1:229" x14ac:dyDescent="0.35">
       <c r="A6" s="3" t="s">
+        <v>235</v>
+      </c>
+      <c r="B6" s="3" t="s">
         <v>236</v>
       </c>
-      <c r="B6" s="3" t="s">
+      <c r="C6" s="3" t="s">
         <v>237</v>
-      </c>
-      <c r="C6" s="3" t="s">
-        <v>238</v>
       </c>
       <c r="D6" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E6" s="3" t="s">
+        <v>213</v>
+      </c>
+      <c r="F6" s="3" t="s">
         <v>214</v>
       </c>
-      <c r="F6" s="3" t="s">
-        <v>215</v>
-      </c>
       <c r="G6" s="3" t="s">
+        <v>238</v>
+      </c>
+      <c r="H6" s="3" t="s">
         <v>239</v>
-      </c>
-      <c r="H6" s="3" t="s">
-        <v>240</v>
       </c>
     </row>
   </sheetData>
@@ -12179,33 +12179,33 @@
         <v>35</v>
       </c>
       <c r="G1" s="2" t="s">
+        <v>221</v>
+      </c>
+      <c r="H1" s="2" t="s">
         <v>222</v>
-      </c>
-      <c r="H1" s="2" t="s">
-        <v>223</v>
       </c>
     </row>
     <row r="2" spans="1:229" s="4" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A2" s="3" t="s">
+        <v>240</v>
+      </c>
+      <c r="B2" s="3" t="s">
         <v>241</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="C2" s="3" t="s">
         <v>242</v>
-      </c>
-      <c r="C2" s="3" t="s">
-        <v>243</v>
       </c>
       <c r="D2" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E2" s="3" t="s">
+        <v>213</v>
+      </c>
+      <c r="F2" s="3" t="s">
         <v>214</v>
       </c>
-      <c r="F2" s="3" t="s">
-        <v>215</v>
-      </c>
       <c r="G2" s="3" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="H2" s="3" t="s">
         <v>131</v>
@@ -12434,80 +12434,80 @@
     </row>
     <row r="3" spans="1:229" x14ac:dyDescent="0.35">
       <c r="A3" s="3" t="s">
+        <v>243</v>
+      </c>
+      <c r="B3" s="3" t="s">
         <v>244</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="C3" s="3" t="s">
         <v>245</v>
-      </c>
-      <c r="C3" s="3" t="s">
-        <v>246</v>
       </c>
       <c r="D3" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E3" s="3" t="s">
+        <v>213</v>
+      </c>
+      <c r="F3" s="3" t="s">
         <v>214</v>
       </c>
-      <c r="F3" s="3" t="s">
-        <v>215</v>
-      </c>
       <c r="G3" s="3" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
     </row>
     <row r="4" spans="1:229" x14ac:dyDescent="0.35">
       <c r="A4" s="3" t="s">
+        <v>247</v>
+      </c>
+      <c r="B4" s="3" t="s">
         <v>248</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="C4" s="3" t="s">
         <v>249</v>
-      </c>
-      <c r="C4" s="3" t="s">
-        <v>250</v>
       </c>
       <c r="D4" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E4" s="3" t="s">
+        <v>213</v>
+      </c>
+      <c r="F4" s="3" t="s">
         <v>214</v>
       </c>
-      <c r="F4" s="3" t="s">
-        <v>215</v>
-      </c>
       <c r="G4" s="3" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
     </row>
     <row r="5" spans="1:229" x14ac:dyDescent="0.35">
       <c r="A5" s="3" t="s">
+        <v>251</v>
+      </c>
+      <c r="B5" s="3" t="s">
         <v>252</v>
       </c>
-      <c r="B5" s="3" t="s">
+      <c r="C5" s="3" t="s">
         <v>253</v>
-      </c>
-      <c r="C5" s="3" t="s">
-        <v>254</v>
       </c>
       <c r="D5" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E5" s="3" t="s">
+        <v>213</v>
+      </c>
+      <c r="F5" s="3" t="s">
         <v>214</v>
       </c>
-      <c r="F5" s="3" t="s">
-        <v>215</v>
-      </c>
       <c r="G5" s="3" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="H5" s="3" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
     </row>
   </sheetData>
@@ -12550,33 +12550,33 @@
         <v>35</v>
       </c>
       <c r="G1" s="2" t="s">
+        <v>221</v>
+      </c>
+      <c r="H1" s="2" t="s">
         <v>222</v>
-      </c>
-      <c r="H1" s="2" t="s">
-        <v>223</v>
       </c>
     </row>
     <row r="2" spans="1:229" s="4" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A2" s="3" t="s">
+        <v>255</v>
+      </c>
+      <c r="B2" s="3" t="s">
         <v>256</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="C2" s="3" t="s">
         <v>257</v>
-      </c>
-      <c r="C2" s="3" t="s">
-        <v>258</v>
       </c>
       <c r="D2" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E2" s="3" t="s">
+        <v>213</v>
+      </c>
+      <c r="F2" s="3" t="s">
         <v>214</v>
       </c>
-      <c r="F2" s="3" t="s">
-        <v>215</v>
-      </c>
       <c r="G2" s="3" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="H2" s="3" t="s">
         <v>140</v>
@@ -12805,132 +12805,132 @@
     </row>
     <row r="3" spans="1:229" x14ac:dyDescent="0.35">
       <c r="A3" s="3" t="s">
+        <v>258</v>
+      </c>
+      <c r="B3" s="3" t="s">
         <v>259</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="C3" s="3" t="s">
         <v>260</v>
-      </c>
-      <c r="C3" s="3" t="s">
-        <v>261</v>
       </c>
       <c r="D3" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E3" s="3" t="s">
+        <v>213</v>
+      </c>
+      <c r="F3" s="3" t="s">
         <v>214</v>
       </c>
-      <c r="F3" s="3" t="s">
-        <v>215</v>
-      </c>
       <c r="G3" s="3" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
     </row>
     <row r="4" spans="1:229" x14ac:dyDescent="0.35">
       <c r="A4" s="3" t="s">
+        <v>262</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>264</v>
+      </c>
+      <c r="C4" s="3" t="s">
         <v>263</v>
-      </c>
-      <c r="B4" s="3" t="s">
-        <v>265</v>
-      </c>
-      <c r="C4" s="3" t="s">
-        <v>264</v>
       </c>
       <c r="D4" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E4" s="3" t="s">
+        <v>213</v>
+      </c>
+      <c r="F4" s="3" t="s">
         <v>214</v>
       </c>
-      <c r="F4" s="3" t="s">
-        <v>215</v>
-      </c>
       <c r="G4" s="3" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
     </row>
     <row r="5" spans="1:229" x14ac:dyDescent="0.35">
       <c r="A5" s="8" t="s">
+        <v>266</v>
+      </c>
+      <c r="B5" s="8" t="s">
         <v>267</v>
       </c>
-      <c r="B5" s="8" t="s">
+      <c r="C5" s="8" t="s">
         <v>268</v>
-      </c>
-      <c r="C5" s="8" t="s">
-        <v>269</v>
       </c>
       <c r="D5" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E5" s="3" t="s">
+        <v>213</v>
+      </c>
+      <c r="F5" s="3" t="s">
         <v>214</v>
       </c>
-      <c r="F5" s="3" t="s">
-        <v>215</v>
-      </c>
       <c r="G5" s="3" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="H5" s="3" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
     </row>
     <row r="6" spans="1:229" x14ac:dyDescent="0.35">
       <c r="A6" s="3" t="s">
+        <v>270</v>
+      </c>
+      <c r="B6" s="3" t="s">
         <v>271</v>
       </c>
-      <c r="B6" s="3" t="s">
+      <c r="C6" s="3" t="s">
         <v>272</v>
-      </c>
-      <c r="C6" s="3" t="s">
-        <v>273</v>
       </c>
       <c r="D6" s="7" t="s">
         <v>0</v>
       </c>
       <c r="E6" s="3" t="s">
+        <v>213</v>
+      </c>
+      <c r="F6" s="3" t="s">
         <v>214</v>
       </c>
-      <c r="F6" s="3" t="s">
-        <v>215</v>
-      </c>
       <c r="G6" s="3" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="H6" s="3" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
     </row>
     <row r="7" spans="1:229" x14ac:dyDescent="0.35">
       <c r="A7" s="3" t="s">
+        <v>274</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>276</v>
+      </c>
+      <c r="C7" s="3" t="s">
         <v>275</v>
-      </c>
-      <c r="B7" s="3" t="s">
-        <v>277</v>
-      </c>
-      <c r="C7" s="3" t="s">
-        <v>276</v>
       </c>
       <c r="D7" s="7" t="s">
         <v>0</v>
       </c>
       <c r="E7" s="3" t="s">
+        <v>213</v>
+      </c>
+      <c r="F7" s="3" t="s">
         <v>214</v>
       </c>
-      <c r="F7" s="3" t="s">
-        <v>215</v>
-      </c>
       <c r="G7" s="3" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="H7" s="3" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
     </row>
   </sheetData>
@@ -12974,33 +12974,33 @@
         <v>35</v>
       </c>
       <c r="G1" s="2" t="s">
+        <v>221</v>
+      </c>
+      <c r="H1" s="2" t="s">
         <v>222</v>
-      </c>
-      <c r="H1" s="2" t="s">
-        <v>223</v>
       </c>
     </row>
     <row r="2" spans="1:229" s="4" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A2" s="3" t="s">
+        <v>278</v>
+      </c>
+      <c r="B2" s="3" t="s">
         <v>279</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="C2" s="3" t="s">
         <v>280</v>
-      </c>
-      <c r="C2" s="3" t="s">
-        <v>281</v>
       </c>
       <c r="D2" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E2" s="3" t="s">
+        <v>213</v>
+      </c>
+      <c r="F2" s="3" t="s">
         <v>214</v>
       </c>
-      <c r="F2" s="3" t="s">
-        <v>215</v>
-      </c>
       <c r="G2" s="3" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="H2" s="3" t="s">
         <v>145</v>
@@ -13229,106 +13229,106 @@
     </row>
     <row r="3" spans="1:229" x14ac:dyDescent="0.35">
       <c r="A3" s="3" t="s">
+        <v>281</v>
+      </c>
+      <c r="B3" s="3" t="s">
         <v>282</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="C3" s="3" t="s">
         <v>283</v>
-      </c>
-      <c r="C3" s="3" t="s">
-        <v>284</v>
       </c>
       <c r="D3" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E3" s="3" t="s">
+        <v>213</v>
+      </c>
+      <c r="F3" s="3" t="s">
         <v>214</v>
       </c>
-      <c r="F3" s="3" t="s">
-        <v>215</v>
-      </c>
       <c r="G3" s="3" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
     </row>
     <row r="4" spans="1:229" x14ac:dyDescent="0.35">
       <c r="A4" s="3" t="s">
+        <v>285</v>
+      </c>
+      <c r="B4" s="3" t="s">
         <v>286</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="C4" s="3" t="s">
         <v>287</v>
-      </c>
-      <c r="C4" s="3" t="s">
-        <v>288</v>
       </c>
       <c r="D4" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E4" s="3" t="s">
+        <v>213</v>
+      </c>
+      <c r="F4" s="3" t="s">
         <v>214</v>
       </c>
-      <c r="F4" s="3" t="s">
-        <v>215</v>
-      </c>
       <c r="G4" s="3" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
     <row r="5" spans="1:229" x14ac:dyDescent="0.35">
       <c r="A5" s="8" t="s">
+        <v>289</v>
+      </c>
+      <c r="B5" s="8" t="s">
         <v>290</v>
       </c>
-      <c r="B5" s="8" t="s">
+      <c r="C5" s="8" t="s">
         <v>291</v>
-      </c>
-      <c r="C5" s="8" t="s">
-        <v>292</v>
       </c>
       <c r="D5" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E5" s="3" t="s">
+        <v>213</v>
+      </c>
+      <c r="F5" s="3" t="s">
         <v>214</v>
       </c>
-      <c r="F5" s="3" t="s">
-        <v>215</v>
-      </c>
       <c r="G5" s="3" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="H5" s="3" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
     </row>
     <row r="6" spans="1:229" x14ac:dyDescent="0.35">
       <c r="A6" s="3" t="s">
+        <v>293</v>
+      </c>
+      <c r="B6" s="3" t="s">
         <v>294</v>
       </c>
-      <c r="B6" s="3" t="s">
+      <c r="C6" s="3" t="s">
         <v>295</v>
-      </c>
-      <c r="C6" s="3" t="s">
-        <v>296</v>
       </c>
       <c r="D6" s="7" t="s">
         <v>0</v>
       </c>
       <c r="E6" s="3" t="s">
+        <v>213</v>
+      </c>
+      <c r="F6" s="3" t="s">
         <v>214</v>
       </c>
-      <c r="F6" s="3" t="s">
-        <v>215</v>
-      </c>
       <c r="G6" s="3" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="H6" s="3" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
     </row>
   </sheetData>
@@ -13589,33 +13589,33 @@
         <v>35</v>
       </c>
       <c r="G1" s="2" t="s">
+        <v>221</v>
+      </c>
+      <c r="H1" s="2" t="s">
         <v>222</v>
-      </c>
-      <c r="H1" s="2" t="s">
-        <v>223</v>
       </c>
     </row>
     <row r="2" spans="1:229" s="4" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A2" s="3" t="s">
+        <v>297</v>
+      </c>
+      <c r="B2" s="3" t="s">
         <v>298</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="C2" s="3" t="s">
         <v>299</v>
-      </c>
-      <c r="C2" s="3" t="s">
-        <v>300</v>
       </c>
       <c r="D2" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E2" s="3" t="s">
+        <v>213</v>
+      </c>
+      <c r="F2" s="3" t="s">
         <v>214</v>
       </c>
-      <c r="F2" s="3" t="s">
-        <v>215</v>
-      </c>
       <c r="G2" s="3" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="H2" s="3" t="s">
         <v>162</v>
@@ -13844,80 +13844,80 @@
     </row>
     <row r="3" spans="1:229" x14ac:dyDescent="0.35">
       <c r="A3" s="3" t="s">
+        <v>300</v>
+      </c>
+      <c r="B3" s="3" t="s">
         <v>301</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="C3" s="3" t="s">
         <v>302</v>
-      </c>
-      <c r="C3" s="3" t="s">
-        <v>303</v>
       </c>
       <c r="D3" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E3" s="3" t="s">
+        <v>213</v>
+      </c>
+      <c r="F3" s="3" t="s">
         <v>214</v>
       </c>
-      <c r="F3" s="3" t="s">
-        <v>215</v>
-      </c>
       <c r="G3" s="3" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
     </row>
     <row r="4" spans="1:229" x14ac:dyDescent="0.35">
       <c r="A4" s="3" t="s">
+        <v>304</v>
+      </c>
+      <c r="B4" s="3" t="s">
         <v>305</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="C4" s="3" t="s">
         <v>306</v>
-      </c>
-      <c r="C4" s="3" t="s">
-        <v>307</v>
       </c>
       <c r="D4" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E4" s="3" t="s">
+        <v>213</v>
+      </c>
+      <c r="F4" s="3" t="s">
         <v>214</v>
       </c>
-      <c r="F4" s="3" t="s">
-        <v>215</v>
-      </c>
       <c r="G4" s="3" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
     </row>
     <row r="5" spans="1:229" x14ac:dyDescent="0.35">
       <c r="A5" s="3" t="s">
+        <v>308</v>
+      </c>
+      <c r="B5" s="3" t="s">
         <v>309</v>
       </c>
-      <c r="B5" s="3" t="s">
+      <c r="C5" s="3" t="s">
         <v>310</v>
-      </c>
-      <c r="C5" s="3" t="s">
-        <v>311</v>
       </c>
       <c r="D5" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E5" s="3" t="s">
+        <v>213</v>
+      </c>
+      <c r="F5" s="3" t="s">
         <v>214</v>
       </c>
-      <c r="F5" s="3" t="s">
-        <v>215</v>
-      </c>
       <c r="G5" s="3" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="H5" s="3" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
     </row>
   </sheetData>
@@ -13960,33 +13960,33 @@
         <v>35</v>
       </c>
       <c r="G1" s="2" t="s">
+        <v>221</v>
+      </c>
+      <c r="H1" s="2" t="s">
         <v>222</v>
-      </c>
-      <c r="H1" s="2" t="s">
-        <v>223</v>
       </c>
     </row>
     <row r="2" spans="1:229" s="4" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A2" s="3" t="s">
+        <v>312</v>
+      </c>
+      <c r="B2" s="3" t="s">
         <v>313</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="C2" s="3" t="s">
         <v>314</v>
-      </c>
-      <c r="C2" s="3" t="s">
-        <v>315</v>
       </c>
       <c r="D2" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E2" s="3" t="s">
+        <v>213</v>
+      </c>
+      <c r="F2" s="3" t="s">
         <v>214</v>
       </c>
-      <c r="F2" s="3" t="s">
-        <v>215</v>
-      </c>
       <c r="G2" s="3" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="H2" s="3" t="s">
         <v>168</v>
@@ -14215,132 +14215,132 @@
     </row>
     <row r="3" spans="1:229" x14ac:dyDescent="0.35">
       <c r="A3" s="3" t="s">
+        <v>315</v>
+      </c>
+      <c r="B3" s="3" t="s">
         <v>316</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="C3" s="3" t="s">
         <v>317</v>
-      </c>
-      <c r="C3" s="3" t="s">
-        <v>318</v>
       </c>
       <c r="D3" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E3" s="3" t="s">
+        <v>213</v>
+      </c>
+      <c r="F3" s="3" t="s">
         <v>214</v>
       </c>
-      <c r="F3" s="3" t="s">
-        <v>215</v>
-      </c>
       <c r="G3" s="3" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
     </row>
     <row r="4" spans="1:229" x14ac:dyDescent="0.35">
       <c r="A4" s="3" t="s">
+        <v>319</v>
+      </c>
+      <c r="B4" s="3" t="s">
         <v>320</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="C4" s="3" t="s">
         <v>321</v>
-      </c>
-      <c r="C4" s="3" t="s">
-        <v>322</v>
       </c>
       <c r="D4" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E4" s="3" t="s">
+        <v>213</v>
+      </c>
+      <c r="F4" s="3" t="s">
         <v>214</v>
       </c>
-      <c r="F4" s="3" t="s">
-        <v>215</v>
-      </c>
       <c r="G4" s="3" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
     </row>
     <row r="5" spans="1:229" x14ac:dyDescent="0.35">
       <c r="A5" s="8" t="s">
+        <v>323</v>
+      </c>
+      <c r="B5" s="8" t="s">
         <v>324</v>
       </c>
-      <c r="B5" s="8" t="s">
+      <c r="C5" s="8" t="s">
         <v>325</v>
-      </c>
-      <c r="C5" s="8" t="s">
-        <v>326</v>
       </c>
       <c r="D5" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E5" s="3" t="s">
+        <v>213</v>
+      </c>
+      <c r="F5" s="3" t="s">
         <v>214</v>
       </c>
-      <c r="F5" s="3" t="s">
-        <v>215</v>
-      </c>
       <c r="G5" s="3" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="H5" s="3" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
     </row>
     <row r="6" spans="1:229" x14ac:dyDescent="0.35">
       <c r="A6" s="3" t="s">
+        <v>327</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>329</v>
+      </c>
+      <c r="C6" s="3" t="s">
         <v>328</v>
-      </c>
-      <c r="B6" s="3" t="s">
-        <v>330</v>
-      </c>
-      <c r="C6" s="3" t="s">
-        <v>329</v>
       </c>
       <c r="D6" s="7" t="s">
         <v>0</v>
       </c>
       <c r="E6" s="3" t="s">
+        <v>213</v>
+      </c>
+      <c r="F6" s="3" t="s">
         <v>214</v>
       </c>
-      <c r="F6" s="3" t="s">
-        <v>215</v>
-      </c>
       <c r="G6" s="3" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="H6" s="3" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
     </row>
     <row r="7" spans="1:229" x14ac:dyDescent="0.35">
       <c r="A7" s="3" t="s">
+        <v>331</v>
+      </c>
+      <c r="B7" s="3" t="s">
         <v>332</v>
       </c>
-      <c r="B7" s="3" t="s">
+      <c r="C7" s="3" t="s">
         <v>333</v>
-      </c>
-      <c r="C7" s="3" t="s">
-        <v>334</v>
       </c>
       <c r="D7" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E7" s="3" t="s">
+        <v>213</v>
+      </c>
+      <c r="F7" s="3" t="s">
         <v>214</v>
       </c>
-      <c r="F7" s="3" t="s">
-        <v>215</v>
-      </c>
       <c r="G7" s="3" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="H7" s="3" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
     </row>
   </sheetData>
@@ -14383,33 +14383,33 @@
         <v>35</v>
       </c>
       <c r="G1" s="2" t="s">
+        <v>221</v>
+      </c>
+      <c r="H1" s="2" t="s">
         <v>222</v>
-      </c>
-      <c r="H1" s="2" t="s">
-        <v>223</v>
       </c>
     </row>
     <row r="2" spans="1:229" s="4" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A2" s="3" t="s">
+        <v>335</v>
+      </c>
+      <c r="B2" s="3" t="s">
         <v>336</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="C2" s="3" t="s">
         <v>337</v>
-      </c>
-      <c r="C2" s="3" t="s">
-        <v>338</v>
       </c>
       <c r="D2" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E2" s="3" t="s">
+        <v>213</v>
+      </c>
+      <c r="F2" s="3" t="s">
         <v>214</v>
       </c>
-      <c r="F2" s="3" t="s">
-        <v>215</v>
-      </c>
       <c r="G2" s="3" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="H2" s="3" t="s">
         <v>176</v>
@@ -14638,132 +14638,132 @@
     </row>
     <row r="3" spans="1:229" x14ac:dyDescent="0.35">
       <c r="A3" s="3" t="s">
+        <v>338</v>
+      </c>
+      <c r="B3" s="3" t="s">
         <v>339</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="C3" s="3" t="s">
         <v>340</v>
-      </c>
-      <c r="C3" s="3" t="s">
-        <v>341</v>
       </c>
       <c r="D3" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E3" s="3" t="s">
+        <v>213</v>
+      </c>
+      <c r="F3" s="3" t="s">
         <v>214</v>
       </c>
-      <c r="F3" s="3" t="s">
-        <v>215</v>
-      </c>
       <c r="G3" s="3" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
     </row>
     <row r="4" spans="1:229" x14ac:dyDescent="0.35">
       <c r="A4" s="3" t="s">
+        <v>342</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>344</v>
+      </c>
+      <c r="C4" s="3" t="s">
         <v>343</v>
-      </c>
-      <c r="B4" s="3" t="s">
-        <v>345</v>
-      </c>
-      <c r="C4" s="3" t="s">
-        <v>344</v>
       </c>
       <c r="D4" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E4" s="3" t="s">
+        <v>213</v>
+      </c>
+      <c r="F4" s="3" t="s">
         <v>214</v>
       </c>
-      <c r="F4" s="3" t="s">
-        <v>215</v>
-      </c>
       <c r="G4" s="3" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
     </row>
     <row r="5" spans="1:229" x14ac:dyDescent="0.35">
       <c r="A5" s="8" t="s">
+        <v>346</v>
+      </c>
+      <c r="B5" s="8" t="s">
         <v>347</v>
       </c>
-      <c r="B5" s="8" t="s">
+      <c r="C5" s="8" t="s">
         <v>348</v>
-      </c>
-      <c r="C5" s="8" t="s">
-        <v>349</v>
       </c>
       <c r="D5" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E5" s="3" t="s">
+        <v>213</v>
+      </c>
+      <c r="F5" s="3" t="s">
         <v>214</v>
       </c>
-      <c r="F5" s="3" t="s">
-        <v>215</v>
-      </c>
       <c r="G5" s="3" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="H5" s="3" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
     </row>
     <row r="6" spans="1:229" x14ac:dyDescent="0.35">
       <c r="A6" s="3" t="s">
+        <v>350</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>352</v>
+      </c>
+      <c r="C6" s="3" t="s">
         <v>351</v>
-      </c>
-      <c r="B6" s="3" t="s">
-        <v>353</v>
-      </c>
-      <c r="C6" s="3" t="s">
-        <v>352</v>
       </c>
       <c r="D6" s="7" t="s">
         <v>0</v>
       </c>
       <c r="E6" s="3" t="s">
+        <v>213</v>
+      </c>
+      <c r="F6" s="3" t="s">
         <v>214</v>
       </c>
-      <c r="F6" s="3" t="s">
-        <v>215</v>
-      </c>
       <c r="G6" s="3" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="H6" s="3" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
     </row>
     <row r="7" spans="1:229" x14ac:dyDescent="0.35">
       <c r="A7" s="3" t="s">
+        <v>354</v>
+      </c>
+      <c r="B7" s="3" t="s">
         <v>355</v>
       </c>
-      <c r="B7" s="3" t="s">
+      <c r="C7" s="3" t="s">
         <v>356</v>
-      </c>
-      <c r="C7" s="3" t="s">
-        <v>357</v>
       </c>
       <c r="D7" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E7" s="3" t="s">
+        <v>213</v>
+      </c>
+      <c r="F7" s="3" t="s">
         <v>214</v>
       </c>
-      <c r="F7" s="3" t="s">
-        <v>215</v>
-      </c>
       <c r="G7" s="3" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="H7" s="3" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
     </row>
   </sheetData>
@@ -14806,33 +14806,33 @@
         <v>35</v>
       </c>
       <c r="G1" s="2" t="s">
+        <v>221</v>
+      </c>
+      <c r="H1" s="2" t="s">
         <v>222</v>
-      </c>
-      <c r="H1" s="2" t="s">
-        <v>223</v>
       </c>
     </row>
     <row r="2" spans="1:229" s="4" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A2" s="3" t="s">
+        <v>367</v>
+      </c>
+      <c r="B2" s="3" t="s">
         <v>368</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="C2" s="3" t="s">
         <v>369</v>
-      </c>
-      <c r="C2" s="3" t="s">
-        <v>370</v>
       </c>
       <c r="D2" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E2" s="3" t="s">
+        <v>213</v>
+      </c>
+      <c r="F2" s="3" t="s">
         <v>214</v>
       </c>
-      <c r="F2" s="3" t="s">
-        <v>215</v>
-      </c>
       <c r="G2" s="3" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="H2" s="3" t="s">
         <v>184</v>
@@ -15061,210 +15061,210 @@
     </row>
     <row r="3" spans="1:229" x14ac:dyDescent="0.35">
       <c r="A3" s="3" t="s">
+        <v>370</v>
+      </c>
+      <c r="B3" s="3" t="s">
         <v>371</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="C3" s="3" t="s">
         <v>372</v>
-      </c>
-      <c r="C3" s="3" t="s">
-        <v>373</v>
       </c>
       <c r="D3" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E3" s="3" t="s">
+        <v>213</v>
+      </c>
+      <c r="F3" s="3" t="s">
         <v>214</v>
       </c>
-      <c r="F3" s="3" t="s">
-        <v>215</v>
-      </c>
       <c r="G3" s="3" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
     </row>
     <row r="4" spans="1:229" x14ac:dyDescent="0.35">
       <c r="A4" s="3" t="s">
+        <v>374</v>
+      </c>
+      <c r="B4" s="3" t="s">
         <v>375</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="C4" s="3" t="s">
         <v>376</v>
-      </c>
-      <c r="C4" s="3" t="s">
-        <v>377</v>
       </c>
       <c r="D4" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E4" s="3" t="s">
+        <v>213</v>
+      </c>
+      <c r="F4" s="3" t="s">
         <v>214</v>
       </c>
-      <c r="F4" s="3" t="s">
-        <v>215</v>
-      </c>
       <c r="G4" s="3" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
     </row>
     <row r="5" spans="1:229" x14ac:dyDescent="0.35">
       <c r="A5" s="8" t="s">
+        <v>378</v>
+      </c>
+      <c r="B5" s="8" t="s">
         <v>379</v>
       </c>
-      <c r="B5" s="8" t="s">
+      <c r="C5" s="8" t="s">
         <v>380</v>
-      </c>
-      <c r="C5" s="8" t="s">
-        <v>381</v>
       </c>
       <c r="D5" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E5" s="3" t="s">
+        <v>213</v>
+      </c>
+      <c r="F5" s="3" t="s">
         <v>214</v>
       </c>
-      <c r="F5" s="3" t="s">
-        <v>215</v>
-      </c>
       <c r="G5" s="3" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="H5" s="3" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
     </row>
     <row r="6" spans="1:229" x14ac:dyDescent="0.35">
       <c r="A6" s="3" t="s">
+        <v>382</v>
+      </c>
+      <c r="B6" s="3" t="s">
         <v>383</v>
       </c>
-      <c r="B6" s="3" t="s">
+      <c r="C6" s="3" t="s">
         <v>384</v>
-      </c>
-      <c r="C6" s="3" t="s">
-        <v>385</v>
       </c>
       <c r="D6" s="7" t="s">
         <v>0</v>
       </c>
       <c r="E6" s="3" t="s">
+        <v>213</v>
+      </c>
+      <c r="F6" s="3" t="s">
         <v>214</v>
       </c>
-      <c r="F6" s="3" t="s">
-        <v>215</v>
-      </c>
       <c r="G6" s="3" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="H6" s="3" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
     </row>
     <row r="7" spans="1:229" x14ac:dyDescent="0.35">
       <c r="A7" s="3" t="s">
+        <v>386</v>
+      </c>
+      <c r="B7" s="3" t="s">
         <v>387</v>
       </c>
-      <c r="B7" s="3" t="s">
+      <c r="C7" s="3" t="s">
         <v>388</v>
-      </c>
-      <c r="C7" s="3" t="s">
-        <v>389</v>
       </c>
       <c r="D7" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E7" s="3" t="s">
+        <v>213</v>
+      </c>
+      <c r="F7" s="3" t="s">
         <v>214</v>
       </c>
-      <c r="F7" s="3" t="s">
-        <v>215</v>
-      </c>
       <c r="G7" s="3" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="H7" s="3" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
     </row>
     <row r="8" spans="1:229" x14ac:dyDescent="0.35">
       <c r="A8" s="3" t="s">
+        <v>390</v>
+      </c>
+      <c r="B8" s="3" t="s">
         <v>391</v>
       </c>
-      <c r="B8" s="3" t="s">
+      <c r="C8" s="3" t="s">
         <v>392</v>
-      </c>
-      <c r="C8" s="3" t="s">
-        <v>393</v>
       </c>
       <c r="D8" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E8" s="3" t="s">
+        <v>213</v>
+      </c>
+      <c r="F8" s="3" t="s">
         <v>214</v>
       </c>
-      <c r="F8" s="3" t="s">
-        <v>215</v>
-      </c>
       <c r="G8" s="3" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="H8" s="3" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
     </row>
     <row r="9" spans="1:229" x14ac:dyDescent="0.35">
       <c r="A9" s="3" t="s">
+        <v>394</v>
+      </c>
+      <c r="B9" s="3" t="s">
         <v>395</v>
       </c>
-      <c r="B9" s="3" t="s">
+      <c r="C9" s="3" t="s">
         <v>396</v>
-      </c>
-      <c r="C9" s="3" t="s">
-        <v>397</v>
       </c>
       <c r="D9" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E9" s="3" t="s">
+        <v>213</v>
+      </c>
+      <c r="F9" s="3" t="s">
         <v>214</v>
       </c>
-      <c r="F9" s="3" t="s">
-        <v>215</v>
-      </c>
       <c r="G9" s="3" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="H9" s="3" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
     </row>
     <row r="10" spans="1:229" x14ac:dyDescent="0.35">
       <c r="A10" s="3" t="s">
+        <v>398</v>
+      </c>
+      <c r="B10" s="3" t="s">
         <v>399</v>
       </c>
-      <c r="B10" s="3" t="s">
+      <c r="C10" s="3" t="s">
         <v>400</v>
-      </c>
-      <c r="C10" s="3" t="s">
-        <v>401</v>
       </c>
       <c r="D10" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E10" s="3" t="s">
+        <v>213</v>
+      </c>
+      <c r="F10" s="3" t="s">
         <v>214</v>
       </c>
-      <c r="F10" s="3" t="s">
-        <v>215</v>
-      </c>
       <c r="G10" s="3" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="H10" s="3" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
     </row>
   </sheetData>
@@ -15308,33 +15308,33 @@
         <v>35</v>
       </c>
       <c r="G1" s="2" t="s">
+        <v>221</v>
+      </c>
+      <c r="H1" s="2" t="s">
         <v>222</v>
-      </c>
-      <c r="H1" s="2" t="s">
-        <v>223</v>
       </c>
     </row>
     <row r="2" spans="1:229" s="4" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A2" s="3" t="s">
+        <v>402</v>
+      </c>
+      <c r="B2" s="3" t="s">
         <v>403</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="C2" s="3" t="s">
         <v>404</v>
-      </c>
-      <c r="C2" s="3" t="s">
-        <v>405</v>
       </c>
       <c r="D2" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E2" s="3" t="s">
+        <v>213</v>
+      </c>
+      <c r="F2" s="3" t="s">
         <v>214</v>
       </c>
-      <c r="F2" s="3" t="s">
-        <v>215</v>
-      </c>
       <c r="G2" s="3" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="H2" s="3" t="s">
         <v>195</v>
@@ -15563,158 +15563,158 @@
     </row>
     <row r="3" spans="1:229" x14ac:dyDescent="0.35">
       <c r="A3" s="3" t="s">
+        <v>405</v>
+      </c>
+      <c r="B3" s="3" t="s">
         <v>406</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="C3" s="3" t="s">
         <v>407</v>
-      </c>
-      <c r="C3" s="3" t="s">
-        <v>408</v>
       </c>
       <c r="D3" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E3" s="3" t="s">
+        <v>213</v>
+      </c>
+      <c r="F3" s="3" t="s">
         <v>214</v>
       </c>
-      <c r="F3" s="3" t="s">
-        <v>215</v>
-      </c>
       <c r="G3" s="3" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
     </row>
     <row r="4" spans="1:229" x14ac:dyDescent="0.35">
       <c r="A4" s="3" t="s">
+        <v>409</v>
+      </c>
+      <c r="B4" s="3" t="s">
         <v>410</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="C4" s="3" t="s">
         <v>411</v>
-      </c>
-      <c r="C4" s="3" t="s">
-        <v>412</v>
       </c>
       <c r="D4" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E4" s="3" t="s">
+        <v>213</v>
+      </c>
+      <c r="F4" s="3" t="s">
         <v>214</v>
       </c>
-      <c r="F4" s="3" t="s">
-        <v>215</v>
-      </c>
       <c r="G4" s="3" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>413</v>
+        <v>412</v>
       </c>
     </row>
     <row r="5" spans="1:229" x14ac:dyDescent="0.35">
       <c r="A5" s="8" t="s">
+        <v>413</v>
+      </c>
+      <c r="B5" s="8" t="s">
         <v>414</v>
       </c>
-      <c r="B5" s="8" t="s">
+      <c r="C5" s="8" t="s">
         <v>415</v>
-      </c>
-      <c r="C5" s="8" t="s">
-        <v>416</v>
       </c>
       <c r="D5" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E5" s="3" t="s">
+        <v>213</v>
+      </c>
+      <c r="F5" s="3" t="s">
         <v>214</v>
       </c>
-      <c r="F5" s="3" t="s">
-        <v>215</v>
-      </c>
       <c r="G5" s="3" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="H5" s="3" t="s">
-        <v>417</v>
+        <v>416</v>
       </c>
     </row>
     <row r="6" spans="1:229" x14ac:dyDescent="0.35">
       <c r="A6" s="3" t="s">
+        <v>417</v>
+      </c>
+      <c r="B6" s="3" t="s">
         <v>418</v>
       </c>
-      <c r="B6" s="3" t="s">
+      <c r="C6" s="3" t="s">
         <v>419</v>
-      </c>
-      <c r="C6" s="3" t="s">
-        <v>420</v>
       </c>
       <c r="D6" s="7" t="s">
         <v>0</v>
       </c>
       <c r="E6" s="3" t="s">
+        <v>213</v>
+      </c>
+      <c r="F6" s="3" t="s">
         <v>214</v>
       </c>
-      <c r="F6" s="3" t="s">
-        <v>215</v>
-      </c>
       <c r="G6" s="3" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="H6" s="3" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
     </row>
     <row r="7" spans="1:229" x14ac:dyDescent="0.35">
       <c r="A7" s="3" t="s">
+        <v>421</v>
+      </c>
+      <c r="B7" s="3" t="s">
         <v>422</v>
       </c>
-      <c r="B7" s="3" t="s">
+      <c r="C7" s="3" t="s">
         <v>423</v>
-      </c>
-      <c r="C7" s="3" t="s">
-        <v>424</v>
       </c>
       <c r="D7" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E7" s="3" t="s">
+        <v>213</v>
+      </c>
+      <c r="F7" s="3" t="s">
         <v>214</v>
       </c>
-      <c r="F7" s="3" t="s">
-        <v>215</v>
-      </c>
       <c r="G7" s="3" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="H7" s="3" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
     </row>
     <row r="8" spans="1:229" x14ac:dyDescent="0.35">
       <c r="A8" s="9" t="s">
+        <v>425</v>
+      </c>
+      <c r="B8" s="9" t="s">
         <v>426</v>
       </c>
-      <c r="B8" s="9" t="s">
+      <c r="C8" s="9" t="s">
         <v>427</v>
-      </c>
-      <c r="C8" s="9" t="s">
-        <v>428</v>
       </c>
       <c r="D8" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E8" s="3" t="s">
+        <v>213</v>
+      </c>
+      <c r="F8" s="3" t="s">
         <v>214</v>
       </c>
-      <c r="F8" s="3" t="s">
-        <v>215</v>
-      </c>
       <c r="G8" s="3" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="H8" s="9" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
     </row>
   </sheetData>
@@ -15758,22 +15758,22 @@
     </row>
     <row r="2" spans="1:1029" x14ac:dyDescent="0.35">
       <c r="A2" s="3" t="s">
+        <v>359</v>
+      </c>
+      <c r="B2" s="3" t="s">
         <v>360</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="C2" s="3" t="s">
         <v>361</v>
-      </c>
-      <c r="C2" s="3" t="s">
-        <v>362</v>
       </c>
       <c r="D2" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
     </row>
     <row r="3" spans="1:1029" x14ac:dyDescent="0.35">
@@ -15790,7 +15790,7 @@
         <v>0</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="F3" s="10" t="s">
         <v>81</v>
@@ -15810,7 +15810,7 @@
         <v>0</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="F4" s="3" t="s">
         <v>112</v>
@@ -15818,22 +15818,22 @@
     </row>
     <row r="5" spans="1:1029" s="4" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A5" s="3" t="s">
+        <v>433</v>
+      </c>
+      <c r="B5" s="3" t="s">
         <v>434</v>
       </c>
-      <c r="B5" s="3" t="s">
+      <c r="C5" s="3" t="s">
         <v>435</v>
-      </c>
-      <c r="C5" s="3" t="s">
-        <v>436</v>
       </c>
       <c r="D5" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>437</v>
+        <v>436</v>
       </c>
       <c r="G5"/>
       <c r="H5"/>
@@ -16873,7 +16873,7 @@
         <v>0</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="F6" s="10" t="s">
         <v>85</v>
@@ -16893,7 +16893,7 @@
         <v>0</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="F7" s="3" t="s">
         <v>77</v>
@@ -16901,22 +16901,22 @@
     </row>
     <row r="8" spans="1:1029" s="4" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A8" s="3" t="s">
+        <v>437</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>439</v>
+      </c>
+      <c r="C8" s="3" t="s">
         <v>438</v>
-      </c>
-      <c r="B8" s="3" t="s">
-        <v>440</v>
-      </c>
-      <c r="C8" s="3" t="s">
-        <v>439</v>
       </c>
       <c r="D8" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E8" s="3" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="F8" s="3" t="s">
-        <v>449</v>
+        <v>448</v>
       </c>
       <c r="G8"/>
       <c r="H8"/>
@@ -17944,42 +17944,42 @@
     </row>
     <row r="9" spans="1:1029" x14ac:dyDescent="0.35">
       <c r="A9" s="3" t="s">
+        <v>440</v>
+      </c>
+      <c r="B9" s="3" t="s">
         <v>441</v>
       </c>
-      <c r="B9" s="3" t="s">
+      <c r="C9" s="3" t="s">
         <v>442</v>
-      </c>
-      <c r="C9" s="3" t="s">
-        <v>443</v>
       </c>
       <c r="D9" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E9" s="3" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="F9" s="3" t="s">
-        <v>444</v>
+        <v>443</v>
       </c>
     </row>
     <row r="10" spans="1:1029" x14ac:dyDescent="0.35">
       <c r="A10" s="3" t="s">
+        <v>444</v>
+      </c>
+      <c r="B10" s="3" t="s">
         <v>445</v>
       </c>
-      <c r="B10" s="3" t="s">
+      <c r="C10" s="3" t="s">
         <v>446</v>
-      </c>
-      <c r="C10" s="3" t="s">
-        <v>447</v>
       </c>
       <c r="D10" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E10" s="3" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="F10" s="3" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
     </row>
     <row r="11" spans="1:1029" x14ac:dyDescent="0.35">
@@ -17996,7 +17996,7 @@
         <v>0</v>
       </c>
       <c r="E11" s="3" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="F11" s="10" t="s">
         <v>73</v>
@@ -18016,7 +18016,7 @@
         <v>0</v>
       </c>
       <c r="E12" s="3" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="F12" s="3" t="s">
         <v>108</v>
@@ -18548,13 +18548,13 @@
     </row>
     <row r="4" spans="1:229" s="4" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A4" s="3" t="s">
+        <v>363</v>
+      </c>
+      <c r="B4" s="3" t="s">
         <v>364</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="C4" s="3" t="s">
         <v>365</v>
-      </c>
-      <c r="C4" s="3" t="s">
-        <v>366</v>
       </c>
       <c r="D4" s="3" t="s">
         <v>0</v>
@@ -18563,7 +18563,7 @@
         <v>89</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="G4"/>
       <c r="H4"/>

</xml_diff>

<commit_message>
Privacy Policy US#15 Improve missing oe inaccurate info US#169 Business area fix #198
</commit_message>
<xml_diff>
--- a/testdata.xlsx
+++ b/testdata.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sshiwani\workspace\find-information-products-services-tests\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{24635E98-D493-4C20-BE24-573CC1FCB0CA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{297BEE1D-61DC-4366-971F-AE90EFF1E76A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="22780" windowHeight="14540" firstSheet="14" activeTab="15" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="22780" windowHeight="14540" firstSheet="13" activeTab="15" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="category_phase" sheetId="1" r:id="rId1"/>
@@ -28,15 +28,17 @@
     <sheet name="usergroup_ParentorCarer_list" sheetId="13" r:id="rId13"/>
     <sheet name="usergroup_ProfExtUserofDfE_list" sheetId="14" r:id="rId14"/>
     <sheet name="usergroup_SocialCWorkforce_list" sheetId="15" r:id="rId15"/>
-    <sheet name="UGSubcategory_AdultLearner" sheetId="16" r:id="rId16"/>
-    <sheet name="UGSubcategory_CareersAdviser" sheetId="17" r:id="rId17"/>
-    <sheet name="UGSubcategory_ChildOrYoungPers" sheetId="18" r:id="rId18"/>
-    <sheet name="UGSubcategory_DfEWorkforce" sheetId="19" r:id="rId19"/>
-    <sheet name="UGSubcategory_Employer" sheetId="20" r:id="rId20"/>
-    <sheet name="UGSubcategory_LAWorkforce" sheetId="21" r:id="rId21"/>
-    <sheet name="UGSubcategory_NEETOrCareerSeek" sheetId="22" r:id="rId22"/>
-    <sheet name="UGSubcategory_ParentOrCarer" sheetId="23" r:id="rId23"/>
-    <sheet name="UGSubcateg_ProfExtUserofDfEData" sheetId="24" r:id="rId24"/>
+    <sheet name="Sheet2" sheetId="26" r:id="rId16"/>
+    <sheet name="UGSubcategory_AdultLearner" sheetId="16" r:id="rId17"/>
+    <sheet name="UGSubcategory_CareersAdviser" sheetId="17" r:id="rId18"/>
+    <sheet name="UGSubcategory_ChildOrYoungPers" sheetId="18" r:id="rId19"/>
+    <sheet name="UGSubcategory_DfEWorkforce" sheetId="19" r:id="rId20"/>
+    <sheet name="UGSubcategory_Employer" sheetId="20" r:id="rId21"/>
+    <sheet name="UGSubcategory_LAWorkforce" sheetId="21" r:id="rId22"/>
+    <sheet name="UGSubcategory_NEETOrCareerSeek" sheetId="22" r:id="rId23"/>
+    <sheet name="UGSubcategory_ParentOrCarer" sheetId="23" r:id="rId24"/>
+    <sheet name="UGSubcateg_ProfExtUserofDfEData" sheetId="24" r:id="rId25"/>
+    <sheet name="Sheet1" sheetId="25" r:id="rId26"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -48,7 +50,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="889" uniqueCount="450">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="897" uniqueCount="450">
   <si>
     <t>Search and filter products and services</t>
   </si>
@@ -260,18 +262,6 @@
     <t>#channel-web</t>
   </si>
   <si>
-    <t>products?group=skills</t>
-  </si>
-  <si>
-    <t>ul.moj-filter-tags li a:has-text('skills')</t>
-  </si>
-  <si>
-    <t>Remove this filter skills</t>
-  </si>
-  <si>
-    <t>#group-skills</t>
-  </si>
-  <si>
     <t>products?group=operations-and-infrastructure</t>
   </si>
   <si>
@@ -284,30 +274,6 @@
     <t>#group-operations-and-infrastructure</t>
   </si>
   <si>
-    <t>products?group=cxd</t>
-  </si>
-  <si>
-    <t>ul.moj-filter-tags li a:has-text('cxd')</t>
-  </si>
-  <si>
-    <t>Remove this filter cxd</t>
-  </si>
-  <si>
-    <t>#group-cxd</t>
-  </si>
-  <si>
-    <t>products?group=funding</t>
-  </si>
-  <si>
-    <t>ul.moj-filter-tags li a:has-text('funding')</t>
-  </si>
-  <si>
-    <t>Remove this filter funding</t>
-  </si>
-  <si>
-    <t>#group-funding</t>
-  </si>
-  <si>
     <t>products?type=api</t>
   </si>
   <si>
@@ -1398,6 +1364,42 @@
   </si>
   <si>
     <t>Remove this filter Adult learner (18+)</t>
+  </si>
+  <si>
+    <t>products?group=customer-experience-and-design</t>
+  </si>
+  <si>
+    <t>Remove this filter customer-experience-and-design</t>
+  </si>
+  <si>
+    <t>ul.moj-filter-tags li a:has-text('customer-experience-and-design')</t>
+  </si>
+  <si>
+    <t>#group-customer-experience-and-design</t>
+  </si>
+  <si>
+    <t>Remove this filter funding-and-financial-oversight</t>
+  </si>
+  <si>
+    <t>products?group=funding-and-financial-oversight</t>
+  </si>
+  <si>
+    <t>ul.moj-filter-tags li a:has-text('funding-and-financial-oversight')</t>
+  </si>
+  <si>
+    <t>#group-funding-and-financial-oversight</t>
+  </si>
+  <si>
+    <t>products?group=skills-and-growth</t>
+  </si>
+  <si>
+    <t>ul.moj-filter-tags li a:has-text('skills-and-growth')</t>
+  </si>
+  <si>
+    <t>Remove this filter skills-and-growth</t>
+  </si>
+  <si>
+    <t>#group-skills-and-growth</t>
   </si>
 </sst>
 </file>
@@ -1419,7 +1421,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1447,12 +1449,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="6"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.59999389629810485"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1532,7 +1528,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
@@ -1543,7 +1539,6 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -4183,13 +4178,13 @@
     </row>
     <row r="4" spans="1:1149" s="5" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A4" s="3" t="s">
-        <v>429</v>
+        <v>417</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>430</v>
+        <v>418</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>431</v>
+        <v>419</v>
       </c>
       <c r="D4" s="3" t="s">
         <v>0</v>
@@ -4198,7 +4193,7 @@
         <v>1</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>432</v>
+        <v>420</v>
       </c>
       <c r="G4"/>
       <c r="H4"/>
@@ -11176,64 +11171,64 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" s="6" t="s">
-        <v>114</v>
+        <v>102</v>
       </c>
       <c r="B1" s="6" t="s">
-        <v>115</v>
+        <v>103</v>
       </c>
       <c r="C1" s="6" t="s">
-        <v>116</v>
+        <v>104</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" s="3" t="s">
-        <v>160</v>
+        <v>148</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>119</v>
+        <v>107</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>161</v>
+        <v>149</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="14" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B3" s="3" t="s">
-        <v>127</v>
+        <v>115</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>128</v>
+        <v>116</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.35">
       <c r="B4" s="3" t="s">
-        <v>125</v>
+        <v>113</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>126</v>
+        <v>114</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A5" s="3" t="s">
-        <v>162</v>
+        <v>150</v>
       </c>
       <c r="B5" s="3"/>
       <c r="C5" s="3"/>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A6" s="3" t="s">
-        <v>163</v>
+        <v>151</v>
       </c>
       <c r="B6" s="3"/>
       <c r="C6" s="3"/>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A7" s="3" t="s">
-        <v>164</v>
+        <v>152</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A8" s="3" t="s">
-        <v>165</v>
+        <v>153</v>
       </c>
     </row>
   </sheetData>
@@ -11253,78 +11248,78 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" s="6" t="s">
-        <v>114</v>
+        <v>102</v>
       </c>
       <c r="B1" s="6" t="s">
-        <v>115</v>
+        <v>103</v>
       </c>
       <c r="C1" s="6" t="s">
-        <v>116</v>
+        <v>104</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" s="3" t="s">
-        <v>166</v>
+        <v>154</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>119</v>
+        <v>107</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>167</v>
+        <v>155</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="14" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B3" s="3" t="s">
-        <v>127</v>
+        <v>115</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>128</v>
+        <v>116</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.35">
       <c r="B4" s="3" t="s">
-        <v>125</v>
+        <v>113</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>126</v>
+        <v>114</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A5" s="3" t="s">
-        <v>168</v>
+        <v>156</v>
       </c>
       <c r="B5" s="3"/>
       <c r="C5" s="3"/>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A6" s="3" t="s">
-        <v>169</v>
+        <v>157</v>
       </c>
       <c r="B6" s="3"/>
       <c r="C6" s="3"/>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A7" s="3" t="s">
-        <v>170</v>
+        <v>158</v>
       </c>
       <c r="B7" s="3"/>
       <c r="C7" s="3"/>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A8" s="3" t="s">
-        <v>171</v>
+        <v>159</v>
       </c>
       <c r="B8" s="3"/>
       <c r="C8" s="3"/>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A9" s="3" t="s">
-        <v>172</v>
+        <v>160</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A10" s="3" t="s">
-        <v>173</v>
+        <v>161</v>
       </c>
     </row>
   </sheetData>
@@ -11345,78 +11340,78 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" s="6" t="s">
-        <v>114</v>
+        <v>102</v>
       </c>
       <c r="B1" s="6" t="s">
-        <v>115</v>
+        <v>103</v>
       </c>
       <c r="C1" s="6" t="s">
-        <v>116</v>
+        <v>104</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" s="3" t="s">
-        <v>174</v>
+        <v>162</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>119</v>
+        <v>107</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>175</v>
+        <v>163</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="14" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B3" s="3" t="s">
-        <v>127</v>
+        <v>115</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>128</v>
+        <v>116</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.35">
       <c r="B4" s="3" t="s">
-        <v>125</v>
+        <v>113</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>126</v>
+        <v>114</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A5" s="3" t="s">
-        <v>176</v>
+        <v>164</v>
       </c>
       <c r="B5" s="3"/>
       <c r="C5" s="3"/>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A6" s="3" t="s">
-        <v>177</v>
+        <v>165</v>
       </c>
       <c r="B6" s="3"/>
       <c r="C6" s="3"/>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A7" s="3" t="s">
-        <v>178</v>
+        <v>166</v>
       </c>
       <c r="B7" s="3"/>
       <c r="C7" s="3"/>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A8" s="3" t="s">
-        <v>179</v>
+        <v>167</v>
       </c>
       <c r="B8" s="3"/>
       <c r="C8" s="3"/>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A9" s="3" t="s">
-        <v>180</v>
+        <v>168</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A10" s="3" t="s">
-        <v>181</v>
+        <v>169</v>
       </c>
     </row>
   </sheetData>
@@ -11436,99 +11431,99 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" s="6" t="s">
-        <v>114</v>
+        <v>102</v>
       </c>
       <c r="B1" s="6" t="s">
-        <v>115</v>
+        <v>103</v>
       </c>
       <c r="C1" s="6" t="s">
-        <v>116</v>
+        <v>104</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" s="3" t="s">
-        <v>182</v>
+        <v>170</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>119</v>
+        <v>107</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>183</v>
+        <v>171</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="14" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B3" s="3" t="s">
-        <v>127</v>
+        <v>115</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>128</v>
+        <v>116</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.35">
       <c r="B4" s="3" t="s">
-        <v>125</v>
+        <v>113</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>126</v>
+        <v>114</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A5" s="3" t="s">
-        <v>184</v>
+        <v>172</v>
       </c>
       <c r="B5" s="3"/>
       <c r="C5" s="3"/>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A6" s="3" t="s">
-        <v>185</v>
+        <v>173</v>
       </c>
       <c r="B6" s="3"/>
       <c r="C6" s="3"/>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A7" s="3" t="s">
-        <v>186</v>
+        <v>174</v>
       </c>
       <c r="B7" s="3"/>
       <c r="C7" s="3"/>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A8" s="3" t="s">
-        <v>187</v>
+        <v>175</v>
       </c>
       <c r="B8" s="3"/>
       <c r="C8" s="3"/>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A9" s="3" t="s">
-        <v>188</v>
+        <v>176</v>
       </c>
       <c r="B9" s="3"/>
       <c r="C9" s="3"/>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A10" s="3" t="s">
-        <v>189</v>
+        <v>177</v>
       </c>
       <c r="B10" s="3"/>
       <c r="C10" s="3"/>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A11" s="3" t="s">
-        <v>190</v>
+        <v>178</v>
       </c>
       <c r="B11" s="3"/>
       <c r="C11" s="3"/>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A12" s="3" t="s">
-        <v>191</v>
+        <v>179</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A13" s="3" t="s">
-        <v>192</v>
+        <v>180</v>
       </c>
     </row>
   </sheetData>
@@ -11548,85 +11543,85 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" s="6" t="s">
-        <v>114</v>
+        <v>102</v>
       </c>
       <c r="B1" s="6" t="s">
-        <v>115</v>
+        <v>103</v>
       </c>
       <c r="C1" s="6" t="s">
-        <v>116</v>
+        <v>104</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" s="3" t="s">
-        <v>193</v>
+        <v>181</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>119</v>
+        <v>107</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>194</v>
+        <v>182</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="14" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B3" s="3" t="s">
-        <v>127</v>
+        <v>115</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>128</v>
+        <v>116</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.35">
       <c r="B4" s="3" t="s">
-        <v>125</v>
+        <v>113</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>126</v>
+        <v>114</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A5" s="3" t="s">
-        <v>195</v>
+        <v>183</v>
       </c>
       <c r="B5" s="3"/>
       <c r="C5" s="3"/>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A6" s="3" t="s">
-        <v>196</v>
+        <v>184</v>
       </c>
       <c r="B6" s="3"/>
       <c r="C6" s="3"/>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A7" s="3" t="s">
-        <v>197</v>
+        <v>185</v>
       </c>
       <c r="B7" s="3"/>
       <c r="C7" s="3"/>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A8" s="3" t="s">
-        <v>198</v>
+        <v>186</v>
       </c>
       <c r="B8" s="3"/>
       <c r="C8" s="3"/>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A9" s="3" t="s">
-        <v>199</v>
+        <v>187</v>
       </c>
       <c r="B9" s="3"/>
       <c r="C9" s="3"/>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A10" s="3" t="s">
-        <v>200</v>
+        <v>188</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A11" s="3" t="s">
-        <v>201</v>
+        <v>189</v>
       </c>
     </row>
   </sheetData>
@@ -11646,99 +11641,99 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" s="6" t="s">
-        <v>114</v>
+        <v>102</v>
       </c>
       <c r="B1" s="6" t="s">
-        <v>115</v>
+        <v>103</v>
       </c>
       <c r="C1" s="6" t="s">
-        <v>116</v>
+        <v>104</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" s="3" t="s">
-        <v>202</v>
+        <v>190</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>119</v>
+        <v>107</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>203</v>
+        <v>191</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="14" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B3" s="3" t="s">
-        <v>127</v>
+        <v>115</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>128</v>
+        <v>116</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.35">
       <c r="B4" s="3" t="s">
-        <v>125</v>
+        <v>113</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>126</v>
+        <v>114</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A5" s="3" t="s">
-        <v>204</v>
+        <v>192</v>
       </c>
       <c r="B5" s="3"/>
       <c r="C5" s="3"/>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A6" s="3" t="s">
-        <v>205</v>
+        <v>193</v>
       </c>
       <c r="B6" s="3"/>
       <c r="C6" s="3"/>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A7" s="3" t="s">
-        <v>206</v>
+        <v>194</v>
       </c>
       <c r="B7" s="3"/>
       <c r="C7" s="3"/>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A8" s="3" t="s">
-        <v>207</v>
+        <v>195</v>
       </c>
       <c r="B8" s="3"/>
       <c r="C8" s="3"/>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A9" s="3" t="s">
-        <v>208</v>
+        <v>196</v>
       </c>
       <c r="B9" s="3"/>
       <c r="C9" s="3"/>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A10" s="3" t="s">
-        <v>209</v>
+        <v>197</v>
       </c>
       <c r="B10" s="3"/>
       <c r="C10" s="3"/>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A11" s="3" t="s">
-        <v>210</v>
+        <v>198</v>
       </c>
       <c r="B11" s="3"/>
       <c r="C11" s="3"/>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A12" s="3" t="s">
-        <v>211</v>
+        <v>199</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A13" s="3" t="s">
-        <v>212</v>
+        <v>200</v>
       </c>
     </row>
   </sheetData>
@@ -11747,6 +11742,91 @@
 </file>
 
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8B03D9F5-4C72-4FCD-8443-70945EFA9D2B}">
+  <dimension ref="A1:C12"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="54.1796875" customWidth="1"/>
+    <col min="2" max="2" width="47.453125" customWidth="1"/>
+    <col min="3" max="3" width="43.90625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A1" s="3" t="s">
+        <v>190</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>107</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="B2" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="B3" s="3" t="s">
+        <v>113</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A4" s="3" t="s">
+        <v>192</v>
+      </c>
+      <c r="B4" s="3"/>
+      <c r="C4" s="3"/>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A5" s="3"/>
+      <c r="B5" s="3"/>
+      <c r="C5" s="3"/>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A6" s="3"/>
+      <c r="B6" s="3"/>
+      <c r="C6" s="3"/>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A7" s="3"/>
+      <c r="B7" s="3"/>
+      <c r="C7" s="3"/>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A8" s="3"/>
+      <c r="B8" s="3"/>
+      <c r="C8" s="3"/>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A9" s="3"/>
+      <c r="B9" s="3"/>
+      <c r="C9" s="3"/>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A10" s="3"/>
+      <c r="B10" s="3"/>
+      <c r="C10" s="3"/>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A11" s="3"/>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A12" s="3"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FB5527F7-85DB-4F8E-B4B3-EC8453E599E1}">
   <dimension ref="A1:HU6"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -11781,36 +11861,36 @@
         <v>35</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>221</v>
+        <v>209</v>
       </c>
       <c r="H1" s="2" t="s">
-        <v>222</v>
+        <v>210</v>
       </c>
     </row>
     <row r="2" spans="1:229" s="4" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A2" s="3" t="s">
-        <v>216</v>
+        <v>204</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>215</v>
+        <v>203</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>449</v>
+        <v>437</v>
       </c>
       <c r="D2" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>213</v>
+        <v>201</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>214</v>
+        <v>202</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>223</v>
+        <v>211</v>
       </c>
       <c r="H2" s="3" t="s">
-        <v>120</v>
+        <v>108</v>
       </c>
       <c r="I2"/>
       <c r="J2"/>
@@ -12036,106 +12116,106 @@
     </row>
     <row r="3" spans="1:229" x14ac:dyDescent="0.35">
       <c r="A3" s="3" t="s">
-        <v>217</v>
+        <v>205</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>219</v>
+        <v>207</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>220</v>
+        <v>208</v>
       </c>
       <c r="D3" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E3" s="3" t="s">
+        <v>201</v>
+      </c>
+      <c r="F3" s="3" t="s">
+        <v>202</v>
+      </c>
+      <c r="G3" s="3" t="s">
+        <v>212</v>
+      </c>
+      <c r="H3" s="3" t="s">
         <v>213</v>
-      </c>
-      <c r="F3" s="3" t="s">
-        <v>214</v>
-      </c>
-      <c r="G3" s="3" t="s">
-        <v>224</v>
-      </c>
-      <c r="H3" s="3" t="s">
-        <v>225</v>
       </c>
     </row>
     <row r="4" spans="1:229" x14ac:dyDescent="0.35">
       <c r="A4" s="3" t="s">
-        <v>218</v>
+        <v>206</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>226</v>
+        <v>214</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>227</v>
+        <v>215</v>
       </c>
       <c r="D4" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>213</v>
+        <v>201</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>214</v>
+        <v>202</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>228</v>
+        <v>216</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>229</v>
+        <v>217</v>
       </c>
     </row>
     <row r="5" spans="1:229" x14ac:dyDescent="0.35">
       <c r="A5" s="3" t="s">
-        <v>230</v>
+        <v>218</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>231</v>
+        <v>219</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>232</v>
+        <v>220</v>
       </c>
       <c r="D5" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>213</v>
+        <v>201</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>214</v>
+        <v>202</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>233</v>
+        <v>221</v>
       </c>
       <c r="H5" s="3" t="s">
-        <v>234</v>
+        <v>222</v>
       </c>
     </row>
     <row r="6" spans="1:229" x14ac:dyDescent="0.35">
       <c r="A6" s="3" t="s">
-        <v>235</v>
+        <v>223</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>236</v>
+        <v>224</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>237</v>
+        <v>225</v>
       </c>
       <c r="D6" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>213</v>
+        <v>201</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>214</v>
+        <v>202</v>
       </c>
       <c r="G6" s="3" t="s">
-        <v>238</v>
+        <v>226</v>
       </c>
       <c r="H6" s="3" t="s">
-        <v>239</v>
+        <v>227</v>
       </c>
     </row>
   </sheetData>
@@ -12144,7 +12224,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A99CF6C3-F305-48A2-AB80-2C2D7CE6460C}">
   <dimension ref="A1:HU5"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -12179,36 +12259,36 @@
         <v>35</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>221</v>
+        <v>209</v>
       </c>
       <c r="H1" s="2" t="s">
-        <v>222</v>
+        <v>210</v>
       </c>
     </row>
     <row r="2" spans="1:229" s="4" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A2" s="3" t="s">
-        <v>240</v>
+        <v>228</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>241</v>
+        <v>229</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>242</v>
+        <v>230</v>
       </c>
       <c r="D2" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>213</v>
+        <v>201</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>214</v>
+        <v>202</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>223</v>
+        <v>211</v>
       </c>
       <c r="H2" s="3" t="s">
-        <v>131</v>
+        <v>119</v>
       </c>
       <c r="I2"/>
       <c r="J2"/>
@@ -12434,80 +12514,80 @@
     </row>
     <row r="3" spans="1:229" x14ac:dyDescent="0.35">
       <c r="A3" s="3" t="s">
-        <v>243</v>
+        <v>231</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>244</v>
+        <v>232</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>245</v>
+        <v>233</v>
       </c>
       <c r="D3" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>213</v>
+        <v>201</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>214</v>
+        <v>202</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>223</v>
+        <v>211</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>246</v>
+        <v>234</v>
       </c>
     </row>
     <row r="4" spans="1:229" x14ac:dyDescent="0.35">
       <c r="A4" s="3" t="s">
-        <v>247</v>
+        <v>235</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>248</v>
+        <v>236</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>249</v>
+        <v>237</v>
       </c>
       <c r="D4" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>213</v>
+        <v>201</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>214</v>
+        <v>202</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>223</v>
+        <v>211</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>250</v>
+        <v>238</v>
       </c>
     </row>
     <row r="5" spans="1:229" x14ac:dyDescent="0.35">
       <c r="A5" s="3" t="s">
-        <v>251</v>
+        <v>239</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>252</v>
+        <v>240</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>253</v>
+        <v>241</v>
       </c>
       <c r="D5" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>213</v>
+        <v>201</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>214</v>
+        <v>202</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>223</v>
+        <v>211</v>
       </c>
       <c r="H5" s="3" t="s">
-        <v>254</v>
+        <v>242</v>
       </c>
     </row>
   </sheetData>
@@ -12515,7 +12595,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5EFF0597-7FD1-4E6A-AA71-DB9F9FAB97A9}">
   <dimension ref="A1:HU7"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -12550,36 +12630,36 @@
         <v>35</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>221</v>
+        <v>209</v>
       </c>
       <c r="H1" s="2" t="s">
-        <v>222</v>
+        <v>210</v>
       </c>
     </row>
     <row r="2" spans="1:229" s="4" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A2" s="3" t="s">
-        <v>255</v>
+        <v>243</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>256</v>
+        <v>244</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>257</v>
+        <v>245</v>
       </c>
       <c r="D2" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>213</v>
+        <v>201</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>214</v>
+        <v>202</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>223</v>
+        <v>211</v>
       </c>
       <c r="H2" s="3" t="s">
-        <v>140</v>
+        <v>128</v>
       </c>
       <c r="I2"/>
       <c r="J2"/>
@@ -12805,132 +12885,132 @@
     </row>
     <row r="3" spans="1:229" x14ac:dyDescent="0.35">
       <c r="A3" s="3" t="s">
-        <v>258</v>
+        <v>246</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>259</v>
+        <v>247</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>260</v>
+        <v>248</v>
       </c>
       <c r="D3" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>213</v>
+        <v>201</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>214</v>
+        <v>202</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>223</v>
+        <v>211</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>261</v>
+        <v>249</v>
       </c>
     </row>
     <row r="4" spans="1:229" x14ac:dyDescent="0.35">
       <c r="A4" s="3" t="s">
-        <v>262</v>
+        <v>250</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>264</v>
+        <v>252</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>263</v>
+        <v>251</v>
       </c>
       <c r="D4" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>213</v>
+        <v>201</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>214</v>
+        <v>202</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>223</v>
+        <v>211</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>265</v>
+        <v>253</v>
       </c>
     </row>
     <row r="5" spans="1:229" x14ac:dyDescent="0.35">
       <c r="A5" s="8" t="s">
-        <v>266</v>
+        <v>254</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>267</v>
+        <v>255</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>268</v>
+        <v>256</v>
       </c>
       <c r="D5" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>213</v>
+        <v>201</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>214</v>
+        <v>202</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>223</v>
+        <v>211</v>
       </c>
       <c r="H5" s="3" t="s">
-        <v>269</v>
+        <v>257</v>
       </c>
     </row>
     <row r="6" spans="1:229" x14ac:dyDescent="0.35">
       <c r="A6" s="3" t="s">
-        <v>270</v>
+        <v>258</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>271</v>
+        <v>259</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>272</v>
+        <v>260</v>
       </c>
       <c r="D6" s="7" t="s">
         <v>0</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>213</v>
+        <v>201</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>214</v>
+        <v>202</v>
       </c>
       <c r="G6" s="3" t="s">
-        <v>223</v>
+        <v>211</v>
       </c>
       <c r="H6" s="3" t="s">
-        <v>273</v>
+        <v>261</v>
       </c>
     </row>
     <row r="7" spans="1:229" x14ac:dyDescent="0.35">
       <c r="A7" s="3" t="s">
-        <v>274</v>
+        <v>262</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>276</v>
+        <v>264</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>275</v>
+        <v>263</v>
       </c>
       <c r="D7" s="7" t="s">
         <v>0</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>213</v>
+        <v>201</v>
       </c>
       <c r="F7" s="3" t="s">
-        <v>214</v>
+        <v>202</v>
       </c>
       <c r="G7" s="3" t="s">
-        <v>223</v>
+        <v>211</v>
       </c>
       <c r="H7" s="3" t="s">
-        <v>277</v>
+        <v>265</v>
       </c>
     </row>
   </sheetData>
@@ -12939,7 +13019,225 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B2DC696B-E1A8-430C-BC9E-87DD1A6FBE9F}">
+  <dimension ref="A1:F10"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="33.08984375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="43.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="32.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="33.36328125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="29.90625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="25.36328125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A2" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="F2" s="3" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A3" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>101</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="F3" s="3" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A4" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="F4" s="3" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A5" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>91</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="F5" s="3" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A6" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="D6" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="E6" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="F6" s="3" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A7" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="E7" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="F7" s="3" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A8" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="D8" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="E8" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="F8" s="3" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A9" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="D9" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="E9" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="F9" s="3" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A10" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="D10" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="E10" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="F10" s="3" t="s">
+        <v>69</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9F4A57AC-4620-4875-88AE-9F5C739A9042}">
   <dimension ref="A1:HU6"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -12974,36 +13272,36 @@
         <v>35</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>221</v>
+        <v>209</v>
       </c>
       <c r="H1" s="2" t="s">
-        <v>222</v>
+        <v>210</v>
       </c>
     </row>
     <row r="2" spans="1:229" s="4" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A2" s="3" t="s">
-        <v>278</v>
+        <v>266</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>279</v>
+        <v>267</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>280</v>
+        <v>268</v>
       </c>
       <c r="D2" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>213</v>
+        <v>201</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>214</v>
+        <v>202</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>223</v>
+        <v>211</v>
       </c>
       <c r="H2" s="3" t="s">
-        <v>145</v>
+        <v>133</v>
       </c>
       <c r="I2"/>
       <c r="J2"/>
@@ -13229,106 +13527,106 @@
     </row>
     <row r="3" spans="1:229" x14ac:dyDescent="0.35">
       <c r="A3" s="3" t="s">
-        <v>281</v>
+        <v>269</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>282</v>
+        <v>270</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>283</v>
+        <v>271</v>
       </c>
       <c r="D3" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>213</v>
+        <v>201</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>214</v>
+        <v>202</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>223</v>
+        <v>211</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>284</v>
+        <v>272</v>
       </c>
     </row>
     <row r="4" spans="1:229" x14ac:dyDescent="0.35">
       <c r="A4" s="3" t="s">
-        <v>285</v>
+        <v>273</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>286</v>
+        <v>274</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>287</v>
+        <v>275</v>
       </c>
       <c r="D4" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>213</v>
+        <v>201</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>214</v>
+        <v>202</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>223</v>
+        <v>211</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>288</v>
+        <v>276</v>
       </c>
     </row>
     <row r="5" spans="1:229" x14ac:dyDescent="0.35">
       <c r="A5" s="8" t="s">
-        <v>289</v>
+        <v>277</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>290</v>
+        <v>278</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>291</v>
+        <v>279</v>
       </c>
       <c r="D5" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>213</v>
+        <v>201</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>214</v>
+        <v>202</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>223</v>
+        <v>211</v>
       </c>
       <c r="H5" s="3" t="s">
-        <v>292</v>
+        <v>280</v>
       </c>
     </row>
     <row r="6" spans="1:229" x14ac:dyDescent="0.35">
       <c r="A6" s="3" t="s">
-        <v>293</v>
+        <v>281</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>294</v>
+        <v>282</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>295</v>
+        <v>283</v>
       </c>
       <c r="D6" s="7" t="s">
         <v>0</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>213</v>
+        <v>201</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>214</v>
+        <v>202</v>
       </c>
       <c r="G6" s="3" t="s">
-        <v>223</v>
+        <v>211</v>
       </c>
       <c r="H6" s="3" t="s">
-        <v>296</v>
+        <v>284</v>
       </c>
     </row>
   </sheetData>
@@ -13336,225 +13634,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B2DC696B-E1A8-430C-BC9E-87DD1A6FBE9F}">
-  <dimension ref="A1:F10"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
-  <cols>
-    <col min="1" max="1" width="33.08984375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="43.54296875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="32.1796875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="33.36328125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="29.90625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="25.36328125" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A1" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="F1" s="2" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="3" t="s">
-        <v>38</v>
-      </c>
-      <c r="B2" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="C2" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="D2" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="E2" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="F2" s="3" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="3" t="s">
-        <v>41</v>
-      </c>
-      <c r="B3" s="3" t="s">
-        <v>113</v>
-      </c>
-      <c r="C3" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="D3" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="E3" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="F3" s="3" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="3" t="s">
-        <v>45</v>
-      </c>
-      <c r="B4" s="3" t="s">
-        <v>44</v>
-      </c>
-      <c r="C4" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="D4" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="E4" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="F4" s="3" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="B5" s="3" t="s">
-        <v>103</v>
-      </c>
-      <c r="C5" s="3" t="s">
-        <v>104</v>
-      </c>
-      <c r="D5" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="E5" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="F5" s="3" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="3" t="s">
-        <v>50</v>
-      </c>
-      <c r="B6" s="3" t="s">
-        <v>51</v>
-      </c>
-      <c r="C6" s="3" t="s">
-        <v>52</v>
-      </c>
-      <c r="D6" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="E6" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="F6" s="3" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A7" s="3" t="s">
-        <v>54</v>
-      </c>
-      <c r="B7" s="3" t="s">
-        <v>55</v>
-      </c>
-      <c r="C7" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="D7" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="E7" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="F7" s="3" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A8" s="3" t="s">
-        <v>58</v>
-      </c>
-      <c r="B8" s="3" t="s">
-        <v>59</v>
-      </c>
-      <c r="C8" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="D8" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="E8" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="F8" s="3" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A9" s="3" t="s">
-        <v>62</v>
-      </c>
-      <c r="B9" s="3" t="s">
-        <v>63</v>
-      </c>
-      <c r="C9" s="3" t="s">
-        <v>64</v>
-      </c>
-      <c r="D9" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="E9" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="F9" s="3" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A10" s="3" t="s">
-        <v>66</v>
-      </c>
-      <c r="B10" s="3" t="s">
-        <v>67</v>
-      </c>
-      <c r="C10" s="3" t="s">
-        <v>68</v>
-      </c>
-      <c r="D10" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="E10" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="F10" s="3" t="s">
-        <v>69</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6C1C130F-0899-4810-82F6-950C9CB07234}">
   <dimension ref="A1:HU5"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -13589,36 +13669,36 @@
         <v>35</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>221</v>
+        <v>209</v>
       </c>
       <c r="H1" s="2" t="s">
-        <v>222</v>
+        <v>210</v>
       </c>
     </row>
     <row r="2" spans="1:229" s="4" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A2" s="3" t="s">
-        <v>297</v>
+        <v>285</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>298</v>
+        <v>286</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>299</v>
+        <v>287</v>
       </c>
       <c r="D2" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>213</v>
+        <v>201</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>214</v>
+        <v>202</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>223</v>
+        <v>211</v>
       </c>
       <c r="H2" s="3" t="s">
-        <v>162</v>
+        <v>150</v>
       </c>
       <c r="I2"/>
       <c r="J2"/>
@@ -13844,80 +13924,80 @@
     </row>
     <row r="3" spans="1:229" x14ac:dyDescent="0.35">
       <c r="A3" s="3" t="s">
-        <v>300</v>
+        <v>288</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>301</v>
+        <v>289</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>302</v>
+        <v>290</v>
       </c>
       <c r="D3" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>213</v>
+        <v>201</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>214</v>
+        <v>202</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>223</v>
+        <v>211</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>303</v>
+        <v>291</v>
       </c>
     </row>
     <row r="4" spans="1:229" x14ac:dyDescent="0.35">
       <c r="A4" s="3" t="s">
-        <v>304</v>
+        <v>292</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>305</v>
+        <v>293</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>306</v>
+        <v>294</v>
       </c>
       <c r="D4" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>213</v>
+        <v>201</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>214</v>
+        <v>202</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>223</v>
+        <v>211</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>307</v>
+        <v>295</v>
       </c>
     </row>
     <row r="5" spans="1:229" x14ac:dyDescent="0.35">
       <c r="A5" s="3" t="s">
-        <v>308</v>
+        <v>296</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>309</v>
+        <v>297</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>310</v>
+        <v>298</v>
       </c>
       <c r="D5" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>213</v>
+        <v>201</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>214</v>
+        <v>202</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>223</v>
+        <v>211</v>
       </c>
       <c r="H5" s="3" t="s">
-        <v>311</v>
+        <v>299</v>
       </c>
     </row>
   </sheetData>
@@ -13925,7 +14005,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4AB9395B-D522-49AD-B790-5334356249F6}">
   <dimension ref="A1:HU7"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -13960,36 +14040,36 @@
         <v>35</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>221</v>
+        <v>209</v>
       </c>
       <c r="H1" s="2" t="s">
-        <v>222</v>
+        <v>210</v>
       </c>
     </row>
     <row r="2" spans="1:229" s="4" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A2" s="3" t="s">
-        <v>312</v>
+        <v>300</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>313</v>
+        <v>301</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>314</v>
+        <v>302</v>
       </c>
       <c r="D2" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>213</v>
+        <v>201</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>214</v>
+        <v>202</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>223</v>
+        <v>211</v>
       </c>
       <c r="H2" s="3" t="s">
-        <v>168</v>
+        <v>156</v>
       </c>
       <c r="I2"/>
       <c r="J2"/>
@@ -14215,132 +14295,132 @@
     </row>
     <row r="3" spans="1:229" x14ac:dyDescent="0.35">
       <c r="A3" s="3" t="s">
-        <v>315</v>
+        <v>303</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>316</v>
+        <v>304</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>317</v>
+        <v>305</v>
       </c>
       <c r="D3" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>213</v>
+        <v>201</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>214</v>
+        <v>202</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>223</v>
+        <v>211</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>318</v>
+        <v>306</v>
       </c>
     </row>
     <row r="4" spans="1:229" x14ac:dyDescent="0.35">
       <c r="A4" s="3" t="s">
-        <v>319</v>
+        <v>307</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>320</v>
+        <v>308</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>321</v>
+        <v>309</v>
       </c>
       <c r="D4" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>213</v>
+        <v>201</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>214</v>
+        <v>202</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>223</v>
+        <v>211</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>322</v>
+        <v>310</v>
       </c>
     </row>
     <row r="5" spans="1:229" x14ac:dyDescent="0.35">
       <c r="A5" s="8" t="s">
-        <v>323</v>
+        <v>311</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>324</v>
+        <v>312</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>325</v>
+        <v>313</v>
       </c>
       <c r="D5" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>213</v>
+        <v>201</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>214</v>
+        <v>202</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>223</v>
+        <v>211</v>
       </c>
       <c r="H5" s="3" t="s">
-        <v>326</v>
+        <v>314</v>
       </c>
     </row>
     <row r="6" spans="1:229" x14ac:dyDescent="0.35">
       <c r="A6" s="3" t="s">
-        <v>327</v>
+        <v>315</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>329</v>
+        <v>317</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>328</v>
+        <v>316</v>
       </c>
       <c r="D6" s="7" t="s">
         <v>0</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>213</v>
+        <v>201</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>214</v>
+        <v>202</v>
       </c>
       <c r="G6" s="3" t="s">
-        <v>223</v>
+        <v>211</v>
       </c>
       <c r="H6" s="3" t="s">
-        <v>330</v>
+        <v>318</v>
       </c>
     </row>
     <row r="7" spans="1:229" x14ac:dyDescent="0.35">
       <c r="A7" s="3" t="s">
-        <v>331</v>
+        <v>319</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>332</v>
+        <v>320</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>333</v>
+        <v>321</v>
       </c>
       <c r="D7" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>213</v>
+        <v>201</v>
       </c>
       <c r="F7" s="3" t="s">
-        <v>214</v>
+        <v>202</v>
       </c>
       <c r="G7" s="3" t="s">
-        <v>223</v>
+        <v>211</v>
       </c>
       <c r="H7" s="3" t="s">
-        <v>334</v>
+        <v>322</v>
       </c>
     </row>
   </sheetData>
@@ -14348,7 +14428,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BEE91763-AD0C-4544-A433-3B50C88AEB79}">
   <dimension ref="A1:HU7"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -14383,36 +14463,36 @@
         <v>35</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>221</v>
+        <v>209</v>
       </c>
       <c r="H1" s="2" t="s">
-        <v>222</v>
+        <v>210</v>
       </c>
     </row>
     <row r="2" spans="1:229" s="4" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A2" s="3" t="s">
-        <v>335</v>
+        <v>323</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>336</v>
+        <v>324</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>337</v>
+        <v>325</v>
       </c>
       <c r="D2" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>213</v>
+        <v>201</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>214</v>
+        <v>202</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>223</v>
+        <v>211</v>
       </c>
       <c r="H2" s="3" t="s">
-        <v>176</v>
+        <v>164</v>
       </c>
       <c r="I2"/>
       <c r="J2"/>
@@ -14638,132 +14718,132 @@
     </row>
     <row r="3" spans="1:229" x14ac:dyDescent="0.35">
       <c r="A3" s="3" t="s">
-        <v>338</v>
+        <v>326</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>339</v>
+        <v>327</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>340</v>
+        <v>328</v>
       </c>
       <c r="D3" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>213</v>
+        <v>201</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>214</v>
+        <v>202</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>223</v>
+        <v>211</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>341</v>
+        <v>329</v>
       </c>
     </row>
     <row r="4" spans="1:229" x14ac:dyDescent="0.35">
       <c r="A4" s="3" t="s">
-        <v>342</v>
+        <v>330</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>344</v>
+        <v>332</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>343</v>
+        <v>331</v>
       </c>
       <c r="D4" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>213</v>
+        <v>201</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>214</v>
+        <v>202</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>223</v>
+        <v>211</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>345</v>
+        <v>333</v>
       </c>
     </row>
     <row r="5" spans="1:229" x14ac:dyDescent="0.35">
       <c r="A5" s="8" t="s">
-        <v>346</v>
+        <v>334</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>347</v>
+        <v>335</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>348</v>
+        <v>336</v>
       </c>
       <c r="D5" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>213</v>
+        <v>201</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>214</v>
+        <v>202</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>223</v>
+        <v>211</v>
       </c>
       <c r="H5" s="3" t="s">
-        <v>349</v>
+        <v>337</v>
       </c>
     </row>
     <row r="6" spans="1:229" x14ac:dyDescent="0.35">
       <c r="A6" s="3" t="s">
-        <v>350</v>
+        <v>338</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>352</v>
+        <v>340</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>351</v>
+        <v>339</v>
       </c>
       <c r="D6" s="7" t="s">
         <v>0</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>213</v>
+        <v>201</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>214</v>
+        <v>202</v>
       </c>
       <c r="G6" s="3" t="s">
-        <v>223</v>
+        <v>211</v>
       </c>
       <c r="H6" s="3" t="s">
-        <v>353</v>
+        <v>341</v>
       </c>
     </row>
     <row r="7" spans="1:229" x14ac:dyDescent="0.35">
       <c r="A7" s="3" t="s">
-        <v>354</v>
+        <v>342</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>355</v>
+        <v>343</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>356</v>
+        <v>344</v>
       </c>
       <c r="D7" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>213</v>
+        <v>201</v>
       </c>
       <c r="F7" s="3" t="s">
-        <v>214</v>
+        <v>202</v>
       </c>
       <c r="G7" s="3" t="s">
-        <v>223</v>
+        <v>211</v>
       </c>
       <c r="H7" s="3" t="s">
-        <v>357</v>
+        <v>345</v>
       </c>
     </row>
   </sheetData>
@@ -14771,7 +14851,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{20DD36AA-F163-4AAB-BD30-4AE6290CCAE7}">
   <dimension ref="A1:HU10"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -14806,36 +14886,36 @@
         <v>35</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>221</v>
+        <v>209</v>
       </c>
       <c r="H1" s="2" t="s">
-        <v>222</v>
+        <v>210</v>
       </c>
     </row>
     <row r="2" spans="1:229" s="4" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A2" s="3" t="s">
-        <v>367</v>
+        <v>355</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>368</v>
+        <v>356</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>369</v>
+        <v>357</v>
       </c>
       <c r="D2" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>213</v>
+        <v>201</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>214</v>
+        <v>202</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>223</v>
+        <v>211</v>
       </c>
       <c r="H2" s="3" t="s">
-        <v>184</v>
+        <v>172</v>
       </c>
       <c r="I2"/>
       <c r="J2"/>
@@ -15061,210 +15141,210 @@
     </row>
     <row r="3" spans="1:229" x14ac:dyDescent="0.35">
       <c r="A3" s="3" t="s">
-        <v>370</v>
+        <v>358</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>371</v>
+        <v>359</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>372</v>
+        <v>360</v>
       </c>
       <c r="D3" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>213</v>
+        <v>201</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>214</v>
+        <v>202</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>223</v>
+        <v>211</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>373</v>
+        <v>361</v>
       </c>
     </row>
     <row r="4" spans="1:229" x14ac:dyDescent="0.35">
       <c r="A4" s="3" t="s">
-        <v>374</v>
+        <v>362</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>375</v>
+        <v>363</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>376</v>
+        <v>364</v>
       </c>
       <c r="D4" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>213</v>
+        <v>201</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>214</v>
+        <v>202</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>223</v>
+        <v>211</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>377</v>
+        <v>365</v>
       </c>
     </row>
     <row r="5" spans="1:229" x14ac:dyDescent="0.35">
       <c r="A5" s="8" t="s">
-        <v>378</v>
+        <v>366</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>379</v>
+        <v>367</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>380</v>
+        <v>368</v>
       </c>
       <c r="D5" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>213</v>
+        <v>201</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>214</v>
+        <v>202</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>223</v>
+        <v>211</v>
       </c>
       <c r="H5" s="3" t="s">
-        <v>381</v>
+        <v>369</v>
       </c>
     </row>
     <row r="6" spans="1:229" x14ac:dyDescent="0.35">
       <c r="A6" s="3" t="s">
-        <v>382</v>
+        <v>370</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>383</v>
+        <v>371</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>384</v>
+        <v>372</v>
       </c>
       <c r="D6" s="7" t="s">
         <v>0</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>213</v>
+        <v>201</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>214</v>
+        <v>202</v>
       </c>
       <c r="G6" s="3" t="s">
-        <v>223</v>
+        <v>211</v>
       </c>
       <c r="H6" s="3" t="s">
-        <v>385</v>
+        <v>373</v>
       </c>
     </row>
     <row r="7" spans="1:229" x14ac:dyDescent="0.35">
       <c r="A7" s="3" t="s">
-        <v>386</v>
+        <v>374</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>387</v>
+        <v>375</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>388</v>
+        <v>376</v>
       </c>
       <c r="D7" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>213</v>
+        <v>201</v>
       </c>
       <c r="F7" s="3" t="s">
-        <v>214</v>
+        <v>202</v>
       </c>
       <c r="G7" s="3" t="s">
-        <v>223</v>
+        <v>211</v>
       </c>
       <c r="H7" s="3" t="s">
-        <v>389</v>
+        <v>377</v>
       </c>
     </row>
     <row r="8" spans="1:229" x14ac:dyDescent="0.35">
       <c r="A8" s="3" t="s">
-        <v>390</v>
+        <v>378</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>391</v>
+        <v>379</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>392</v>
+        <v>380</v>
       </c>
       <c r="D8" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E8" s="3" t="s">
-        <v>213</v>
+        <v>201</v>
       </c>
       <c r="F8" s="3" t="s">
-        <v>214</v>
+        <v>202</v>
       </c>
       <c r="G8" s="3" t="s">
-        <v>223</v>
+        <v>211</v>
       </c>
       <c r="H8" s="3" t="s">
-        <v>393</v>
+        <v>381</v>
       </c>
     </row>
     <row r="9" spans="1:229" x14ac:dyDescent="0.35">
       <c r="A9" s="3" t="s">
-        <v>394</v>
+        <v>382</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>395</v>
+        <v>383</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>396</v>
+        <v>384</v>
       </c>
       <c r="D9" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E9" s="3" t="s">
-        <v>213</v>
+        <v>201</v>
       </c>
       <c r="F9" s="3" t="s">
-        <v>214</v>
+        <v>202</v>
       </c>
       <c r="G9" s="3" t="s">
-        <v>223</v>
+        <v>211</v>
       </c>
       <c r="H9" s="3" t="s">
-        <v>397</v>
+        <v>385</v>
       </c>
     </row>
     <row r="10" spans="1:229" x14ac:dyDescent="0.35">
       <c r="A10" s="3" t="s">
-        <v>398</v>
+        <v>386</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>399</v>
+        <v>387</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>400</v>
+        <v>388</v>
       </c>
       <c r="D10" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E10" s="3" t="s">
-        <v>213</v>
+        <v>201</v>
       </c>
       <c r="F10" s="3" t="s">
-        <v>214</v>
+        <v>202</v>
       </c>
       <c r="G10" s="3" t="s">
-        <v>223</v>
+        <v>211</v>
       </c>
       <c r="H10" s="3" t="s">
-        <v>401</v>
+        <v>389</v>
       </c>
     </row>
   </sheetData>
@@ -15273,7 +15353,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C6EE6111-FDB3-4B43-8820-BBF68AAFCD6D}">
   <dimension ref="A1:HU8"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -15308,36 +15388,36 @@
         <v>35</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>221</v>
+        <v>209</v>
       </c>
       <c r="H1" s="2" t="s">
-        <v>222</v>
+        <v>210</v>
       </c>
     </row>
     <row r="2" spans="1:229" s="4" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A2" s="3" t="s">
-        <v>402</v>
+        <v>390</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>403</v>
+        <v>391</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>404</v>
+        <v>392</v>
       </c>
       <c r="D2" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>213</v>
+        <v>201</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>214</v>
+        <v>202</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>223</v>
+        <v>211</v>
       </c>
       <c r="H2" s="3" t="s">
-        <v>195</v>
+        <v>183</v>
       </c>
       <c r="I2"/>
       <c r="J2"/>
@@ -15563,162 +15643,171 @@
     </row>
     <row r="3" spans="1:229" x14ac:dyDescent="0.35">
       <c r="A3" s="3" t="s">
-        <v>405</v>
+        <v>393</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>406</v>
+        <v>394</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>407</v>
+        <v>395</v>
       </c>
       <c r="D3" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>213</v>
+        <v>201</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>214</v>
+        <v>202</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>223</v>
+        <v>211</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>408</v>
+        <v>396</v>
       </c>
     </row>
     <row r="4" spans="1:229" x14ac:dyDescent="0.35">
       <c r="A4" s="3" t="s">
-        <v>409</v>
+        <v>397</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>410</v>
+        <v>398</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>411</v>
+        <v>399</v>
       </c>
       <c r="D4" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>213</v>
+        <v>201</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>214</v>
+        <v>202</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>223</v>
+        <v>211</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>412</v>
+        <v>400</v>
       </c>
     </row>
     <row r="5" spans="1:229" x14ac:dyDescent="0.35">
       <c r="A5" s="8" t="s">
-        <v>413</v>
+        <v>401</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>414</v>
+        <v>402</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>415</v>
+        <v>403</v>
       </c>
       <c r="D5" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>213</v>
+        <v>201</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>214</v>
+        <v>202</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>223</v>
+        <v>211</v>
       </c>
       <c r="H5" s="3" t="s">
-        <v>416</v>
+        <v>404</v>
       </c>
     </row>
     <row r="6" spans="1:229" x14ac:dyDescent="0.35">
       <c r="A6" s="3" t="s">
-        <v>417</v>
+        <v>405</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>418</v>
+        <v>406</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>419</v>
+        <v>407</v>
       </c>
       <c r="D6" s="7" t="s">
         <v>0</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>213</v>
+        <v>201</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>214</v>
+        <v>202</v>
       </c>
       <c r="G6" s="3" t="s">
-        <v>223</v>
+        <v>211</v>
       </c>
       <c r="H6" s="3" t="s">
-        <v>420</v>
+        <v>408</v>
       </c>
     </row>
     <row r="7" spans="1:229" x14ac:dyDescent="0.35">
       <c r="A7" s="3" t="s">
-        <v>421</v>
+        <v>409</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>422</v>
+        <v>410</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>423</v>
+        <v>411</v>
       </c>
       <c r="D7" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>213</v>
+        <v>201</v>
       </c>
       <c r="F7" s="3" t="s">
-        <v>214</v>
+        <v>202</v>
       </c>
       <c r="G7" s="3" t="s">
-        <v>223</v>
+        <v>211</v>
       </c>
       <c r="H7" s="3" t="s">
-        <v>424</v>
+        <v>412</v>
       </c>
     </row>
     <row r="8" spans="1:229" x14ac:dyDescent="0.35">
       <c r="A8" s="9" t="s">
-        <v>425</v>
+        <v>413</v>
       </c>
       <c r="B8" s="9" t="s">
-        <v>426</v>
+        <v>414</v>
       </c>
       <c r="C8" s="9" t="s">
-        <v>427</v>
+        <v>415</v>
       </c>
       <c r="D8" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E8" s="3" t="s">
-        <v>213</v>
+        <v>201</v>
       </c>
       <c r="F8" s="3" t="s">
-        <v>214</v>
+        <v>202</v>
       </c>
       <c r="G8" s="3" t="s">
-        <v>223</v>
+        <v>211</v>
       </c>
       <c r="H8" s="9" t="s">
-        <v>428</v>
+        <v>416</v>
       </c>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E6428663-7558-48F1-8CD3-947F03FFD4CC}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -15728,12 +15817,12 @@
   <dimension ref="A1:AMO12"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="40.54296875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="52.7265625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="41.36328125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="43.08984375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="55.26953125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="43.90625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="33.36328125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="34.54296875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="32.7265625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="35.26953125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:1029" x14ac:dyDescent="0.35">
@@ -15758,82 +15847,82 @@
     </row>
     <row r="2" spans="1:1029" x14ac:dyDescent="0.35">
       <c r="A2" s="3" t="s">
-        <v>359</v>
+        <v>347</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>360</v>
+        <v>348</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>361</v>
+        <v>349</v>
       </c>
       <c r="D2" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>358</v>
+        <v>346</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>362</v>
+        <v>350</v>
       </c>
     </row>
     <row r="3" spans="1:1029" x14ac:dyDescent="0.35">
-      <c r="A3" s="10" t="s">
-        <v>78</v>
-      </c>
-      <c r="B3" s="10" t="s">
-        <v>79</v>
-      </c>
-      <c r="C3" s="10" t="s">
-        <v>80</v>
+      <c r="A3" s="3" t="s">
+        <v>438</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>440</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>439</v>
       </c>
       <c r="D3" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>358</v>
-      </c>
-      <c r="F3" s="10" t="s">
-        <v>81</v>
+        <v>346</v>
+      </c>
+      <c r="F3" s="3" t="s">
+        <v>441</v>
       </c>
     </row>
     <row r="4" spans="1:1029" x14ac:dyDescent="0.35">
       <c r="A4" s="3" t="s">
-        <v>109</v>
+        <v>97</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>110</v>
+        <v>98</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>111</v>
+        <v>99</v>
       </c>
       <c r="D4" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>358</v>
+        <v>346</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>112</v>
+        <v>100</v>
       </c>
     </row>
     <row r="5" spans="1:1029" s="4" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A5" s="3" t="s">
-        <v>433</v>
+        <v>421</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>434</v>
+        <v>422</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>435</v>
+        <v>423</v>
       </c>
       <c r="D5" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>358</v>
+        <v>346</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>436</v>
+        <v>424</v>
       </c>
       <c r="G5"/>
       <c r="H5"/>
@@ -16860,63 +16949,63 @@
       <c r="AMO5"/>
     </row>
     <row r="6" spans="1:1029" x14ac:dyDescent="0.35">
-      <c r="A6" s="10" t="s">
-        <v>82</v>
-      </c>
-      <c r="B6" s="10" t="s">
-        <v>83</v>
-      </c>
-      <c r="C6" s="10" t="s">
-        <v>84</v>
+      <c r="A6" s="3" t="s">
+        <v>443</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>444</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>442</v>
       </c>
       <c r="D6" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>358</v>
-      </c>
-      <c r="F6" s="10" t="s">
-        <v>85</v>
+        <v>346</v>
+      </c>
+      <c r="F6" s="3" t="s">
+        <v>445</v>
       </c>
     </row>
     <row r="7" spans="1:1029" x14ac:dyDescent="0.35">
       <c r="A7" s="3" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="D7" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>358</v>
+        <v>346</v>
       </c>
       <c r="F7" s="3" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
     </row>
     <row r="8" spans="1:1029" s="4" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A8" s="3" t="s">
-        <v>437</v>
+        <v>425</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>439</v>
+        <v>427</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>438</v>
+        <v>426</v>
       </c>
       <c r="D8" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E8" s="3" t="s">
-        <v>358</v>
+        <v>346</v>
       </c>
       <c r="F8" s="3" t="s">
-        <v>448</v>
+        <v>436</v>
       </c>
       <c r="G8"/>
       <c r="H8"/>
@@ -17944,82 +18033,82 @@
     </row>
     <row r="9" spans="1:1029" x14ac:dyDescent="0.35">
       <c r="A9" s="3" t="s">
-        <v>440</v>
+        <v>428</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>441</v>
+        <v>429</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>442</v>
+        <v>430</v>
       </c>
       <c r="D9" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E9" s="3" t="s">
-        <v>358</v>
+        <v>346</v>
       </c>
       <c r="F9" s="3" t="s">
-        <v>443</v>
+        <v>431</v>
       </c>
     </row>
     <row r="10" spans="1:1029" x14ac:dyDescent="0.35">
       <c r="A10" s="3" t="s">
-        <v>444</v>
+        <v>432</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>445</v>
+        <v>433</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>446</v>
+        <v>434</v>
       </c>
       <c r="D10" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E10" s="3" t="s">
-        <v>358</v>
+        <v>346</v>
       </c>
       <c r="F10" s="3" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="11" spans="1:1029" x14ac:dyDescent="0.35">
+      <c r="A11" s="3" t="s">
+        <v>446</v>
+      </c>
+      <c r="B11" s="3" t="s">
         <v>447</v>
       </c>
-    </row>
-    <row r="11" spans="1:1029" x14ac:dyDescent="0.35">
-      <c r="A11" s="10" t="s">
-        <v>70</v>
-      </c>
-      <c r="B11" s="10" t="s">
-        <v>71</v>
-      </c>
-      <c r="C11" s="10" t="s">
-        <v>72</v>
+      <c r="C11" s="3" t="s">
+        <v>448</v>
       </c>
       <c r="D11" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E11" s="3" t="s">
-        <v>358</v>
-      </c>
-      <c r="F11" s="10" t="s">
-        <v>73</v>
+        <v>346</v>
+      </c>
+      <c r="F11" s="3" t="s">
+        <v>449</v>
       </c>
     </row>
     <row r="12" spans="1:1029" x14ac:dyDescent="0.35">
       <c r="A12" s="3" t="s">
-        <v>105</v>
+        <v>93</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>106</v>
+        <v>94</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>107</v>
+        <v>95</v>
       </c>
       <c r="D12" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E12" s="3" t="s">
-        <v>358</v>
+        <v>346</v>
       </c>
       <c r="F12" s="3" t="s">
-        <v>108</v>
+        <v>96</v>
       </c>
     </row>
   </sheetData>
@@ -18062,22 +18151,22 @@
     </row>
     <row r="2" spans="1:229" s="4" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A2" s="3" t="s">
-        <v>86</v>
+        <v>74</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>87</v>
+        <v>75</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>88</v>
+        <v>76</v>
       </c>
       <c r="D2" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>89</v>
+        <v>77</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>90</v>
+        <v>78</v>
       </c>
       <c r="G2"/>
       <c r="H2"/>
@@ -18305,22 +18394,22 @@
     </row>
     <row r="3" spans="1:229" s="4" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A3" s="3" t="s">
-        <v>91</v>
+        <v>79</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>92</v>
+        <v>80</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>93</v>
+        <v>81</v>
       </c>
       <c r="D3" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>89</v>
+        <v>77</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>94</v>
+        <v>82</v>
       </c>
       <c r="G3"/>
       <c r="H3"/>
@@ -18548,22 +18637,22 @@
     </row>
     <row r="4" spans="1:229" s="4" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A4" s="3" t="s">
-        <v>363</v>
+        <v>351</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>364</v>
+        <v>352</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>365</v>
+        <v>353</v>
       </c>
       <c r="D4" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>89</v>
+        <v>77</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>366</v>
+        <v>354</v>
       </c>
       <c r="G4"/>
       <c r="H4"/>
@@ -18791,42 +18880,42 @@
     </row>
     <row r="5" spans="1:229" x14ac:dyDescent="0.35">
       <c r="A5" s="3" t="s">
-        <v>95</v>
+        <v>83</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>96</v>
+        <v>84</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>97</v>
+        <v>85</v>
       </c>
       <c r="D5" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>89</v>
+        <v>77</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>98</v>
+        <v>86</v>
       </c>
     </row>
     <row r="6" spans="1:229" x14ac:dyDescent="0.35">
       <c r="A6" s="3" t="s">
-        <v>99</v>
+        <v>87</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>100</v>
+        <v>88</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>101</v>
+        <v>89</v>
       </c>
       <c r="D6" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>89</v>
+        <v>77</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>102</v>
+        <v>90</v>
       </c>
     </row>
   </sheetData>
@@ -18846,71 +18935,71 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" s="6" t="s">
-        <v>114</v>
+        <v>102</v>
       </c>
       <c r="B1" s="6" t="s">
-        <v>115</v>
+        <v>103</v>
       </c>
       <c r="C1" s="6" t="s">
-        <v>116</v>
+        <v>104</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" s="3" t="s">
-        <v>117</v>
+        <v>105</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>119</v>
+        <v>107</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>118</v>
+        <v>106</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="14" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B3" s="3" t="s">
-        <v>127</v>
+        <v>115</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>128</v>
+        <v>116</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.35">
       <c r="B4" s="3" t="s">
-        <v>125</v>
+        <v>113</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>126</v>
+        <v>114</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A5" s="3" t="s">
-        <v>120</v>
+        <v>108</v>
       </c>
       <c r="B5" s="3"/>
       <c r="C5" s="3"/>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A6" s="3" t="s">
-        <v>121</v>
+        <v>109</v>
       </c>
       <c r="B6" s="3"/>
       <c r="C6" s="3"/>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A7" s="3" t="s">
-        <v>122</v>
+        <v>110</v>
       </c>
       <c r="B7" s="3"/>
       <c r="C7" s="3"/>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A8" s="3" t="s">
-        <v>123</v>
+        <v>111</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A9" s="3" t="s">
-        <v>124</v>
+        <v>112</v>
       </c>
     </row>
   </sheetData>
@@ -18929,64 +19018,64 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" s="6" t="s">
-        <v>114</v>
+        <v>102</v>
       </c>
       <c r="B1" s="6" t="s">
-        <v>115</v>
+        <v>103</v>
       </c>
       <c r="C1" s="6" t="s">
-        <v>116</v>
+        <v>104</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" s="3" t="s">
-        <v>129</v>
+        <v>117</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>119</v>
+        <v>107</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>130</v>
+        <v>118</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="14" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B3" s="3" t="s">
-        <v>127</v>
+        <v>115</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>128</v>
+        <v>116</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.35">
       <c r="B4" s="3" t="s">
-        <v>125</v>
+        <v>113</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>126</v>
+        <v>114</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A5" s="3" t="s">
-        <v>131</v>
+        <v>119</v>
       </c>
       <c r="B5" s="3"/>
       <c r="C5" s="3"/>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A6" s="3" t="s">
-        <v>132</v>
+        <v>120</v>
       </c>
       <c r="B6" s="3"/>
       <c r="C6" s="3"/>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A7" s="3" t="s">
-        <v>133</v>
+        <v>121</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A8" s="3" t="s">
-        <v>134</v>
+        <v>122</v>
       </c>
     </row>
   </sheetData>
@@ -19005,78 +19094,78 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" s="6" t="s">
-        <v>114</v>
+        <v>102</v>
       </c>
       <c r="B1" s="6" t="s">
-        <v>115</v>
+        <v>103</v>
       </c>
       <c r="C1" s="6" t="s">
-        <v>116</v>
+        <v>104</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" s="3" t="s">
-        <v>135</v>
+        <v>123</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>119</v>
+        <v>107</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>136</v>
+        <v>124</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="14" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B3" s="3" t="s">
-        <v>127</v>
+        <v>115</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>128</v>
+        <v>116</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.35">
       <c r="B4" s="3" t="s">
-        <v>125</v>
+        <v>113</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>126</v>
+        <v>114</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A5" s="3" t="s">
-        <v>140</v>
+        <v>128</v>
       </c>
       <c r="B5" s="3"/>
       <c r="C5" s="3"/>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A6" s="3" t="s">
-        <v>139</v>
+        <v>127</v>
       </c>
       <c r="B6" s="3"/>
       <c r="C6" s="3"/>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A7" s="3" t="s">
-        <v>138</v>
+        <v>126</v>
       </c>
       <c r="B7" s="3"/>
       <c r="C7" s="3"/>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A8" s="3" t="s">
-        <v>137</v>
+        <v>125</v>
       </c>
       <c r="B8" s="3"/>
       <c r="C8" s="3"/>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A9" s="3" t="s">
-        <v>141</v>
+        <v>129</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A10" s="3" t="s">
-        <v>142</v>
+        <v>130</v>
       </c>
     </row>
   </sheetData>
@@ -19096,71 +19185,71 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" s="6" t="s">
-        <v>114</v>
+        <v>102</v>
       </c>
       <c r="B1" s="6" t="s">
-        <v>115</v>
+        <v>103</v>
       </c>
       <c r="C1" s="6" t="s">
-        <v>116</v>
+        <v>104</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" s="3" t="s">
-        <v>143</v>
+        <v>131</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>119</v>
+        <v>107</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>144</v>
+        <v>132</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="14" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B3" s="3" t="s">
-        <v>127</v>
+        <v>115</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>128</v>
+        <v>116</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.35">
       <c r="B4" s="3" t="s">
-        <v>125</v>
+        <v>113</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>126</v>
+        <v>114</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A5" s="3" t="s">
-        <v>145</v>
+        <v>133</v>
       </c>
       <c r="B5" s="3"/>
       <c r="C5" s="3"/>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A6" s="3" t="s">
-        <v>146</v>
+        <v>134</v>
       </c>
       <c r="B6" s="3"/>
       <c r="C6" s="3"/>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A7" s="3" t="s">
-        <v>147</v>
+        <v>135</v>
       </c>
       <c r="B7" s="3"/>
       <c r="C7" s="3"/>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A8" s="3" t="s">
-        <v>148</v>
+        <v>136</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A9" s="3" t="s">
-        <v>149</v>
+        <v>137</v>
       </c>
     </row>
   </sheetData>
@@ -19180,92 +19269,92 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" s="6" t="s">
-        <v>114</v>
+        <v>102</v>
       </c>
       <c r="B1" s="6" t="s">
-        <v>115</v>
+        <v>103</v>
       </c>
       <c r="C1" s="6" t="s">
-        <v>116</v>
+        <v>104</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" s="3" t="s">
-        <v>150</v>
+        <v>138</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>119</v>
+        <v>107</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>151</v>
+        <v>139</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="14" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B3" s="3" t="s">
-        <v>127</v>
+        <v>115</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>128</v>
+        <v>116</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.35">
       <c r="B4" s="3" t="s">
-        <v>125</v>
+        <v>113</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>126</v>
+        <v>114</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A5" s="3" t="s">
-        <v>152</v>
+        <v>140</v>
       </c>
       <c r="B5" s="3"/>
       <c r="C5" s="3"/>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A6" s="3" t="s">
-        <v>153</v>
+        <v>141</v>
       </c>
       <c r="B6" s="3"/>
       <c r="C6" s="3"/>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A7" s="3" t="s">
-        <v>154</v>
+        <v>142</v>
       </c>
       <c r="B7" s="3"/>
       <c r="C7" s="3"/>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A8" s="3" t="s">
-        <v>155</v>
+        <v>143</v>
       </c>
       <c r="B8" s="3"/>
       <c r="C8" s="3"/>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A9" s="3" t="s">
-        <v>156</v>
+        <v>144</v>
       </c>
       <c r="B9" s="3"/>
       <c r="C9" s="3"/>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A10" s="3" t="s">
-        <v>157</v>
+        <v>145</v>
       </c>
       <c r="B10" s="3"/>
       <c r="C10" s="3"/>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A11" s="3" t="s">
-        <v>158</v>
+        <v>146</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A12" s="3" t="s">
-        <v>159</v>
+        <v>147</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Added test cases for Social Care Workforce US#101
</commit_message>
<xml_diff>
--- a/testdata.xlsx
+++ b/testdata.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sshiwani\workspace\find-information-products-services-tests\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{297BEE1D-61DC-4366-971F-AE90EFF1E76A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B5106E12-4C7B-4221-B5AE-6E364F41D686}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="22780" windowHeight="14540" firstSheet="13" activeTab="15" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="22780" windowHeight="14540" firstSheet="14" activeTab="15" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="category_phase" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
     <sheet name="usergroup_ParentorCarer_list" sheetId="13" r:id="rId13"/>
     <sheet name="usergroup_ProfExtUserofDfE_list" sheetId="14" r:id="rId14"/>
     <sheet name="usergroup_SocialCWorkforce_list" sheetId="15" r:id="rId15"/>
-    <sheet name="Sheet2" sheetId="26" r:id="rId16"/>
+    <sheet name="usergroup_SocialWorker_list" sheetId="26" r:id="rId16"/>
     <sheet name="UGSubcategory_AdultLearner" sheetId="16" r:id="rId17"/>
     <sheet name="UGSubcategory_CareersAdviser" sheetId="17" r:id="rId18"/>
     <sheet name="UGSubcategory_ChildOrYoungPers" sheetId="18" r:id="rId19"/>
@@ -38,7 +38,7 @@
     <sheet name="UGSubcategory_NEETOrCareerSeek" sheetId="22" r:id="rId23"/>
     <sheet name="UGSubcategory_ParentOrCarer" sheetId="23" r:id="rId24"/>
     <sheet name="UGSubcateg_ProfExtUserofDfEData" sheetId="24" r:id="rId25"/>
-    <sheet name="Sheet1" sheetId="25" r:id="rId26"/>
+    <sheet name="UGSubcategory_SCWorkforce" sheetId="25" r:id="rId26"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -50,7 +50,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="897" uniqueCount="450">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="977" uniqueCount="488">
   <si>
     <t>Search and filter products and services</t>
   </si>
@@ -1400,6 +1400,120 @@
   </si>
   <si>
     <t>#group-skills-and-growth</t>
+  </si>
+  <si>
+    <t>categories/user-group/social-care-workforce/social-worker</t>
+  </si>
+  <si>
+    <t>Browse products in Social worker</t>
+  </si>
+  <si>
+    <t>Chief Social Worker for Children and Families</t>
+  </si>
+  <si>
+    <t>Child Protection Lead Practitioner</t>
+  </si>
+  <si>
+    <t>Practice leader (social worker)</t>
+  </si>
+  <si>
+    <t>Practice supervisor (social worker)</t>
+  </si>
+  <si>
+    <t>Principal Child and Family Social Worker</t>
+  </si>
+  <si>
+    <t>products?userGroup=social-care-workforce</t>
+  </si>
+  <si>
+    <t>ul.moj-filter-tags li a:has-text('Social care workforce')</t>
+  </si>
+  <si>
+    <t>Remove this filter Social care workforce</t>
+  </si>
+  <si>
+    <t>products?userGroup=childrens-care-home-workforce</t>
+  </si>
+  <si>
+    <t>ul.moj-filter-tags li a:has-text(" Children's care home workforce  (Social care workforce)")</t>
+  </si>
+  <si>
+    <t>Remove this filter Children's care home workforce  (Social care workforce)</t>
+  </si>
+  <si>
+    <t>Children's care home workforce  (Social care workforce)</t>
+  </si>
+  <si>
+    <t>products?userGroup=childrens-centre-staff-member</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Remove this filter Children's centre staff member </t>
+  </si>
+  <si>
+    <t>Children's centre staff member  (Social care workforce)</t>
+  </si>
+  <si>
+    <t>ul.moj-filter-tags li a:has-text(" Children's centre staff member ")</t>
+  </si>
+  <si>
+    <t>products?userGroup=early-intervention-practitioner</t>
+  </si>
+  <si>
+    <t>ul.moj-filter-tags li a:has-text('Early intervention practitioner  (Social care workforce)')</t>
+  </si>
+  <si>
+    <t>Remove this filter Early intervention practitioner  (Social care workforce)</t>
+  </si>
+  <si>
+    <t>Early intervention practitioner  (Social care workforce)</t>
+  </si>
+  <si>
+    <t>ul.moj-filter-tags li a:has-text(' Early intervention support worker  (Social care workforce)')</t>
+  </si>
+  <si>
+    <t>products?userGroup=category-value-3</t>
+  </si>
+  <si>
+    <t>Remove this filter Early intervention support worker  (Social care workforce)</t>
+  </si>
+  <si>
+    <t>Early intervention support worker  (Social care workforce)</t>
+  </si>
+  <si>
+    <t>products?userGroup=family-hub-practitioner</t>
+  </si>
+  <si>
+    <t>ul.moj-filter-tags li a:has-text(' Family hub practitioner  (Social care workforce)')</t>
+  </si>
+  <si>
+    <t>Remove this filter Family hub practitioner  (Social care workforce)</t>
+  </si>
+  <si>
+    <t>Family hub practitioner  (Social care workforce)</t>
+  </si>
+  <si>
+    <t>products?userGroup=family-support-worker</t>
+  </si>
+  <si>
+    <t>ul.moj-filter-tags li a:has-text(' Family support worker  (Social care workforce)')</t>
+  </si>
+  <si>
+    <t>Remove this filter Family support worker  (Social care workforce)</t>
+  </si>
+  <si>
+    <t>Family support worker  (Social care workforce)</t>
+  </si>
+  <si>
+    <t>products?userGroup=personal-adviser-social-care-workforce</t>
+  </si>
+  <si>
+    <t>ul.moj-filter-tags li a:has-text(' Personal adviser (social care workforce)  (Social care workforce)')</t>
+  </si>
+  <si>
+    <t>Remove this filter Personal adviser (social care workforce)  (Social care workforce)</t>
+  </si>
+  <si>
+    <t>Personal adviser (social care workforce)  (Social care workforce)</t>
   </si>
 </sst>
 </file>
@@ -11743,7 +11857,7 @@
 
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8B03D9F5-4C72-4FCD-8443-70945EFA9D2B}">
-  <dimension ref="A1:C12"/>
+  <dimension ref="A1:C10"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="54.1796875" customWidth="1"/>
@@ -11752,74 +11866,84 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A1" s="3" t="s">
-        <v>190</v>
-      </c>
-      <c r="B1" s="3" t="s">
+      <c r="A1" s="6" t="s">
+        <v>102</v>
+      </c>
+      <c r="B1" s="6" t="s">
+        <v>103</v>
+      </c>
+      <c r="C1" s="6" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A2" s="3" t="s">
+        <v>450</v>
+      </c>
+      <c r="B2" s="3" t="s">
         <v>107</v>
       </c>
-      <c r="C1" s="3" t="s">
-        <v>191</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="B2" s="3" t="s">
-        <v>115</v>
-      </c>
       <c r="C2" s="3" t="s">
-        <v>116</v>
+        <v>451</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.35">
       <c r="B3" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="B4" s="3" t="s">
         <v>113</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="C4" s="3" t="s">
         <v>114</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A4" s="3" t="s">
-        <v>192</v>
-      </c>
-      <c r="B4" s="3"/>
-      <c r="C4" s="3"/>
-    </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A5" s="3"/>
+      <c r="A5" s="3" t="s">
+        <v>200</v>
+      </c>
       <c r="B5" s="3"/>
       <c r="C5" s="3"/>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A6" s="3"/>
+      <c r="A6" s="3" t="s">
+        <v>452</v>
+      </c>
       <c r="B6" s="3"/>
       <c r="C6" s="3"/>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A7" s="3"/>
+      <c r="A7" s="3" t="s">
+        <v>453</v>
+      </c>
       <c r="B7" s="3"/>
       <c r="C7" s="3"/>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A8" s="3"/>
+      <c r="A8" s="3" t="s">
+        <v>454</v>
+      </c>
       <c r="B8" s="3"/>
       <c r="C8" s="3"/>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A9" s="3"/>
+      <c r="A9" s="3" t="s">
+        <v>455</v>
+      </c>
       <c r="B9" s="3"/>
       <c r="C9" s="3"/>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A10" s="3"/>
+      <c r="A10" s="3" t="s">
+        <v>456</v>
+      </c>
       <c r="B10" s="3"/>
       <c r="C10" s="3"/>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A11" s="3"/>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A12" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -15805,9 +15929,476 @@
 
 <file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E6428663-7558-48F1-8CD3-947F03FFD4CC}">
-  <dimension ref="A1"/>
+  <dimension ref="A1:HU9"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
-  <sheetData/>
+  <cols>
+    <col min="1" max="1" width="50.90625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="52.26953125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="42.453125" customWidth="1"/>
+    <col min="4" max="4" width="33.36328125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="33.08984375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="17.08984375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="40.81640625" customWidth="1"/>
+    <col min="8" max="8" width="57.08984375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:229" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>209</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="2" spans="1:229" s="4" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A2" s="3" t="s">
+        <v>457</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>458</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>459</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>201</v>
+      </c>
+      <c r="F2" s="3" t="s">
+        <v>202</v>
+      </c>
+      <c r="G2" s="3" t="s">
+        <v>211</v>
+      </c>
+      <c r="H2" s="3" t="s">
+        <v>192</v>
+      </c>
+      <c r="I2"/>
+      <c r="J2"/>
+      <c r="K2"/>
+      <c r="L2"/>
+      <c r="M2"/>
+      <c r="N2"/>
+      <c r="O2"/>
+      <c r="P2"/>
+      <c r="Q2"/>
+      <c r="R2"/>
+      <c r="S2"/>
+      <c r="T2"/>
+      <c r="U2"/>
+      <c r="V2"/>
+      <c r="W2"/>
+      <c r="X2"/>
+      <c r="Y2"/>
+      <c r="Z2"/>
+      <c r="AA2"/>
+      <c r="AB2"/>
+      <c r="AC2"/>
+      <c r="AD2"/>
+      <c r="AE2"/>
+      <c r="AF2"/>
+      <c r="AG2"/>
+      <c r="AH2"/>
+      <c r="AI2"/>
+      <c r="AJ2"/>
+      <c r="AK2"/>
+      <c r="AL2"/>
+      <c r="AM2"/>
+      <c r="AN2"/>
+      <c r="AO2"/>
+      <c r="AP2"/>
+      <c r="AQ2"/>
+      <c r="AR2"/>
+      <c r="AS2"/>
+      <c r="AT2"/>
+      <c r="AU2"/>
+      <c r="AV2"/>
+      <c r="AW2"/>
+      <c r="AX2"/>
+      <c r="AY2"/>
+      <c r="AZ2"/>
+      <c r="BA2"/>
+      <c r="BB2"/>
+      <c r="BC2"/>
+      <c r="BD2"/>
+      <c r="BE2"/>
+      <c r="BF2"/>
+      <c r="BG2"/>
+      <c r="BH2"/>
+      <c r="BI2"/>
+      <c r="BJ2"/>
+      <c r="BK2"/>
+      <c r="BL2"/>
+      <c r="BM2"/>
+      <c r="BN2"/>
+      <c r="BO2"/>
+      <c r="BP2"/>
+      <c r="BQ2"/>
+      <c r="BR2"/>
+      <c r="BS2"/>
+      <c r="BT2"/>
+      <c r="BU2"/>
+      <c r="BV2"/>
+      <c r="BW2"/>
+      <c r="BX2"/>
+      <c r="BY2"/>
+      <c r="BZ2"/>
+      <c r="CA2"/>
+      <c r="CB2"/>
+      <c r="CC2"/>
+      <c r="CD2"/>
+      <c r="CE2"/>
+      <c r="CF2"/>
+      <c r="CG2"/>
+      <c r="CH2"/>
+      <c r="CI2"/>
+      <c r="CJ2"/>
+      <c r="CK2"/>
+      <c r="CL2"/>
+      <c r="CM2"/>
+      <c r="CN2"/>
+      <c r="CO2"/>
+      <c r="CP2"/>
+      <c r="CQ2"/>
+      <c r="CR2"/>
+      <c r="CS2"/>
+      <c r="CT2"/>
+      <c r="CU2"/>
+      <c r="CV2"/>
+      <c r="CW2"/>
+      <c r="CX2"/>
+      <c r="CY2"/>
+      <c r="CZ2"/>
+      <c r="DA2"/>
+      <c r="DB2"/>
+      <c r="DC2"/>
+      <c r="DD2"/>
+      <c r="DE2"/>
+      <c r="DF2"/>
+      <c r="DG2"/>
+      <c r="DH2"/>
+      <c r="DI2"/>
+      <c r="DJ2"/>
+      <c r="DK2"/>
+      <c r="DL2"/>
+      <c r="DM2"/>
+      <c r="DN2"/>
+      <c r="DO2"/>
+      <c r="DP2"/>
+      <c r="DQ2"/>
+      <c r="DR2"/>
+      <c r="DS2"/>
+      <c r="DT2"/>
+      <c r="DU2"/>
+      <c r="DV2"/>
+      <c r="DW2"/>
+      <c r="DX2"/>
+      <c r="DY2"/>
+      <c r="DZ2"/>
+      <c r="EA2"/>
+      <c r="EB2"/>
+      <c r="EC2"/>
+      <c r="ED2"/>
+      <c r="EE2"/>
+      <c r="EF2"/>
+      <c r="EG2"/>
+      <c r="EH2"/>
+      <c r="EI2"/>
+      <c r="EJ2"/>
+      <c r="EK2"/>
+      <c r="EL2"/>
+      <c r="EM2"/>
+      <c r="EN2"/>
+      <c r="EO2"/>
+      <c r="EP2"/>
+      <c r="EQ2"/>
+      <c r="ER2"/>
+      <c r="ES2"/>
+      <c r="ET2"/>
+      <c r="EU2"/>
+      <c r="EV2"/>
+      <c r="EW2"/>
+      <c r="EX2"/>
+      <c r="EY2"/>
+      <c r="EZ2"/>
+      <c r="FA2"/>
+      <c r="FB2"/>
+      <c r="FC2"/>
+      <c r="FD2"/>
+      <c r="FE2"/>
+      <c r="FF2"/>
+      <c r="FG2"/>
+      <c r="FH2"/>
+      <c r="FI2"/>
+      <c r="FJ2"/>
+      <c r="FK2"/>
+      <c r="FL2"/>
+      <c r="FM2"/>
+      <c r="FN2"/>
+      <c r="FO2"/>
+      <c r="FP2"/>
+      <c r="FQ2"/>
+      <c r="FR2"/>
+      <c r="FS2"/>
+      <c r="FT2"/>
+      <c r="FU2"/>
+      <c r="FV2"/>
+      <c r="FW2"/>
+      <c r="FX2"/>
+      <c r="FY2"/>
+      <c r="FZ2"/>
+      <c r="GA2"/>
+      <c r="GB2"/>
+      <c r="GC2"/>
+      <c r="GD2"/>
+      <c r="GE2"/>
+      <c r="GF2"/>
+      <c r="GG2"/>
+      <c r="GH2"/>
+      <c r="GI2"/>
+      <c r="GJ2"/>
+      <c r="GK2"/>
+      <c r="GL2"/>
+      <c r="GM2"/>
+      <c r="GN2"/>
+      <c r="GO2"/>
+      <c r="GP2"/>
+      <c r="GQ2"/>
+      <c r="GR2"/>
+      <c r="GS2"/>
+      <c r="GT2"/>
+      <c r="GU2"/>
+      <c r="GV2"/>
+      <c r="GW2"/>
+      <c r="GX2"/>
+      <c r="GY2"/>
+      <c r="GZ2"/>
+      <c r="HA2"/>
+      <c r="HB2"/>
+      <c r="HC2"/>
+      <c r="HD2"/>
+      <c r="HE2"/>
+      <c r="HF2"/>
+      <c r="HG2"/>
+      <c r="HH2"/>
+      <c r="HI2"/>
+      <c r="HJ2"/>
+      <c r="HK2"/>
+      <c r="HL2"/>
+      <c r="HM2"/>
+      <c r="HN2"/>
+      <c r="HO2"/>
+      <c r="HP2"/>
+      <c r="HQ2"/>
+      <c r="HR2"/>
+      <c r="HS2"/>
+      <c r="HT2"/>
+      <c r="HU2"/>
+    </row>
+    <row r="3" spans="1:229" x14ac:dyDescent="0.35">
+      <c r="A3" s="3" t="s">
+        <v>460</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>461</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>462</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>201</v>
+      </c>
+      <c r="F3" s="3" t="s">
+        <v>202</v>
+      </c>
+      <c r="G3" s="3" t="s">
+        <v>211</v>
+      </c>
+      <c r="H3" s="3" t="s">
+        <v>463</v>
+      </c>
+    </row>
+    <row r="4" spans="1:229" x14ac:dyDescent="0.35">
+      <c r="A4" s="3" t="s">
+        <v>464</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>467</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>465</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>201</v>
+      </c>
+      <c r="F4" s="3" t="s">
+        <v>202</v>
+      </c>
+      <c r="G4" s="3" t="s">
+        <v>211</v>
+      </c>
+      <c r="H4" s="3" t="s">
+        <v>466</v>
+      </c>
+    </row>
+    <row r="5" spans="1:229" x14ac:dyDescent="0.35">
+      <c r="A5" s="8" t="s">
+        <v>468</v>
+      </c>
+      <c r="B5" s="8" t="s">
+        <v>469</v>
+      </c>
+      <c r="C5" s="8" t="s">
+        <v>470</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>201</v>
+      </c>
+      <c r="F5" s="3" t="s">
+        <v>202</v>
+      </c>
+      <c r="G5" s="3" t="s">
+        <v>211</v>
+      </c>
+      <c r="H5" s="3" t="s">
+        <v>471</v>
+      </c>
+    </row>
+    <row r="6" spans="1:229" x14ac:dyDescent="0.35">
+      <c r="A6" s="3" t="s">
+        <v>473</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>472</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>474</v>
+      </c>
+      <c r="D6" s="7" t="s">
+        <v>0</v>
+      </c>
+      <c r="E6" s="3" t="s">
+        <v>201</v>
+      </c>
+      <c r="F6" s="3" t="s">
+        <v>202</v>
+      </c>
+      <c r="G6" s="3" t="s">
+        <v>211</v>
+      </c>
+      <c r="H6" s="3" t="s">
+        <v>475</v>
+      </c>
+    </row>
+    <row r="7" spans="1:229" x14ac:dyDescent="0.35">
+      <c r="A7" s="3" t="s">
+        <v>476</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>477</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>478</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="E7" s="3" t="s">
+        <v>201</v>
+      </c>
+      <c r="F7" s="3" t="s">
+        <v>202</v>
+      </c>
+      <c r="G7" s="3" t="s">
+        <v>211</v>
+      </c>
+      <c r="H7" s="3" t="s">
+        <v>479</v>
+      </c>
+    </row>
+    <row r="8" spans="1:229" x14ac:dyDescent="0.35">
+      <c r="A8" s="3" t="s">
+        <v>480</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>481</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>482</v>
+      </c>
+      <c r="D8" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="E8" s="3" t="s">
+        <v>201</v>
+      </c>
+      <c r="F8" s="3" t="s">
+        <v>202</v>
+      </c>
+      <c r="G8" s="3" t="s">
+        <v>211</v>
+      </c>
+      <c r="H8" s="3" t="s">
+        <v>483</v>
+      </c>
+    </row>
+    <row r="9" spans="1:229" x14ac:dyDescent="0.35">
+      <c r="A9" s="3" t="s">
+        <v>484</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>485</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>486</v>
+      </c>
+      <c r="D9" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="E9" s="3" t="s">
+        <v>201</v>
+      </c>
+      <c r="F9" s="3" t="s">
+        <v>202</v>
+      </c>
+      <c r="G9" s="3" t="s">
+        <v>211</v>
+      </c>
+      <c r="H9" s="3" t="s">
+        <v>487</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Added testcases for Social Worker US#128 Updated framework for maximizing window
</commit_message>
<xml_diff>
--- a/testdata.xlsx
+++ b/testdata.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sshiwani\workspace\find-information-products-services-tests\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B5106E12-4C7B-4221-B5AE-6E364F41D686}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B074F4D3-2814-4AA5-8B40-1FC99FED345C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="22780" windowHeight="14540" firstSheet="14" activeTab="15" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="22780" windowHeight="14540" firstSheet="10" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="category_phase" sheetId="1" r:id="rId1"/>
@@ -39,6 +39,7 @@
     <sheet name="UGSubcategory_ParentOrCarer" sheetId="23" r:id="rId24"/>
     <sheet name="UGSubcateg_ProfExtUserofDfEData" sheetId="24" r:id="rId25"/>
     <sheet name="UGSubcategory_SCWorkforce" sheetId="25" r:id="rId26"/>
+    <sheet name="UGSubcategory_SocialWorker" sheetId="27" r:id="rId27"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -50,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="977" uniqueCount="488">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1033" uniqueCount="512">
   <si>
     <t>Search and filter products and services</t>
   </si>
@@ -1514,6 +1515,78 @@
   </si>
   <si>
     <t>Personal adviser (social care workforce)  (Social care workforce)</t>
+  </si>
+  <si>
+    <t>products?userGroup=social-worker</t>
+  </si>
+  <si>
+    <t>ul.moj-filter-tags li a:has-text(' Social worker  (Social care workforce)')</t>
+  </si>
+  <si>
+    <t>Remove this filter Social worker  (Social care workforce)</t>
+  </si>
+  <si>
+    <t>Social worker  (Social care workforce)</t>
+  </si>
+  <si>
+    <t>products?userGroup=chief-social-worker-for-children-and-families</t>
+  </si>
+  <si>
+    <t>ul.moj-filter-tags li a:has-text(' Chief Social Worker for Children and Families ')</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Remove this filter Chief Social Worker for Children and Families </t>
+  </si>
+  <si>
+    <t>Chief Social Worker for Children and Families  (Social worker)</t>
+  </si>
+  <si>
+    <t>products?userGroup=child-protection-lead-practitioner</t>
+  </si>
+  <si>
+    <t>ul.moj-filter-tags li a:has-text(' Child Protection Lead Practitioner ')</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Remove this filter Child Protection Lead Practitioner </t>
+  </si>
+  <si>
+    <t>Child Protection Lead Practitioner  (Social worker)</t>
+  </si>
+  <si>
+    <t>products?userGroup=practice-leader-social-worker</t>
+  </si>
+  <si>
+    <t>ul.moj-filter-tags li a:has-text(' Practice leader (social worker) ')</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Remove this filter Practice leader (social worker) </t>
+  </si>
+  <si>
+    <t>Practice leader (social worker)  (Social worker)</t>
+  </si>
+  <si>
+    <t>products?userGroup=practice-supervisor-social-worker</t>
+  </si>
+  <si>
+    <t>ul.moj-filter-tags li a:has-text(' Practice supervisor (social worker) ')</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Remove this filter Practice supervisor (social worker) </t>
+  </si>
+  <si>
+    <t>Practice supervisor (social worker)  (Social worker)</t>
+  </si>
+  <si>
+    <t>ul.moj-filter-tags li a:has-text(' Principal Child and Family Social Worker ')</t>
+  </si>
+  <si>
+    <t>products?userGroup=principal-child-and-family-social-worker</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Remove this filter Principal Child and Family Social Worker </t>
+  </si>
+  <si>
+    <t>Principal Child and Family Social Worker  (Social worker)</t>
   </si>
 </sst>
 </file>
@@ -16403,6 +16476,429 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2A4E3580-B709-4E66-9F6E-B7F9948D7FD3}">
+  <dimension ref="A1:HU7"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="50.90625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="52.26953125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="42.453125" customWidth="1"/>
+    <col min="4" max="4" width="33.36328125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="33.08984375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="17.08984375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="40.81640625" customWidth="1"/>
+    <col min="8" max="8" width="57.08984375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:229" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>209</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="2" spans="1:229" s="4" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A2" s="3" t="s">
+        <v>488</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>489</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>490</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>201</v>
+      </c>
+      <c r="F2" s="3" t="s">
+        <v>202</v>
+      </c>
+      <c r="G2" s="3" t="s">
+        <v>211</v>
+      </c>
+      <c r="H2" s="3" t="s">
+        <v>491</v>
+      </c>
+      <c r="I2"/>
+      <c r="J2"/>
+      <c r="K2"/>
+      <c r="L2"/>
+      <c r="M2"/>
+      <c r="N2"/>
+      <c r="O2"/>
+      <c r="P2"/>
+      <c r="Q2"/>
+      <c r="R2"/>
+      <c r="S2"/>
+      <c r="T2"/>
+      <c r="U2"/>
+      <c r="V2"/>
+      <c r="W2"/>
+      <c r="X2"/>
+      <c r="Y2"/>
+      <c r="Z2"/>
+      <c r="AA2"/>
+      <c r="AB2"/>
+      <c r="AC2"/>
+      <c r="AD2"/>
+      <c r="AE2"/>
+      <c r="AF2"/>
+      <c r="AG2"/>
+      <c r="AH2"/>
+      <c r="AI2"/>
+      <c r="AJ2"/>
+      <c r="AK2"/>
+      <c r="AL2"/>
+      <c r="AM2"/>
+      <c r="AN2"/>
+      <c r="AO2"/>
+      <c r="AP2"/>
+      <c r="AQ2"/>
+      <c r="AR2"/>
+      <c r="AS2"/>
+      <c r="AT2"/>
+      <c r="AU2"/>
+      <c r="AV2"/>
+      <c r="AW2"/>
+      <c r="AX2"/>
+      <c r="AY2"/>
+      <c r="AZ2"/>
+      <c r="BA2"/>
+      <c r="BB2"/>
+      <c r="BC2"/>
+      <c r="BD2"/>
+      <c r="BE2"/>
+      <c r="BF2"/>
+      <c r="BG2"/>
+      <c r="BH2"/>
+      <c r="BI2"/>
+      <c r="BJ2"/>
+      <c r="BK2"/>
+      <c r="BL2"/>
+      <c r="BM2"/>
+      <c r="BN2"/>
+      <c r="BO2"/>
+      <c r="BP2"/>
+      <c r="BQ2"/>
+      <c r="BR2"/>
+      <c r="BS2"/>
+      <c r="BT2"/>
+      <c r="BU2"/>
+      <c r="BV2"/>
+      <c r="BW2"/>
+      <c r="BX2"/>
+      <c r="BY2"/>
+      <c r="BZ2"/>
+      <c r="CA2"/>
+      <c r="CB2"/>
+      <c r="CC2"/>
+      <c r="CD2"/>
+      <c r="CE2"/>
+      <c r="CF2"/>
+      <c r="CG2"/>
+      <c r="CH2"/>
+      <c r="CI2"/>
+      <c r="CJ2"/>
+      <c r="CK2"/>
+      <c r="CL2"/>
+      <c r="CM2"/>
+      <c r="CN2"/>
+      <c r="CO2"/>
+      <c r="CP2"/>
+      <c r="CQ2"/>
+      <c r="CR2"/>
+      <c r="CS2"/>
+      <c r="CT2"/>
+      <c r="CU2"/>
+      <c r="CV2"/>
+      <c r="CW2"/>
+      <c r="CX2"/>
+      <c r="CY2"/>
+      <c r="CZ2"/>
+      <c r="DA2"/>
+      <c r="DB2"/>
+      <c r="DC2"/>
+      <c r="DD2"/>
+      <c r="DE2"/>
+      <c r="DF2"/>
+      <c r="DG2"/>
+      <c r="DH2"/>
+      <c r="DI2"/>
+      <c r="DJ2"/>
+      <c r="DK2"/>
+      <c r="DL2"/>
+      <c r="DM2"/>
+      <c r="DN2"/>
+      <c r="DO2"/>
+      <c r="DP2"/>
+      <c r="DQ2"/>
+      <c r="DR2"/>
+      <c r="DS2"/>
+      <c r="DT2"/>
+      <c r="DU2"/>
+      <c r="DV2"/>
+      <c r="DW2"/>
+      <c r="DX2"/>
+      <c r="DY2"/>
+      <c r="DZ2"/>
+      <c r="EA2"/>
+      <c r="EB2"/>
+      <c r="EC2"/>
+      <c r="ED2"/>
+      <c r="EE2"/>
+      <c r="EF2"/>
+      <c r="EG2"/>
+      <c r="EH2"/>
+      <c r="EI2"/>
+      <c r="EJ2"/>
+      <c r="EK2"/>
+      <c r="EL2"/>
+      <c r="EM2"/>
+      <c r="EN2"/>
+      <c r="EO2"/>
+      <c r="EP2"/>
+      <c r="EQ2"/>
+      <c r="ER2"/>
+      <c r="ES2"/>
+      <c r="ET2"/>
+      <c r="EU2"/>
+      <c r="EV2"/>
+      <c r="EW2"/>
+      <c r="EX2"/>
+      <c r="EY2"/>
+      <c r="EZ2"/>
+      <c r="FA2"/>
+      <c r="FB2"/>
+      <c r="FC2"/>
+      <c r="FD2"/>
+      <c r="FE2"/>
+      <c r="FF2"/>
+      <c r="FG2"/>
+      <c r="FH2"/>
+      <c r="FI2"/>
+      <c r="FJ2"/>
+      <c r="FK2"/>
+      <c r="FL2"/>
+      <c r="FM2"/>
+      <c r="FN2"/>
+      <c r="FO2"/>
+      <c r="FP2"/>
+      <c r="FQ2"/>
+      <c r="FR2"/>
+      <c r="FS2"/>
+      <c r="FT2"/>
+      <c r="FU2"/>
+      <c r="FV2"/>
+      <c r="FW2"/>
+      <c r="FX2"/>
+      <c r="FY2"/>
+      <c r="FZ2"/>
+      <c r="GA2"/>
+      <c r="GB2"/>
+      <c r="GC2"/>
+      <c r="GD2"/>
+      <c r="GE2"/>
+      <c r="GF2"/>
+      <c r="GG2"/>
+      <c r="GH2"/>
+      <c r="GI2"/>
+      <c r="GJ2"/>
+      <c r="GK2"/>
+      <c r="GL2"/>
+      <c r="GM2"/>
+      <c r="GN2"/>
+      <c r="GO2"/>
+      <c r="GP2"/>
+      <c r="GQ2"/>
+      <c r="GR2"/>
+      <c r="GS2"/>
+      <c r="GT2"/>
+      <c r="GU2"/>
+      <c r="GV2"/>
+      <c r="GW2"/>
+      <c r="GX2"/>
+      <c r="GY2"/>
+      <c r="GZ2"/>
+      <c r="HA2"/>
+      <c r="HB2"/>
+      <c r="HC2"/>
+      <c r="HD2"/>
+      <c r="HE2"/>
+      <c r="HF2"/>
+      <c r="HG2"/>
+      <c r="HH2"/>
+      <c r="HI2"/>
+      <c r="HJ2"/>
+      <c r="HK2"/>
+      <c r="HL2"/>
+      <c r="HM2"/>
+      <c r="HN2"/>
+      <c r="HO2"/>
+      <c r="HP2"/>
+      <c r="HQ2"/>
+      <c r="HR2"/>
+      <c r="HS2"/>
+      <c r="HT2"/>
+      <c r="HU2"/>
+    </row>
+    <row r="3" spans="1:229" x14ac:dyDescent="0.35">
+      <c r="A3" s="3" t="s">
+        <v>492</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>493</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>494</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>201</v>
+      </c>
+      <c r="F3" s="3" t="s">
+        <v>202</v>
+      </c>
+      <c r="G3" s="3" t="s">
+        <v>211</v>
+      </c>
+      <c r="H3" s="3" t="s">
+        <v>495</v>
+      </c>
+    </row>
+    <row r="4" spans="1:229" x14ac:dyDescent="0.35">
+      <c r="A4" s="3" t="s">
+        <v>496</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>497</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>498</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>201</v>
+      </c>
+      <c r="F4" s="3" t="s">
+        <v>202</v>
+      </c>
+      <c r="G4" s="3" t="s">
+        <v>211</v>
+      </c>
+      <c r="H4" s="3" t="s">
+        <v>499</v>
+      </c>
+    </row>
+    <row r="5" spans="1:229" x14ac:dyDescent="0.35">
+      <c r="A5" s="8" t="s">
+        <v>500</v>
+      </c>
+      <c r="B5" s="8" t="s">
+        <v>501</v>
+      </c>
+      <c r="C5" s="8" t="s">
+        <v>502</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>201</v>
+      </c>
+      <c r="F5" s="3" t="s">
+        <v>202</v>
+      </c>
+      <c r="G5" s="3" t="s">
+        <v>211</v>
+      </c>
+      <c r="H5" s="3" t="s">
+        <v>503</v>
+      </c>
+    </row>
+    <row r="6" spans="1:229" x14ac:dyDescent="0.35">
+      <c r="A6" s="3" t="s">
+        <v>504</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>505</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>506</v>
+      </c>
+      <c r="D6" s="7" t="s">
+        <v>0</v>
+      </c>
+      <c r="E6" s="3" t="s">
+        <v>201</v>
+      </c>
+      <c r="F6" s="3" t="s">
+        <v>202</v>
+      </c>
+      <c r="G6" s="3" t="s">
+        <v>211</v>
+      </c>
+      <c r="H6" s="3" t="s">
+        <v>507</v>
+      </c>
+    </row>
+    <row r="7" spans="1:229" x14ac:dyDescent="0.35">
+      <c r="A7" s="3" t="s">
+        <v>509</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>508</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>510</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="E7" s="3" t="s">
+        <v>201</v>
+      </c>
+      <c r="F7" s="3" t="s">
+        <v>202</v>
+      </c>
+      <c r="G7" s="3" t="s">
+        <v>211</v>
+      </c>
+      <c r="H7" s="3" t="s">
+        <v>511</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F9169CA5-09CB-4ADC-8EEE-AB383FD3DBB7}">
   <dimension ref="A1:AMO12"/>

</xml_diff>

<commit_message>
Added test cases for Academy Trust Workforce subcategory page US#130 and Education Provider subcategory page US#94
</commit_message>
<xml_diff>
--- a/testdata.xlsx
+++ b/testdata.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sshiwani\workspace\find-information-products-services-tests\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B074F4D3-2814-4AA5-8B40-1FC99FED345C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0AA9572B-ED4F-4DF7-BF30-28BE31D05844}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="22780" windowHeight="14540" firstSheet="10" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="22780" windowHeight="14540" firstSheet="28" activeTab="29" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="category_phase" sheetId="1" r:id="rId1"/>
@@ -29,17 +29,20 @@
     <sheet name="usergroup_ProfExtUserofDfE_list" sheetId="14" r:id="rId14"/>
     <sheet name="usergroup_SocialCWorkforce_list" sheetId="15" r:id="rId15"/>
     <sheet name="usergroup_SocialWorker_list" sheetId="26" r:id="rId16"/>
-    <sheet name="UGSubcategory_AdultLearner" sheetId="16" r:id="rId17"/>
-    <sheet name="UGSubcategory_CareersAdviser" sheetId="17" r:id="rId18"/>
-    <sheet name="UGSubcategory_ChildOrYoungPers" sheetId="18" r:id="rId19"/>
-    <sheet name="UGSubcategory_DfEWorkforce" sheetId="19" r:id="rId20"/>
-    <sheet name="UGSubcategory_Employer" sheetId="20" r:id="rId21"/>
-    <sheet name="UGSubcategory_LAWorkforce" sheetId="21" r:id="rId22"/>
-    <sheet name="UGSubcategory_NEETOrCareerSeek" sheetId="22" r:id="rId23"/>
-    <sheet name="UGSubcategory_ParentOrCarer" sheetId="23" r:id="rId24"/>
-    <sheet name="UGSubcateg_ProfExtUserofDfEData" sheetId="24" r:id="rId25"/>
-    <sheet name="UGSubcategory_SCWorkforce" sheetId="25" r:id="rId26"/>
-    <sheet name="UGSubcategory_SocialWorker" sheetId="27" r:id="rId27"/>
+    <sheet name="UG_EPEYAcademyTruWorkforce_list" sheetId="30" r:id="rId17"/>
+    <sheet name="UGSubcategory_AdultLearner" sheetId="16" r:id="rId18"/>
+    <sheet name="UGSubcategory_CareersAdviser" sheetId="17" r:id="rId19"/>
+    <sheet name="UGSubcategory_ChildOrYoungPers" sheetId="18" r:id="rId20"/>
+    <sheet name="UGSubcategory_DfEWorkforce" sheetId="19" r:id="rId21"/>
+    <sheet name="UGSubcategory_Employer" sheetId="20" r:id="rId22"/>
+    <sheet name="UGSubcategory_LAWorkforce" sheetId="21" r:id="rId23"/>
+    <sheet name="UGSubcategory_NEETOrCareerSeek" sheetId="22" r:id="rId24"/>
+    <sheet name="UGSubcategory_ParentOrCarer" sheetId="23" r:id="rId25"/>
+    <sheet name="UGSubcateg_ProfExtUserofDfEData" sheetId="24" r:id="rId26"/>
+    <sheet name="UGSubcategory_SCWorkforce" sheetId="25" r:id="rId27"/>
+    <sheet name="UGSubcategory_SocialWorker" sheetId="27" r:id="rId28"/>
+    <sheet name="UGSubcategory_EPandEYWorkforce" sheetId="29" r:id="rId29"/>
+    <sheet name="EPEYSubcateg_AcademyTWorkforce" sheetId="31" r:id="rId30"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -51,7 +54,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1033" uniqueCount="512">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1166" uniqueCount="571">
   <si>
     <t>Search and filter products and services</t>
   </si>
@@ -1587,6 +1590,183 @@
   </si>
   <si>
     <t>Principal Child and Family Social Worker  (Social worker)</t>
+  </si>
+  <si>
+    <t>products?userGroup=education-provider-and-early-years-workforce</t>
+  </si>
+  <si>
+    <t>ul.moj-filter-tags li a:has-text(' Education provider and early years workforce')</t>
+  </si>
+  <si>
+    <t>Remove this filter Education provider and early years workforce</t>
+  </si>
+  <si>
+    <t>categories/user-group/education-provider-and-early-years-workforce/academy-and-trust-workforce</t>
+  </si>
+  <si>
+    <t>Browse products in Academy and trust workforce</t>
+  </si>
+  <si>
+    <t>Academy governor</t>
+  </si>
+  <si>
+    <t>Academy headteacher (primary)</t>
+  </si>
+  <si>
+    <t>Academy headteacher (secondary)</t>
+  </si>
+  <si>
+    <t>Academy higher level teaching assistant</t>
+  </si>
+  <si>
+    <t>Academy school business professional</t>
+  </si>
+  <si>
+    <t>Academy support staff</t>
+  </si>
+  <si>
+    <t>Academy teacher (primary)</t>
+  </si>
+  <si>
+    <t>Academy teacher (secondary)</t>
+  </si>
+  <si>
+    <t>Academy teaching assistant</t>
+  </si>
+  <si>
+    <t>Academy trustee</t>
+  </si>
+  <si>
+    <t>products?userGroup=academy-and-trust-workforce</t>
+  </si>
+  <si>
+    <t>ul.moj-filter-tags li a:has-text(' Academy and trust workforce  (Education provider and early years workforce)')</t>
+  </si>
+  <si>
+    <t>Remove this filter Academy and trust workforce  (Education provider and early years workforce)</t>
+  </si>
+  <si>
+    <t>Academy and trust workforce  (Education provider and early years workforce)</t>
+  </si>
+  <si>
+    <t>ul.moj-filter-tags li a:has-text(' Academy governor  (Academy and trust workforce)')</t>
+  </si>
+  <si>
+    <t>products?userGroup=academy-governor</t>
+  </si>
+  <si>
+    <t>Remove this filter Academy governor  (Academy and trust workforce)</t>
+  </si>
+  <si>
+    <t>Academy governor  (Academy and trust workforce)</t>
+  </si>
+  <si>
+    <t>products?userGroup=academy-headteacher-primary</t>
+  </si>
+  <si>
+    <t>ul.moj-filter-tags li a:has-text(' Academy headteacher (primary)  (Academy and trust workforce)')</t>
+  </si>
+  <si>
+    <t>Remove this filter Academy headteacher (primary)  (Academy and trust workforce)</t>
+  </si>
+  <si>
+    <t>Academy headteacher (primary)  (Academy and trust workforce)</t>
+  </si>
+  <si>
+    <t>products?userGroup=academy-headteacher-secondary</t>
+  </si>
+  <si>
+    <t>ul.moj-filter-tags li a:has-text(' Academy headteacher (secondary)  (Academy and trust workforce)')</t>
+  </si>
+  <si>
+    <t>Remove this filter Academy headteacher (secondary)  (Academy and trust workforce)</t>
+  </si>
+  <si>
+    <t>Academy headteacher (secondary)  (Academy and trust workforce)</t>
+  </si>
+  <si>
+    <t>products?userGroup=academy-higher-level-teaching-assistant</t>
+  </si>
+  <si>
+    <t>ul.moj-filter-tags li a:has-text(' Academy higher level teaching assistant ')</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Remove this filter Academy higher level teaching assistant </t>
+  </si>
+  <si>
+    <t>Academy higher level teaching assistant  (Academy and trust workforce)</t>
+  </si>
+  <si>
+    <t>products?userGroup=academy-school-business-professional</t>
+  </si>
+  <si>
+    <t>ul.moj-filter-tags li a:has-text(' Academy school business professional  (Academy and trust workforce)')</t>
+  </si>
+  <si>
+    <t>Remove this filter Academy school business professional  (Academy and trust workforce)</t>
+  </si>
+  <si>
+    <t>Academy school business professional  (Academy and trust workforce)</t>
+  </si>
+  <si>
+    <t>products?userGroup=academy-support-staff</t>
+  </si>
+  <si>
+    <t>ul.moj-filter-tags li a:has-text(' Academy support staff  (Academy and trust workforce)')</t>
+  </si>
+  <si>
+    <t>Remove this filter Academy support staff  (Academy and trust workforce)</t>
+  </si>
+  <si>
+    <t>Academy support staff  (Academy and trust workforce)</t>
+  </si>
+  <si>
+    <t>products?userGroup=academy-teacher-primary</t>
+  </si>
+  <si>
+    <t>ul.moj-filter-tags li a:has-text(' Academy teacher (primary)  (Academy and trust workforce)')</t>
+  </si>
+  <si>
+    <t>Academy teacher (primary)  (Academy and trust workforce)</t>
+  </si>
+  <si>
+    <t>Remove this filter Academy teacher (primary)  (Academy and trust workforce)</t>
+  </si>
+  <si>
+    <t>products?userGroup=academy-teacher-secondary</t>
+  </si>
+  <si>
+    <t>ul.moj-filter-tags li a:has-text(' Academy teacher (secondary)  (Academy and trust workforce)')</t>
+  </si>
+  <si>
+    <t>Remove this filter Academy teacher (secondary)  (Academy and trust workforce)</t>
+  </si>
+  <si>
+    <t>Academy teacher (secondary)  (Academy and trust workforce)</t>
+  </si>
+  <si>
+    <t>products?userGroup=academy-teaching-assistant</t>
+  </si>
+  <si>
+    <t>ul.moj-filter-tags li a:has-text(' Academy teaching assistant ')</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Remove this filter Academy teaching assistant </t>
+  </si>
+  <si>
+    <t>Academy teaching assistant  (Academy and trust workforce)</t>
+  </si>
+  <si>
+    <t>products?userGroup=academy-trustee</t>
+  </si>
+  <si>
+    <t>ul.moj-filter-tags li a:has-text(' Academy trustee ')</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Remove this filter Academy trustee </t>
+  </si>
+  <si>
+    <t>Academy trustee  (Academy and trust workforce)</t>
   </si>
 </sst>
 </file>
@@ -1640,7 +1820,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="6">
+  <borders count="7">
     <border>
       <left/>
       <right/>
@@ -1711,11 +1891,24 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
@@ -1726,6 +1919,7 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="6" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -12024,6 +12218,136 @@
 </file>
 
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9E55FD73-18AE-49C9-9000-5AF4367B4AE3}">
+  <dimension ref="A1:C15"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="54.1796875" customWidth="1"/>
+    <col min="2" max="2" width="47.453125" customWidth="1"/>
+    <col min="3" max="3" width="43.90625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A1" s="6" t="s">
+        <v>102</v>
+      </c>
+      <c r="B1" s="6" t="s">
+        <v>103</v>
+      </c>
+      <c r="C1" s="6" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A2" s="3" t="s">
+        <v>515</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>107</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>516</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="B3" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="B4" s="3" t="s">
+        <v>113</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A5" s="3" t="s">
+        <v>141</v>
+      </c>
+      <c r="B5" s="3"/>
+      <c r="C5" s="3"/>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A6" s="3" t="s">
+        <v>517</v>
+      </c>
+      <c r="B6" s="3"/>
+      <c r="C6" s="3"/>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A7" s="3" t="s">
+        <v>518</v>
+      </c>
+      <c r="B7" s="3"/>
+      <c r="C7" s="3"/>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A8" s="3" t="s">
+        <v>519</v>
+      </c>
+      <c r="B8" s="3"/>
+      <c r="C8" s="3"/>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A9" s="3" t="s">
+        <v>520</v>
+      </c>
+      <c r="B9" s="3"/>
+      <c r="C9" s="3"/>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A10" s="3" t="s">
+        <v>521</v>
+      </c>
+      <c r="B10" s="3"/>
+      <c r="C10" s="3"/>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A11" s="3" t="s">
+        <v>522</v>
+      </c>
+      <c r="B11" s="3"/>
+      <c r="C11" s="3"/>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A12" s="3" t="s">
+        <v>523</v>
+      </c>
+      <c r="B12" s="3"/>
+      <c r="C12" s="3"/>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A13" s="3" t="s">
+        <v>524</v>
+      </c>
+      <c r="B13" s="3"/>
+      <c r="C13" s="3"/>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A14" s="3" t="s">
+        <v>525</v>
+      </c>
+      <c r="B14" s="3"/>
+      <c r="C14" s="3"/>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A15" s="3" t="s">
+        <v>526</v>
+      </c>
+      <c r="B15" s="3"/>
+      <c r="C15" s="3"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FB5527F7-85DB-4F8E-B4B3-EC8453E599E1}">
   <dimension ref="A1:HU6"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -12421,7 +12745,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A99CF6C3-F305-48A2-AB80-2C2D7CE6460C}">
   <dimension ref="A1:HU5"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -12792,7 +13116,225 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B2DC696B-E1A8-430C-BC9E-87DD1A6FBE9F}">
+  <dimension ref="A1:F10"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="33.08984375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="43.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="32.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="33.36328125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="29.90625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="25.36328125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A2" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="F2" s="3" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A3" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>101</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="F3" s="3" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A4" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="F4" s="3" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A5" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>91</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="F5" s="3" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A6" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="D6" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="E6" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="F6" s="3" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A7" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="E7" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="F7" s="3" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A8" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="D8" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="E8" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="F8" s="3" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A9" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="D9" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="E9" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="F9" s="3" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A10" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="D10" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="E10" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="F10" s="3" t="s">
+        <v>69</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5EFF0597-7FD1-4E6A-AA71-DB9F9FAB97A9}">
   <dimension ref="A1:HU7"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -13216,225 +13758,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B2DC696B-E1A8-430C-BC9E-87DD1A6FBE9F}">
-  <dimension ref="A1:F10"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
-  <cols>
-    <col min="1" max="1" width="33.08984375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="43.54296875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="32.1796875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="33.36328125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="29.90625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="25.36328125" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A1" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="F1" s="2" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="3" t="s">
-        <v>38</v>
-      </c>
-      <c r="B2" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="C2" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="D2" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="E2" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="F2" s="3" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="3" t="s">
-        <v>41</v>
-      </c>
-      <c r="B3" s="3" t="s">
-        <v>101</v>
-      </c>
-      <c r="C3" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="D3" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="E3" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="F3" s="3" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="3" t="s">
-        <v>45</v>
-      </c>
-      <c r="B4" s="3" t="s">
-        <v>44</v>
-      </c>
-      <c r="C4" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="D4" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="E4" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="F4" s="3" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="B5" s="3" t="s">
-        <v>91</v>
-      </c>
-      <c r="C5" s="3" t="s">
-        <v>92</v>
-      </c>
-      <c r="D5" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="E5" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="F5" s="3" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="3" t="s">
-        <v>50</v>
-      </c>
-      <c r="B6" s="3" t="s">
-        <v>51</v>
-      </c>
-      <c r="C6" s="3" t="s">
-        <v>52</v>
-      </c>
-      <c r="D6" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="E6" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="F6" s="3" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A7" s="3" t="s">
-        <v>54</v>
-      </c>
-      <c r="B7" s="3" t="s">
-        <v>55</v>
-      </c>
-      <c r="C7" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="D7" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="E7" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="F7" s="3" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A8" s="3" t="s">
-        <v>58</v>
-      </c>
-      <c r="B8" s="3" t="s">
-        <v>59</v>
-      </c>
-      <c r="C8" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="D8" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="E8" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="F8" s="3" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A9" s="3" t="s">
-        <v>62</v>
-      </c>
-      <c r="B9" s="3" t="s">
-        <v>63</v>
-      </c>
-      <c r="C9" s="3" t="s">
-        <v>64</v>
-      </c>
-      <c r="D9" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="E9" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="F9" s="3" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A10" s="3" t="s">
-        <v>66</v>
-      </c>
-      <c r="B10" s="3" t="s">
-        <v>67</v>
-      </c>
-      <c r="C10" s="3" t="s">
-        <v>68</v>
-      </c>
-      <c r="D10" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="E10" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="F10" s="3" t="s">
-        <v>69</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9F4A57AC-4620-4875-88AE-9F5C739A9042}">
   <dimension ref="A1:HU6"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -13831,7 +14155,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6C1C130F-0899-4810-82F6-950C9CB07234}">
   <dimension ref="A1:HU5"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -14202,7 +14526,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4AB9395B-D522-49AD-B790-5334356249F6}">
   <dimension ref="A1:HU7"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -14625,7 +14949,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BEE91763-AD0C-4544-A433-3B50C88AEB79}">
   <dimension ref="A1:HU7"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -15048,7 +15372,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{20DD36AA-F163-4AAB-BD30-4AE6290CCAE7}">
   <dimension ref="A1:HU10"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -15550,7 +15874,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C6EE6111-FDB3-4B43-8820-BBF68AAFCD6D}">
   <dimension ref="A1:HU8"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -16000,7 +16324,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E6428663-7558-48F1-8CD3-947F03FFD4CC}">
   <dimension ref="A1:HU9"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -16476,7 +16800,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2A4E3580-B709-4E66-9F6E-B7F9948D7FD3}">
   <dimension ref="A1:HU7"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -16893,6 +17217,299 @@
       <c r="H7" s="3" t="s">
         <v>511</v>
       </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet29.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{95706458-CD50-4C74-87C4-ABAE617927AD}">
+  <dimension ref="A1:HU2"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="50.90625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="52.26953125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="42.453125" customWidth="1"/>
+    <col min="4" max="4" width="33.36328125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="33.08984375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="17.08984375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="40.81640625" customWidth="1"/>
+    <col min="8" max="8" width="57.08984375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:229" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>209</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="2" spans="1:229" s="4" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A2" s="3" t="s">
+        <v>512</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>513</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>514</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>201</v>
+      </c>
+      <c r="F2" s="3" t="s">
+        <v>202</v>
+      </c>
+      <c r="G2" s="3" t="s">
+        <v>211</v>
+      </c>
+      <c r="H2" s="3" t="s">
+        <v>140</v>
+      </c>
+      <c r="I2"/>
+      <c r="J2"/>
+      <c r="K2"/>
+      <c r="L2"/>
+      <c r="M2"/>
+      <c r="N2"/>
+      <c r="O2"/>
+      <c r="P2"/>
+      <c r="Q2"/>
+      <c r="R2"/>
+      <c r="S2"/>
+      <c r="T2"/>
+      <c r="U2"/>
+      <c r="V2"/>
+      <c r="W2"/>
+      <c r="X2"/>
+      <c r="Y2"/>
+      <c r="Z2"/>
+      <c r="AA2"/>
+      <c r="AB2"/>
+      <c r="AC2"/>
+      <c r="AD2"/>
+      <c r="AE2"/>
+      <c r="AF2"/>
+      <c r="AG2"/>
+      <c r="AH2"/>
+      <c r="AI2"/>
+      <c r="AJ2"/>
+      <c r="AK2"/>
+      <c r="AL2"/>
+      <c r="AM2"/>
+      <c r="AN2"/>
+      <c r="AO2"/>
+      <c r="AP2"/>
+      <c r="AQ2"/>
+      <c r="AR2"/>
+      <c r="AS2"/>
+      <c r="AT2"/>
+      <c r="AU2"/>
+      <c r="AV2"/>
+      <c r="AW2"/>
+      <c r="AX2"/>
+      <c r="AY2"/>
+      <c r="AZ2"/>
+      <c r="BA2"/>
+      <c r="BB2"/>
+      <c r="BC2"/>
+      <c r="BD2"/>
+      <c r="BE2"/>
+      <c r="BF2"/>
+      <c r="BG2"/>
+      <c r="BH2"/>
+      <c r="BI2"/>
+      <c r="BJ2"/>
+      <c r="BK2"/>
+      <c r="BL2"/>
+      <c r="BM2"/>
+      <c r="BN2"/>
+      <c r="BO2"/>
+      <c r="BP2"/>
+      <c r="BQ2"/>
+      <c r="BR2"/>
+      <c r="BS2"/>
+      <c r="BT2"/>
+      <c r="BU2"/>
+      <c r="BV2"/>
+      <c r="BW2"/>
+      <c r="BX2"/>
+      <c r="BY2"/>
+      <c r="BZ2"/>
+      <c r="CA2"/>
+      <c r="CB2"/>
+      <c r="CC2"/>
+      <c r="CD2"/>
+      <c r="CE2"/>
+      <c r="CF2"/>
+      <c r="CG2"/>
+      <c r="CH2"/>
+      <c r="CI2"/>
+      <c r="CJ2"/>
+      <c r="CK2"/>
+      <c r="CL2"/>
+      <c r="CM2"/>
+      <c r="CN2"/>
+      <c r="CO2"/>
+      <c r="CP2"/>
+      <c r="CQ2"/>
+      <c r="CR2"/>
+      <c r="CS2"/>
+      <c r="CT2"/>
+      <c r="CU2"/>
+      <c r="CV2"/>
+      <c r="CW2"/>
+      <c r="CX2"/>
+      <c r="CY2"/>
+      <c r="CZ2"/>
+      <c r="DA2"/>
+      <c r="DB2"/>
+      <c r="DC2"/>
+      <c r="DD2"/>
+      <c r="DE2"/>
+      <c r="DF2"/>
+      <c r="DG2"/>
+      <c r="DH2"/>
+      <c r="DI2"/>
+      <c r="DJ2"/>
+      <c r="DK2"/>
+      <c r="DL2"/>
+      <c r="DM2"/>
+      <c r="DN2"/>
+      <c r="DO2"/>
+      <c r="DP2"/>
+      <c r="DQ2"/>
+      <c r="DR2"/>
+      <c r="DS2"/>
+      <c r="DT2"/>
+      <c r="DU2"/>
+      <c r="DV2"/>
+      <c r="DW2"/>
+      <c r="DX2"/>
+      <c r="DY2"/>
+      <c r="DZ2"/>
+      <c r="EA2"/>
+      <c r="EB2"/>
+      <c r="EC2"/>
+      <c r="ED2"/>
+      <c r="EE2"/>
+      <c r="EF2"/>
+      <c r="EG2"/>
+      <c r="EH2"/>
+      <c r="EI2"/>
+      <c r="EJ2"/>
+      <c r="EK2"/>
+      <c r="EL2"/>
+      <c r="EM2"/>
+      <c r="EN2"/>
+      <c r="EO2"/>
+      <c r="EP2"/>
+      <c r="EQ2"/>
+      <c r="ER2"/>
+      <c r="ES2"/>
+      <c r="ET2"/>
+      <c r="EU2"/>
+      <c r="EV2"/>
+      <c r="EW2"/>
+      <c r="EX2"/>
+      <c r="EY2"/>
+      <c r="EZ2"/>
+      <c r="FA2"/>
+      <c r="FB2"/>
+      <c r="FC2"/>
+      <c r="FD2"/>
+      <c r="FE2"/>
+      <c r="FF2"/>
+      <c r="FG2"/>
+      <c r="FH2"/>
+      <c r="FI2"/>
+      <c r="FJ2"/>
+      <c r="FK2"/>
+      <c r="FL2"/>
+      <c r="FM2"/>
+      <c r="FN2"/>
+      <c r="FO2"/>
+      <c r="FP2"/>
+      <c r="FQ2"/>
+      <c r="FR2"/>
+      <c r="FS2"/>
+      <c r="FT2"/>
+      <c r="FU2"/>
+      <c r="FV2"/>
+      <c r="FW2"/>
+      <c r="FX2"/>
+      <c r="FY2"/>
+      <c r="FZ2"/>
+      <c r="GA2"/>
+      <c r="GB2"/>
+      <c r="GC2"/>
+      <c r="GD2"/>
+      <c r="GE2"/>
+      <c r="GF2"/>
+      <c r="GG2"/>
+      <c r="GH2"/>
+      <c r="GI2"/>
+      <c r="GJ2"/>
+      <c r="GK2"/>
+      <c r="GL2"/>
+      <c r="GM2"/>
+      <c r="GN2"/>
+      <c r="GO2"/>
+      <c r="GP2"/>
+      <c r="GQ2"/>
+      <c r="GR2"/>
+      <c r="GS2"/>
+      <c r="GT2"/>
+      <c r="GU2"/>
+      <c r="GV2"/>
+      <c r="GW2"/>
+      <c r="GX2"/>
+      <c r="GY2"/>
+      <c r="GZ2"/>
+      <c r="HA2"/>
+      <c r="HB2"/>
+      <c r="HC2"/>
+      <c r="HD2"/>
+      <c r="HE2"/>
+      <c r="HF2"/>
+      <c r="HG2"/>
+      <c r="HH2"/>
+      <c r="HI2"/>
+      <c r="HJ2"/>
+      <c r="HK2"/>
+      <c r="HL2"/>
+      <c r="HM2"/>
+      <c r="HN2"/>
+      <c r="HO2"/>
+      <c r="HP2"/>
+      <c r="HQ2"/>
+      <c r="HR2"/>
+      <c r="HS2"/>
+      <c r="HT2"/>
+      <c r="HU2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -19203,6 +19820,560 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet30.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1AD86191-7CFE-4ED9-9129-FF78170AB51E}">
+  <dimension ref="A1:HU12"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="50.90625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="52.26953125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="42.453125" customWidth="1"/>
+    <col min="4" max="4" width="33.36328125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="33.08984375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="17.08984375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="40.81640625" customWidth="1"/>
+    <col min="8" max="8" width="65.54296875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:229" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>209</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="2" spans="1:229" s="4" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A2" s="3" t="s">
+        <v>527</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>528</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>529</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>201</v>
+      </c>
+      <c r="F2" s="3" t="s">
+        <v>202</v>
+      </c>
+      <c r="G2" s="3" t="s">
+        <v>211</v>
+      </c>
+      <c r="H2" s="3" t="s">
+        <v>530</v>
+      </c>
+      <c r="I2"/>
+      <c r="J2"/>
+      <c r="K2"/>
+      <c r="L2"/>
+      <c r="M2"/>
+      <c r="N2"/>
+      <c r="O2"/>
+      <c r="P2"/>
+      <c r="Q2"/>
+      <c r="R2"/>
+      <c r="S2"/>
+      <c r="T2"/>
+      <c r="U2"/>
+      <c r="V2"/>
+      <c r="W2"/>
+      <c r="X2"/>
+      <c r="Y2"/>
+      <c r="Z2"/>
+      <c r="AA2"/>
+      <c r="AB2"/>
+      <c r="AC2"/>
+      <c r="AD2"/>
+      <c r="AE2"/>
+      <c r="AF2"/>
+      <c r="AG2"/>
+      <c r="AH2"/>
+      <c r="AI2"/>
+      <c r="AJ2"/>
+      <c r="AK2"/>
+      <c r="AL2"/>
+      <c r="AM2"/>
+      <c r="AN2"/>
+      <c r="AO2"/>
+      <c r="AP2"/>
+      <c r="AQ2"/>
+      <c r="AR2"/>
+      <c r="AS2"/>
+      <c r="AT2"/>
+      <c r="AU2"/>
+      <c r="AV2"/>
+      <c r="AW2"/>
+      <c r="AX2"/>
+      <c r="AY2"/>
+      <c r="AZ2"/>
+      <c r="BA2"/>
+      <c r="BB2"/>
+      <c r="BC2"/>
+      <c r="BD2"/>
+      <c r="BE2"/>
+      <c r="BF2"/>
+      <c r="BG2"/>
+      <c r="BH2"/>
+      <c r="BI2"/>
+      <c r="BJ2"/>
+      <c r="BK2"/>
+      <c r="BL2"/>
+      <c r="BM2"/>
+      <c r="BN2"/>
+      <c r="BO2"/>
+      <c r="BP2"/>
+      <c r="BQ2"/>
+      <c r="BR2"/>
+      <c r="BS2"/>
+      <c r="BT2"/>
+      <c r="BU2"/>
+      <c r="BV2"/>
+      <c r="BW2"/>
+      <c r="BX2"/>
+      <c r="BY2"/>
+      <c r="BZ2"/>
+      <c r="CA2"/>
+      <c r="CB2"/>
+      <c r="CC2"/>
+      <c r="CD2"/>
+      <c r="CE2"/>
+      <c r="CF2"/>
+      <c r="CG2"/>
+      <c r="CH2"/>
+      <c r="CI2"/>
+      <c r="CJ2"/>
+      <c r="CK2"/>
+      <c r="CL2"/>
+      <c r="CM2"/>
+      <c r="CN2"/>
+      <c r="CO2"/>
+      <c r="CP2"/>
+      <c r="CQ2"/>
+      <c r="CR2"/>
+      <c r="CS2"/>
+      <c r="CT2"/>
+      <c r="CU2"/>
+      <c r="CV2"/>
+      <c r="CW2"/>
+      <c r="CX2"/>
+      <c r="CY2"/>
+      <c r="CZ2"/>
+      <c r="DA2"/>
+      <c r="DB2"/>
+      <c r="DC2"/>
+      <c r="DD2"/>
+      <c r="DE2"/>
+      <c r="DF2"/>
+      <c r="DG2"/>
+      <c r="DH2"/>
+      <c r="DI2"/>
+      <c r="DJ2"/>
+      <c r="DK2"/>
+      <c r="DL2"/>
+      <c r="DM2"/>
+      <c r="DN2"/>
+      <c r="DO2"/>
+      <c r="DP2"/>
+      <c r="DQ2"/>
+      <c r="DR2"/>
+      <c r="DS2"/>
+      <c r="DT2"/>
+      <c r="DU2"/>
+      <c r="DV2"/>
+      <c r="DW2"/>
+      <c r="DX2"/>
+      <c r="DY2"/>
+      <c r="DZ2"/>
+      <c r="EA2"/>
+      <c r="EB2"/>
+      <c r="EC2"/>
+      <c r="ED2"/>
+      <c r="EE2"/>
+      <c r="EF2"/>
+      <c r="EG2"/>
+      <c r="EH2"/>
+      <c r="EI2"/>
+      <c r="EJ2"/>
+      <c r="EK2"/>
+      <c r="EL2"/>
+      <c r="EM2"/>
+      <c r="EN2"/>
+      <c r="EO2"/>
+      <c r="EP2"/>
+      <c r="EQ2"/>
+      <c r="ER2"/>
+      <c r="ES2"/>
+      <c r="ET2"/>
+      <c r="EU2"/>
+      <c r="EV2"/>
+      <c r="EW2"/>
+      <c r="EX2"/>
+      <c r="EY2"/>
+      <c r="EZ2"/>
+      <c r="FA2"/>
+      <c r="FB2"/>
+      <c r="FC2"/>
+      <c r="FD2"/>
+      <c r="FE2"/>
+      <c r="FF2"/>
+      <c r="FG2"/>
+      <c r="FH2"/>
+      <c r="FI2"/>
+      <c r="FJ2"/>
+      <c r="FK2"/>
+      <c r="FL2"/>
+      <c r="FM2"/>
+      <c r="FN2"/>
+      <c r="FO2"/>
+      <c r="FP2"/>
+      <c r="FQ2"/>
+      <c r="FR2"/>
+      <c r="FS2"/>
+      <c r="FT2"/>
+      <c r="FU2"/>
+      <c r="FV2"/>
+      <c r="FW2"/>
+      <c r="FX2"/>
+      <c r="FY2"/>
+      <c r="FZ2"/>
+      <c r="GA2"/>
+      <c r="GB2"/>
+      <c r="GC2"/>
+      <c r="GD2"/>
+      <c r="GE2"/>
+      <c r="GF2"/>
+      <c r="GG2"/>
+      <c r="GH2"/>
+      <c r="GI2"/>
+      <c r="GJ2"/>
+      <c r="GK2"/>
+      <c r="GL2"/>
+      <c r="GM2"/>
+      <c r="GN2"/>
+      <c r="GO2"/>
+      <c r="GP2"/>
+      <c r="GQ2"/>
+      <c r="GR2"/>
+      <c r="GS2"/>
+      <c r="GT2"/>
+      <c r="GU2"/>
+      <c r="GV2"/>
+      <c r="GW2"/>
+      <c r="GX2"/>
+      <c r="GY2"/>
+      <c r="GZ2"/>
+      <c r="HA2"/>
+      <c r="HB2"/>
+      <c r="HC2"/>
+      <c r="HD2"/>
+      <c r="HE2"/>
+      <c r="HF2"/>
+      <c r="HG2"/>
+      <c r="HH2"/>
+      <c r="HI2"/>
+      <c r="HJ2"/>
+      <c r="HK2"/>
+      <c r="HL2"/>
+      <c r="HM2"/>
+      <c r="HN2"/>
+      <c r="HO2"/>
+      <c r="HP2"/>
+      <c r="HQ2"/>
+      <c r="HR2"/>
+      <c r="HS2"/>
+      <c r="HT2"/>
+      <c r="HU2"/>
+    </row>
+    <row r="3" spans="1:229" x14ac:dyDescent="0.35">
+      <c r="A3" s="3" t="s">
+        <v>532</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>531</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>533</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>201</v>
+      </c>
+      <c r="F3" s="3" t="s">
+        <v>202</v>
+      </c>
+      <c r="G3" s="3" t="s">
+        <v>211</v>
+      </c>
+      <c r="H3" s="3" t="s">
+        <v>534</v>
+      </c>
+    </row>
+    <row r="4" spans="1:229" x14ac:dyDescent="0.35">
+      <c r="A4" s="3" t="s">
+        <v>535</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>536</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>537</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>201</v>
+      </c>
+      <c r="F4" s="3" t="s">
+        <v>202</v>
+      </c>
+      <c r="G4" s="3" t="s">
+        <v>211</v>
+      </c>
+      <c r="H4" s="3" t="s">
+        <v>538</v>
+      </c>
+    </row>
+    <row r="5" spans="1:229" x14ac:dyDescent="0.35">
+      <c r="A5" s="8" t="s">
+        <v>539</v>
+      </c>
+      <c r="B5" s="8" t="s">
+        <v>540</v>
+      </c>
+      <c r="C5" s="8" t="s">
+        <v>541</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>201</v>
+      </c>
+      <c r="F5" s="3" t="s">
+        <v>202</v>
+      </c>
+      <c r="G5" s="3" t="s">
+        <v>211</v>
+      </c>
+      <c r="H5" s="3" t="s">
+        <v>542</v>
+      </c>
+    </row>
+    <row r="6" spans="1:229" x14ac:dyDescent="0.35">
+      <c r="A6" s="3" t="s">
+        <v>543</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>544</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>545</v>
+      </c>
+      <c r="D6" s="7" t="s">
+        <v>0</v>
+      </c>
+      <c r="E6" s="3" t="s">
+        <v>201</v>
+      </c>
+      <c r="F6" s="3" t="s">
+        <v>202</v>
+      </c>
+      <c r="G6" s="3" t="s">
+        <v>211</v>
+      </c>
+      <c r="H6" s="3" t="s">
+        <v>546</v>
+      </c>
+    </row>
+    <row r="7" spans="1:229" x14ac:dyDescent="0.35">
+      <c r="A7" s="3" t="s">
+        <v>547</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>548</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>549</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="E7" s="3" t="s">
+        <v>201</v>
+      </c>
+      <c r="F7" s="3" t="s">
+        <v>202</v>
+      </c>
+      <c r="G7" s="3" t="s">
+        <v>211</v>
+      </c>
+      <c r="H7" s="3" t="s">
+        <v>550</v>
+      </c>
+    </row>
+    <row r="8" spans="1:229" x14ac:dyDescent="0.35">
+      <c r="A8" s="3" t="s">
+        <v>551</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>552</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>553</v>
+      </c>
+      <c r="D8" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="E8" s="3" t="s">
+        <v>201</v>
+      </c>
+      <c r="F8" s="3" t="s">
+        <v>202</v>
+      </c>
+      <c r="G8" s="10" t="s">
+        <v>211</v>
+      </c>
+      <c r="H8" s="3" t="s">
+        <v>554</v>
+      </c>
+    </row>
+    <row r="9" spans="1:229" x14ac:dyDescent="0.35">
+      <c r="A9" s="3" t="s">
+        <v>555</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>556</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>558</v>
+      </c>
+      <c r="D9" s="7" t="s">
+        <v>0</v>
+      </c>
+      <c r="E9" s="3" t="s">
+        <v>201</v>
+      </c>
+      <c r="F9" s="3" t="s">
+        <v>202</v>
+      </c>
+      <c r="G9" s="10" t="s">
+        <v>211</v>
+      </c>
+      <c r="H9" s="3" t="s">
+        <v>557</v>
+      </c>
+    </row>
+    <row r="10" spans="1:229" x14ac:dyDescent="0.35">
+      <c r="A10" s="3" t="s">
+        <v>559</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>560</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>561</v>
+      </c>
+      <c r="D10" s="7" t="s">
+        <v>0</v>
+      </c>
+      <c r="E10" s="3" t="s">
+        <v>201</v>
+      </c>
+      <c r="F10" s="3" t="s">
+        <v>202</v>
+      </c>
+      <c r="G10" s="10" t="s">
+        <v>211</v>
+      </c>
+      <c r="H10" s="3" t="s">
+        <v>562</v>
+      </c>
+    </row>
+    <row r="11" spans="1:229" x14ac:dyDescent="0.35">
+      <c r="A11" s="3" t="s">
+        <v>563</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>564</v>
+      </c>
+      <c r="C11" s="3" t="s">
+        <v>565</v>
+      </c>
+      <c r="D11" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="E11" s="3" t="s">
+        <v>201</v>
+      </c>
+      <c r="F11" s="3" t="s">
+        <v>202</v>
+      </c>
+      <c r="G11" s="10" t="s">
+        <v>211</v>
+      </c>
+      <c r="H11" s="3" t="s">
+        <v>566</v>
+      </c>
+    </row>
+    <row r="12" spans="1:229" x14ac:dyDescent="0.35">
+      <c r="A12" s="3" t="s">
+        <v>567</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>568</v>
+      </c>
+      <c r="C12" s="3" t="s">
+        <v>569</v>
+      </c>
+      <c r="D12" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="E12" s="3" t="s">
+        <v>201</v>
+      </c>
+      <c r="F12" s="3" t="s">
+        <v>202</v>
+      </c>
+      <c r="G12" s="10" t="s">
+        <v>211</v>
+      </c>
+      <c r="H12" s="3" t="s">
+        <v>570</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{005D001A-3768-4392-8BD8-510250183310}">
   <dimension ref="A1:HU6"/>

</xml_diff>

<commit_message>
Added test cases for Alternative provision setting workforce US#131 and Early years workforce US#132
</commit_message>
<xml_diff>
--- a/testdata.xlsx
+++ b/testdata.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sshiwani\workspace\find-information-products-services-tests\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0AA9572B-ED4F-4DF7-BF30-28BE31D05844}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{03279657-AE4E-4469-BDE8-A24A591A0385}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="22780" windowHeight="14540" firstSheet="28" activeTab="29" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="22780" windowHeight="14540" firstSheet="32" activeTab="33" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="category_phase" sheetId="1" r:id="rId1"/>
@@ -30,19 +30,23 @@
     <sheet name="usergroup_SocialCWorkforce_list" sheetId="15" r:id="rId15"/>
     <sheet name="usergroup_SocialWorker_list" sheetId="26" r:id="rId16"/>
     <sheet name="UG_EPEYAcademyTruWorkforce_list" sheetId="30" r:id="rId17"/>
-    <sheet name="UGSubcategory_AdultLearner" sheetId="16" r:id="rId18"/>
-    <sheet name="UGSubcategory_CareersAdviser" sheetId="17" r:id="rId19"/>
-    <sheet name="UGSubcategory_ChildOrYoungPers" sheetId="18" r:id="rId20"/>
-    <sheet name="UGSubcategory_DfEWorkforce" sheetId="19" r:id="rId21"/>
-    <sheet name="UGSubcategory_Employer" sheetId="20" r:id="rId22"/>
-    <sheet name="UGSubcategory_LAWorkforce" sheetId="21" r:id="rId23"/>
-    <sheet name="UGSubcategory_NEETOrCareerSeek" sheetId="22" r:id="rId24"/>
-    <sheet name="UGSubcategory_ParentOrCarer" sheetId="23" r:id="rId25"/>
-    <sheet name="UGSubcateg_ProfExtUserofDfEData" sheetId="24" r:id="rId26"/>
-    <sheet name="UGSubcategory_SCWorkforce" sheetId="25" r:id="rId27"/>
-    <sheet name="UGSubcategory_SocialWorker" sheetId="27" r:id="rId28"/>
-    <sheet name="UGSubcategory_EPandEYWorkforce" sheetId="29" r:id="rId29"/>
-    <sheet name="EPEYSubcateg_AcademyTWorkforce" sheetId="31" r:id="rId30"/>
+    <sheet name="UG_EPEYAltProvSetWorkforce_list" sheetId="32" r:id="rId18"/>
+    <sheet name="UG_EPEYEarlyYearsWorkforce_list" sheetId="35" r:id="rId19"/>
+    <sheet name="UGSubcategory_AdultLearner" sheetId="16" r:id="rId20"/>
+    <sheet name="UGSubcategory_CareersAdviser" sheetId="17" r:id="rId21"/>
+    <sheet name="UGSubcategory_ChildOrYoungPers" sheetId="18" r:id="rId22"/>
+    <sheet name="UGSubcategory_DfEWorkforce" sheetId="19" r:id="rId23"/>
+    <sheet name="UGSubcategory_Employer" sheetId="20" r:id="rId24"/>
+    <sheet name="UGSubcategory_LAWorkforce" sheetId="21" r:id="rId25"/>
+    <sheet name="UGSubcategory_NEETOrCareerSeek" sheetId="22" r:id="rId26"/>
+    <sheet name="UGSubcategory_ParentOrCarer" sheetId="23" r:id="rId27"/>
+    <sheet name="UGSubcateg_ProfExtUserofDfEData" sheetId="24" r:id="rId28"/>
+    <sheet name="UGSubcategory_SCWorkforce" sheetId="25" r:id="rId29"/>
+    <sheet name="UGSubcategory_SocialWorker" sheetId="27" r:id="rId30"/>
+    <sheet name="UGSubcategory_EPandEYWorkforce" sheetId="29" r:id="rId31"/>
+    <sheet name="EPEYSubcateg_AcademyTWorkforce" sheetId="31" r:id="rId32"/>
+    <sheet name="EPEYSubcateg_AltProSetWorkforce" sheetId="33" r:id="rId33"/>
+    <sheet name="EPEYSubcateg_EarlyYearsWorkforc" sheetId="34" r:id="rId34"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -54,7 +58,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1166" uniqueCount="571">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1255" uniqueCount="602">
   <si>
     <t>Search and filter products and services</t>
   </si>
@@ -1767,6 +1771,99 @@
   </si>
   <si>
     <t>Academy trustee  (Academy and trust workforce)</t>
+  </si>
+  <si>
+    <t>categories/user-group/education-provider-and-early-years-workforce/alternative-provision-setting-workforce</t>
+  </si>
+  <si>
+    <t>Browse products in Alternative provision setting workforce</t>
+  </si>
+  <si>
+    <t>Alternative provision setting mentor</t>
+  </si>
+  <si>
+    <t>Alternative provision setting support assistant</t>
+  </si>
+  <si>
+    <t>Alternative provision setting teacher</t>
+  </si>
+  <si>
+    <t>products?userGroup=alternative-provision-setting-workforce</t>
+  </si>
+  <si>
+    <t>ul.moj-filter-tags li a:has-text(' Alternative provision setting workforce ')</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Remove this filter Alternative provision setting workforce </t>
+  </si>
+  <si>
+    <t>Alternative provision setting workforce  (Education provider and early years workforce)</t>
+  </si>
+  <si>
+    <t>products?userGroup=alternative-provision-setting-mentor</t>
+  </si>
+  <si>
+    <t>ul.moj-filter-tags li a:has-text(' Alternative provision setting mentor ')</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Remove this filter Alternative provision setting mentor </t>
+  </si>
+  <si>
+    <t>Alternative provision setting mentor  (Alternative provision setting workforce)</t>
+  </si>
+  <si>
+    <t>products?userGroup=alternative-provision-setting-support-assistant</t>
+  </si>
+  <si>
+    <t>ul.moj-filter-tags li a:has-text(' alternative-provision-setting-support-assistant')</t>
+  </si>
+  <si>
+    <t>Remove this filter alternative-provision-setting-support-assistant</t>
+  </si>
+  <si>
+    <t>products?userGroup=alternative-provision-setting-teacher</t>
+  </si>
+  <si>
+    <t>ul.moj-filter-tags li a:has-text(' Alternative provision setting teacher  (Alternative provision setting workforce)')</t>
+  </si>
+  <si>
+    <t>Remove this filter Alternative provision setting teacher  (Alternative provision setting workforce)</t>
+  </si>
+  <si>
+    <t>Alternative provision setting teacher  (Alternative provision setting workforce)</t>
+  </si>
+  <si>
+    <t>categories/user-group/education-provider-and-early-years-workforce/early-years-workforce</t>
+  </si>
+  <si>
+    <t>Browse products in Early years workforce</t>
+  </si>
+  <si>
+    <t>Early years teacher</t>
+  </si>
+  <si>
+    <t>products?userGroup=early-years-workforce</t>
+  </si>
+  <si>
+    <t>ul.moj-filter-tags li a:has-text(' Early years workforce  (Education provider and early years workforce)')</t>
+  </si>
+  <si>
+    <t>Remove this filter Early years workforce  (Education provider and early years workforce)</t>
+  </si>
+  <si>
+    <t>Early years workforce  (Education provider and early years workforce)</t>
+  </si>
+  <si>
+    <t>products?userGroup=early-years-teacher</t>
+  </si>
+  <si>
+    <t>ul.moj-filter-tags li a:has-text(' Early years teacher  (Early years workforce)')</t>
+  </si>
+  <si>
+    <t>Remove this filter Early years teacher  (Early years workforce)</t>
+  </si>
+  <si>
+    <t>Early years teacher  (Early years workforce)</t>
   </si>
 </sst>
 </file>
@@ -1788,7 +1885,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1816,6 +1913,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="6"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1908,7 +2011,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
@@ -1920,6 +2023,7 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="6" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -12348,6 +12452,372 @@
 </file>
 
 <file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3235E800-0517-4419-BDEC-02DDE8FA7B7F}">
+  <dimension ref="A1:C8"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="54.1796875" customWidth="1"/>
+    <col min="2" max="2" width="47.453125" customWidth="1"/>
+    <col min="3" max="3" width="50.36328125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A1" s="6" t="s">
+        <v>102</v>
+      </c>
+      <c r="B1" s="6" t="s">
+        <v>103</v>
+      </c>
+      <c r="C1" s="6" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A2" s="3" t="s">
+        <v>571</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>107</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>572</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="B3" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="B4" s="3" t="s">
+        <v>113</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A5" s="3" t="s">
+        <v>142</v>
+      </c>
+      <c r="B5" s="3"/>
+      <c r="C5" s="3"/>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A6" s="3" t="s">
+        <v>573</v>
+      </c>
+      <c r="B6" s="3"/>
+      <c r="C6" s="3"/>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A7" s="3" t="s">
+        <v>574</v>
+      </c>
+      <c r="B7" s="3"/>
+      <c r="C7" s="3"/>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A8" s="3" t="s">
+        <v>575</v>
+      </c>
+      <c r="B8" s="3"/>
+      <c r="C8" s="3"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FF697B66-4B1C-421E-AABA-D2FBFBB56C35}">
+  <dimension ref="A1:C6"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="54.1796875" customWidth="1"/>
+    <col min="2" max="2" width="47.453125" customWidth="1"/>
+    <col min="3" max="3" width="50.36328125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A1" s="6" t="s">
+        <v>102</v>
+      </c>
+      <c r="B1" s="6" t="s">
+        <v>103</v>
+      </c>
+      <c r="C1" s="6" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A2" s="3" t="s">
+        <v>591</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>107</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>592</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="B3" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="B4" s="3" t="s">
+        <v>113</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A5" s="3" t="s">
+        <v>143</v>
+      </c>
+      <c r="B5" s="3"/>
+      <c r="C5" s="3"/>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A6" s="3" t="s">
+        <v>593</v>
+      </c>
+      <c r="B6" s="3"/>
+      <c r="C6" s="3"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B2DC696B-E1A8-430C-BC9E-87DD1A6FBE9F}">
+  <dimension ref="A1:F10"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="33.08984375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="43.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="32.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="33.36328125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="29.90625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="25.36328125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A2" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="F2" s="3" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A3" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>101</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="F3" s="3" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A4" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="F4" s="3" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A5" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>91</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="F5" s="3" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A6" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="D6" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="E6" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="F6" s="3" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A7" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="E7" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="F7" s="3" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A8" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="D8" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="E8" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="F8" s="3" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A9" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="D9" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="E9" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="F9" s="3" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A10" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="D10" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="E10" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="F10" s="3" t="s">
+        <v>69</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FB5527F7-85DB-4F8E-B4B3-EC8453E599E1}">
   <dimension ref="A1:HU6"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -12745,7 +13215,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A99CF6C3-F305-48A2-AB80-2C2D7CE6460C}">
   <dimension ref="A1:HU5"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -13116,225 +13586,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B2DC696B-E1A8-430C-BC9E-87DD1A6FBE9F}">
-  <dimension ref="A1:F10"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
-  <cols>
-    <col min="1" max="1" width="33.08984375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="43.54296875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="32.1796875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="33.36328125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="29.90625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="25.36328125" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A1" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="F1" s="2" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="3" t="s">
-        <v>38</v>
-      </c>
-      <c r="B2" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="C2" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="D2" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="E2" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="F2" s="3" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="3" t="s">
-        <v>41</v>
-      </c>
-      <c r="B3" s="3" t="s">
-        <v>101</v>
-      </c>
-      <c r="C3" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="D3" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="E3" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="F3" s="3" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="3" t="s">
-        <v>45</v>
-      </c>
-      <c r="B4" s="3" t="s">
-        <v>44</v>
-      </c>
-      <c r="C4" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="D4" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="E4" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="F4" s="3" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="B5" s="3" t="s">
-        <v>91</v>
-      </c>
-      <c r="C5" s="3" t="s">
-        <v>92</v>
-      </c>
-      <c r="D5" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="E5" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="F5" s="3" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="3" t="s">
-        <v>50</v>
-      </c>
-      <c r="B6" s="3" t="s">
-        <v>51</v>
-      </c>
-      <c r="C6" s="3" t="s">
-        <v>52</v>
-      </c>
-      <c r="D6" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="E6" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="F6" s="3" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A7" s="3" t="s">
-        <v>54</v>
-      </c>
-      <c r="B7" s="3" t="s">
-        <v>55</v>
-      </c>
-      <c r="C7" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="D7" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="E7" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="F7" s="3" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A8" s="3" t="s">
-        <v>58</v>
-      </c>
-      <c r="B8" s="3" t="s">
-        <v>59</v>
-      </c>
-      <c r="C8" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="D8" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="E8" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="F8" s="3" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A9" s="3" t="s">
-        <v>62</v>
-      </c>
-      <c r="B9" s="3" t="s">
-        <v>63</v>
-      </c>
-      <c r="C9" s="3" t="s">
-        <v>64</v>
-      </c>
-      <c r="D9" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="E9" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="F9" s="3" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A10" s="3" t="s">
-        <v>66</v>
-      </c>
-      <c r="B10" s="3" t="s">
-        <v>67</v>
-      </c>
-      <c r="C10" s="3" t="s">
-        <v>68</v>
-      </c>
-      <c r="D10" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="E10" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="F10" s="3" t="s">
-        <v>69</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5EFF0597-7FD1-4E6A-AA71-DB9F9FAB97A9}">
   <dimension ref="A1:HU7"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -13758,7 +14010,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9F4A57AC-4620-4875-88AE-9F5C739A9042}">
   <dimension ref="A1:HU6"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -14155,7 +14407,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6C1C130F-0899-4810-82F6-950C9CB07234}">
   <dimension ref="A1:HU5"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -14526,7 +14778,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4AB9395B-D522-49AD-B790-5334356249F6}">
   <dimension ref="A1:HU7"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -14949,7 +15201,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BEE91763-AD0C-4544-A433-3B50C88AEB79}">
   <dimension ref="A1:HU7"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -15372,7 +15624,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{20DD36AA-F163-4AAB-BD30-4AE6290CCAE7}">
   <dimension ref="A1:HU10"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -15874,7 +16126,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C6EE6111-FDB3-4B43-8820-BBF68AAFCD6D}">
   <dimension ref="A1:HU8"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -16324,7 +16576,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet29.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E6428663-7558-48F1-8CD3-947F03FFD4CC}">
   <dimension ref="A1:HU9"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -16796,722 +17048,6 @@
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2A4E3580-B709-4E66-9F6E-B7F9948D7FD3}">
-  <dimension ref="A1:HU7"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
-  <cols>
-    <col min="1" max="1" width="50.90625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="52.26953125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="42.453125" customWidth="1"/>
-    <col min="4" max="4" width="33.36328125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="33.08984375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="17.08984375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="40.81640625" customWidth="1"/>
-    <col min="8" max="8" width="57.08984375" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:229" x14ac:dyDescent="0.35">
-      <c r="A1" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="F1" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="G1" s="2" t="s">
-        <v>209</v>
-      </c>
-      <c r="H1" s="2" t="s">
-        <v>210</v>
-      </c>
-    </row>
-    <row r="2" spans="1:229" s="4" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="3" t="s">
-        <v>488</v>
-      </c>
-      <c r="B2" s="3" t="s">
-        <v>489</v>
-      </c>
-      <c r="C2" s="3" t="s">
-        <v>490</v>
-      </c>
-      <c r="D2" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="E2" s="3" t="s">
-        <v>201</v>
-      </c>
-      <c r="F2" s="3" t="s">
-        <v>202</v>
-      </c>
-      <c r="G2" s="3" t="s">
-        <v>211</v>
-      </c>
-      <c r="H2" s="3" t="s">
-        <v>491</v>
-      </c>
-      <c r="I2"/>
-      <c r="J2"/>
-      <c r="K2"/>
-      <c r="L2"/>
-      <c r="M2"/>
-      <c r="N2"/>
-      <c r="O2"/>
-      <c r="P2"/>
-      <c r="Q2"/>
-      <c r="R2"/>
-      <c r="S2"/>
-      <c r="T2"/>
-      <c r="U2"/>
-      <c r="V2"/>
-      <c r="W2"/>
-      <c r="X2"/>
-      <c r="Y2"/>
-      <c r="Z2"/>
-      <c r="AA2"/>
-      <c r="AB2"/>
-      <c r="AC2"/>
-      <c r="AD2"/>
-      <c r="AE2"/>
-      <c r="AF2"/>
-      <c r="AG2"/>
-      <c r="AH2"/>
-      <c r="AI2"/>
-      <c r="AJ2"/>
-      <c r="AK2"/>
-      <c r="AL2"/>
-      <c r="AM2"/>
-      <c r="AN2"/>
-      <c r="AO2"/>
-      <c r="AP2"/>
-      <c r="AQ2"/>
-      <c r="AR2"/>
-      <c r="AS2"/>
-      <c r="AT2"/>
-      <c r="AU2"/>
-      <c r="AV2"/>
-      <c r="AW2"/>
-      <c r="AX2"/>
-      <c r="AY2"/>
-      <c r="AZ2"/>
-      <c r="BA2"/>
-      <c r="BB2"/>
-      <c r="BC2"/>
-      <c r="BD2"/>
-      <c r="BE2"/>
-      <c r="BF2"/>
-      <c r="BG2"/>
-      <c r="BH2"/>
-      <c r="BI2"/>
-      <c r="BJ2"/>
-      <c r="BK2"/>
-      <c r="BL2"/>
-      <c r="BM2"/>
-      <c r="BN2"/>
-      <c r="BO2"/>
-      <c r="BP2"/>
-      <c r="BQ2"/>
-      <c r="BR2"/>
-      <c r="BS2"/>
-      <c r="BT2"/>
-      <c r="BU2"/>
-      <c r="BV2"/>
-      <c r="BW2"/>
-      <c r="BX2"/>
-      <c r="BY2"/>
-      <c r="BZ2"/>
-      <c r="CA2"/>
-      <c r="CB2"/>
-      <c r="CC2"/>
-      <c r="CD2"/>
-      <c r="CE2"/>
-      <c r="CF2"/>
-      <c r="CG2"/>
-      <c r="CH2"/>
-      <c r="CI2"/>
-      <c r="CJ2"/>
-      <c r="CK2"/>
-      <c r="CL2"/>
-      <c r="CM2"/>
-      <c r="CN2"/>
-      <c r="CO2"/>
-      <c r="CP2"/>
-      <c r="CQ2"/>
-      <c r="CR2"/>
-      <c r="CS2"/>
-      <c r="CT2"/>
-      <c r="CU2"/>
-      <c r="CV2"/>
-      <c r="CW2"/>
-      <c r="CX2"/>
-      <c r="CY2"/>
-      <c r="CZ2"/>
-      <c r="DA2"/>
-      <c r="DB2"/>
-      <c r="DC2"/>
-      <c r="DD2"/>
-      <c r="DE2"/>
-      <c r="DF2"/>
-      <c r="DG2"/>
-      <c r="DH2"/>
-      <c r="DI2"/>
-      <c r="DJ2"/>
-      <c r="DK2"/>
-      <c r="DL2"/>
-      <c r="DM2"/>
-      <c r="DN2"/>
-      <c r="DO2"/>
-      <c r="DP2"/>
-      <c r="DQ2"/>
-      <c r="DR2"/>
-      <c r="DS2"/>
-      <c r="DT2"/>
-      <c r="DU2"/>
-      <c r="DV2"/>
-      <c r="DW2"/>
-      <c r="DX2"/>
-      <c r="DY2"/>
-      <c r="DZ2"/>
-      <c r="EA2"/>
-      <c r="EB2"/>
-      <c r="EC2"/>
-      <c r="ED2"/>
-      <c r="EE2"/>
-      <c r="EF2"/>
-      <c r="EG2"/>
-      <c r="EH2"/>
-      <c r="EI2"/>
-      <c r="EJ2"/>
-      <c r="EK2"/>
-      <c r="EL2"/>
-      <c r="EM2"/>
-      <c r="EN2"/>
-      <c r="EO2"/>
-      <c r="EP2"/>
-      <c r="EQ2"/>
-      <c r="ER2"/>
-      <c r="ES2"/>
-      <c r="ET2"/>
-      <c r="EU2"/>
-      <c r="EV2"/>
-      <c r="EW2"/>
-      <c r="EX2"/>
-      <c r="EY2"/>
-      <c r="EZ2"/>
-      <c r="FA2"/>
-      <c r="FB2"/>
-      <c r="FC2"/>
-      <c r="FD2"/>
-      <c r="FE2"/>
-      <c r="FF2"/>
-      <c r="FG2"/>
-      <c r="FH2"/>
-      <c r="FI2"/>
-      <c r="FJ2"/>
-      <c r="FK2"/>
-      <c r="FL2"/>
-      <c r="FM2"/>
-      <c r="FN2"/>
-      <c r="FO2"/>
-      <c r="FP2"/>
-      <c r="FQ2"/>
-      <c r="FR2"/>
-      <c r="FS2"/>
-      <c r="FT2"/>
-      <c r="FU2"/>
-      <c r="FV2"/>
-      <c r="FW2"/>
-      <c r="FX2"/>
-      <c r="FY2"/>
-      <c r="FZ2"/>
-      <c r="GA2"/>
-      <c r="GB2"/>
-      <c r="GC2"/>
-      <c r="GD2"/>
-      <c r="GE2"/>
-      <c r="GF2"/>
-      <c r="GG2"/>
-      <c r="GH2"/>
-      <c r="GI2"/>
-      <c r="GJ2"/>
-      <c r="GK2"/>
-      <c r="GL2"/>
-      <c r="GM2"/>
-      <c r="GN2"/>
-      <c r="GO2"/>
-      <c r="GP2"/>
-      <c r="GQ2"/>
-      <c r="GR2"/>
-      <c r="GS2"/>
-      <c r="GT2"/>
-      <c r="GU2"/>
-      <c r="GV2"/>
-      <c r="GW2"/>
-      <c r="GX2"/>
-      <c r="GY2"/>
-      <c r="GZ2"/>
-      <c r="HA2"/>
-      <c r="HB2"/>
-      <c r="HC2"/>
-      <c r="HD2"/>
-      <c r="HE2"/>
-      <c r="HF2"/>
-      <c r="HG2"/>
-      <c r="HH2"/>
-      <c r="HI2"/>
-      <c r="HJ2"/>
-      <c r="HK2"/>
-      <c r="HL2"/>
-      <c r="HM2"/>
-      <c r="HN2"/>
-      <c r="HO2"/>
-      <c r="HP2"/>
-      <c r="HQ2"/>
-      <c r="HR2"/>
-      <c r="HS2"/>
-      <c r="HT2"/>
-      <c r="HU2"/>
-    </row>
-    <row r="3" spans="1:229" x14ac:dyDescent="0.35">
-      <c r="A3" s="3" t="s">
-        <v>492</v>
-      </c>
-      <c r="B3" s="3" t="s">
-        <v>493</v>
-      </c>
-      <c r="C3" s="3" t="s">
-        <v>494</v>
-      </c>
-      <c r="D3" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="E3" s="3" t="s">
-        <v>201</v>
-      </c>
-      <c r="F3" s="3" t="s">
-        <v>202</v>
-      </c>
-      <c r="G3" s="3" t="s">
-        <v>211</v>
-      </c>
-      <c r="H3" s="3" t="s">
-        <v>495</v>
-      </c>
-    </row>
-    <row r="4" spans="1:229" x14ac:dyDescent="0.35">
-      <c r="A4" s="3" t="s">
-        <v>496</v>
-      </c>
-      <c r="B4" s="3" t="s">
-        <v>497</v>
-      </c>
-      <c r="C4" s="3" t="s">
-        <v>498</v>
-      </c>
-      <c r="D4" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="E4" s="3" t="s">
-        <v>201</v>
-      </c>
-      <c r="F4" s="3" t="s">
-        <v>202</v>
-      </c>
-      <c r="G4" s="3" t="s">
-        <v>211</v>
-      </c>
-      <c r="H4" s="3" t="s">
-        <v>499</v>
-      </c>
-    </row>
-    <row r="5" spans="1:229" x14ac:dyDescent="0.35">
-      <c r="A5" s="8" t="s">
-        <v>500</v>
-      </c>
-      <c r="B5" s="8" t="s">
-        <v>501</v>
-      </c>
-      <c r="C5" s="8" t="s">
-        <v>502</v>
-      </c>
-      <c r="D5" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="E5" s="3" t="s">
-        <v>201</v>
-      </c>
-      <c r="F5" s="3" t="s">
-        <v>202</v>
-      </c>
-      <c r="G5" s="3" t="s">
-        <v>211</v>
-      </c>
-      <c r="H5" s="3" t="s">
-        <v>503</v>
-      </c>
-    </row>
-    <row r="6" spans="1:229" x14ac:dyDescent="0.35">
-      <c r="A6" s="3" t="s">
-        <v>504</v>
-      </c>
-      <c r="B6" s="3" t="s">
-        <v>505</v>
-      </c>
-      <c r="C6" s="3" t="s">
-        <v>506</v>
-      </c>
-      <c r="D6" s="7" t="s">
-        <v>0</v>
-      </c>
-      <c r="E6" s="3" t="s">
-        <v>201</v>
-      </c>
-      <c r="F6" s="3" t="s">
-        <v>202</v>
-      </c>
-      <c r="G6" s="3" t="s">
-        <v>211</v>
-      </c>
-      <c r="H6" s="3" t="s">
-        <v>507</v>
-      </c>
-    </row>
-    <row r="7" spans="1:229" x14ac:dyDescent="0.35">
-      <c r="A7" s="3" t="s">
-        <v>509</v>
-      </c>
-      <c r="B7" s="3" t="s">
-        <v>508</v>
-      </c>
-      <c r="C7" s="3" t="s">
-        <v>510</v>
-      </c>
-      <c r="D7" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="E7" s="3" t="s">
-        <v>201</v>
-      </c>
-      <c r="F7" s="3" t="s">
-        <v>202</v>
-      </c>
-      <c r="G7" s="3" t="s">
-        <v>211</v>
-      </c>
-      <c r="H7" s="3" t="s">
-        <v>511</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet29.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{95706458-CD50-4C74-87C4-ABAE617927AD}">
-  <dimension ref="A1:HU2"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
-  <cols>
-    <col min="1" max="1" width="50.90625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="52.26953125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="42.453125" customWidth="1"/>
-    <col min="4" max="4" width="33.36328125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="33.08984375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="17.08984375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="40.81640625" customWidth="1"/>
-    <col min="8" max="8" width="57.08984375" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:229" x14ac:dyDescent="0.35">
-      <c r="A1" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="F1" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="G1" s="2" t="s">
-        <v>209</v>
-      </c>
-      <c r="H1" s="2" t="s">
-        <v>210</v>
-      </c>
-    </row>
-    <row r="2" spans="1:229" s="4" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="3" t="s">
-        <v>512</v>
-      </c>
-      <c r="B2" s="3" t="s">
-        <v>513</v>
-      </c>
-      <c r="C2" s="3" t="s">
-        <v>514</v>
-      </c>
-      <c r="D2" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="E2" s="3" t="s">
-        <v>201</v>
-      </c>
-      <c r="F2" s="3" t="s">
-        <v>202</v>
-      </c>
-      <c r="G2" s="3" t="s">
-        <v>211</v>
-      </c>
-      <c r="H2" s="3" t="s">
-        <v>140</v>
-      </c>
-      <c r="I2"/>
-      <c r="J2"/>
-      <c r="K2"/>
-      <c r="L2"/>
-      <c r="M2"/>
-      <c r="N2"/>
-      <c r="O2"/>
-      <c r="P2"/>
-      <c r="Q2"/>
-      <c r="R2"/>
-      <c r="S2"/>
-      <c r="T2"/>
-      <c r="U2"/>
-      <c r="V2"/>
-      <c r="W2"/>
-      <c r="X2"/>
-      <c r="Y2"/>
-      <c r="Z2"/>
-      <c r="AA2"/>
-      <c r="AB2"/>
-      <c r="AC2"/>
-      <c r="AD2"/>
-      <c r="AE2"/>
-      <c r="AF2"/>
-      <c r="AG2"/>
-      <c r="AH2"/>
-      <c r="AI2"/>
-      <c r="AJ2"/>
-      <c r="AK2"/>
-      <c r="AL2"/>
-      <c r="AM2"/>
-      <c r="AN2"/>
-      <c r="AO2"/>
-      <c r="AP2"/>
-      <c r="AQ2"/>
-      <c r="AR2"/>
-      <c r="AS2"/>
-      <c r="AT2"/>
-      <c r="AU2"/>
-      <c r="AV2"/>
-      <c r="AW2"/>
-      <c r="AX2"/>
-      <c r="AY2"/>
-      <c r="AZ2"/>
-      <c r="BA2"/>
-      <c r="BB2"/>
-      <c r="BC2"/>
-      <c r="BD2"/>
-      <c r="BE2"/>
-      <c r="BF2"/>
-      <c r="BG2"/>
-      <c r="BH2"/>
-      <c r="BI2"/>
-      <c r="BJ2"/>
-      <c r="BK2"/>
-      <c r="BL2"/>
-      <c r="BM2"/>
-      <c r="BN2"/>
-      <c r="BO2"/>
-      <c r="BP2"/>
-      <c r="BQ2"/>
-      <c r="BR2"/>
-      <c r="BS2"/>
-      <c r="BT2"/>
-      <c r="BU2"/>
-      <c r="BV2"/>
-      <c r="BW2"/>
-      <c r="BX2"/>
-      <c r="BY2"/>
-      <c r="BZ2"/>
-      <c r="CA2"/>
-      <c r="CB2"/>
-      <c r="CC2"/>
-      <c r="CD2"/>
-      <c r="CE2"/>
-      <c r="CF2"/>
-      <c r="CG2"/>
-      <c r="CH2"/>
-      <c r="CI2"/>
-      <c r="CJ2"/>
-      <c r="CK2"/>
-      <c r="CL2"/>
-      <c r="CM2"/>
-      <c r="CN2"/>
-      <c r="CO2"/>
-      <c r="CP2"/>
-      <c r="CQ2"/>
-      <c r="CR2"/>
-      <c r="CS2"/>
-      <c r="CT2"/>
-      <c r="CU2"/>
-      <c r="CV2"/>
-      <c r="CW2"/>
-      <c r="CX2"/>
-      <c r="CY2"/>
-      <c r="CZ2"/>
-      <c r="DA2"/>
-      <c r="DB2"/>
-      <c r="DC2"/>
-      <c r="DD2"/>
-      <c r="DE2"/>
-      <c r="DF2"/>
-      <c r="DG2"/>
-      <c r="DH2"/>
-      <c r="DI2"/>
-      <c r="DJ2"/>
-      <c r="DK2"/>
-      <c r="DL2"/>
-      <c r="DM2"/>
-      <c r="DN2"/>
-      <c r="DO2"/>
-      <c r="DP2"/>
-      <c r="DQ2"/>
-      <c r="DR2"/>
-      <c r="DS2"/>
-      <c r="DT2"/>
-      <c r="DU2"/>
-      <c r="DV2"/>
-      <c r="DW2"/>
-      <c r="DX2"/>
-      <c r="DY2"/>
-      <c r="DZ2"/>
-      <c r="EA2"/>
-      <c r="EB2"/>
-      <c r="EC2"/>
-      <c r="ED2"/>
-      <c r="EE2"/>
-      <c r="EF2"/>
-      <c r="EG2"/>
-      <c r="EH2"/>
-      <c r="EI2"/>
-      <c r="EJ2"/>
-      <c r="EK2"/>
-      <c r="EL2"/>
-      <c r="EM2"/>
-      <c r="EN2"/>
-      <c r="EO2"/>
-      <c r="EP2"/>
-      <c r="EQ2"/>
-      <c r="ER2"/>
-      <c r="ES2"/>
-      <c r="ET2"/>
-      <c r="EU2"/>
-      <c r="EV2"/>
-      <c r="EW2"/>
-      <c r="EX2"/>
-      <c r="EY2"/>
-      <c r="EZ2"/>
-      <c r="FA2"/>
-      <c r="FB2"/>
-      <c r="FC2"/>
-      <c r="FD2"/>
-      <c r="FE2"/>
-      <c r="FF2"/>
-      <c r="FG2"/>
-      <c r="FH2"/>
-      <c r="FI2"/>
-      <c r="FJ2"/>
-      <c r="FK2"/>
-      <c r="FL2"/>
-      <c r="FM2"/>
-      <c r="FN2"/>
-      <c r="FO2"/>
-      <c r="FP2"/>
-      <c r="FQ2"/>
-      <c r="FR2"/>
-      <c r="FS2"/>
-      <c r="FT2"/>
-      <c r="FU2"/>
-      <c r="FV2"/>
-      <c r="FW2"/>
-      <c r="FX2"/>
-      <c r="FY2"/>
-      <c r="FZ2"/>
-      <c r="GA2"/>
-      <c r="GB2"/>
-      <c r="GC2"/>
-      <c r="GD2"/>
-      <c r="GE2"/>
-      <c r="GF2"/>
-      <c r="GG2"/>
-      <c r="GH2"/>
-      <c r="GI2"/>
-      <c r="GJ2"/>
-      <c r="GK2"/>
-      <c r="GL2"/>
-      <c r="GM2"/>
-      <c r="GN2"/>
-      <c r="GO2"/>
-      <c r="GP2"/>
-      <c r="GQ2"/>
-      <c r="GR2"/>
-      <c r="GS2"/>
-      <c r="GT2"/>
-      <c r="GU2"/>
-      <c r="GV2"/>
-      <c r="GW2"/>
-      <c r="GX2"/>
-      <c r="GY2"/>
-      <c r="GZ2"/>
-      <c r="HA2"/>
-      <c r="HB2"/>
-      <c r="HC2"/>
-      <c r="HD2"/>
-      <c r="HE2"/>
-      <c r="HF2"/>
-      <c r="HG2"/>
-      <c r="HH2"/>
-      <c r="HI2"/>
-      <c r="HJ2"/>
-      <c r="HK2"/>
-      <c r="HL2"/>
-      <c r="HM2"/>
-      <c r="HN2"/>
-      <c r="HO2"/>
-      <c r="HP2"/>
-      <c r="HQ2"/>
-      <c r="HR2"/>
-      <c r="HS2"/>
-      <c r="HT2"/>
-      <c r="HU2"/>
-    </row>
-  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -19821,8 +19357,8 @@
 </file>
 
 <file path=xl/worksheets/sheet30.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1AD86191-7CFE-4ED9-9129-FF78170AB51E}">
-  <dimension ref="A1:HU12"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2A4E3580-B709-4E66-9F6E-B7F9948D7FD3}">
+  <dimension ref="A1:HU7"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="50.90625" bestFit="1" customWidth="1"/>
@@ -19832,7 +19368,7 @@
     <col min="5" max="5" width="33.08984375" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="17.08984375" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="40.81640625" customWidth="1"/>
-    <col min="8" max="8" width="65.54296875" customWidth="1"/>
+    <col min="8" max="8" width="57.08984375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:229" x14ac:dyDescent="0.35">
@@ -19863,13 +19399,13 @@
     </row>
     <row r="2" spans="1:229" s="4" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A2" s="3" t="s">
-        <v>527</v>
+        <v>488</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>528</v>
+        <v>489</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>529</v>
+        <v>490</v>
       </c>
       <c r="D2" s="3" t="s">
         <v>0</v>
@@ -19884,7 +19420,7 @@
         <v>211</v>
       </c>
       <c r="H2" s="3" t="s">
-        <v>530</v>
+        <v>491</v>
       </c>
       <c r="I2"/>
       <c r="J2"/>
@@ -20110,6 +19646,722 @@
     </row>
     <row r="3" spans="1:229" x14ac:dyDescent="0.35">
       <c r="A3" s="3" t="s">
+        <v>492</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>493</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>494</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>201</v>
+      </c>
+      <c r="F3" s="3" t="s">
+        <v>202</v>
+      </c>
+      <c r="G3" s="3" t="s">
+        <v>211</v>
+      </c>
+      <c r="H3" s="3" t="s">
+        <v>495</v>
+      </c>
+    </row>
+    <row r="4" spans="1:229" x14ac:dyDescent="0.35">
+      <c r="A4" s="3" t="s">
+        <v>496</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>497</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>498</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>201</v>
+      </c>
+      <c r="F4" s="3" t="s">
+        <v>202</v>
+      </c>
+      <c r="G4" s="3" t="s">
+        <v>211</v>
+      </c>
+      <c r="H4" s="3" t="s">
+        <v>499</v>
+      </c>
+    </row>
+    <row r="5" spans="1:229" x14ac:dyDescent="0.35">
+      <c r="A5" s="8" t="s">
+        <v>500</v>
+      </c>
+      <c r="B5" s="8" t="s">
+        <v>501</v>
+      </c>
+      <c r="C5" s="8" t="s">
+        <v>502</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>201</v>
+      </c>
+      <c r="F5" s="3" t="s">
+        <v>202</v>
+      </c>
+      <c r="G5" s="3" t="s">
+        <v>211</v>
+      </c>
+      <c r="H5" s="3" t="s">
+        <v>503</v>
+      </c>
+    </row>
+    <row r="6" spans="1:229" x14ac:dyDescent="0.35">
+      <c r="A6" s="3" t="s">
+        <v>504</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>505</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>506</v>
+      </c>
+      <c r="D6" s="7" t="s">
+        <v>0</v>
+      </c>
+      <c r="E6" s="3" t="s">
+        <v>201</v>
+      </c>
+      <c r="F6" s="3" t="s">
+        <v>202</v>
+      </c>
+      <c r="G6" s="3" t="s">
+        <v>211</v>
+      </c>
+      <c r="H6" s="3" t="s">
+        <v>507</v>
+      </c>
+    </row>
+    <row r="7" spans="1:229" x14ac:dyDescent="0.35">
+      <c r="A7" s="3" t="s">
+        <v>509</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>508</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>510</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="E7" s="3" t="s">
+        <v>201</v>
+      </c>
+      <c r="F7" s="3" t="s">
+        <v>202</v>
+      </c>
+      <c r="G7" s="3" t="s">
+        <v>211</v>
+      </c>
+      <c r="H7" s="3" t="s">
+        <v>511</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet31.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{95706458-CD50-4C74-87C4-ABAE617927AD}">
+  <dimension ref="A1:HU2"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="50.90625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="52.26953125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="42.453125" customWidth="1"/>
+    <col min="4" max="4" width="33.36328125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="33.08984375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="17.08984375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="40.81640625" customWidth="1"/>
+    <col min="8" max="8" width="57.08984375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:229" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>209</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="2" spans="1:229" s="4" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A2" s="3" t="s">
+        <v>512</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>513</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>514</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>201</v>
+      </c>
+      <c r="F2" s="3" t="s">
+        <v>202</v>
+      </c>
+      <c r="G2" s="3" t="s">
+        <v>211</v>
+      </c>
+      <c r="H2" s="3" t="s">
+        <v>140</v>
+      </c>
+      <c r="I2"/>
+      <c r="J2"/>
+      <c r="K2"/>
+      <c r="L2"/>
+      <c r="M2"/>
+      <c r="N2"/>
+      <c r="O2"/>
+      <c r="P2"/>
+      <c r="Q2"/>
+      <c r="R2"/>
+      <c r="S2"/>
+      <c r="T2"/>
+      <c r="U2"/>
+      <c r="V2"/>
+      <c r="W2"/>
+      <c r="X2"/>
+      <c r="Y2"/>
+      <c r="Z2"/>
+      <c r="AA2"/>
+      <c r="AB2"/>
+      <c r="AC2"/>
+      <c r="AD2"/>
+      <c r="AE2"/>
+      <c r="AF2"/>
+      <c r="AG2"/>
+      <c r="AH2"/>
+      <c r="AI2"/>
+      <c r="AJ2"/>
+      <c r="AK2"/>
+      <c r="AL2"/>
+      <c r="AM2"/>
+      <c r="AN2"/>
+      <c r="AO2"/>
+      <c r="AP2"/>
+      <c r="AQ2"/>
+      <c r="AR2"/>
+      <c r="AS2"/>
+      <c r="AT2"/>
+      <c r="AU2"/>
+      <c r="AV2"/>
+      <c r="AW2"/>
+      <c r="AX2"/>
+      <c r="AY2"/>
+      <c r="AZ2"/>
+      <c r="BA2"/>
+      <c r="BB2"/>
+      <c r="BC2"/>
+      <c r="BD2"/>
+      <c r="BE2"/>
+      <c r="BF2"/>
+      <c r="BG2"/>
+      <c r="BH2"/>
+      <c r="BI2"/>
+      <c r="BJ2"/>
+      <c r="BK2"/>
+      <c r="BL2"/>
+      <c r="BM2"/>
+      <c r="BN2"/>
+      <c r="BO2"/>
+      <c r="BP2"/>
+      <c r="BQ2"/>
+      <c r="BR2"/>
+      <c r="BS2"/>
+      <c r="BT2"/>
+      <c r="BU2"/>
+      <c r="BV2"/>
+      <c r="BW2"/>
+      <c r="BX2"/>
+      <c r="BY2"/>
+      <c r="BZ2"/>
+      <c r="CA2"/>
+      <c r="CB2"/>
+      <c r="CC2"/>
+      <c r="CD2"/>
+      <c r="CE2"/>
+      <c r="CF2"/>
+      <c r="CG2"/>
+      <c r="CH2"/>
+      <c r="CI2"/>
+      <c r="CJ2"/>
+      <c r="CK2"/>
+      <c r="CL2"/>
+      <c r="CM2"/>
+      <c r="CN2"/>
+      <c r="CO2"/>
+      <c r="CP2"/>
+      <c r="CQ2"/>
+      <c r="CR2"/>
+      <c r="CS2"/>
+      <c r="CT2"/>
+      <c r="CU2"/>
+      <c r="CV2"/>
+      <c r="CW2"/>
+      <c r="CX2"/>
+      <c r="CY2"/>
+      <c r="CZ2"/>
+      <c r="DA2"/>
+      <c r="DB2"/>
+      <c r="DC2"/>
+      <c r="DD2"/>
+      <c r="DE2"/>
+      <c r="DF2"/>
+      <c r="DG2"/>
+      <c r="DH2"/>
+      <c r="DI2"/>
+      <c r="DJ2"/>
+      <c r="DK2"/>
+      <c r="DL2"/>
+      <c r="DM2"/>
+      <c r="DN2"/>
+      <c r="DO2"/>
+      <c r="DP2"/>
+      <c r="DQ2"/>
+      <c r="DR2"/>
+      <c r="DS2"/>
+      <c r="DT2"/>
+      <c r="DU2"/>
+      <c r="DV2"/>
+      <c r="DW2"/>
+      <c r="DX2"/>
+      <c r="DY2"/>
+      <c r="DZ2"/>
+      <c r="EA2"/>
+      <c r="EB2"/>
+      <c r="EC2"/>
+      <c r="ED2"/>
+      <c r="EE2"/>
+      <c r="EF2"/>
+      <c r="EG2"/>
+      <c r="EH2"/>
+      <c r="EI2"/>
+      <c r="EJ2"/>
+      <c r="EK2"/>
+      <c r="EL2"/>
+      <c r="EM2"/>
+      <c r="EN2"/>
+      <c r="EO2"/>
+      <c r="EP2"/>
+      <c r="EQ2"/>
+      <c r="ER2"/>
+      <c r="ES2"/>
+      <c r="ET2"/>
+      <c r="EU2"/>
+      <c r="EV2"/>
+      <c r="EW2"/>
+      <c r="EX2"/>
+      <c r="EY2"/>
+      <c r="EZ2"/>
+      <c r="FA2"/>
+      <c r="FB2"/>
+      <c r="FC2"/>
+      <c r="FD2"/>
+      <c r="FE2"/>
+      <c r="FF2"/>
+      <c r="FG2"/>
+      <c r="FH2"/>
+      <c r="FI2"/>
+      <c r="FJ2"/>
+      <c r="FK2"/>
+      <c r="FL2"/>
+      <c r="FM2"/>
+      <c r="FN2"/>
+      <c r="FO2"/>
+      <c r="FP2"/>
+      <c r="FQ2"/>
+      <c r="FR2"/>
+      <c r="FS2"/>
+      <c r="FT2"/>
+      <c r="FU2"/>
+      <c r="FV2"/>
+      <c r="FW2"/>
+      <c r="FX2"/>
+      <c r="FY2"/>
+      <c r="FZ2"/>
+      <c r="GA2"/>
+      <c r="GB2"/>
+      <c r="GC2"/>
+      <c r="GD2"/>
+      <c r="GE2"/>
+      <c r="GF2"/>
+      <c r="GG2"/>
+      <c r="GH2"/>
+      <c r="GI2"/>
+      <c r="GJ2"/>
+      <c r="GK2"/>
+      <c r="GL2"/>
+      <c r="GM2"/>
+      <c r="GN2"/>
+      <c r="GO2"/>
+      <c r="GP2"/>
+      <c r="GQ2"/>
+      <c r="GR2"/>
+      <c r="GS2"/>
+      <c r="GT2"/>
+      <c r="GU2"/>
+      <c r="GV2"/>
+      <c r="GW2"/>
+      <c r="GX2"/>
+      <c r="GY2"/>
+      <c r="GZ2"/>
+      <c r="HA2"/>
+      <c r="HB2"/>
+      <c r="HC2"/>
+      <c r="HD2"/>
+      <c r="HE2"/>
+      <c r="HF2"/>
+      <c r="HG2"/>
+      <c r="HH2"/>
+      <c r="HI2"/>
+      <c r="HJ2"/>
+      <c r="HK2"/>
+      <c r="HL2"/>
+      <c r="HM2"/>
+      <c r="HN2"/>
+      <c r="HO2"/>
+      <c r="HP2"/>
+      <c r="HQ2"/>
+      <c r="HR2"/>
+      <c r="HS2"/>
+      <c r="HT2"/>
+      <c r="HU2"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet32.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1AD86191-7CFE-4ED9-9129-FF78170AB51E}">
+  <dimension ref="A1:HU12"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="50.90625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="52.26953125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="42.453125" customWidth="1"/>
+    <col min="4" max="4" width="33.36328125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="33.08984375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="17.08984375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="40.81640625" customWidth="1"/>
+    <col min="8" max="8" width="65.54296875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:229" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>209</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="2" spans="1:229" s="4" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A2" s="3" t="s">
+        <v>527</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>528</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>529</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>201</v>
+      </c>
+      <c r="F2" s="3" t="s">
+        <v>202</v>
+      </c>
+      <c r="G2" s="3" t="s">
+        <v>211</v>
+      </c>
+      <c r="H2" s="3" t="s">
+        <v>530</v>
+      </c>
+      <c r="I2"/>
+      <c r="J2"/>
+      <c r="K2"/>
+      <c r="L2"/>
+      <c r="M2"/>
+      <c r="N2"/>
+      <c r="O2"/>
+      <c r="P2"/>
+      <c r="Q2"/>
+      <c r="R2"/>
+      <c r="S2"/>
+      <c r="T2"/>
+      <c r="U2"/>
+      <c r="V2"/>
+      <c r="W2"/>
+      <c r="X2"/>
+      <c r="Y2"/>
+      <c r="Z2"/>
+      <c r="AA2"/>
+      <c r="AB2"/>
+      <c r="AC2"/>
+      <c r="AD2"/>
+      <c r="AE2"/>
+      <c r="AF2"/>
+      <c r="AG2"/>
+      <c r="AH2"/>
+      <c r="AI2"/>
+      <c r="AJ2"/>
+      <c r="AK2"/>
+      <c r="AL2"/>
+      <c r="AM2"/>
+      <c r="AN2"/>
+      <c r="AO2"/>
+      <c r="AP2"/>
+      <c r="AQ2"/>
+      <c r="AR2"/>
+      <c r="AS2"/>
+      <c r="AT2"/>
+      <c r="AU2"/>
+      <c r="AV2"/>
+      <c r="AW2"/>
+      <c r="AX2"/>
+      <c r="AY2"/>
+      <c r="AZ2"/>
+      <c r="BA2"/>
+      <c r="BB2"/>
+      <c r="BC2"/>
+      <c r="BD2"/>
+      <c r="BE2"/>
+      <c r="BF2"/>
+      <c r="BG2"/>
+      <c r="BH2"/>
+      <c r="BI2"/>
+      <c r="BJ2"/>
+      <c r="BK2"/>
+      <c r="BL2"/>
+      <c r="BM2"/>
+      <c r="BN2"/>
+      <c r="BO2"/>
+      <c r="BP2"/>
+      <c r="BQ2"/>
+      <c r="BR2"/>
+      <c r="BS2"/>
+      <c r="BT2"/>
+      <c r="BU2"/>
+      <c r="BV2"/>
+      <c r="BW2"/>
+      <c r="BX2"/>
+      <c r="BY2"/>
+      <c r="BZ2"/>
+      <c r="CA2"/>
+      <c r="CB2"/>
+      <c r="CC2"/>
+      <c r="CD2"/>
+      <c r="CE2"/>
+      <c r="CF2"/>
+      <c r="CG2"/>
+      <c r="CH2"/>
+      <c r="CI2"/>
+      <c r="CJ2"/>
+      <c r="CK2"/>
+      <c r="CL2"/>
+      <c r="CM2"/>
+      <c r="CN2"/>
+      <c r="CO2"/>
+      <c r="CP2"/>
+      <c r="CQ2"/>
+      <c r="CR2"/>
+      <c r="CS2"/>
+      <c r="CT2"/>
+      <c r="CU2"/>
+      <c r="CV2"/>
+      <c r="CW2"/>
+      <c r="CX2"/>
+      <c r="CY2"/>
+      <c r="CZ2"/>
+      <c r="DA2"/>
+      <c r="DB2"/>
+      <c r="DC2"/>
+      <c r="DD2"/>
+      <c r="DE2"/>
+      <c r="DF2"/>
+      <c r="DG2"/>
+      <c r="DH2"/>
+      <c r="DI2"/>
+      <c r="DJ2"/>
+      <c r="DK2"/>
+      <c r="DL2"/>
+      <c r="DM2"/>
+      <c r="DN2"/>
+      <c r="DO2"/>
+      <c r="DP2"/>
+      <c r="DQ2"/>
+      <c r="DR2"/>
+      <c r="DS2"/>
+      <c r="DT2"/>
+      <c r="DU2"/>
+      <c r="DV2"/>
+      <c r="DW2"/>
+      <c r="DX2"/>
+      <c r="DY2"/>
+      <c r="DZ2"/>
+      <c r="EA2"/>
+      <c r="EB2"/>
+      <c r="EC2"/>
+      <c r="ED2"/>
+      <c r="EE2"/>
+      <c r="EF2"/>
+      <c r="EG2"/>
+      <c r="EH2"/>
+      <c r="EI2"/>
+      <c r="EJ2"/>
+      <c r="EK2"/>
+      <c r="EL2"/>
+      <c r="EM2"/>
+      <c r="EN2"/>
+      <c r="EO2"/>
+      <c r="EP2"/>
+      <c r="EQ2"/>
+      <c r="ER2"/>
+      <c r="ES2"/>
+      <c r="ET2"/>
+      <c r="EU2"/>
+      <c r="EV2"/>
+      <c r="EW2"/>
+      <c r="EX2"/>
+      <c r="EY2"/>
+      <c r="EZ2"/>
+      <c r="FA2"/>
+      <c r="FB2"/>
+      <c r="FC2"/>
+      <c r="FD2"/>
+      <c r="FE2"/>
+      <c r="FF2"/>
+      <c r="FG2"/>
+      <c r="FH2"/>
+      <c r="FI2"/>
+      <c r="FJ2"/>
+      <c r="FK2"/>
+      <c r="FL2"/>
+      <c r="FM2"/>
+      <c r="FN2"/>
+      <c r="FO2"/>
+      <c r="FP2"/>
+      <c r="FQ2"/>
+      <c r="FR2"/>
+      <c r="FS2"/>
+      <c r="FT2"/>
+      <c r="FU2"/>
+      <c r="FV2"/>
+      <c r="FW2"/>
+      <c r="FX2"/>
+      <c r="FY2"/>
+      <c r="FZ2"/>
+      <c r="GA2"/>
+      <c r="GB2"/>
+      <c r="GC2"/>
+      <c r="GD2"/>
+      <c r="GE2"/>
+      <c r="GF2"/>
+      <c r="GG2"/>
+      <c r="GH2"/>
+      <c r="GI2"/>
+      <c r="GJ2"/>
+      <c r="GK2"/>
+      <c r="GL2"/>
+      <c r="GM2"/>
+      <c r="GN2"/>
+      <c r="GO2"/>
+      <c r="GP2"/>
+      <c r="GQ2"/>
+      <c r="GR2"/>
+      <c r="GS2"/>
+      <c r="GT2"/>
+      <c r="GU2"/>
+      <c r="GV2"/>
+      <c r="GW2"/>
+      <c r="GX2"/>
+      <c r="GY2"/>
+      <c r="GZ2"/>
+      <c r="HA2"/>
+      <c r="HB2"/>
+      <c r="HC2"/>
+      <c r="HD2"/>
+      <c r="HE2"/>
+      <c r="HF2"/>
+      <c r="HG2"/>
+      <c r="HH2"/>
+      <c r="HI2"/>
+      <c r="HJ2"/>
+      <c r="HK2"/>
+      <c r="HL2"/>
+      <c r="HM2"/>
+      <c r="HN2"/>
+      <c r="HO2"/>
+      <c r="HP2"/>
+      <c r="HQ2"/>
+      <c r="HR2"/>
+      <c r="HS2"/>
+      <c r="HT2"/>
+      <c r="HU2"/>
+    </row>
+    <row r="3" spans="1:229" x14ac:dyDescent="0.35">
+      <c r="A3" s="3" t="s">
         <v>532</v>
       </c>
       <c r="B3" s="3" t="s">
@@ -20370,6 +20622,694 @@
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet33.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{24EB34D0-BCF8-4F57-88CC-AC842687528F}">
+  <dimension ref="A1:HU5"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="52.453125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="52.26953125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="42.453125" customWidth="1"/>
+    <col min="4" max="4" width="33.36328125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="33.08984375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="17.08984375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="40.81640625" customWidth="1"/>
+    <col min="8" max="8" width="65.54296875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:229" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>209</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="2" spans="1:229" s="4" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A2" s="3" t="s">
+        <v>576</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>577</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>578</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>201</v>
+      </c>
+      <c r="F2" s="3" t="s">
+        <v>202</v>
+      </c>
+      <c r="G2" s="3" t="s">
+        <v>211</v>
+      </c>
+      <c r="H2" s="3" t="s">
+        <v>579</v>
+      </c>
+      <c r="I2"/>
+      <c r="J2"/>
+      <c r="K2"/>
+      <c r="L2"/>
+      <c r="M2"/>
+      <c r="N2"/>
+      <c r="O2"/>
+      <c r="P2"/>
+      <c r="Q2"/>
+      <c r="R2"/>
+      <c r="S2"/>
+      <c r="T2"/>
+      <c r="U2"/>
+      <c r="V2"/>
+      <c r="W2"/>
+      <c r="X2"/>
+      <c r="Y2"/>
+      <c r="Z2"/>
+      <c r="AA2"/>
+      <c r="AB2"/>
+      <c r="AC2"/>
+      <c r="AD2"/>
+      <c r="AE2"/>
+      <c r="AF2"/>
+      <c r="AG2"/>
+      <c r="AH2"/>
+      <c r="AI2"/>
+      <c r="AJ2"/>
+      <c r="AK2"/>
+      <c r="AL2"/>
+      <c r="AM2"/>
+      <c r="AN2"/>
+      <c r="AO2"/>
+      <c r="AP2"/>
+      <c r="AQ2"/>
+      <c r="AR2"/>
+      <c r="AS2"/>
+      <c r="AT2"/>
+      <c r="AU2"/>
+      <c r="AV2"/>
+      <c r="AW2"/>
+      <c r="AX2"/>
+      <c r="AY2"/>
+      <c r="AZ2"/>
+      <c r="BA2"/>
+      <c r="BB2"/>
+      <c r="BC2"/>
+      <c r="BD2"/>
+      <c r="BE2"/>
+      <c r="BF2"/>
+      <c r="BG2"/>
+      <c r="BH2"/>
+      <c r="BI2"/>
+      <c r="BJ2"/>
+      <c r="BK2"/>
+      <c r="BL2"/>
+      <c r="BM2"/>
+      <c r="BN2"/>
+      <c r="BO2"/>
+      <c r="BP2"/>
+      <c r="BQ2"/>
+      <c r="BR2"/>
+      <c r="BS2"/>
+      <c r="BT2"/>
+      <c r="BU2"/>
+      <c r="BV2"/>
+      <c r="BW2"/>
+      <c r="BX2"/>
+      <c r="BY2"/>
+      <c r="BZ2"/>
+      <c r="CA2"/>
+      <c r="CB2"/>
+      <c r="CC2"/>
+      <c r="CD2"/>
+      <c r="CE2"/>
+      <c r="CF2"/>
+      <c r="CG2"/>
+      <c r="CH2"/>
+      <c r="CI2"/>
+      <c r="CJ2"/>
+      <c r="CK2"/>
+      <c r="CL2"/>
+      <c r="CM2"/>
+      <c r="CN2"/>
+      <c r="CO2"/>
+      <c r="CP2"/>
+      <c r="CQ2"/>
+      <c r="CR2"/>
+      <c r="CS2"/>
+      <c r="CT2"/>
+      <c r="CU2"/>
+      <c r="CV2"/>
+      <c r="CW2"/>
+      <c r="CX2"/>
+      <c r="CY2"/>
+      <c r="CZ2"/>
+      <c r="DA2"/>
+      <c r="DB2"/>
+      <c r="DC2"/>
+      <c r="DD2"/>
+      <c r="DE2"/>
+      <c r="DF2"/>
+      <c r="DG2"/>
+      <c r="DH2"/>
+      <c r="DI2"/>
+      <c r="DJ2"/>
+      <c r="DK2"/>
+      <c r="DL2"/>
+      <c r="DM2"/>
+      <c r="DN2"/>
+      <c r="DO2"/>
+      <c r="DP2"/>
+      <c r="DQ2"/>
+      <c r="DR2"/>
+      <c r="DS2"/>
+      <c r="DT2"/>
+      <c r="DU2"/>
+      <c r="DV2"/>
+      <c r="DW2"/>
+      <c r="DX2"/>
+      <c r="DY2"/>
+      <c r="DZ2"/>
+      <c r="EA2"/>
+      <c r="EB2"/>
+      <c r="EC2"/>
+      <c r="ED2"/>
+      <c r="EE2"/>
+      <c r="EF2"/>
+      <c r="EG2"/>
+      <c r="EH2"/>
+      <c r="EI2"/>
+      <c r="EJ2"/>
+      <c r="EK2"/>
+      <c r="EL2"/>
+      <c r="EM2"/>
+      <c r="EN2"/>
+      <c r="EO2"/>
+      <c r="EP2"/>
+      <c r="EQ2"/>
+      <c r="ER2"/>
+      <c r="ES2"/>
+      <c r="ET2"/>
+      <c r="EU2"/>
+      <c r="EV2"/>
+      <c r="EW2"/>
+      <c r="EX2"/>
+      <c r="EY2"/>
+      <c r="EZ2"/>
+      <c r="FA2"/>
+      <c r="FB2"/>
+      <c r="FC2"/>
+      <c r="FD2"/>
+      <c r="FE2"/>
+      <c r="FF2"/>
+      <c r="FG2"/>
+      <c r="FH2"/>
+      <c r="FI2"/>
+      <c r="FJ2"/>
+      <c r="FK2"/>
+      <c r="FL2"/>
+      <c r="FM2"/>
+      <c r="FN2"/>
+      <c r="FO2"/>
+      <c r="FP2"/>
+      <c r="FQ2"/>
+      <c r="FR2"/>
+      <c r="FS2"/>
+      <c r="FT2"/>
+      <c r="FU2"/>
+      <c r="FV2"/>
+      <c r="FW2"/>
+      <c r="FX2"/>
+      <c r="FY2"/>
+      <c r="FZ2"/>
+      <c r="GA2"/>
+      <c r="GB2"/>
+      <c r="GC2"/>
+      <c r="GD2"/>
+      <c r="GE2"/>
+      <c r="GF2"/>
+      <c r="GG2"/>
+      <c r="GH2"/>
+      <c r="GI2"/>
+      <c r="GJ2"/>
+      <c r="GK2"/>
+      <c r="GL2"/>
+      <c r="GM2"/>
+      <c r="GN2"/>
+      <c r="GO2"/>
+      <c r="GP2"/>
+      <c r="GQ2"/>
+      <c r="GR2"/>
+      <c r="GS2"/>
+      <c r="GT2"/>
+      <c r="GU2"/>
+      <c r="GV2"/>
+      <c r="GW2"/>
+      <c r="GX2"/>
+      <c r="GY2"/>
+      <c r="GZ2"/>
+      <c r="HA2"/>
+      <c r="HB2"/>
+      <c r="HC2"/>
+      <c r="HD2"/>
+      <c r="HE2"/>
+      <c r="HF2"/>
+      <c r="HG2"/>
+      <c r="HH2"/>
+      <c r="HI2"/>
+      <c r="HJ2"/>
+      <c r="HK2"/>
+      <c r="HL2"/>
+      <c r="HM2"/>
+      <c r="HN2"/>
+      <c r="HO2"/>
+      <c r="HP2"/>
+      <c r="HQ2"/>
+      <c r="HR2"/>
+      <c r="HS2"/>
+      <c r="HT2"/>
+      <c r="HU2"/>
+    </row>
+    <row r="3" spans="1:229" x14ac:dyDescent="0.35">
+      <c r="A3" s="3" t="s">
+        <v>580</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>581</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>582</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>201</v>
+      </c>
+      <c r="F3" s="3" t="s">
+        <v>202</v>
+      </c>
+      <c r="G3" s="3" t="s">
+        <v>211</v>
+      </c>
+      <c r="H3" s="3" t="s">
+        <v>583</v>
+      </c>
+    </row>
+    <row r="4" spans="1:229" x14ac:dyDescent="0.35">
+      <c r="A4" s="11" t="s">
+        <v>584</v>
+      </c>
+      <c r="B4" s="11" t="s">
+        <v>585</v>
+      </c>
+      <c r="C4" s="11" t="s">
+        <v>586</v>
+      </c>
+      <c r="D4" s="11" t="s">
+        <v>0</v>
+      </c>
+      <c r="E4" s="11" t="s">
+        <v>201</v>
+      </c>
+      <c r="F4" s="11" t="s">
+        <v>202</v>
+      </c>
+      <c r="G4" s="11" t="s">
+        <v>211</v>
+      </c>
+      <c r="H4" s="11"/>
+    </row>
+    <row r="5" spans="1:229" x14ac:dyDescent="0.35">
+      <c r="A5" s="3" t="s">
+        <v>587</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>588</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>589</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>201</v>
+      </c>
+      <c r="F5" s="3" t="s">
+        <v>202</v>
+      </c>
+      <c r="G5" s="3" t="s">
+        <v>211</v>
+      </c>
+      <c r="H5" s="3" t="s">
+        <v>590</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet34.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7271F742-0542-4B33-AEE2-20AE8A69F475}">
+  <dimension ref="A1:HU3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="52.453125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="52.26953125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="42.453125" customWidth="1"/>
+    <col min="4" max="4" width="33.36328125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="33.08984375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="17.08984375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="40.81640625" customWidth="1"/>
+    <col min="8" max="8" width="65.54296875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:229" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>209</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="2" spans="1:229" s="4" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A2" s="3" t="s">
+        <v>594</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>595</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>596</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>201</v>
+      </c>
+      <c r="F2" s="3" t="s">
+        <v>202</v>
+      </c>
+      <c r="G2" s="3" t="s">
+        <v>211</v>
+      </c>
+      <c r="H2" s="3" t="s">
+        <v>597</v>
+      </c>
+      <c r="I2"/>
+      <c r="J2"/>
+      <c r="K2"/>
+      <c r="L2"/>
+      <c r="M2"/>
+      <c r="N2"/>
+      <c r="O2"/>
+      <c r="P2"/>
+      <c r="Q2"/>
+      <c r="R2"/>
+      <c r="S2"/>
+      <c r="T2"/>
+      <c r="U2"/>
+      <c r="V2"/>
+      <c r="W2"/>
+      <c r="X2"/>
+      <c r="Y2"/>
+      <c r="Z2"/>
+      <c r="AA2"/>
+      <c r="AB2"/>
+      <c r="AC2"/>
+      <c r="AD2"/>
+      <c r="AE2"/>
+      <c r="AF2"/>
+      <c r="AG2"/>
+      <c r="AH2"/>
+      <c r="AI2"/>
+      <c r="AJ2"/>
+      <c r="AK2"/>
+      <c r="AL2"/>
+      <c r="AM2"/>
+      <c r="AN2"/>
+      <c r="AO2"/>
+      <c r="AP2"/>
+      <c r="AQ2"/>
+      <c r="AR2"/>
+      <c r="AS2"/>
+      <c r="AT2"/>
+      <c r="AU2"/>
+      <c r="AV2"/>
+      <c r="AW2"/>
+      <c r="AX2"/>
+      <c r="AY2"/>
+      <c r="AZ2"/>
+      <c r="BA2"/>
+      <c r="BB2"/>
+      <c r="BC2"/>
+      <c r="BD2"/>
+      <c r="BE2"/>
+      <c r="BF2"/>
+      <c r="BG2"/>
+      <c r="BH2"/>
+      <c r="BI2"/>
+      <c r="BJ2"/>
+      <c r="BK2"/>
+      <c r="BL2"/>
+      <c r="BM2"/>
+      <c r="BN2"/>
+      <c r="BO2"/>
+      <c r="BP2"/>
+      <c r="BQ2"/>
+      <c r="BR2"/>
+      <c r="BS2"/>
+      <c r="BT2"/>
+      <c r="BU2"/>
+      <c r="BV2"/>
+      <c r="BW2"/>
+      <c r="BX2"/>
+      <c r="BY2"/>
+      <c r="BZ2"/>
+      <c r="CA2"/>
+      <c r="CB2"/>
+      <c r="CC2"/>
+      <c r="CD2"/>
+      <c r="CE2"/>
+      <c r="CF2"/>
+      <c r="CG2"/>
+      <c r="CH2"/>
+      <c r="CI2"/>
+      <c r="CJ2"/>
+      <c r="CK2"/>
+      <c r="CL2"/>
+      <c r="CM2"/>
+      <c r="CN2"/>
+      <c r="CO2"/>
+      <c r="CP2"/>
+      <c r="CQ2"/>
+      <c r="CR2"/>
+      <c r="CS2"/>
+      <c r="CT2"/>
+      <c r="CU2"/>
+      <c r="CV2"/>
+      <c r="CW2"/>
+      <c r="CX2"/>
+      <c r="CY2"/>
+      <c r="CZ2"/>
+      <c r="DA2"/>
+      <c r="DB2"/>
+      <c r="DC2"/>
+      <c r="DD2"/>
+      <c r="DE2"/>
+      <c r="DF2"/>
+      <c r="DG2"/>
+      <c r="DH2"/>
+      <c r="DI2"/>
+      <c r="DJ2"/>
+      <c r="DK2"/>
+      <c r="DL2"/>
+      <c r="DM2"/>
+      <c r="DN2"/>
+      <c r="DO2"/>
+      <c r="DP2"/>
+      <c r="DQ2"/>
+      <c r="DR2"/>
+      <c r="DS2"/>
+      <c r="DT2"/>
+      <c r="DU2"/>
+      <c r="DV2"/>
+      <c r="DW2"/>
+      <c r="DX2"/>
+      <c r="DY2"/>
+      <c r="DZ2"/>
+      <c r="EA2"/>
+      <c r="EB2"/>
+      <c r="EC2"/>
+      <c r="ED2"/>
+      <c r="EE2"/>
+      <c r="EF2"/>
+      <c r="EG2"/>
+      <c r="EH2"/>
+      <c r="EI2"/>
+      <c r="EJ2"/>
+      <c r="EK2"/>
+      <c r="EL2"/>
+      <c r="EM2"/>
+      <c r="EN2"/>
+      <c r="EO2"/>
+      <c r="EP2"/>
+      <c r="EQ2"/>
+      <c r="ER2"/>
+      <c r="ES2"/>
+      <c r="ET2"/>
+      <c r="EU2"/>
+      <c r="EV2"/>
+      <c r="EW2"/>
+      <c r="EX2"/>
+      <c r="EY2"/>
+      <c r="EZ2"/>
+      <c r="FA2"/>
+      <c r="FB2"/>
+      <c r="FC2"/>
+      <c r="FD2"/>
+      <c r="FE2"/>
+      <c r="FF2"/>
+      <c r="FG2"/>
+      <c r="FH2"/>
+      <c r="FI2"/>
+      <c r="FJ2"/>
+      <c r="FK2"/>
+      <c r="FL2"/>
+      <c r="FM2"/>
+      <c r="FN2"/>
+      <c r="FO2"/>
+      <c r="FP2"/>
+      <c r="FQ2"/>
+      <c r="FR2"/>
+      <c r="FS2"/>
+      <c r="FT2"/>
+      <c r="FU2"/>
+      <c r="FV2"/>
+      <c r="FW2"/>
+      <c r="FX2"/>
+      <c r="FY2"/>
+      <c r="FZ2"/>
+      <c r="GA2"/>
+      <c r="GB2"/>
+      <c r="GC2"/>
+      <c r="GD2"/>
+      <c r="GE2"/>
+      <c r="GF2"/>
+      <c r="GG2"/>
+      <c r="GH2"/>
+      <c r="GI2"/>
+      <c r="GJ2"/>
+      <c r="GK2"/>
+      <c r="GL2"/>
+      <c r="GM2"/>
+      <c r="GN2"/>
+      <c r="GO2"/>
+      <c r="GP2"/>
+      <c r="GQ2"/>
+      <c r="GR2"/>
+      <c r="GS2"/>
+      <c r="GT2"/>
+      <c r="GU2"/>
+      <c r="GV2"/>
+      <c r="GW2"/>
+      <c r="GX2"/>
+      <c r="GY2"/>
+      <c r="GZ2"/>
+      <c r="HA2"/>
+      <c r="HB2"/>
+      <c r="HC2"/>
+      <c r="HD2"/>
+      <c r="HE2"/>
+      <c r="HF2"/>
+      <c r="HG2"/>
+      <c r="HH2"/>
+      <c r="HI2"/>
+      <c r="HJ2"/>
+      <c r="HK2"/>
+      <c r="HL2"/>
+      <c r="HM2"/>
+      <c r="HN2"/>
+      <c r="HO2"/>
+      <c r="HP2"/>
+      <c r="HQ2"/>
+      <c r="HR2"/>
+      <c r="HS2"/>
+      <c r="HT2"/>
+      <c r="HU2"/>
+    </row>
+    <row r="3" spans="1:229" x14ac:dyDescent="0.35">
+      <c r="A3" s="3" t="s">
+        <v>598</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>599</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>600</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>201</v>
+      </c>
+      <c r="F3" s="3" t="s">
+        <v>202</v>
+      </c>
+      <c r="G3" s="3" t="s">
+        <v>211</v>
+      </c>
+      <c r="H3" s="3" t="s">
+        <v>601</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Added test cases for - Subcategory for page: Further education workforce #133
</commit_message>
<xml_diff>
--- a/testdata.xlsx
+++ b/testdata.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sshiwani\workspace\find-information-products-services-tests\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{03279657-AE4E-4469-BDE8-A24A591A0385}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6DC67814-7EC6-4595-B980-9CA1061BB621}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="22780" windowHeight="14540" firstSheet="32" activeTab="33" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="22780" windowHeight="14540" firstSheet="18" activeTab="19" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="category_phase" sheetId="1" r:id="rId1"/>
@@ -32,21 +32,23 @@
     <sheet name="UG_EPEYAcademyTruWorkforce_list" sheetId="30" r:id="rId17"/>
     <sheet name="UG_EPEYAltProvSetWorkforce_list" sheetId="32" r:id="rId18"/>
     <sheet name="UG_EPEYEarlyYearsWorkforce_list" sheetId="35" r:id="rId19"/>
-    <sheet name="UGSubcategory_AdultLearner" sheetId="16" r:id="rId20"/>
-    <sheet name="UGSubcategory_CareersAdviser" sheetId="17" r:id="rId21"/>
-    <sheet name="UGSubcategory_ChildOrYoungPers" sheetId="18" r:id="rId22"/>
-    <sheet name="UGSubcategory_DfEWorkforce" sheetId="19" r:id="rId23"/>
-    <sheet name="UGSubcategory_Employer" sheetId="20" r:id="rId24"/>
-    <sheet name="UGSubcategory_LAWorkforce" sheetId="21" r:id="rId25"/>
-    <sheet name="UGSubcategory_NEETOrCareerSeek" sheetId="22" r:id="rId26"/>
-    <sheet name="UGSubcategory_ParentOrCarer" sheetId="23" r:id="rId27"/>
-    <sheet name="UGSubcateg_ProfExtUserofDfEData" sheetId="24" r:id="rId28"/>
-    <sheet name="UGSubcategory_SCWorkforce" sheetId="25" r:id="rId29"/>
-    <sheet name="UGSubcategory_SocialWorker" sheetId="27" r:id="rId30"/>
-    <sheet name="UGSubcategory_EPandEYWorkforce" sheetId="29" r:id="rId31"/>
-    <sheet name="EPEYSubcateg_AcademyTWorkforce" sheetId="31" r:id="rId32"/>
-    <sheet name="EPEYSubcateg_AltProSetWorkforce" sheetId="33" r:id="rId33"/>
-    <sheet name="EPEYSubcateg_EarlyYearsWorkforc" sheetId="34" r:id="rId34"/>
+    <sheet name="UG_EPEYFurtherEduWorkforce_list" sheetId="37" r:id="rId20"/>
+    <sheet name="UGSubcategory_AdultLearner" sheetId="16" r:id="rId21"/>
+    <sheet name="UGSubcategory_CareersAdviser" sheetId="17" r:id="rId22"/>
+    <sheet name="UGSubcategory_ChildOrYoungPers" sheetId="18" r:id="rId23"/>
+    <sheet name="UGSubcategory_DfEWorkforce" sheetId="19" r:id="rId24"/>
+    <sheet name="UGSubcategory_Employer" sheetId="20" r:id="rId25"/>
+    <sheet name="UGSubcategory_LAWorkforce" sheetId="21" r:id="rId26"/>
+    <sheet name="UGSubcategory_NEETOrCareerSeek" sheetId="22" r:id="rId27"/>
+    <sheet name="UGSubcategory_ParentOrCarer" sheetId="23" r:id="rId28"/>
+    <sheet name="UGSubcateg_ProfExtUserofDfEData" sheetId="24" r:id="rId29"/>
+    <sheet name="UGSubcategory_SCWorkforce" sheetId="25" r:id="rId30"/>
+    <sheet name="UGSubcategory_SocialWorker" sheetId="27" r:id="rId31"/>
+    <sheet name="UGSubcategory_EPandEYWorkforce" sheetId="29" r:id="rId32"/>
+    <sheet name="EPEYSubcateg_AcademyTWorkforce" sheetId="31" r:id="rId33"/>
+    <sheet name="EPEYSubcateg_AltProSetWorkforce" sheetId="33" r:id="rId34"/>
+    <sheet name="EPEYSubcatg_EarlyYearsWorkforce" sheetId="34" r:id="rId35"/>
+    <sheet name="EPEYSubcatg_FurtherEduWorkforce" sheetId="36" r:id="rId36"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -58,7 +60,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1255" uniqueCount="602">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1308" uniqueCount="622">
   <si>
     <t>Search and filter products and services</t>
   </si>
@@ -1864,6 +1866,66 @@
   </si>
   <si>
     <t>Early years teacher  (Early years workforce)</t>
+  </si>
+  <si>
+    <t>categories/user-group/education-provider-and-early-years-workforce/further-education-workforce</t>
+  </si>
+  <si>
+    <t>Browse products in Further education workforce</t>
+  </si>
+  <si>
+    <t>College leader</t>
+  </si>
+  <si>
+    <t>College support staff</t>
+  </si>
+  <si>
+    <t>Lecturer (further education)</t>
+  </si>
+  <si>
+    <t>products?userGroup=further-education-workforce</t>
+  </si>
+  <si>
+    <t>ul.moj-filter-tags li a:has-text(' further-education-workforce')</t>
+  </si>
+  <si>
+    <t>Remove this filter further-education-workforce</t>
+  </si>
+  <si>
+    <t>products?userGroup=college-leader</t>
+  </si>
+  <si>
+    <t>ul.moj-filter-tags li a:has-text(' College leader  (Further education workforce)')</t>
+  </si>
+  <si>
+    <t>Remove this filter College leader  (Further education workforce)</t>
+  </si>
+  <si>
+    <t>College leader  (Further education workforce)</t>
+  </si>
+  <si>
+    <t>products?userGroup=college-support-staff</t>
+  </si>
+  <si>
+    <t>ul.moj-filter-tags li a:has-text(' College support staff  (Further education workforce)')</t>
+  </si>
+  <si>
+    <t>Remove this filter College support staff  (Further education workforce)</t>
+  </si>
+  <si>
+    <t>College support staff  (Further education workforce)</t>
+  </si>
+  <si>
+    <t>products?userGroup=lecturer-further-education</t>
+  </si>
+  <si>
+    <t>ul.moj-filter-tags li a:has-text(' Lecturer (further education) ')</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Remove this filter Lecturer (further education) </t>
+  </si>
+  <si>
+    <t>Lecturer (further education)  (Further education workforce)</t>
   </si>
 </sst>
 </file>
@@ -12818,6 +12880,87 @@
 </file>
 
 <file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{85EB819D-F775-4E64-97E5-4F6BB5F27AC7}">
+  <dimension ref="A1:C8"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="54.1796875" customWidth="1"/>
+    <col min="2" max="2" width="47.453125" customWidth="1"/>
+    <col min="3" max="3" width="50.36328125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A1" s="6" t="s">
+        <v>102</v>
+      </c>
+      <c r="B1" s="6" t="s">
+        <v>103</v>
+      </c>
+      <c r="C1" s="6" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A2" s="3" t="s">
+        <v>602</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>107</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>603</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="B3" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="B4" s="3" t="s">
+        <v>113</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A5" s="3" t="s">
+        <v>144</v>
+      </c>
+      <c r="B5" s="3"/>
+      <c r="C5" s="3"/>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A6" s="3" t="s">
+        <v>604</v>
+      </c>
+      <c r="B6" s="3"/>
+      <c r="C6" s="3"/>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A7" s="3" t="s">
+        <v>605</v>
+      </c>
+      <c r="B7" s="3"/>
+      <c r="C7" s="3"/>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A8" s="3" t="s">
+        <v>606</v>
+      </c>
+      <c r="B8" s="3"/>
+      <c r="C8" s="3"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FB5527F7-85DB-4F8E-B4B3-EC8453E599E1}">
   <dimension ref="A1:HU6"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -13215,7 +13358,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A99CF6C3-F305-48A2-AB80-2C2D7CE6460C}">
   <dimension ref="A1:HU5"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -13586,7 +13729,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5EFF0597-7FD1-4E6A-AA71-DB9F9FAB97A9}">
   <dimension ref="A1:HU7"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -14010,7 +14153,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9F4A57AC-4620-4875-88AE-9F5C739A9042}">
   <dimension ref="A1:HU6"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -14407,7 +14550,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6C1C130F-0899-4810-82F6-950C9CB07234}">
   <dimension ref="A1:HU5"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -14778,7 +14921,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4AB9395B-D522-49AD-B790-5334356249F6}">
   <dimension ref="A1:HU7"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -15201,7 +15344,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BEE91763-AD0C-4544-A433-3B50C88AEB79}">
   <dimension ref="A1:HU7"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -15624,7 +15767,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{20DD36AA-F163-4AAB-BD30-4AE6290CCAE7}">
   <dimension ref="A1:HU10"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -16126,7 +16269,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet29.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C6EE6111-FDB3-4B43-8820-BBF68AAFCD6D}">
   <dimension ref="A1:HU8"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -16568,482 +16711,6 @@
       </c>
       <c r="H8" s="9" t="s">
         <v>416</v>
-      </c>
-    </row>
-  </sheetData>
-  <phoneticPr fontId="1" type="noConversion"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet29.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E6428663-7558-48F1-8CD3-947F03FFD4CC}">
-  <dimension ref="A1:HU9"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
-  <cols>
-    <col min="1" max="1" width="50.90625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="52.26953125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="42.453125" customWidth="1"/>
-    <col min="4" max="4" width="33.36328125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="33.08984375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="17.08984375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="40.81640625" customWidth="1"/>
-    <col min="8" max="8" width="57.08984375" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:229" x14ac:dyDescent="0.35">
-      <c r="A1" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="F1" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="G1" s="2" t="s">
-        <v>209</v>
-      </c>
-      <c r="H1" s="2" t="s">
-        <v>210</v>
-      </c>
-    </row>
-    <row r="2" spans="1:229" s="4" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="3" t="s">
-        <v>457</v>
-      </c>
-      <c r="B2" s="3" t="s">
-        <v>458</v>
-      </c>
-      <c r="C2" s="3" t="s">
-        <v>459</v>
-      </c>
-      <c r="D2" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="E2" s="3" t="s">
-        <v>201</v>
-      </c>
-      <c r="F2" s="3" t="s">
-        <v>202</v>
-      </c>
-      <c r="G2" s="3" t="s">
-        <v>211</v>
-      </c>
-      <c r="H2" s="3" t="s">
-        <v>192</v>
-      </c>
-      <c r="I2"/>
-      <c r="J2"/>
-      <c r="K2"/>
-      <c r="L2"/>
-      <c r="M2"/>
-      <c r="N2"/>
-      <c r="O2"/>
-      <c r="P2"/>
-      <c r="Q2"/>
-      <c r="R2"/>
-      <c r="S2"/>
-      <c r="T2"/>
-      <c r="U2"/>
-      <c r="V2"/>
-      <c r="W2"/>
-      <c r="X2"/>
-      <c r="Y2"/>
-      <c r="Z2"/>
-      <c r="AA2"/>
-      <c r="AB2"/>
-      <c r="AC2"/>
-      <c r="AD2"/>
-      <c r="AE2"/>
-      <c r="AF2"/>
-      <c r="AG2"/>
-      <c r="AH2"/>
-      <c r="AI2"/>
-      <c r="AJ2"/>
-      <c r="AK2"/>
-      <c r="AL2"/>
-      <c r="AM2"/>
-      <c r="AN2"/>
-      <c r="AO2"/>
-      <c r="AP2"/>
-      <c r="AQ2"/>
-      <c r="AR2"/>
-      <c r="AS2"/>
-      <c r="AT2"/>
-      <c r="AU2"/>
-      <c r="AV2"/>
-      <c r="AW2"/>
-      <c r="AX2"/>
-      <c r="AY2"/>
-      <c r="AZ2"/>
-      <c r="BA2"/>
-      <c r="BB2"/>
-      <c r="BC2"/>
-      <c r="BD2"/>
-      <c r="BE2"/>
-      <c r="BF2"/>
-      <c r="BG2"/>
-      <c r="BH2"/>
-      <c r="BI2"/>
-      <c r="BJ2"/>
-      <c r="BK2"/>
-      <c r="BL2"/>
-      <c r="BM2"/>
-      <c r="BN2"/>
-      <c r="BO2"/>
-      <c r="BP2"/>
-      <c r="BQ2"/>
-      <c r="BR2"/>
-      <c r="BS2"/>
-      <c r="BT2"/>
-      <c r="BU2"/>
-      <c r="BV2"/>
-      <c r="BW2"/>
-      <c r="BX2"/>
-      <c r="BY2"/>
-      <c r="BZ2"/>
-      <c r="CA2"/>
-      <c r="CB2"/>
-      <c r="CC2"/>
-      <c r="CD2"/>
-      <c r="CE2"/>
-      <c r="CF2"/>
-      <c r="CG2"/>
-      <c r="CH2"/>
-      <c r="CI2"/>
-      <c r="CJ2"/>
-      <c r="CK2"/>
-      <c r="CL2"/>
-      <c r="CM2"/>
-      <c r="CN2"/>
-      <c r="CO2"/>
-      <c r="CP2"/>
-      <c r="CQ2"/>
-      <c r="CR2"/>
-      <c r="CS2"/>
-      <c r="CT2"/>
-      <c r="CU2"/>
-      <c r="CV2"/>
-      <c r="CW2"/>
-      <c r="CX2"/>
-      <c r="CY2"/>
-      <c r="CZ2"/>
-      <c r="DA2"/>
-      <c r="DB2"/>
-      <c r="DC2"/>
-      <c r="DD2"/>
-      <c r="DE2"/>
-      <c r="DF2"/>
-      <c r="DG2"/>
-      <c r="DH2"/>
-      <c r="DI2"/>
-      <c r="DJ2"/>
-      <c r="DK2"/>
-      <c r="DL2"/>
-      <c r="DM2"/>
-      <c r="DN2"/>
-      <c r="DO2"/>
-      <c r="DP2"/>
-      <c r="DQ2"/>
-      <c r="DR2"/>
-      <c r="DS2"/>
-      <c r="DT2"/>
-      <c r="DU2"/>
-      <c r="DV2"/>
-      <c r="DW2"/>
-      <c r="DX2"/>
-      <c r="DY2"/>
-      <c r="DZ2"/>
-      <c r="EA2"/>
-      <c r="EB2"/>
-      <c r="EC2"/>
-      <c r="ED2"/>
-      <c r="EE2"/>
-      <c r="EF2"/>
-      <c r="EG2"/>
-      <c r="EH2"/>
-      <c r="EI2"/>
-      <c r="EJ2"/>
-      <c r="EK2"/>
-      <c r="EL2"/>
-      <c r="EM2"/>
-      <c r="EN2"/>
-      <c r="EO2"/>
-      <c r="EP2"/>
-      <c r="EQ2"/>
-      <c r="ER2"/>
-      <c r="ES2"/>
-      <c r="ET2"/>
-      <c r="EU2"/>
-      <c r="EV2"/>
-      <c r="EW2"/>
-      <c r="EX2"/>
-      <c r="EY2"/>
-      <c r="EZ2"/>
-      <c r="FA2"/>
-      <c r="FB2"/>
-      <c r="FC2"/>
-      <c r="FD2"/>
-      <c r="FE2"/>
-      <c r="FF2"/>
-      <c r="FG2"/>
-      <c r="FH2"/>
-      <c r="FI2"/>
-      <c r="FJ2"/>
-      <c r="FK2"/>
-      <c r="FL2"/>
-      <c r="FM2"/>
-      <c r="FN2"/>
-      <c r="FO2"/>
-      <c r="FP2"/>
-      <c r="FQ2"/>
-      <c r="FR2"/>
-      <c r="FS2"/>
-      <c r="FT2"/>
-      <c r="FU2"/>
-      <c r="FV2"/>
-      <c r="FW2"/>
-      <c r="FX2"/>
-      <c r="FY2"/>
-      <c r="FZ2"/>
-      <c r="GA2"/>
-      <c r="GB2"/>
-      <c r="GC2"/>
-      <c r="GD2"/>
-      <c r="GE2"/>
-      <c r="GF2"/>
-      <c r="GG2"/>
-      <c r="GH2"/>
-      <c r="GI2"/>
-      <c r="GJ2"/>
-      <c r="GK2"/>
-      <c r="GL2"/>
-      <c r="GM2"/>
-      <c r="GN2"/>
-      <c r="GO2"/>
-      <c r="GP2"/>
-      <c r="GQ2"/>
-      <c r="GR2"/>
-      <c r="GS2"/>
-      <c r="GT2"/>
-      <c r="GU2"/>
-      <c r="GV2"/>
-      <c r="GW2"/>
-      <c r="GX2"/>
-      <c r="GY2"/>
-      <c r="GZ2"/>
-      <c r="HA2"/>
-      <c r="HB2"/>
-      <c r="HC2"/>
-      <c r="HD2"/>
-      <c r="HE2"/>
-      <c r="HF2"/>
-      <c r="HG2"/>
-      <c r="HH2"/>
-      <c r="HI2"/>
-      <c r="HJ2"/>
-      <c r="HK2"/>
-      <c r="HL2"/>
-      <c r="HM2"/>
-      <c r="HN2"/>
-      <c r="HO2"/>
-      <c r="HP2"/>
-      <c r="HQ2"/>
-      <c r="HR2"/>
-      <c r="HS2"/>
-      <c r="HT2"/>
-      <c r="HU2"/>
-    </row>
-    <row r="3" spans="1:229" x14ac:dyDescent="0.35">
-      <c r="A3" s="3" t="s">
-        <v>460</v>
-      </c>
-      <c r="B3" s="3" t="s">
-        <v>461</v>
-      </c>
-      <c r="C3" s="3" t="s">
-        <v>462</v>
-      </c>
-      <c r="D3" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="E3" s="3" t="s">
-        <v>201</v>
-      </c>
-      <c r="F3" s="3" t="s">
-        <v>202</v>
-      </c>
-      <c r="G3" s="3" t="s">
-        <v>211</v>
-      </c>
-      <c r="H3" s="3" t="s">
-        <v>463</v>
-      </c>
-    </row>
-    <row r="4" spans="1:229" x14ac:dyDescent="0.35">
-      <c r="A4" s="3" t="s">
-        <v>464</v>
-      </c>
-      <c r="B4" s="3" t="s">
-        <v>467</v>
-      </c>
-      <c r="C4" s="3" t="s">
-        <v>465</v>
-      </c>
-      <c r="D4" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="E4" s="3" t="s">
-        <v>201</v>
-      </c>
-      <c r="F4" s="3" t="s">
-        <v>202</v>
-      </c>
-      <c r="G4" s="3" t="s">
-        <v>211</v>
-      </c>
-      <c r="H4" s="3" t="s">
-        <v>466</v>
-      </c>
-    </row>
-    <row r="5" spans="1:229" x14ac:dyDescent="0.35">
-      <c r="A5" s="8" t="s">
-        <v>468</v>
-      </c>
-      <c r="B5" s="8" t="s">
-        <v>469</v>
-      </c>
-      <c r="C5" s="8" t="s">
-        <v>470</v>
-      </c>
-      <c r="D5" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="E5" s="3" t="s">
-        <v>201</v>
-      </c>
-      <c r="F5" s="3" t="s">
-        <v>202</v>
-      </c>
-      <c r="G5" s="3" t="s">
-        <v>211</v>
-      </c>
-      <c r="H5" s="3" t="s">
-        <v>471</v>
-      </c>
-    </row>
-    <row r="6" spans="1:229" x14ac:dyDescent="0.35">
-      <c r="A6" s="3" t="s">
-        <v>473</v>
-      </c>
-      <c r="B6" s="3" t="s">
-        <v>472</v>
-      </c>
-      <c r="C6" s="3" t="s">
-        <v>474</v>
-      </c>
-      <c r="D6" s="7" t="s">
-        <v>0</v>
-      </c>
-      <c r="E6" s="3" t="s">
-        <v>201</v>
-      </c>
-      <c r="F6" s="3" t="s">
-        <v>202</v>
-      </c>
-      <c r="G6" s="3" t="s">
-        <v>211</v>
-      </c>
-      <c r="H6" s="3" t="s">
-        <v>475</v>
-      </c>
-    </row>
-    <row r="7" spans="1:229" x14ac:dyDescent="0.35">
-      <c r="A7" s="3" t="s">
-        <v>476</v>
-      </c>
-      <c r="B7" s="3" t="s">
-        <v>477</v>
-      </c>
-      <c r="C7" s="3" t="s">
-        <v>478</v>
-      </c>
-      <c r="D7" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="E7" s="3" t="s">
-        <v>201</v>
-      </c>
-      <c r="F7" s="3" t="s">
-        <v>202</v>
-      </c>
-      <c r="G7" s="3" t="s">
-        <v>211</v>
-      </c>
-      <c r="H7" s="3" t="s">
-        <v>479</v>
-      </c>
-    </row>
-    <row r="8" spans="1:229" x14ac:dyDescent="0.35">
-      <c r="A8" s="3" t="s">
-        <v>480</v>
-      </c>
-      <c r="B8" s="3" t="s">
-        <v>481</v>
-      </c>
-      <c r="C8" s="3" t="s">
-        <v>482</v>
-      </c>
-      <c r="D8" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="E8" s="3" t="s">
-        <v>201</v>
-      </c>
-      <c r="F8" s="3" t="s">
-        <v>202</v>
-      </c>
-      <c r="G8" s="3" t="s">
-        <v>211</v>
-      </c>
-      <c r="H8" s="3" t="s">
-        <v>483</v>
-      </c>
-    </row>
-    <row r="9" spans="1:229" x14ac:dyDescent="0.35">
-      <c r="A9" s="3" t="s">
-        <v>484</v>
-      </c>
-      <c r="B9" s="3" t="s">
-        <v>485</v>
-      </c>
-      <c r="C9" s="3" t="s">
-        <v>486</v>
-      </c>
-      <c r="D9" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="E9" s="3" t="s">
-        <v>201</v>
-      </c>
-      <c r="F9" s="3" t="s">
-        <v>202</v>
-      </c>
-      <c r="G9" s="3" t="s">
-        <v>211</v>
-      </c>
-      <c r="H9" s="3" t="s">
-        <v>487</v>
       </c>
     </row>
   </sheetData>
@@ -19357,8 +19024,8 @@
 </file>
 
 <file path=xl/worksheets/sheet30.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2A4E3580-B709-4E66-9F6E-B7F9948D7FD3}">
-  <dimension ref="A1:HU7"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E6428663-7558-48F1-8CD3-947F03FFD4CC}">
+  <dimension ref="A1:HU9"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="50.90625" bestFit="1" customWidth="1"/>
@@ -19399,13 +19066,13 @@
     </row>
     <row r="2" spans="1:229" s="4" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A2" s="3" t="s">
-        <v>488</v>
+        <v>457</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>489</v>
+        <v>458</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>490</v>
+        <v>459</v>
       </c>
       <c r="D2" s="3" t="s">
         <v>0</v>
@@ -19420,7 +19087,7 @@
         <v>211</v>
       </c>
       <c r="H2" s="3" t="s">
-        <v>491</v>
+        <v>192</v>
       </c>
       <c r="I2"/>
       <c r="J2"/>
@@ -19646,13 +19313,13 @@
     </row>
     <row r="3" spans="1:229" x14ac:dyDescent="0.35">
       <c r="A3" s="3" t="s">
-        <v>492</v>
+        <v>460</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>493</v>
+        <v>461</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>494</v>
+        <v>462</v>
       </c>
       <c r="D3" s="3" t="s">
         <v>0</v>
@@ -19667,18 +19334,18 @@
         <v>211</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>495</v>
+        <v>463</v>
       </c>
     </row>
     <row r="4" spans="1:229" x14ac:dyDescent="0.35">
       <c r="A4" s="3" t="s">
-        <v>496</v>
+        <v>464</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>497</v>
+        <v>467</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>498</v>
+        <v>465</v>
       </c>
       <c r="D4" s="3" t="s">
         <v>0</v>
@@ -19693,18 +19360,18 @@
         <v>211</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>499</v>
+        <v>466</v>
       </c>
     </row>
     <row r="5" spans="1:229" x14ac:dyDescent="0.35">
       <c r="A5" s="8" t="s">
-        <v>500</v>
+        <v>468</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>501</v>
+        <v>469</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>502</v>
+        <v>470</v>
       </c>
       <c r="D5" s="3" t="s">
         <v>0</v>
@@ -19719,18 +19386,18 @@
         <v>211</v>
       </c>
       <c r="H5" s="3" t="s">
-        <v>503</v>
+        <v>471</v>
       </c>
     </row>
     <row r="6" spans="1:229" x14ac:dyDescent="0.35">
       <c r="A6" s="3" t="s">
-        <v>504</v>
+        <v>473</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>505</v>
+        <v>472</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>506</v>
+        <v>474</v>
       </c>
       <c r="D6" s="7" t="s">
         <v>0</v>
@@ -19745,18 +19412,18 @@
         <v>211</v>
       </c>
       <c r="H6" s="3" t="s">
-        <v>507</v>
+        <v>475</v>
       </c>
     </row>
     <row r="7" spans="1:229" x14ac:dyDescent="0.35">
       <c r="A7" s="3" t="s">
-        <v>509</v>
+        <v>476</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>508</v>
+        <v>477</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>510</v>
+        <v>478</v>
       </c>
       <c r="D7" s="3" t="s">
         <v>0</v>
@@ -19771,17 +19438,70 @@
         <v>211</v>
       </c>
       <c r="H7" s="3" t="s">
-        <v>511</v>
+        <v>479</v>
+      </c>
+    </row>
+    <row r="8" spans="1:229" x14ac:dyDescent="0.35">
+      <c r="A8" s="3" t="s">
+        <v>480</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>481</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>482</v>
+      </c>
+      <c r="D8" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="E8" s="3" t="s">
+        <v>201</v>
+      </c>
+      <c r="F8" s="3" t="s">
+        <v>202</v>
+      </c>
+      <c r="G8" s="3" t="s">
+        <v>211</v>
+      </c>
+      <c r="H8" s="3" t="s">
+        <v>483</v>
+      </c>
+    </row>
+    <row r="9" spans="1:229" x14ac:dyDescent="0.35">
+      <c r="A9" s="3" t="s">
+        <v>484</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>485</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>486</v>
+      </c>
+      <c r="D9" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="E9" s="3" t="s">
+        <v>201</v>
+      </c>
+      <c r="F9" s="3" t="s">
+        <v>202</v>
+      </c>
+      <c r="G9" s="3" t="s">
+        <v>211</v>
+      </c>
+      <c r="H9" s="3" t="s">
+        <v>487</v>
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet31.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{95706458-CD50-4C74-87C4-ABAE617927AD}">
-  <dimension ref="A1:HU2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2A4E3580-B709-4E66-9F6E-B7F9948D7FD3}">
+  <dimension ref="A1:HU7"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="50.90625" bestFit="1" customWidth="1"/>
@@ -19822,13 +19542,13 @@
     </row>
     <row r="2" spans="1:229" s="4" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A2" s="3" t="s">
-        <v>512</v>
+        <v>488</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>513</v>
+        <v>489</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>514</v>
+        <v>490</v>
       </c>
       <c r="D2" s="3" t="s">
         <v>0</v>
@@ -19843,7 +19563,7 @@
         <v>211</v>
       </c>
       <c r="H2" s="3" t="s">
-        <v>140</v>
+        <v>491</v>
       </c>
       <c r="I2"/>
       <c r="J2"/>
@@ -20067,14 +19787,144 @@
       <c r="HT2"/>
       <c r="HU2"/>
     </row>
+    <row r="3" spans="1:229" x14ac:dyDescent="0.35">
+      <c r="A3" s="3" t="s">
+        <v>492</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>493</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>494</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>201</v>
+      </c>
+      <c r="F3" s="3" t="s">
+        <v>202</v>
+      </c>
+      <c r="G3" s="3" t="s">
+        <v>211</v>
+      </c>
+      <c r="H3" s="3" t="s">
+        <v>495</v>
+      </c>
+    </row>
+    <row r="4" spans="1:229" x14ac:dyDescent="0.35">
+      <c r="A4" s="3" t="s">
+        <v>496</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>497</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>498</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>201</v>
+      </c>
+      <c r="F4" s="3" t="s">
+        <v>202</v>
+      </c>
+      <c r="G4" s="3" t="s">
+        <v>211</v>
+      </c>
+      <c r="H4" s="3" t="s">
+        <v>499</v>
+      </c>
+    </row>
+    <row r="5" spans="1:229" x14ac:dyDescent="0.35">
+      <c r="A5" s="8" t="s">
+        <v>500</v>
+      </c>
+      <c r="B5" s="8" t="s">
+        <v>501</v>
+      </c>
+      <c r="C5" s="8" t="s">
+        <v>502</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>201</v>
+      </c>
+      <c r="F5" s="3" t="s">
+        <v>202</v>
+      </c>
+      <c r="G5" s="3" t="s">
+        <v>211</v>
+      </c>
+      <c r="H5" s="3" t="s">
+        <v>503</v>
+      </c>
+    </row>
+    <row r="6" spans="1:229" x14ac:dyDescent="0.35">
+      <c r="A6" s="3" t="s">
+        <v>504</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>505</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>506</v>
+      </c>
+      <c r="D6" s="7" t="s">
+        <v>0</v>
+      </c>
+      <c r="E6" s="3" t="s">
+        <v>201</v>
+      </c>
+      <c r="F6" s="3" t="s">
+        <v>202</v>
+      </c>
+      <c r="G6" s="3" t="s">
+        <v>211</v>
+      </c>
+      <c r="H6" s="3" t="s">
+        <v>507</v>
+      </c>
+    </row>
+    <row r="7" spans="1:229" x14ac:dyDescent="0.35">
+      <c r="A7" s="3" t="s">
+        <v>509</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>508</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>510</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="E7" s="3" t="s">
+        <v>201</v>
+      </c>
+      <c r="F7" s="3" t="s">
+        <v>202</v>
+      </c>
+      <c r="G7" s="3" t="s">
+        <v>211</v>
+      </c>
+      <c r="H7" s="3" t="s">
+        <v>511</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet32.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1AD86191-7CFE-4ED9-9129-FF78170AB51E}">
-  <dimension ref="A1:HU12"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{95706458-CD50-4C74-87C4-ABAE617927AD}">
+  <dimension ref="A1:HU2"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="50.90625" bestFit="1" customWidth="1"/>
@@ -20084,7 +19934,7 @@
     <col min="5" max="5" width="33.08984375" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="17.08984375" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="40.81640625" customWidth="1"/>
-    <col min="8" max="8" width="65.54296875" customWidth="1"/>
+    <col min="8" max="8" width="57.08984375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:229" x14ac:dyDescent="0.35">
@@ -20115,13 +19965,13 @@
     </row>
     <row r="2" spans="1:229" s="4" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A2" s="3" t="s">
-        <v>527</v>
+        <v>512</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>528</v>
+        <v>513</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>529</v>
+        <v>514</v>
       </c>
       <c r="D2" s="3" t="s">
         <v>0</v>
@@ -20136,7 +19986,7 @@
         <v>211</v>
       </c>
       <c r="H2" s="3" t="s">
-        <v>530</v>
+        <v>140</v>
       </c>
       <c r="I2"/>
       <c r="J2"/>
@@ -20360,278 +20210,17 @@
       <c r="HT2"/>
       <c r="HU2"/>
     </row>
-    <row r="3" spans="1:229" x14ac:dyDescent="0.35">
-      <c r="A3" s="3" t="s">
-        <v>532</v>
-      </c>
-      <c r="B3" s="3" t="s">
-        <v>531</v>
-      </c>
-      <c r="C3" s="3" t="s">
-        <v>533</v>
-      </c>
-      <c r="D3" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="E3" s="3" t="s">
-        <v>201</v>
-      </c>
-      <c r="F3" s="3" t="s">
-        <v>202</v>
-      </c>
-      <c r="G3" s="3" t="s">
-        <v>211</v>
-      </c>
-      <c r="H3" s="3" t="s">
-        <v>534</v>
-      </c>
-    </row>
-    <row r="4" spans="1:229" x14ac:dyDescent="0.35">
-      <c r="A4" s="3" t="s">
-        <v>535</v>
-      </c>
-      <c r="B4" s="3" t="s">
-        <v>536</v>
-      </c>
-      <c r="C4" s="3" t="s">
-        <v>537</v>
-      </c>
-      <c r="D4" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="E4" s="3" t="s">
-        <v>201</v>
-      </c>
-      <c r="F4" s="3" t="s">
-        <v>202</v>
-      </c>
-      <c r="G4" s="3" t="s">
-        <v>211</v>
-      </c>
-      <c r="H4" s="3" t="s">
-        <v>538</v>
-      </c>
-    </row>
-    <row r="5" spans="1:229" x14ac:dyDescent="0.35">
-      <c r="A5" s="8" t="s">
-        <v>539</v>
-      </c>
-      <c r="B5" s="8" t="s">
-        <v>540</v>
-      </c>
-      <c r="C5" s="8" t="s">
-        <v>541</v>
-      </c>
-      <c r="D5" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="E5" s="3" t="s">
-        <v>201</v>
-      </c>
-      <c r="F5" s="3" t="s">
-        <v>202</v>
-      </c>
-      <c r="G5" s="3" t="s">
-        <v>211</v>
-      </c>
-      <c r="H5" s="3" t="s">
-        <v>542</v>
-      </c>
-    </row>
-    <row r="6" spans="1:229" x14ac:dyDescent="0.35">
-      <c r="A6" s="3" t="s">
-        <v>543</v>
-      </c>
-      <c r="B6" s="3" t="s">
-        <v>544</v>
-      </c>
-      <c r="C6" s="3" t="s">
-        <v>545</v>
-      </c>
-      <c r="D6" s="7" t="s">
-        <v>0</v>
-      </c>
-      <c r="E6" s="3" t="s">
-        <v>201</v>
-      </c>
-      <c r="F6" s="3" t="s">
-        <v>202</v>
-      </c>
-      <c r="G6" s="3" t="s">
-        <v>211</v>
-      </c>
-      <c r="H6" s="3" t="s">
-        <v>546</v>
-      </c>
-    </row>
-    <row r="7" spans="1:229" x14ac:dyDescent="0.35">
-      <c r="A7" s="3" t="s">
-        <v>547</v>
-      </c>
-      <c r="B7" s="3" t="s">
-        <v>548</v>
-      </c>
-      <c r="C7" s="3" t="s">
-        <v>549</v>
-      </c>
-      <c r="D7" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="E7" s="3" t="s">
-        <v>201</v>
-      </c>
-      <c r="F7" s="3" t="s">
-        <v>202</v>
-      </c>
-      <c r="G7" s="3" t="s">
-        <v>211</v>
-      </c>
-      <c r="H7" s="3" t="s">
-        <v>550</v>
-      </c>
-    </row>
-    <row r="8" spans="1:229" x14ac:dyDescent="0.35">
-      <c r="A8" s="3" t="s">
-        <v>551</v>
-      </c>
-      <c r="B8" s="3" t="s">
-        <v>552</v>
-      </c>
-      <c r="C8" s="3" t="s">
-        <v>553</v>
-      </c>
-      <c r="D8" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="E8" s="3" t="s">
-        <v>201</v>
-      </c>
-      <c r="F8" s="3" t="s">
-        <v>202</v>
-      </c>
-      <c r="G8" s="10" t="s">
-        <v>211</v>
-      </c>
-      <c r="H8" s="3" t="s">
-        <v>554</v>
-      </c>
-    </row>
-    <row r="9" spans="1:229" x14ac:dyDescent="0.35">
-      <c r="A9" s="3" t="s">
-        <v>555</v>
-      </c>
-      <c r="B9" s="3" t="s">
-        <v>556</v>
-      </c>
-      <c r="C9" s="3" t="s">
-        <v>558</v>
-      </c>
-      <c r="D9" s="7" t="s">
-        <v>0</v>
-      </c>
-      <c r="E9" s="3" t="s">
-        <v>201</v>
-      </c>
-      <c r="F9" s="3" t="s">
-        <v>202</v>
-      </c>
-      <c r="G9" s="10" t="s">
-        <v>211</v>
-      </c>
-      <c r="H9" s="3" t="s">
-        <v>557</v>
-      </c>
-    </row>
-    <row r="10" spans="1:229" x14ac:dyDescent="0.35">
-      <c r="A10" s="3" t="s">
-        <v>559</v>
-      </c>
-      <c r="B10" s="3" t="s">
-        <v>560</v>
-      </c>
-      <c r="C10" s="3" t="s">
-        <v>561</v>
-      </c>
-      <c r="D10" s="7" t="s">
-        <v>0</v>
-      </c>
-      <c r="E10" s="3" t="s">
-        <v>201</v>
-      </c>
-      <c r="F10" s="3" t="s">
-        <v>202</v>
-      </c>
-      <c r="G10" s="10" t="s">
-        <v>211</v>
-      </c>
-      <c r="H10" s="3" t="s">
-        <v>562</v>
-      </c>
-    </row>
-    <row r="11" spans="1:229" x14ac:dyDescent="0.35">
-      <c r="A11" s="3" t="s">
-        <v>563</v>
-      </c>
-      <c r="B11" s="3" t="s">
-        <v>564</v>
-      </c>
-      <c r="C11" s="3" t="s">
-        <v>565</v>
-      </c>
-      <c r="D11" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="E11" s="3" t="s">
-        <v>201</v>
-      </c>
-      <c r="F11" s="3" t="s">
-        <v>202</v>
-      </c>
-      <c r="G11" s="10" t="s">
-        <v>211</v>
-      </c>
-      <c r="H11" s="3" t="s">
-        <v>566</v>
-      </c>
-    </row>
-    <row r="12" spans="1:229" x14ac:dyDescent="0.35">
-      <c r="A12" s="3" t="s">
-        <v>567</v>
-      </c>
-      <c r="B12" s="3" t="s">
-        <v>568</v>
-      </c>
-      <c r="C12" s="3" t="s">
-        <v>569</v>
-      </c>
-      <c r="D12" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="E12" s="3" t="s">
-        <v>201</v>
-      </c>
-      <c r="F12" s="3" t="s">
-        <v>202</v>
-      </c>
-      <c r="G12" s="10" t="s">
-        <v>211</v>
-      </c>
-      <c r="H12" s="3" t="s">
-        <v>570</v>
-      </c>
-    </row>
   </sheetData>
-  <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet33.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{24EB34D0-BCF8-4F57-88CC-AC842687528F}">
-  <dimension ref="A1:HU5"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1AD86191-7CFE-4ED9-9129-FF78170AB51E}">
+  <dimension ref="A1:HU12"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="52.453125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="50.90625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="52.26953125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="42.453125" customWidth="1"/>
     <col min="4" max="4" width="33.36328125" bestFit="1" customWidth="1"/>
@@ -20669,13 +20258,13 @@
     </row>
     <row r="2" spans="1:229" s="4" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A2" s="3" t="s">
-        <v>576</v>
+        <v>527</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>577</v>
+        <v>528</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>578</v>
+        <v>529</v>
       </c>
       <c r="D2" s="3" t="s">
         <v>0</v>
@@ -20690,7 +20279,7 @@
         <v>211</v>
       </c>
       <c r="H2" s="3" t="s">
-        <v>579</v>
+        <v>530</v>
       </c>
       <c r="I2"/>
       <c r="J2"/>
@@ -20916,13 +20505,13 @@
     </row>
     <row r="3" spans="1:229" x14ac:dyDescent="0.35">
       <c r="A3" s="3" t="s">
-        <v>580</v>
+        <v>532</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>581</v>
+        <v>531</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>582</v>
+        <v>533</v>
       </c>
       <c r="D3" s="3" t="s">
         <v>0</v>
@@ -20937,42 +20526,44 @@
         <v>211</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>583</v>
+        <v>534</v>
       </c>
     </row>
     <row r="4" spans="1:229" x14ac:dyDescent="0.35">
-      <c r="A4" s="11" t="s">
-        <v>584</v>
-      </c>
-      <c r="B4" s="11" t="s">
-        <v>585</v>
-      </c>
-      <c r="C4" s="11" t="s">
-        <v>586</v>
-      </c>
-      <c r="D4" s="11" t="s">
+      <c r="A4" s="3" t="s">
+        <v>535</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>536</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>537</v>
+      </c>
+      <c r="D4" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="E4" s="11" t="s">
+      <c r="E4" s="3" t="s">
         <v>201</v>
       </c>
-      <c r="F4" s="11" t="s">
+      <c r="F4" s="3" t="s">
         <v>202</v>
       </c>
-      <c r="G4" s="11" t="s">
+      <c r="G4" s="3" t="s">
         <v>211</v>
       </c>
-      <c r="H4" s="11"/>
+      <c r="H4" s="3" t="s">
+        <v>538</v>
+      </c>
     </row>
     <row r="5" spans="1:229" x14ac:dyDescent="0.35">
-      <c r="A5" s="3" t="s">
-        <v>587</v>
-      </c>
-      <c r="B5" s="3" t="s">
-        <v>588</v>
-      </c>
-      <c r="C5" s="3" t="s">
-        <v>589</v>
+      <c r="A5" s="8" t="s">
+        <v>539</v>
+      </c>
+      <c r="B5" s="8" t="s">
+        <v>540</v>
+      </c>
+      <c r="C5" s="8" t="s">
+        <v>541</v>
       </c>
       <c r="D5" s="3" t="s">
         <v>0</v>
@@ -20987,17 +20578,200 @@
         <v>211</v>
       </c>
       <c r="H5" s="3" t="s">
-        <v>590</v>
+        <v>542</v>
+      </c>
+    </row>
+    <row r="6" spans="1:229" x14ac:dyDescent="0.35">
+      <c r="A6" s="3" t="s">
+        <v>543</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>544</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>545</v>
+      </c>
+      <c r="D6" s="7" t="s">
+        <v>0</v>
+      </c>
+      <c r="E6" s="3" t="s">
+        <v>201</v>
+      </c>
+      <c r="F6" s="3" t="s">
+        <v>202</v>
+      </c>
+      <c r="G6" s="3" t="s">
+        <v>211</v>
+      </c>
+      <c r="H6" s="3" t="s">
+        <v>546</v>
+      </c>
+    </row>
+    <row r="7" spans="1:229" x14ac:dyDescent="0.35">
+      <c r="A7" s="3" t="s">
+        <v>547</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>548</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>549</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="E7" s="3" t="s">
+        <v>201</v>
+      </c>
+      <c r="F7" s="3" t="s">
+        <v>202</v>
+      </c>
+      <c r="G7" s="3" t="s">
+        <v>211</v>
+      </c>
+      <c r="H7" s="3" t="s">
+        <v>550</v>
+      </c>
+    </row>
+    <row r="8" spans="1:229" x14ac:dyDescent="0.35">
+      <c r="A8" s="3" t="s">
+        <v>551</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>552</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>553</v>
+      </c>
+      <c r="D8" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="E8" s="3" t="s">
+        <v>201</v>
+      </c>
+      <c r="F8" s="3" t="s">
+        <v>202</v>
+      </c>
+      <c r="G8" s="10" t="s">
+        <v>211</v>
+      </c>
+      <c r="H8" s="3" t="s">
+        <v>554</v>
+      </c>
+    </row>
+    <row r="9" spans="1:229" x14ac:dyDescent="0.35">
+      <c r="A9" s="3" t="s">
+        <v>555</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>556</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>558</v>
+      </c>
+      <c r="D9" s="7" t="s">
+        <v>0</v>
+      </c>
+      <c r="E9" s="3" t="s">
+        <v>201</v>
+      </c>
+      <c r="F9" s="3" t="s">
+        <v>202</v>
+      </c>
+      <c r="G9" s="10" t="s">
+        <v>211</v>
+      </c>
+      <c r="H9" s="3" t="s">
+        <v>557</v>
+      </c>
+    </row>
+    <row r="10" spans="1:229" x14ac:dyDescent="0.35">
+      <c r="A10" s="3" t="s">
+        <v>559</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>560</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>561</v>
+      </c>
+      <c r="D10" s="7" t="s">
+        <v>0</v>
+      </c>
+      <c r="E10" s="3" t="s">
+        <v>201</v>
+      </c>
+      <c r="F10" s="3" t="s">
+        <v>202</v>
+      </c>
+      <c r="G10" s="10" t="s">
+        <v>211</v>
+      </c>
+      <c r="H10" s="3" t="s">
+        <v>562</v>
+      </c>
+    </row>
+    <row r="11" spans="1:229" x14ac:dyDescent="0.35">
+      <c r="A11" s="3" t="s">
+        <v>563</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>564</v>
+      </c>
+      <c r="C11" s="3" t="s">
+        <v>565</v>
+      </c>
+      <c r="D11" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="E11" s="3" t="s">
+        <v>201</v>
+      </c>
+      <c r="F11" s="3" t="s">
+        <v>202</v>
+      </c>
+      <c r="G11" s="10" t="s">
+        <v>211</v>
+      </c>
+      <c r="H11" s="3" t="s">
+        <v>566</v>
+      </c>
+    </row>
+    <row r="12" spans="1:229" x14ac:dyDescent="0.35">
+      <c r="A12" s="3" t="s">
+        <v>567</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>568</v>
+      </c>
+      <c r="C12" s="3" t="s">
+        <v>569</v>
+      </c>
+      <c r="D12" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="E12" s="3" t="s">
+        <v>201</v>
+      </c>
+      <c r="F12" s="3" t="s">
+        <v>202</v>
+      </c>
+      <c r="G12" s="10" t="s">
+        <v>211</v>
+      </c>
+      <c r="H12" s="3" t="s">
+        <v>570</v>
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet34.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7271F742-0542-4B33-AEE2-20AE8A69F475}">
-  <dimension ref="A1:HU3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{24EB34D0-BCF8-4F57-88CC-AC842687528F}">
+  <dimension ref="A1:HU5"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="52.453125" bestFit="1" customWidth="1"/>
@@ -21038,13 +20812,13 @@
     </row>
     <row r="2" spans="1:229" s="4" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A2" s="3" t="s">
-        <v>594</v>
+        <v>576</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>595</v>
+        <v>577</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>596</v>
+        <v>578</v>
       </c>
       <c r="D2" s="3" t="s">
         <v>0</v>
@@ -21059,7 +20833,7 @@
         <v>211</v>
       </c>
       <c r="H2" s="3" t="s">
-        <v>597</v>
+        <v>579</v>
       </c>
       <c r="I2"/>
       <c r="J2"/>
@@ -21285,6 +21059,375 @@
     </row>
     <row r="3" spans="1:229" x14ac:dyDescent="0.35">
       <c r="A3" s="3" t="s">
+        <v>580</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>581</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>582</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>201</v>
+      </c>
+      <c r="F3" s="3" t="s">
+        <v>202</v>
+      </c>
+      <c r="G3" s="3" t="s">
+        <v>211</v>
+      </c>
+      <c r="H3" s="3" t="s">
+        <v>583</v>
+      </c>
+    </row>
+    <row r="4" spans="1:229" x14ac:dyDescent="0.35">
+      <c r="A4" s="11" t="s">
+        <v>584</v>
+      </c>
+      <c r="B4" s="11" t="s">
+        <v>585</v>
+      </c>
+      <c r="C4" s="11" t="s">
+        <v>586</v>
+      </c>
+      <c r="D4" s="11" t="s">
+        <v>0</v>
+      </c>
+      <c r="E4" s="11" t="s">
+        <v>201</v>
+      </c>
+      <c r="F4" s="11" t="s">
+        <v>202</v>
+      </c>
+      <c r="G4" s="11" t="s">
+        <v>211</v>
+      </c>
+      <c r="H4" s="11"/>
+    </row>
+    <row r="5" spans="1:229" x14ac:dyDescent="0.35">
+      <c r="A5" s="3" t="s">
+        <v>587</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>588</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>589</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>201</v>
+      </c>
+      <c r="F5" s="3" t="s">
+        <v>202</v>
+      </c>
+      <c r="G5" s="3" t="s">
+        <v>211</v>
+      </c>
+      <c r="H5" s="3" t="s">
+        <v>590</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet35.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7271F742-0542-4B33-AEE2-20AE8A69F475}">
+  <dimension ref="A1:HU3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="52.453125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="52.26953125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="42.453125" customWidth="1"/>
+    <col min="4" max="4" width="33.36328125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="33.08984375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="17.08984375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="40.81640625" customWidth="1"/>
+    <col min="8" max="8" width="65.54296875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:229" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>209</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="2" spans="1:229" s="4" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A2" s="3" t="s">
+        <v>594</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>595</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>596</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>201</v>
+      </c>
+      <c r="F2" s="3" t="s">
+        <v>202</v>
+      </c>
+      <c r="G2" s="3" t="s">
+        <v>211</v>
+      </c>
+      <c r="H2" s="3" t="s">
+        <v>597</v>
+      </c>
+      <c r="I2"/>
+      <c r="J2"/>
+      <c r="K2"/>
+      <c r="L2"/>
+      <c r="M2"/>
+      <c r="N2"/>
+      <c r="O2"/>
+      <c r="P2"/>
+      <c r="Q2"/>
+      <c r="R2"/>
+      <c r="S2"/>
+      <c r="T2"/>
+      <c r="U2"/>
+      <c r="V2"/>
+      <c r="W2"/>
+      <c r="X2"/>
+      <c r="Y2"/>
+      <c r="Z2"/>
+      <c r="AA2"/>
+      <c r="AB2"/>
+      <c r="AC2"/>
+      <c r="AD2"/>
+      <c r="AE2"/>
+      <c r="AF2"/>
+      <c r="AG2"/>
+      <c r="AH2"/>
+      <c r="AI2"/>
+      <c r="AJ2"/>
+      <c r="AK2"/>
+      <c r="AL2"/>
+      <c r="AM2"/>
+      <c r="AN2"/>
+      <c r="AO2"/>
+      <c r="AP2"/>
+      <c r="AQ2"/>
+      <c r="AR2"/>
+      <c r="AS2"/>
+      <c r="AT2"/>
+      <c r="AU2"/>
+      <c r="AV2"/>
+      <c r="AW2"/>
+      <c r="AX2"/>
+      <c r="AY2"/>
+      <c r="AZ2"/>
+      <c r="BA2"/>
+      <c r="BB2"/>
+      <c r="BC2"/>
+      <c r="BD2"/>
+      <c r="BE2"/>
+      <c r="BF2"/>
+      <c r="BG2"/>
+      <c r="BH2"/>
+      <c r="BI2"/>
+      <c r="BJ2"/>
+      <c r="BK2"/>
+      <c r="BL2"/>
+      <c r="BM2"/>
+      <c r="BN2"/>
+      <c r="BO2"/>
+      <c r="BP2"/>
+      <c r="BQ2"/>
+      <c r="BR2"/>
+      <c r="BS2"/>
+      <c r="BT2"/>
+      <c r="BU2"/>
+      <c r="BV2"/>
+      <c r="BW2"/>
+      <c r="BX2"/>
+      <c r="BY2"/>
+      <c r="BZ2"/>
+      <c r="CA2"/>
+      <c r="CB2"/>
+      <c r="CC2"/>
+      <c r="CD2"/>
+      <c r="CE2"/>
+      <c r="CF2"/>
+      <c r="CG2"/>
+      <c r="CH2"/>
+      <c r="CI2"/>
+      <c r="CJ2"/>
+      <c r="CK2"/>
+      <c r="CL2"/>
+      <c r="CM2"/>
+      <c r="CN2"/>
+      <c r="CO2"/>
+      <c r="CP2"/>
+      <c r="CQ2"/>
+      <c r="CR2"/>
+      <c r="CS2"/>
+      <c r="CT2"/>
+      <c r="CU2"/>
+      <c r="CV2"/>
+      <c r="CW2"/>
+      <c r="CX2"/>
+      <c r="CY2"/>
+      <c r="CZ2"/>
+      <c r="DA2"/>
+      <c r="DB2"/>
+      <c r="DC2"/>
+      <c r="DD2"/>
+      <c r="DE2"/>
+      <c r="DF2"/>
+      <c r="DG2"/>
+      <c r="DH2"/>
+      <c r="DI2"/>
+      <c r="DJ2"/>
+      <c r="DK2"/>
+      <c r="DL2"/>
+      <c r="DM2"/>
+      <c r="DN2"/>
+      <c r="DO2"/>
+      <c r="DP2"/>
+      <c r="DQ2"/>
+      <c r="DR2"/>
+      <c r="DS2"/>
+      <c r="DT2"/>
+      <c r="DU2"/>
+      <c r="DV2"/>
+      <c r="DW2"/>
+      <c r="DX2"/>
+      <c r="DY2"/>
+      <c r="DZ2"/>
+      <c r="EA2"/>
+      <c r="EB2"/>
+      <c r="EC2"/>
+      <c r="ED2"/>
+      <c r="EE2"/>
+      <c r="EF2"/>
+      <c r="EG2"/>
+      <c r="EH2"/>
+      <c r="EI2"/>
+      <c r="EJ2"/>
+      <c r="EK2"/>
+      <c r="EL2"/>
+      <c r="EM2"/>
+      <c r="EN2"/>
+      <c r="EO2"/>
+      <c r="EP2"/>
+      <c r="EQ2"/>
+      <c r="ER2"/>
+      <c r="ES2"/>
+      <c r="ET2"/>
+      <c r="EU2"/>
+      <c r="EV2"/>
+      <c r="EW2"/>
+      <c r="EX2"/>
+      <c r="EY2"/>
+      <c r="EZ2"/>
+      <c r="FA2"/>
+      <c r="FB2"/>
+      <c r="FC2"/>
+      <c r="FD2"/>
+      <c r="FE2"/>
+      <c r="FF2"/>
+      <c r="FG2"/>
+      <c r="FH2"/>
+      <c r="FI2"/>
+      <c r="FJ2"/>
+      <c r="FK2"/>
+      <c r="FL2"/>
+      <c r="FM2"/>
+      <c r="FN2"/>
+      <c r="FO2"/>
+      <c r="FP2"/>
+      <c r="FQ2"/>
+      <c r="FR2"/>
+      <c r="FS2"/>
+      <c r="FT2"/>
+      <c r="FU2"/>
+      <c r="FV2"/>
+      <c r="FW2"/>
+      <c r="FX2"/>
+      <c r="FY2"/>
+      <c r="FZ2"/>
+      <c r="GA2"/>
+      <c r="GB2"/>
+      <c r="GC2"/>
+      <c r="GD2"/>
+      <c r="GE2"/>
+      <c r="GF2"/>
+      <c r="GG2"/>
+      <c r="GH2"/>
+      <c r="GI2"/>
+      <c r="GJ2"/>
+      <c r="GK2"/>
+      <c r="GL2"/>
+      <c r="GM2"/>
+      <c r="GN2"/>
+      <c r="GO2"/>
+      <c r="GP2"/>
+      <c r="GQ2"/>
+      <c r="GR2"/>
+      <c r="GS2"/>
+      <c r="GT2"/>
+      <c r="GU2"/>
+      <c r="GV2"/>
+      <c r="GW2"/>
+      <c r="GX2"/>
+      <c r="GY2"/>
+      <c r="GZ2"/>
+      <c r="HA2"/>
+      <c r="HB2"/>
+      <c r="HC2"/>
+      <c r="HD2"/>
+      <c r="HE2"/>
+      <c r="HF2"/>
+      <c r="HG2"/>
+      <c r="HH2"/>
+      <c r="HI2"/>
+      <c r="HJ2"/>
+      <c r="HK2"/>
+      <c r="HL2"/>
+      <c r="HM2"/>
+      <c r="HN2"/>
+      <c r="HO2"/>
+      <c r="HP2"/>
+      <c r="HQ2"/>
+      <c r="HR2"/>
+      <c r="HS2"/>
+      <c r="HT2"/>
+      <c r="HU2"/>
+    </row>
+    <row r="3" spans="1:229" x14ac:dyDescent="0.35">
+      <c r="A3" s="3" t="s">
         <v>598</v>
       </c>
       <c r="B3" s="3" t="s">
@@ -21310,6 +21453,376 @@
       </c>
     </row>
   </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet36.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{738B4CF9-CA20-4A87-AA62-B89EDC02284E}">
+  <dimension ref="A1:HU5"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="52.453125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="52.26953125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="42.453125" customWidth="1"/>
+    <col min="4" max="4" width="33.36328125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="33.08984375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="17.08984375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="40.81640625" customWidth="1"/>
+    <col min="8" max="8" width="65.54296875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:229" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>209</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="2" spans="1:229" s="4" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A2" s="3" t="s">
+        <v>607</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>608</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>609</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>201</v>
+      </c>
+      <c r="F2" s="3" t="s">
+        <v>202</v>
+      </c>
+      <c r="G2" s="3" t="s">
+        <v>211</v>
+      </c>
+      <c r="H2" s="11"/>
+      <c r="I2"/>
+      <c r="J2"/>
+      <c r="K2"/>
+      <c r="L2"/>
+      <c r="M2"/>
+      <c r="N2"/>
+      <c r="O2"/>
+      <c r="P2"/>
+      <c r="Q2"/>
+      <c r="R2"/>
+      <c r="S2"/>
+      <c r="T2"/>
+      <c r="U2"/>
+      <c r="V2"/>
+      <c r="W2"/>
+      <c r="X2"/>
+      <c r="Y2"/>
+      <c r="Z2"/>
+      <c r="AA2"/>
+      <c r="AB2"/>
+      <c r="AC2"/>
+      <c r="AD2"/>
+      <c r="AE2"/>
+      <c r="AF2"/>
+      <c r="AG2"/>
+      <c r="AH2"/>
+      <c r="AI2"/>
+      <c r="AJ2"/>
+      <c r="AK2"/>
+      <c r="AL2"/>
+      <c r="AM2"/>
+      <c r="AN2"/>
+      <c r="AO2"/>
+      <c r="AP2"/>
+      <c r="AQ2"/>
+      <c r="AR2"/>
+      <c r="AS2"/>
+      <c r="AT2"/>
+      <c r="AU2"/>
+      <c r="AV2"/>
+      <c r="AW2"/>
+      <c r="AX2"/>
+      <c r="AY2"/>
+      <c r="AZ2"/>
+      <c r="BA2"/>
+      <c r="BB2"/>
+      <c r="BC2"/>
+      <c r="BD2"/>
+      <c r="BE2"/>
+      <c r="BF2"/>
+      <c r="BG2"/>
+      <c r="BH2"/>
+      <c r="BI2"/>
+      <c r="BJ2"/>
+      <c r="BK2"/>
+      <c r="BL2"/>
+      <c r="BM2"/>
+      <c r="BN2"/>
+      <c r="BO2"/>
+      <c r="BP2"/>
+      <c r="BQ2"/>
+      <c r="BR2"/>
+      <c r="BS2"/>
+      <c r="BT2"/>
+      <c r="BU2"/>
+      <c r="BV2"/>
+      <c r="BW2"/>
+      <c r="BX2"/>
+      <c r="BY2"/>
+      <c r="BZ2"/>
+      <c r="CA2"/>
+      <c r="CB2"/>
+      <c r="CC2"/>
+      <c r="CD2"/>
+      <c r="CE2"/>
+      <c r="CF2"/>
+      <c r="CG2"/>
+      <c r="CH2"/>
+      <c r="CI2"/>
+      <c r="CJ2"/>
+      <c r="CK2"/>
+      <c r="CL2"/>
+      <c r="CM2"/>
+      <c r="CN2"/>
+      <c r="CO2"/>
+      <c r="CP2"/>
+      <c r="CQ2"/>
+      <c r="CR2"/>
+      <c r="CS2"/>
+      <c r="CT2"/>
+      <c r="CU2"/>
+      <c r="CV2"/>
+      <c r="CW2"/>
+      <c r="CX2"/>
+      <c r="CY2"/>
+      <c r="CZ2"/>
+      <c r="DA2"/>
+      <c r="DB2"/>
+      <c r="DC2"/>
+      <c r="DD2"/>
+      <c r="DE2"/>
+      <c r="DF2"/>
+      <c r="DG2"/>
+      <c r="DH2"/>
+      <c r="DI2"/>
+      <c r="DJ2"/>
+      <c r="DK2"/>
+      <c r="DL2"/>
+      <c r="DM2"/>
+      <c r="DN2"/>
+      <c r="DO2"/>
+      <c r="DP2"/>
+      <c r="DQ2"/>
+      <c r="DR2"/>
+      <c r="DS2"/>
+      <c r="DT2"/>
+      <c r="DU2"/>
+      <c r="DV2"/>
+      <c r="DW2"/>
+      <c r="DX2"/>
+      <c r="DY2"/>
+      <c r="DZ2"/>
+      <c r="EA2"/>
+      <c r="EB2"/>
+      <c r="EC2"/>
+      <c r="ED2"/>
+      <c r="EE2"/>
+      <c r="EF2"/>
+      <c r="EG2"/>
+      <c r="EH2"/>
+      <c r="EI2"/>
+      <c r="EJ2"/>
+      <c r="EK2"/>
+      <c r="EL2"/>
+      <c r="EM2"/>
+      <c r="EN2"/>
+      <c r="EO2"/>
+      <c r="EP2"/>
+      <c r="EQ2"/>
+      <c r="ER2"/>
+      <c r="ES2"/>
+      <c r="ET2"/>
+      <c r="EU2"/>
+      <c r="EV2"/>
+      <c r="EW2"/>
+      <c r="EX2"/>
+      <c r="EY2"/>
+      <c r="EZ2"/>
+      <c r="FA2"/>
+      <c r="FB2"/>
+      <c r="FC2"/>
+      <c r="FD2"/>
+      <c r="FE2"/>
+      <c r="FF2"/>
+      <c r="FG2"/>
+      <c r="FH2"/>
+      <c r="FI2"/>
+      <c r="FJ2"/>
+      <c r="FK2"/>
+      <c r="FL2"/>
+      <c r="FM2"/>
+      <c r="FN2"/>
+      <c r="FO2"/>
+      <c r="FP2"/>
+      <c r="FQ2"/>
+      <c r="FR2"/>
+      <c r="FS2"/>
+      <c r="FT2"/>
+      <c r="FU2"/>
+      <c r="FV2"/>
+      <c r="FW2"/>
+      <c r="FX2"/>
+      <c r="FY2"/>
+      <c r="FZ2"/>
+      <c r="GA2"/>
+      <c r="GB2"/>
+      <c r="GC2"/>
+      <c r="GD2"/>
+      <c r="GE2"/>
+      <c r="GF2"/>
+      <c r="GG2"/>
+      <c r="GH2"/>
+      <c r="GI2"/>
+      <c r="GJ2"/>
+      <c r="GK2"/>
+      <c r="GL2"/>
+      <c r="GM2"/>
+      <c r="GN2"/>
+      <c r="GO2"/>
+      <c r="GP2"/>
+      <c r="GQ2"/>
+      <c r="GR2"/>
+      <c r="GS2"/>
+      <c r="GT2"/>
+      <c r="GU2"/>
+      <c r="GV2"/>
+      <c r="GW2"/>
+      <c r="GX2"/>
+      <c r="GY2"/>
+      <c r="GZ2"/>
+      <c r="HA2"/>
+      <c r="HB2"/>
+      <c r="HC2"/>
+      <c r="HD2"/>
+      <c r="HE2"/>
+      <c r="HF2"/>
+      <c r="HG2"/>
+      <c r="HH2"/>
+      <c r="HI2"/>
+      <c r="HJ2"/>
+      <c r="HK2"/>
+      <c r="HL2"/>
+      <c r="HM2"/>
+      <c r="HN2"/>
+      <c r="HO2"/>
+      <c r="HP2"/>
+      <c r="HQ2"/>
+      <c r="HR2"/>
+      <c r="HS2"/>
+      <c r="HT2"/>
+      <c r="HU2"/>
+    </row>
+    <row r="3" spans="1:229" x14ac:dyDescent="0.35">
+      <c r="A3" s="3" t="s">
+        <v>610</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>611</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>612</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>201</v>
+      </c>
+      <c r="F3" s="3" t="s">
+        <v>202</v>
+      </c>
+      <c r="G3" s="3" t="s">
+        <v>211</v>
+      </c>
+      <c r="H3" s="3" t="s">
+        <v>613</v>
+      </c>
+    </row>
+    <row r="4" spans="1:229" x14ac:dyDescent="0.35">
+      <c r="A4" s="3" t="s">
+        <v>614</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>615</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>616</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>201</v>
+      </c>
+      <c r="F4" s="3" t="s">
+        <v>202</v>
+      </c>
+      <c r="G4" s="3" t="s">
+        <v>211</v>
+      </c>
+      <c r="H4" s="3" t="s">
+        <v>617</v>
+      </c>
+    </row>
+    <row r="5" spans="1:229" x14ac:dyDescent="0.35">
+      <c r="A5" s="3" t="s">
+        <v>618</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>619</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>620</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>201</v>
+      </c>
+      <c r="F5" s="3" t="s">
+        <v>202</v>
+      </c>
+      <c r="G5" s="3" t="s">
+        <v>211</v>
+      </c>
+      <c r="H5" s="3" t="s">
+        <v>621</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Added test cases for Higher Education Workforce Subcategory page US#134
</commit_message>
<xml_diff>
--- a/testdata.xlsx
+++ b/testdata.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sshiwani\workspace\find-information-products-services-tests\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6DC67814-7EC6-4595-B980-9CA1061BB621}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C3998CDD-2D0D-4FE1-90F0-EC349A662F70}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="22780" windowHeight="14540" firstSheet="18" activeTab="19" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="22780" windowHeight="14540" firstSheet="19" activeTab="20" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="category_phase" sheetId="1" r:id="rId1"/>
@@ -33,22 +33,24 @@
     <sheet name="UG_EPEYAltProvSetWorkforce_list" sheetId="32" r:id="rId18"/>
     <sheet name="UG_EPEYEarlyYearsWorkforce_list" sheetId="35" r:id="rId19"/>
     <sheet name="UG_EPEYFurtherEduWorkforce_list" sheetId="37" r:id="rId20"/>
-    <sheet name="UGSubcategory_AdultLearner" sheetId="16" r:id="rId21"/>
-    <sheet name="UGSubcategory_CareersAdviser" sheetId="17" r:id="rId22"/>
-    <sheet name="UGSubcategory_ChildOrYoungPers" sheetId="18" r:id="rId23"/>
-    <sheet name="UGSubcategory_DfEWorkforce" sheetId="19" r:id="rId24"/>
-    <sheet name="UGSubcategory_Employer" sheetId="20" r:id="rId25"/>
-    <sheet name="UGSubcategory_LAWorkforce" sheetId="21" r:id="rId26"/>
-    <sheet name="UGSubcategory_NEETOrCareerSeek" sheetId="22" r:id="rId27"/>
-    <sheet name="UGSubcategory_ParentOrCarer" sheetId="23" r:id="rId28"/>
-    <sheet name="UGSubcateg_ProfExtUserofDfEData" sheetId="24" r:id="rId29"/>
-    <sheet name="UGSubcategory_SCWorkforce" sheetId="25" r:id="rId30"/>
-    <sheet name="UGSubcategory_SocialWorker" sheetId="27" r:id="rId31"/>
-    <sheet name="UGSubcategory_EPandEYWorkforce" sheetId="29" r:id="rId32"/>
-    <sheet name="EPEYSubcateg_AcademyTWorkforce" sheetId="31" r:id="rId33"/>
-    <sheet name="EPEYSubcateg_AltProSetWorkforce" sheetId="33" r:id="rId34"/>
-    <sheet name="EPEYSubcatg_EarlyYearsWorkforce" sheetId="34" r:id="rId35"/>
-    <sheet name="EPEYSubcatg_FurtherEduWorkforce" sheetId="36" r:id="rId36"/>
+    <sheet name="UG_EPEYHigherEduWorkforce_list" sheetId="38" r:id="rId21"/>
+    <sheet name="UGSubcategory_AdultLearner" sheetId="16" r:id="rId22"/>
+    <sheet name="UGSubcategory_CareersAdviser" sheetId="17" r:id="rId23"/>
+    <sheet name="UGSubcategory_ChildOrYoungPers" sheetId="18" r:id="rId24"/>
+    <sheet name="UGSubcategory_DfEWorkforce" sheetId="19" r:id="rId25"/>
+    <sheet name="UGSubcategory_Employer" sheetId="20" r:id="rId26"/>
+    <sheet name="UGSubcategory_LAWorkforce" sheetId="21" r:id="rId27"/>
+    <sheet name="UGSubcategory_NEETOrCareerSeek" sheetId="22" r:id="rId28"/>
+    <sheet name="UGSubcategory_ParentOrCarer" sheetId="23" r:id="rId29"/>
+    <sheet name="UGSubcateg_ProfExtUserofDfEData" sheetId="24" r:id="rId30"/>
+    <sheet name="UGSubcategory_SCWorkforce" sheetId="25" r:id="rId31"/>
+    <sheet name="UGSubcategory_SocialWorker" sheetId="27" r:id="rId32"/>
+    <sheet name="UGSubcategory_EPandEYWorkforce" sheetId="29" r:id="rId33"/>
+    <sheet name="EPEYSubcateg_AcademyTWorkforce" sheetId="31" r:id="rId34"/>
+    <sheet name="EPEYSubcateg_AltProSetWorkforce" sheetId="33" r:id="rId35"/>
+    <sheet name="EPEYSubcatg_EarlyYearsWorkforce" sheetId="34" r:id="rId36"/>
+    <sheet name="EPEYSubcatg_FurtherEduWorkforce" sheetId="36" r:id="rId37"/>
+    <sheet name="EPEYSubcatg_HigherEduWorkforce" sheetId="39" r:id="rId38"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -60,7 +62,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1308" uniqueCount="622">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1362" uniqueCount="643">
   <si>
     <t>Search and filter products and services</t>
   </si>
@@ -1926,6 +1928,69 @@
   </si>
   <si>
     <t>Lecturer (further education)  (Further education workforce)</t>
+  </si>
+  <si>
+    <t>categories/user-group/education-provider-and-early-years-workforce/higher-education-workforce</t>
+  </si>
+  <si>
+    <t>Browse products in Higher education workforce</t>
+  </si>
+  <si>
+    <t>Lecturer (higher education)</t>
+  </si>
+  <si>
+    <t>University leader</t>
+  </si>
+  <si>
+    <t>University support staff</t>
+  </si>
+  <si>
+    <t>products?userGroup=higher-education-workforce</t>
+  </si>
+  <si>
+    <t>ul.moj-filter-tags li a:has-text(' Higher education workforce  (Education provider and early years workforce)')</t>
+  </si>
+  <si>
+    <t>Remove this filter Higher education workforce  (Education provider and early years workforce)</t>
+  </si>
+  <si>
+    <t>Higher education workforce  (Education provider and early years workforce)</t>
+  </si>
+  <si>
+    <t>products?userGroup=lecturer-higher-education</t>
+  </si>
+  <si>
+    <t>ul.moj-filter-tags li a:has-text(' Lecturer (higher education) ')</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Remove this filter Lecturer (higher education) </t>
+  </si>
+  <si>
+    <t>Lecturer (higher education)  (Higher education workforce)</t>
+  </si>
+  <si>
+    <t>ul.moj-filter-tags li a:has-text(' University leader ')</t>
+  </si>
+  <si>
+    <t>products?userGroup=university-leader</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Remove this filter University leader </t>
+  </si>
+  <si>
+    <t>University leader  (Higher education workforce)</t>
+  </si>
+  <si>
+    <t>products?userGroup=university-support-staff</t>
+  </si>
+  <si>
+    <t>ul.moj-filter-tags li a:has-text(' University support staff  (Higher education workforce)')</t>
+  </si>
+  <si>
+    <t>Remove this filter University support staff  (Higher education workforce)</t>
+  </si>
+  <si>
+    <t>University support staff  (Higher education workforce)</t>
   </si>
 </sst>
 </file>
@@ -12961,6 +13026,87 @@
 </file>
 
 <file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F8566466-31D4-4316-960A-E75B8AD62D44}">
+  <dimension ref="A1:C8"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="54.1796875" customWidth="1"/>
+    <col min="2" max="2" width="47.453125" customWidth="1"/>
+    <col min="3" max="3" width="50.36328125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A1" s="6" t="s">
+        <v>102</v>
+      </c>
+      <c r="B1" s="6" t="s">
+        <v>103</v>
+      </c>
+      <c r="C1" s="6" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A2" s="3" t="s">
+        <v>622</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>107</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>623</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="B3" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="B4" s="3" t="s">
+        <v>113</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A5" s="3" t="s">
+        <v>145</v>
+      </c>
+      <c r="B5" s="3"/>
+      <c r="C5" s="3"/>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A6" s="3" t="s">
+        <v>624</v>
+      </c>
+      <c r="B6" s="3"/>
+      <c r="C6" s="3"/>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A7" s="3" t="s">
+        <v>625</v>
+      </c>
+      <c r="B7" s="3"/>
+      <c r="C7" s="3"/>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A8" s="3" t="s">
+        <v>626</v>
+      </c>
+      <c r="B8" s="3"/>
+      <c r="C8" s="3"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FB5527F7-85DB-4F8E-B4B3-EC8453E599E1}">
   <dimension ref="A1:HU6"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -13358,7 +13504,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A99CF6C3-F305-48A2-AB80-2C2D7CE6460C}">
   <dimension ref="A1:HU5"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -13729,7 +13875,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5EFF0597-7FD1-4E6A-AA71-DB9F9FAB97A9}">
   <dimension ref="A1:HU7"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -14153,7 +14299,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9F4A57AC-4620-4875-88AE-9F5C739A9042}">
   <dimension ref="A1:HU6"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -14550,7 +14696,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6C1C130F-0899-4810-82F6-950C9CB07234}">
   <dimension ref="A1:HU5"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -14921,7 +15067,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4AB9395B-D522-49AD-B790-5334356249F6}">
   <dimension ref="A1:HU7"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -15344,7 +15490,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BEE91763-AD0C-4544-A433-3B50C88AEB79}">
   <dimension ref="A1:HU7"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -15767,7 +15913,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet29.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{20DD36AA-F163-4AAB-BD30-4AE6290CCAE7}">
   <dimension ref="A1:HU10"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -16261,456 +16407,6 @@
       </c>
       <c r="H10" s="3" t="s">
         <v>389</v>
-      </c>
-    </row>
-  </sheetData>
-  <phoneticPr fontId="1" type="noConversion"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet29.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C6EE6111-FDB3-4B43-8820-BBF68AAFCD6D}">
-  <dimension ref="A1:HU8"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
-  <cols>
-    <col min="1" max="1" width="50.90625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="52.26953125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="42.453125" customWidth="1"/>
-    <col min="4" max="4" width="33.36328125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="33.08984375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="17.08984375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="40.81640625" customWidth="1"/>
-    <col min="8" max="8" width="62.54296875" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:229" x14ac:dyDescent="0.35">
-      <c r="A1" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="F1" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="G1" s="2" t="s">
-        <v>209</v>
-      </c>
-      <c r="H1" s="2" t="s">
-        <v>210</v>
-      </c>
-    </row>
-    <row r="2" spans="1:229" s="4" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="3" t="s">
-        <v>390</v>
-      </c>
-      <c r="B2" s="3" t="s">
-        <v>391</v>
-      </c>
-      <c r="C2" s="3" t="s">
-        <v>392</v>
-      </c>
-      <c r="D2" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="E2" s="3" t="s">
-        <v>201</v>
-      </c>
-      <c r="F2" s="3" t="s">
-        <v>202</v>
-      </c>
-      <c r="G2" s="3" t="s">
-        <v>211</v>
-      </c>
-      <c r="H2" s="3" t="s">
-        <v>183</v>
-      </c>
-      <c r="I2"/>
-      <c r="J2"/>
-      <c r="K2"/>
-      <c r="L2"/>
-      <c r="M2"/>
-      <c r="N2"/>
-      <c r="O2"/>
-      <c r="P2"/>
-      <c r="Q2"/>
-      <c r="R2"/>
-      <c r="S2"/>
-      <c r="T2"/>
-      <c r="U2"/>
-      <c r="V2"/>
-      <c r="W2"/>
-      <c r="X2"/>
-      <c r="Y2"/>
-      <c r="Z2"/>
-      <c r="AA2"/>
-      <c r="AB2"/>
-      <c r="AC2"/>
-      <c r="AD2"/>
-      <c r="AE2"/>
-      <c r="AF2"/>
-      <c r="AG2"/>
-      <c r="AH2"/>
-      <c r="AI2"/>
-      <c r="AJ2"/>
-      <c r="AK2"/>
-      <c r="AL2"/>
-      <c r="AM2"/>
-      <c r="AN2"/>
-      <c r="AO2"/>
-      <c r="AP2"/>
-      <c r="AQ2"/>
-      <c r="AR2"/>
-      <c r="AS2"/>
-      <c r="AT2"/>
-      <c r="AU2"/>
-      <c r="AV2"/>
-      <c r="AW2"/>
-      <c r="AX2"/>
-      <c r="AY2"/>
-      <c r="AZ2"/>
-      <c r="BA2"/>
-      <c r="BB2"/>
-      <c r="BC2"/>
-      <c r="BD2"/>
-      <c r="BE2"/>
-      <c r="BF2"/>
-      <c r="BG2"/>
-      <c r="BH2"/>
-      <c r="BI2"/>
-      <c r="BJ2"/>
-      <c r="BK2"/>
-      <c r="BL2"/>
-      <c r="BM2"/>
-      <c r="BN2"/>
-      <c r="BO2"/>
-      <c r="BP2"/>
-      <c r="BQ2"/>
-      <c r="BR2"/>
-      <c r="BS2"/>
-      <c r="BT2"/>
-      <c r="BU2"/>
-      <c r="BV2"/>
-      <c r="BW2"/>
-      <c r="BX2"/>
-      <c r="BY2"/>
-      <c r="BZ2"/>
-      <c r="CA2"/>
-      <c r="CB2"/>
-      <c r="CC2"/>
-      <c r="CD2"/>
-      <c r="CE2"/>
-      <c r="CF2"/>
-      <c r="CG2"/>
-      <c r="CH2"/>
-      <c r="CI2"/>
-      <c r="CJ2"/>
-      <c r="CK2"/>
-      <c r="CL2"/>
-      <c r="CM2"/>
-      <c r="CN2"/>
-      <c r="CO2"/>
-      <c r="CP2"/>
-      <c r="CQ2"/>
-      <c r="CR2"/>
-      <c r="CS2"/>
-      <c r="CT2"/>
-      <c r="CU2"/>
-      <c r="CV2"/>
-      <c r="CW2"/>
-      <c r="CX2"/>
-      <c r="CY2"/>
-      <c r="CZ2"/>
-      <c r="DA2"/>
-      <c r="DB2"/>
-      <c r="DC2"/>
-      <c r="DD2"/>
-      <c r="DE2"/>
-      <c r="DF2"/>
-      <c r="DG2"/>
-      <c r="DH2"/>
-      <c r="DI2"/>
-      <c r="DJ2"/>
-      <c r="DK2"/>
-      <c r="DL2"/>
-      <c r="DM2"/>
-      <c r="DN2"/>
-      <c r="DO2"/>
-      <c r="DP2"/>
-      <c r="DQ2"/>
-      <c r="DR2"/>
-      <c r="DS2"/>
-      <c r="DT2"/>
-      <c r="DU2"/>
-      <c r="DV2"/>
-      <c r="DW2"/>
-      <c r="DX2"/>
-      <c r="DY2"/>
-      <c r="DZ2"/>
-      <c r="EA2"/>
-      <c r="EB2"/>
-      <c r="EC2"/>
-      <c r="ED2"/>
-      <c r="EE2"/>
-      <c r="EF2"/>
-      <c r="EG2"/>
-      <c r="EH2"/>
-      <c r="EI2"/>
-      <c r="EJ2"/>
-      <c r="EK2"/>
-      <c r="EL2"/>
-      <c r="EM2"/>
-      <c r="EN2"/>
-      <c r="EO2"/>
-      <c r="EP2"/>
-      <c r="EQ2"/>
-      <c r="ER2"/>
-      <c r="ES2"/>
-      <c r="ET2"/>
-      <c r="EU2"/>
-      <c r="EV2"/>
-      <c r="EW2"/>
-      <c r="EX2"/>
-      <c r="EY2"/>
-      <c r="EZ2"/>
-      <c r="FA2"/>
-      <c r="FB2"/>
-      <c r="FC2"/>
-      <c r="FD2"/>
-      <c r="FE2"/>
-      <c r="FF2"/>
-      <c r="FG2"/>
-      <c r="FH2"/>
-      <c r="FI2"/>
-      <c r="FJ2"/>
-      <c r="FK2"/>
-      <c r="FL2"/>
-      <c r="FM2"/>
-      <c r="FN2"/>
-      <c r="FO2"/>
-      <c r="FP2"/>
-      <c r="FQ2"/>
-      <c r="FR2"/>
-      <c r="FS2"/>
-      <c r="FT2"/>
-      <c r="FU2"/>
-      <c r="FV2"/>
-      <c r="FW2"/>
-      <c r="FX2"/>
-      <c r="FY2"/>
-      <c r="FZ2"/>
-      <c r="GA2"/>
-      <c r="GB2"/>
-      <c r="GC2"/>
-      <c r="GD2"/>
-      <c r="GE2"/>
-      <c r="GF2"/>
-      <c r="GG2"/>
-      <c r="GH2"/>
-      <c r="GI2"/>
-      <c r="GJ2"/>
-      <c r="GK2"/>
-      <c r="GL2"/>
-      <c r="GM2"/>
-      <c r="GN2"/>
-      <c r="GO2"/>
-      <c r="GP2"/>
-      <c r="GQ2"/>
-      <c r="GR2"/>
-      <c r="GS2"/>
-      <c r="GT2"/>
-      <c r="GU2"/>
-      <c r="GV2"/>
-      <c r="GW2"/>
-      <c r="GX2"/>
-      <c r="GY2"/>
-      <c r="GZ2"/>
-      <c r="HA2"/>
-      <c r="HB2"/>
-      <c r="HC2"/>
-      <c r="HD2"/>
-      <c r="HE2"/>
-      <c r="HF2"/>
-      <c r="HG2"/>
-      <c r="HH2"/>
-      <c r="HI2"/>
-      <c r="HJ2"/>
-      <c r="HK2"/>
-      <c r="HL2"/>
-      <c r="HM2"/>
-      <c r="HN2"/>
-      <c r="HO2"/>
-      <c r="HP2"/>
-      <c r="HQ2"/>
-      <c r="HR2"/>
-      <c r="HS2"/>
-      <c r="HT2"/>
-      <c r="HU2"/>
-    </row>
-    <row r="3" spans="1:229" x14ac:dyDescent="0.35">
-      <c r="A3" s="3" t="s">
-        <v>393</v>
-      </c>
-      <c r="B3" s="3" t="s">
-        <v>394</v>
-      </c>
-      <c r="C3" s="3" t="s">
-        <v>395</v>
-      </c>
-      <c r="D3" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="E3" s="3" t="s">
-        <v>201</v>
-      </c>
-      <c r="F3" s="3" t="s">
-        <v>202</v>
-      </c>
-      <c r="G3" s="3" t="s">
-        <v>211</v>
-      </c>
-      <c r="H3" s="3" t="s">
-        <v>396</v>
-      </c>
-    </row>
-    <row r="4" spans="1:229" x14ac:dyDescent="0.35">
-      <c r="A4" s="3" t="s">
-        <v>397</v>
-      </c>
-      <c r="B4" s="3" t="s">
-        <v>398</v>
-      </c>
-      <c r="C4" s="3" t="s">
-        <v>399</v>
-      </c>
-      <c r="D4" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="E4" s="3" t="s">
-        <v>201</v>
-      </c>
-      <c r="F4" s="3" t="s">
-        <v>202</v>
-      </c>
-      <c r="G4" s="3" t="s">
-        <v>211</v>
-      </c>
-      <c r="H4" s="3" t="s">
-        <v>400</v>
-      </c>
-    </row>
-    <row r="5" spans="1:229" x14ac:dyDescent="0.35">
-      <c r="A5" s="8" t="s">
-        <v>401</v>
-      </c>
-      <c r="B5" s="8" t="s">
-        <v>402</v>
-      </c>
-      <c r="C5" s="8" t="s">
-        <v>403</v>
-      </c>
-      <c r="D5" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="E5" s="3" t="s">
-        <v>201</v>
-      </c>
-      <c r="F5" s="3" t="s">
-        <v>202</v>
-      </c>
-      <c r="G5" s="3" t="s">
-        <v>211</v>
-      </c>
-      <c r="H5" s="3" t="s">
-        <v>404</v>
-      </c>
-    </row>
-    <row r="6" spans="1:229" x14ac:dyDescent="0.35">
-      <c r="A6" s="3" t="s">
-        <v>405</v>
-      </c>
-      <c r="B6" s="3" t="s">
-        <v>406</v>
-      </c>
-      <c r="C6" s="3" t="s">
-        <v>407</v>
-      </c>
-      <c r="D6" s="7" t="s">
-        <v>0</v>
-      </c>
-      <c r="E6" s="3" t="s">
-        <v>201</v>
-      </c>
-      <c r="F6" s="3" t="s">
-        <v>202</v>
-      </c>
-      <c r="G6" s="3" t="s">
-        <v>211</v>
-      </c>
-      <c r="H6" s="3" t="s">
-        <v>408</v>
-      </c>
-    </row>
-    <row r="7" spans="1:229" x14ac:dyDescent="0.35">
-      <c r="A7" s="3" t="s">
-        <v>409</v>
-      </c>
-      <c r="B7" s="3" t="s">
-        <v>410</v>
-      </c>
-      <c r="C7" s="3" t="s">
-        <v>411</v>
-      </c>
-      <c r="D7" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="E7" s="3" t="s">
-        <v>201</v>
-      </c>
-      <c r="F7" s="3" t="s">
-        <v>202</v>
-      </c>
-      <c r="G7" s="3" t="s">
-        <v>211</v>
-      </c>
-      <c r="H7" s="3" t="s">
-        <v>412</v>
-      </c>
-    </row>
-    <row r="8" spans="1:229" x14ac:dyDescent="0.35">
-      <c r="A8" s="9" t="s">
-        <v>413</v>
-      </c>
-      <c r="B8" s="9" t="s">
-        <v>414</v>
-      </c>
-      <c r="C8" s="9" t="s">
-        <v>415</v>
-      </c>
-      <c r="D8" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="E8" s="3" t="s">
-        <v>201</v>
-      </c>
-      <c r="F8" s="3" t="s">
-        <v>202</v>
-      </c>
-      <c r="G8" s="3" t="s">
-        <v>211</v>
-      </c>
-      <c r="H8" s="9" t="s">
-        <v>416</v>
       </c>
     </row>
   </sheetData>
@@ -19024,8 +18720,8 @@
 </file>
 
 <file path=xl/worksheets/sheet30.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E6428663-7558-48F1-8CD3-947F03FFD4CC}">
-  <dimension ref="A1:HU9"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C6EE6111-FDB3-4B43-8820-BBF68AAFCD6D}">
+  <dimension ref="A1:HU8"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="50.90625" bestFit="1" customWidth="1"/>
@@ -19035,7 +18731,7 @@
     <col min="5" max="5" width="33.08984375" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="17.08984375" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="40.81640625" customWidth="1"/>
-    <col min="8" max="8" width="57.08984375" customWidth="1"/>
+    <col min="8" max="8" width="62.54296875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:229" x14ac:dyDescent="0.35">
@@ -19066,13 +18762,13 @@
     </row>
     <row r="2" spans="1:229" s="4" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A2" s="3" t="s">
-        <v>457</v>
+        <v>390</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>458</v>
+        <v>391</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>459</v>
+        <v>392</v>
       </c>
       <c r="D2" s="3" t="s">
         <v>0</v>
@@ -19087,7 +18783,7 @@
         <v>211</v>
       </c>
       <c r="H2" s="3" t="s">
-        <v>192</v>
+        <v>183</v>
       </c>
       <c r="I2"/>
       <c r="J2"/>
@@ -19313,13 +19009,13 @@
     </row>
     <row r="3" spans="1:229" x14ac:dyDescent="0.35">
       <c r="A3" s="3" t="s">
-        <v>460</v>
+        <v>393</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>461</v>
+        <v>394</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>462</v>
+        <v>395</v>
       </c>
       <c r="D3" s="3" t="s">
         <v>0</v>
@@ -19334,18 +19030,18 @@
         <v>211</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>463</v>
+        <v>396</v>
       </c>
     </row>
     <row r="4" spans="1:229" x14ac:dyDescent="0.35">
       <c r="A4" s="3" t="s">
-        <v>464</v>
+        <v>397</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>467</v>
+        <v>398</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>465</v>
+        <v>399</v>
       </c>
       <c r="D4" s="3" t="s">
         <v>0</v>
@@ -19360,18 +19056,18 @@
         <v>211</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>466</v>
+        <v>400</v>
       </c>
     </row>
     <row r="5" spans="1:229" x14ac:dyDescent="0.35">
       <c r="A5" s="8" t="s">
-        <v>468</v>
+        <v>401</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>469</v>
+        <v>402</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>470</v>
+        <v>403</v>
       </c>
       <c r="D5" s="3" t="s">
         <v>0</v>
@@ -19386,18 +19082,18 @@
         <v>211</v>
       </c>
       <c r="H5" s="3" t="s">
-        <v>471</v>
+        <v>404</v>
       </c>
     </row>
     <row r="6" spans="1:229" x14ac:dyDescent="0.35">
       <c r="A6" s="3" t="s">
-        <v>473</v>
+        <v>405</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>472</v>
+        <v>406</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>474</v>
+        <v>407</v>
       </c>
       <c r="D6" s="7" t="s">
         <v>0</v>
@@ -19412,18 +19108,18 @@
         <v>211</v>
       </c>
       <c r="H6" s="3" t="s">
-        <v>475</v>
+        <v>408</v>
       </c>
     </row>
     <row r="7" spans="1:229" x14ac:dyDescent="0.35">
       <c r="A7" s="3" t="s">
-        <v>476</v>
+        <v>409</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>477</v>
+        <v>410</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>478</v>
+        <v>411</v>
       </c>
       <c r="D7" s="3" t="s">
         <v>0</v>
@@ -19438,18 +19134,18 @@
         <v>211</v>
       </c>
       <c r="H7" s="3" t="s">
-        <v>479</v>
+        <v>412</v>
       </c>
     </row>
     <row r="8" spans="1:229" x14ac:dyDescent="0.35">
-      <c r="A8" s="3" t="s">
-        <v>480</v>
-      </c>
-      <c r="B8" s="3" t="s">
-        <v>481</v>
-      </c>
-      <c r="C8" s="3" t="s">
-        <v>482</v>
+      <c r="A8" s="9" t="s">
+        <v>413</v>
+      </c>
+      <c r="B8" s="9" t="s">
+        <v>414</v>
+      </c>
+      <c r="C8" s="9" t="s">
+        <v>415</v>
       </c>
       <c r="D8" s="3" t="s">
         <v>0</v>
@@ -19463,34 +19159,8 @@
       <c r="G8" s="3" t="s">
         <v>211</v>
       </c>
-      <c r="H8" s="3" t="s">
-        <v>483</v>
-      </c>
-    </row>
-    <row r="9" spans="1:229" x14ac:dyDescent="0.35">
-      <c r="A9" s="3" t="s">
-        <v>484</v>
-      </c>
-      <c r="B9" s="3" t="s">
-        <v>485</v>
-      </c>
-      <c r="C9" s="3" t="s">
-        <v>486</v>
-      </c>
-      <c r="D9" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="E9" s="3" t="s">
-        <v>201</v>
-      </c>
-      <c r="F9" s="3" t="s">
-        <v>202</v>
-      </c>
-      <c r="G9" s="3" t="s">
-        <v>211</v>
-      </c>
-      <c r="H9" s="3" t="s">
-        <v>487</v>
+      <c r="H8" s="9" t="s">
+        <v>416</v>
       </c>
     </row>
   </sheetData>
@@ -19500,8 +19170,8 @@
 </file>
 
 <file path=xl/worksheets/sheet31.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2A4E3580-B709-4E66-9F6E-B7F9948D7FD3}">
-  <dimension ref="A1:HU7"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E6428663-7558-48F1-8CD3-947F03FFD4CC}">
+  <dimension ref="A1:HU9"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="50.90625" bestFit="1" customWidth="1"/>
@@ -19542,13 +19212,13 @@
     </row>
     <row r="2" spans="1:229" s="4" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A2" s="3" t="s">
-        <v>488</v>
+        <v>457</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>489</v>
+        <v>458</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>490</v>
+        <v>459</v>
       </c>
       <c r="D2" s="3" t="s">
         <v>0</v>
@@ -19563,7 +19233,7 @@
         <v>211</v>
       </c>
       <c r="H2" s="3" t="s">
-        <v>491</v>
+        <v>192</v>
       </c>
       <c r="I2"/>
       <c r="J2"/>
@@ -19789,13 +19459,13 @@
     </row>
     <row r="3" spans="1:229" x14ac:dyDescent="0.35">
       <c r="A3" s="3" t="s">
-        <v>492</v>
+        <v>460</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>493</v>
+        <v>461</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>494</v>
+        <v>462</v>
       </c>
       <c r="D3" s="3" t="s">
         <v>0</v>
@@ -19810,18 +19480,18 @@
         <v>211</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>495</v>
+        <v>463</v>
       </c>
     </row>
     <row r="4" spans="1:229" x14ac:dyDescent="0.35">
       <c r="A4" s="3" t="s">
-        <v>496</v>
+        <v>464</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>497</v>
+        <v>467</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>498</v>
+        <v>465</v>
       </c>
       <c r="D4" s="3" t="s">
         <v>0</v>
@@ -19836,18 +19506,18 @@
         <v>211</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>499</v>
+        <v>466</v>
       </c>
     </row>
     <row r="5" spans="1:229" x14ac:dyDescent="0.35">
       <c r="A5" s="8" t="s">
-        <v>500</v>
+        <v>468</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>501</v>
+        <v>469</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>502</v>
+        <v>470</v>
       </c>
       <c r="D5" s="3" t="s">
         <v>0</v>
@@ -19862,18 +19532,18 @@
         <v>211</v>
       </c>
       <c r="H5" s="3" t="s">
-        <v>503</v>
+        <v>471</v>
       </c>
     </row>
     <row r="6" spans="1:229" x14ac:dyDescent="0.35">
       <c r="A6" s="3" t="s">
-        <v>504</v>
+        <v>473</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>505</v>
+        <v>472</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>506</v>
+        <v>474</v>
       </c>
       <c r="D6" s="7" t="s">
         <v>0</v>
@@ -19888,18 +19558,18 @@
         <v>211</v>
       </c>
       <c r="H6" s="3" t="s">
-        <v>507</v>
+        <v>475</v>
       </c>
     </row>
     <row r="7" spans="1:229" x14ac:dyDescent="0.35">
       <c r="A7" s="3" t="s">
-        <v>509</v>
+        <v>476</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>508</v>
+        <v>477</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>510</v>
+        <v>478</v>
       </c>
       <c r="D7" s="3" t="s">
         <v>0</v>
@@ -19914,17 +19584,70 @@
         <v>211</v>
       </c>
       <c r="H7" s="3" t="s">
-        <v>511</v>
+        <v>479</v>
+      </c>
+    </row>
+    <row r="8" spans="1:229" x14ac:dyDescent="0.35">
+      <c r="A8" s="3" t="s">
+        <v>480</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>481</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>482</v>
+      </c>
+      <c r="D8" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="E8" s="3" t="s">
+        <v>201</v>
+      </c>
+      <c r="F8" s="3" t="s">
+        <v>202</v>
+      </c>
+      <c r="G8" s="3" t="s">
+        <v>211</v>
+      </c>
+      <c r="H8" s="3" t="s">
+        <v>483</v>
+      </c>
+    </row>
+    <row r="9" spans="1:229" x14ac:dyDescent="0.35">
+      <c r="A9" s="3" t="s">
+        <v>484</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>485</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>486</v>
+      </c>
+      <c r="D9" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="E9" s="3" t="s">
+        <v>201</v>
+      </c>
+      <c r="F9" s="3" t="s">
+        <v>202</v>
+      </c>
+      <c r="G9" s="3" t="s">
+        <v>211</v>
+      </c>
+      <c r="H9" s="3" t="s">
+        <v>487</v>
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet32.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{95706458-CD50-4C74-87C4-ABAE617927AD}">
-  <dimension ref="A1:HU2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2A4E3580-B709-4E66-9F6E-B7F9948D7FD3}">
+  <dimension ref="A1:HU7"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="50.90625" bestFit="1" customWidth="1"/>
@@ -19965,13 +19688,13 @@
     </row>
     <row r="2" spans="1:229" s="4" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A2" s="3" t="s">
-        <v>512</v>
+        <v>488</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>513</v>
+        <v>489</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>514</v>
+        <v>490</v>
       </c>
       <c r="D2" s="3" t="s">
         <v>0</v>
@@ -19986,7 +19709,7 @@
         <v>211</v>
       </c>
       <c r="H2" s="3" t="s">
-        <v>140</v>
+        <v>491</v>
       </c>
       <c r="I2"/>
       <c r="J2"/>
@@ -20210,14 +19933,144 @@
       <c r="HT2"/>
       <c r="HU2"/>
     </row>
+    <row r="3" spans="1:229" x14ac:dyDescent="0.35">
+      <c r="A3" s="3" t="s">
+        <v>492</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>493</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>494</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>201</v>
+      </c>
+      <c r="F3" s="3" t="s">
+        <v>202</v>
+      </c>
+      <c r="G3" s="3" t="s">
+        <v>211</v>
+      </c>
+      <c r="H3" s="3" t="s">
+        <v>495</v>
+      </c>
+    </row>
+    <row r="4" spans="1:229" x14ac:dyDescent="0.35">
+      <c r="A4" s="3" t="s">
+        <v>496</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>497</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>498</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>201</v>
+      </c>
+      <c r="F4" s="3" t="s">
+        <v>202</v>
+      </c>
+      <c r="G4" s="3" t="s">
+        <v>211</v>
+      </c>
+      <c r="H4" s="3" t="s">
+        <v>499</v>
+      </c>
+    </row>
+    <row r="5" spans="1:229" x14ac:dyDescent="0.35">
+      <c r="A5" s="8" t="s">
+        <v>500</v>
+      </c>
+      <c r="B5" s="8" t="s">
+        <v>501</v>
+      </c>
+      <c r="C5" s="8" t="s">
+        <v>502</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>201</v>
+      </c>
+      <c r="F5" s="3" t="s">
+        <v>202</v>
+      </c>
+      <c r="G5" s="3" t="s">
+        <v>211</v>
+      </c>
+      <c r="H5" s="3" t="s">
+        <v>503</v>
+      </c>
+    </row>
+    <row r="6" spans="1:229" x14ac:dyDescent="0.35">
+      <c r="A6" s="3" t="s">
+        <v>504</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>505</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>506</v>
+      </c>
+      <c r="D6" s="7" t="s">
+        <v>0</v>
+      </c>
+      <c r="E6" s="3" t="s">
+        <v>201</v>
+      </c>
+      <c r="F6" s="3" t="s">
+        <v>202</v>
+      </c>
+      <c r="G6" s="3" t="s">
+        <v>211</v>
+      </c>
+      <c r="H6" s="3" t="s">
+        <v>507</v>
+      </c>
+    </row>
+    <row r="7" spans="1:229" x14ac:dyDescent="0.35">
+      <c r="A7" s="3" t="s">
+        <v>509</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>508</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>510</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="E7" s="3" t="s">
+        <v>201</v>
+      </c>
+      <c r="F7" s="3" t="s">
+        <v>202</v>
+      </c>
+      <c r="G7" s="3" t="s">
+        <v>211</v>
+      </c>
+      <c r="H7" s="3" t="s">
+        <v>511</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet33.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1AD86191-7CFE-4ED9-9129-FF78170AB51E}">
-  <dimension ref="A1:HU12"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{95706458-CD50-4C74-87C4-ABAE617927AD}">
+  <dimension ref="A1:HU2"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="50.90625" bestFit="1" customWidth="1"/>
@@ -20227,7 +20080,7 @@
     <col min="5" max="5" width="33.08984375" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="17.08984375" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="40.81640625" customWidth="1"/>
-    <col min="8" max="8" width="65.54296875" customWidth="1"/>
+    <col min="8" max="8" width="57.08984375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:229" x14ac:dyDescent="0.35">
@@ -20258,13 +20111,13 @@
     </row>
     <row r="2" spans="1:229" s="4" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A2" s="3" t="s">
-        <v>527</v>
+        <v>512</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>528</v>
+        <v>513</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>529</v>
+        <v>514</v>
       </c>
       <c r="D2" s="3" t="s">
         <v>0</v>
@@ -20279,7 +20132,7 @@
         <v>211</v>
       </c>
       <c r="H2" s="3" t="s">
-        <v>530</v>
+        <v>140</v>
       </c>
       <c r="I2"/>
       <c r="J2"/>
@@ -20503,278 +20356,17 @@
       <c r="HT2"/>
       <c r="HU2"/>
     </row>
-    <row r="3" spans="1:229" x14ac:dyDescent="0.35">
-      <c r="A3" s="3" t="s">
-        <v>532</v>
-      </c>
-      <c r="B3" s="3" t="s">
-        <v>531</v>
-      </c>
-      <c r="C3" s="3" t="s">
-        <v>533</v>
-      </c>
-      <c r="D3" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="E3" s="3" t="s">
-        <v>201</v>
-      </c>
-      <c r="F3" s="3" t="s">
-        <v>202</v>
-      </c>
-      <c r="G3" s="3" t="s">
-        <v>211</v>
-      </c>
-      <c r="H3" s="3" t="s">
-        <v>534</v>
-      </c>
-    </row>
-    <row r="4" spans="1:229" x14ac:dyDescent="0.35">
-      <c r="A4" s="3" t="s">
-        <v>535</v>
-      </c>
-      <c r="B4" s="3" t="s">
-        <v>536</v>
-      </c>
-      <c r="C4" s="3" t="s">
-        <v>537</v>
-      </c>
-      <c r="D4" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="E4" s="3" t="s">
-        <v>201</v>
-      </c>
-      <c r="F4" s="3" t="s">
-        <v>202</v>
-      </c>
-      <c r="G4" s="3" t="s">
-        <v>211</v>
-      </c>
-      <c r="H4" s="3" t="s">
-        <v>538</v>
-      </c>
-    </row>
-    <row r="5" spans="1:229" x14ac:dyDescent="0.35">
-      <c r="A5" s="8" t="s">
-        <v>539</v>
-      </c>
-      <c r="B5" s="8" t="s">
-        <v>540</v>
-      </c>
-      <c r="C5" s="8" t="s">
-        <v>541</v>
-      </c>
-      <c r="D5" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="E5" s="3" t="s">
-        <v>201</v>
-      </c>
-      <c r="F5" s="3" t="s">
-        <v>202</v>
-      </c>
-      <c r="G5" s="3" t="s">
-        <v>211</v>
-      </c>
-      <c r="H5" s="3" t="s">
-        <v>542</v>
-      </c>
-    </row>
-    <row r="6" spans="1:229" x14ac:dyDescent="0.35">
-      <c r="A6" s="3" t="s">
-        <v>543</v>
-      </c>
-      <c r="B6" s="3" t="s">
-        <v>544</v>
-      </c>
-      <c r="C6" s="3" t="s">
-        <v>545</v>
-      </c>
-      <c r="D6" s="7" t="s">
-        <v>0</v>
-      </c>
-      <c r="E6" s="3" t="s">
-        <v>201</v>
-      </c>
-      <c r="F6" s="3" t="s">
-        <v>202</v>
-      </c>
-      <c r="G6" s="3" t="s">
-        <v>211</v>
-      </c>
-      <c r="H6" s="3" t="s">
-        <v>546</v>
-      </c>
-    </row>
-    <row r="7" spans="1:229" x14ac:dyDescent="0.35">
-      <c r="A7" s="3" t="s">
-        <v>547</v>
-      </c>
-      <c r="B7" s="3" t="s">
-        <v>548</v>
-      </c>
-      <c r="C7" s="3" t="s">
-        <v>549</v>
-      </c>
-      <c r="D7" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="E7" s="3" t="s">
-        <v>201</v>
-      </c>
-      <c r="F7" s="3" t="s">
-        <v>202</v>
-      </c>
-      <c r="G7" s="3" t="s">
-        <v>211</v>
-      </c>
-      <c r="H7" s="3" t="s">
-        <v>550</v>
-      </c>
-    </row>
-    <row r="8" spans="1:229" x14ac:dyDescent="0.35">
-      <c r="A8" s="3" t="s">
-        <v>551</v>
-      </c>
-      <c r="B8" s="3" t="s">
-        <v>552</v>
-      </c>
-      <c r="C8" s="3" t="s">
-        <v>553</v>
-      </c>
-      <c r="D8" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="E8" s="3" t="s">
-        <v>201</v>
-      </c>
-      <c r="F8" s="3" t="s">
-        <v>202</v>
-      </c>
-      <c r="G8" s="10" t="s">
-        <v>211</v>
-      </c>
-      <c r="H8" s="3" t="s">
-        <v>554</v>
-      </c>
-    </row>
-    <row r="9" spans="1:229" x14ac:dyDescent="0.35">
-      <c r="A9" s="3" t="s">
-        <v>555</v>
-      </c>
-      <c r="B9" s="3" t="s">
-        <v>556</v>
-      </c>
-      <c r="C9" s="3" t="s">
-        <v>558</v>
-      </c>
-      <c r="D9" s="7" t="s">
-        <v>0</v>
-      </c>
-      <c r="E9" s="3" t="s">
-        <v>201</v>
-      </c>
-      <c r="F9" s="3" t="s">
-        <v>202</v>
-      </c>
-      <c r="G9" s="10" t="s">
-        <v>211</v>
-      </c>
-      <c r="H9" s="3" t="s">
-        <v>557</v>
-      </c>
-    </row>
-    <row r="10" spans="1:229" x14ac:dyDescent="0.35">
-      <c r="A10" s="3" t="s">
-        <v>559</v>
-      </c>
-      <c r="B10" s="3" t="s">
-        <v>560</v>
-      </c>
-      <c r="C10" s="3" t="s">
-        <v>561</v>
-      </c>
-      <c r="D10" s="7" t="s">
-        <v>0</v>
-      </c>
-      <c r="E10" s="3" t="s">
-        <v>201</v>
-      </c>
-      <c r="F10" s="3" t="s">
-        <v>202</v>
-      </c>
-      <c r="G10" s="10" t="s">
-        <v>211</v>
-      </c>
-      <c r="H10" s="3" t="s">
-        <v>562</v>
-      </c>
-    </row>
-    <row r="11" spans="1:229" x14ac:dyDescent="0.35">
-      <c r="A11" s="3" t="s">
-        <v>563</v>
-      </c>
-      <c r="B11" s="3" t="s">
-        <v>564</v>
-      </c>
-      <c r="C11" s="3" t="s">
-        <v>565</v>
-      </c>
-      <c r="D11" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="E11" s="3" t="s">
-        <v>201</v>
-      </c>
-      <c r="F11" s="3" t="s">
-        <v>202</v>
-      </c>
-      <c r="G11" s="10" t="s">
-        <v>211</v>
-      </c>
-      <c r="H11" s="3" t="s">
-        <v>566</v>
-      </c>
-    </row>
-    <row r="12" spans="1:229" x14ac:dyDescent="0.35">
-      <c r="A12" s="3" t="s">
-        <v>567</v>
-      </c>
-      <c r="B12" s="3" t="s">
-        <v>568</v>
-      </c>
-      <c r="C12" s="3" t="s">
-        <v>569</v>
-      </c>
-      <c r="D12" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="E12" s="3" t="s">
-        <v>201</v>
-      </c>
-      <c r="F12" s="3" t="s">
-        <v>202</v>
-      </c>
-      <c r="G12" s="10" t="s">
-        <v>211</v>
-      </c>
-      <c r="H12" s="3" t="s">
-        <v>570</v>
-      </c>
-    </row>
   </sheetData>
-  <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet34.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{24EB34D0-BCF8-4F57-88CC-AC842687528F}">
-  <dimension ref="A1:HU5"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1AD86191-7CFE-4ED9-9129-FF78170AB51E}">
+  <dimension ref="A1:HU12"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="52.453125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="50.90625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="52.26953125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="42.453125" customWidth="1"/>
     <col min="4" max="4" width="33.36328125" bestFit="1" customWidth="1"/>
@@ -20812,13 +20404,13 @@
     </row>
     <row r="2" spans="1:229" s="4" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A2" s="3" t="s">
-        <v>576</v>
+        <v>527</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>577</v>
+        <v>528</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>578</v>
+        <v>529</v>
       </c>
       <c r="D2" s="3" t="s">
         <v>0</v>
@@ -20833,7 +20425,7 @@
         <v>211</v>
       </c>
       <c r="H2" s="3" t="s">
-        <v>579</v>
+        <v>530</v>
       </c>
       <c r="I2"/>
       <c r="J2"/>
@@ -21059,13 +20651,13 @@
     </row>
     <row r="3" spans="1:229" x14ac:dyDescent="0.35">
       <c r="A3" s="3" t="s">
-        <v>580</v>
+        <v>532</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>581</v>
+        <v>531</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>582</v>
+        <v>533</v>
       </c>
       <c r="D3" s="3" t="s">
         <v>0</v>
@@ -21080,42 +20672,44 @@
         <v>211</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>583</v>
+        <v>534</v>
       </c>
     </row>
     <row r="4" spans="1:229" x14ac:dyDescent="0.35">
-      <c r="A4" s="11" t="s">
-        <v>584</v>
-      </c>
-      <c r="B4" s="11" t="s">
-        <v>585</v>
-      </c>
-      <c r="C4" s="11" t="s">
-        <v>586</v>
-      </c>
-      <c r="D4" s="11" t="s">
+      <c r="A4" s="3" t="s">
+        <v>535</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>536</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>537</v>
+      </c>
+      <c r="D4" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="E4" s="11" t="s">
+      <c r="E4" s="3" t="s">
         <v>201</v>
       </c>
-      <c r="F4" s="11" t="s">
+      <c r="F4" s="3" t="s">
         <v>202</v>
       </c>
-      <c r="G4" s="11" t="s">
+      <c r="G4" s="3" t="s">
         <v>211</v>
       </c>
-      <c r="H4" s="11"/>
+      <c r="H4" s="3" t="s">
+        <v>538</v>
+      </c>
     </row>
     <row r="5" spans="1:229" x14ac:dyDescent="0.35">
-      <c r="A5" s="3" t="s">
-        <v>587</v>
-      </c>
-      <c r="B5" s="3" t="s">
-        <v>588</v>
-      </c>
-      <c r="C5" s="3" t="s">
-        <v>589</v>
+      <c r="A5" s="8" t="s">
+        <v>539</v>
+      </c>
+      <c r="B5" s="8" t="s">
+        <v>540</v>
+      </c>
+      <c r="C5" s="8" t="s">
+        <v>541</v>
       </c>
       <c r="D5" s="3" t="s">
         <v>0</v>
@@ -21130,17 +20724,200 @@
         <v>211</v>
       </c>
       <c r="H5" s="3" t="s">
-        <v>590</v>
+        <v>542</v>
+      </c>
+    </row>
+    <row r="6" spans="1:229" x14ac:dyDescent="0.35">
+      <c r="A6" s="3" t="s">
+        <v>543</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>544</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>545</v>
+      </c>
+      <c r="D6" s="7" t="s">
+        <v>0</v>
+      </c>
+      <c r="E6" s="3" t="s">
+        <v>201</v>
+      </c>
+      <c r="F6" s="3" t="s">
+        <v>202</v>
+      </c>
+      <c r="G6" s="3" t="s">
+        <v>211</v>
+      </c>
+      <c r="H6" s="3" t="s">
+        <v>546</v>
+      </c>
+    </row>
+    <row r="7" spans="1:229" x14ac:dyDescent="0.35">
+      <c r="A7" s="3" t="s">
+        <v>547</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>548</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>549</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="E7" s="3" t="s">
+        <v>201</v>
+      </c>
+      <c r="F7" s="3" t="s">
+        <v>202</v>
+      </c>
+      <c r="G7" s="3" t="s">
+        <v>211</v>
+      </c>
+      <c r="H7" s="3" t="s">
+        <v>550</v>
+      </c>
+    </row>
+    <row r="8" spans="1:229" x14ac:dyDescent="0.35">
+      <c r="A8" s="3" t="s">
+        <v>551</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>552</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>553</v>
+      </c>
+      <c r="D8" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="E8" s="3" t="s">
+        <v>201</v>
+      </c>
+      <c r="F8" s="3" t="s">
+        <v>202</v>
+      </c>
+      <c r="G8" s="10" t="s">
+        <v>211</v>
+      </c>
+      <c r="H8" s="3" t="s">
+        <v>554</v>
+      </c>
+    </row>
+    <row r="9" spans="1:229" x14ac:dyDescent="0.35">
+      <c r="A9" s="3" t="s">
+        <v>555</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>556</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>558</v>
+      </c>
+      <c r="D9" s="7" t="s">
+        <v>0</v>
+      </c>
+      <c r="E9" s="3" t="s">
+        <v>201</v>
+      </c>
+      <c r="F9" s="3" t="s">
+        <v>202</v>
+      </c>
+      <c r="G9" s="10" t="s">
+        <v>211</v>
+      </c>
+      <c r="H9" s="3" t="s">
+        <v>557</v>
+      </c>
+    </row>
+    <row r="10" spans="1:229" x14ac:dyDescent="0.35">
+      <c r="A10" s="3" t="s">
+        <v>559</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>560</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>561</v>
+      </c>
+      <c r="D10" s="7" t="s">
+        <v>0</v>
+      </c>
+      <c r="E10" s="3" t="s">
+        <v>201</v>
+      </c>
+      <c r="F10" s="3" t="s">
+        <v>202</v>
+      </c>
+      <c r="G10" s="10" t="s">
+        <v>211</v>
+      </c>
+      <c r="H10" s="3" t="s">
+        <v>562</v>
+      </c>
+    </row>
+    <row r="11" spans="1:229" x14ac:dyDescent="0.35">
+      <c r="A11" s="3" t="s">
+        <v>563</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>564</v>
+      </c>
+      <c r="C11" s="3" t="s">
+        <v>565</v>
+      </c>
+      <c r="D11" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="E11" s="3" t="s">
+        <v>201</v>
+      </c>
+      <c r="F11" s="3" t="s">
+        <v>202</v>
+      </c>
+      <c r="G11" s="10" t="s">
+        <v>211</v>
+      </c>
+      <c r="H11" s="3" t="s">
+        <v>566</v>
+      </c>
+    </row>
+    <row r="12" spans="1:229" x14ac:dyDescent="0.35">
+      <c r="A12" s="3" t="s">
+        <v>567</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>568</v>
+      </c>
+      <c r="C12" s="3" t="s">
+        <v>569</v>
+      </c>
+      <c r="D12" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="E12" s="3" t="s">
+        <v>201</v>
+      </c>
+      <c r="F12" s="3" t="s">
+        <v>202</v>
+      </c>
+      <c r="G12" s="10" t="s">
+        <v>211</v>
+      </c>
+      <c r="H12" s="3" t="s">
+        <v>570</v>
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet35.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7271F742-0542-4B33-AEE2-20AE8A69F475}">
-  <dimension ref="A1:HU3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{24EB34D0-BCF8-4F57-88CC-AC842687528F}">
+  <dimension ref="A1:HU5"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="52.453125" bestFit="1" customWidth="1"/>
@@ -21181,13 +20958,13 @@
     </row>
     <row r="2" spans="1:229" s="4" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A2" s="3" t="s">
-        <v>594</v>
+        <v>576</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>595</v>
+        <v>577</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>596</v>
+        <v>578</v>
       </c>
       <c r="D2" s="3" t="s">
         <v>0</v>
@@ -21202,7 +20979,7 @@
         <v>211</v>
       </c>
       <c r="H2" s="3" t="s">
-        <v>597</v>
+        <v>579</v>
       </c>
       <c r="I2"/>
       <c r="J2"/>
@@ -21428,13 +21205,13 @@
     </row>
     <row r="3" spans="1:229" x14ac:dyDescent="0.35">
       <c r="A3" s="3" t="s">
-        <v>598</v>
+        <v>580</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>599</v>
+        <v>581</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>600</v>
+        <v>582</v>
       </c>
       <c r="D3" s="3" t="s">
         <v>0</v>
@@ -21449,7 +21226,57 @@
         <v>211</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>601</v>
+        <v>583</v>
+      </c>
+    </row>
+    <row r="4" spans="1:229" x14ac:dyDescent="0.35">
+      <c r="A4" s="11" t="s">
+        <v>584</v>
+      </c>
+      <c r="B4" s="11" t="s">
+        <v>585</v>
+      </c>
+      <c r="C4" s="11" t="s">
+        <v>586</v>
+      </c>
+      <c r="D4" s="11" t="s">
+        <v>0</v>
+      </c>
+      <c r="E4" s="11" t="s">
+        <v>201</v>
+      </c>
+      <c r="F4" s="11" t="s">
+        <v>202</v>
+      </c>
+      <c r="G4" s="11" t="s">
+        <v>211</v>
+      </c>
+      <c r="H4" s="11"/>
+    </row>
+    <row r="5" spans="1:229" x14ac:dyDescent="0.35">
+      <c r="A5" s="3" t="s">
+        <v>587</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>588</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>589</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>201</v>
+      </c>
+      <c r="F5" s="3" t="s">
+        <v>202</v>
+      </c>
+      <c r="G5" s="3" t="s">
+        <v>211</v>
+      </c>
+      <c r="H5" s="3" t="s">
+        <v>590</v>
       </c>
     </row>
   </sheetData>
@@ -21458,6 +21285,325 @@
 </file>
 
 <file path=xl/worksheets/sheet36.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7271F742-0542-4B33-AEE2-20AE8A69F475}">
+  <dimension ref="A1:HU3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="52.453125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="52.26953125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="42.453125" customWidth="1"/>
+    <col min="4" max="4" width="33.36328125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="33.08984375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="17.08984375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="40.81640625" customWidth="1"/>
+    <col min="8" max="8" width="65.54296875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:229" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>209</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="2" spans="1:229" s="4" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A2" s="3" t="s">
+        <v>594</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>595</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>596</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>201</v>
+      </c>
+      <c r="F2" s="3" t="s">
+        <v>202</v>
+      </c>
+      <c r="G2" s="3" t="s">
+        <v>211</v>
+      </c>
+      <c r="H2" s="3" t="s">
+        <v>597</v>
+      </c>
+      <c r="I2"/>
+      <c r="J2"/>
+      <c r="K2"/>
+      <c r="L2"/>
+      <c r="M2"/>
+      <c r="N2"/>
+      <c r="O2"/>
+      <c r="P2"/>
+      <c r="Q2"/>
+      <c r="R2"/>
+      <c r="S2"/>
+      <c r="T2"/>
+      <c r="U2"/>
+      <c r="V2"/>
+      <c r="W2"/>
+      <c r="X2"/>
+      <c r="Y2"/>
+      <c r="Z2"/>
+      <c r="AA2"/>
+      <c r="AB2"/>
+      <c r="AC2"/>
+      <c r="AD2"/>
+      <c r="AE2"/>
+      <c r="AF2"/>
+      <c r="AG2"/>
+      <c r="AH2"/>
+      <c r="AI2"/>
+      <c r="AJ2"/>
+      <c r="AK2"/>
+      <c r="AL2"/>
+      <c r="AM2"/>
+      <c r="AN2"/>
+      <c r="AO2"/>
+      <c r="AP2"/>
+      <c r="AQ2"/>
+      <c r="AR2"/>
+      <c r="AS2"/>
+      <c r="AT2"/>
+      <c r="AU2"/>
+      <c r="AV2"/>
+      <c r="AW2"/>
+      <c r="AX2"/>
+      <c r="AY2"/>
+      <c r="AZ2"/>
+      <c r="BA2"/>
+      <c r="BB2"/>
+      <c r="BC2"/>
+      <c r="BD2"/>
+      <c r="BE2"/>
+      <c r="BF2"/>
+      <c r="BG2"/>
+      <c r="BH2"/>
+      <c r="BI2"/>
+      <c r="BJ2"/>
+      <c r="BK2"/>
+      <c r="BL2"/>
+      <c r="BM2"/>
+      <c r="BN2"/>
+      <c r="BO2"/>
+      <c r="BP2"/>
+      <c r="BQ2"/>
+      <c r="BR2"/>
+      <c r="BS2"/>
+      <c r="BT2"/>
+      <c r="BU2"/>
+      <c r="BV2"/>
+      <c r="BW2"/>
+      <c r="BX2"/>
+      <c r="BY2"/>
+      <c r="BZ2"/>
+      <c r="CA2"/>
+      <c r="CB2"/>
+      <c r="CC2"/>
+      <c r="CD2"/>
+      <c r="CE2"/>
+      <c r="CF2"/>
+      <c r="CG2"/>
+      <c r="CH2"/>
+      <c r="CI2"/>
+      <c r="CJ2"/>
+      <c r="CK2"/>
+      <c r="CL2"/>
+      <c r="CM2"/>
+      <c r="CN2"/>
+      <c r="CO2"/>
+      <c r="CP2"/>
+      <c r="CQ2"/>
+      <c r="CR2"/>
+      <c r="CS2"/>
+      <c r="CT2"/>
+      <c r="CU2"/>
+      <c r="CV2"/>
+      <c r="CW2"/>
+      <c r="CX2"/>
+      <c r="CY2"/>
+      <c r="CZ2"/>
+      <c r="DA2"/>
+      <c r="DB2"/>
+      <c r="DC2"/>
+      <c r="DD2"/>
+      <c r="DE2"/>
+      <c r="DF2"/>
+      <c r="DG2"/>
+      <c r="DH2"/>
+      <c r="DI2"/>
+      <c r="DJ2"/>
+      <c r="DK2"/>
+      <c r="DL2"/>
+      <c r="DM2"/>
+      <c r="DN2"/>
+      <c r="DO2"/>
+      <c r="DP2"/>
+      <c r="DQ2"/>
+      <c r="DR2"/>
+      <c r="DS2"/>
+      <c r="DT2"/>
+      <c r="DU2"/>
+      <c r="DV2"/>
+      <c r="DW2"/>
+      <c r="DX2"/>
+      <c r="DY2"/>
+      <c r="DZ2"/>
+      <c r="EA2"/>
+      <c r="EB2"/>
+      <c r="EC2"/>
+      <c r="ED2"/>
+      <c r="EE2"/>
+      <c r="EF2"/>
+      <c r="EG2"/>
+      <c r="EH2"/>
+      <c r="EI2"/>
+      <c r="EJ2"/>
+      <c r="EK2"/>
+      <c r="EL2"/>
+      <c r="EM2"/>
+      <c r="EN2"/>
+      <c r="EO2"/>
+      <c r="EP2"/>
+      <c r="EQ2"/>
+      <c r="ER2"/>
+      <c r="ES2"/>
+      <c r="ET2"/>
+      <c r="EU2"/>
+      <c r="EV2"/>
+      <c r="EW2"/>
+      <c r="EX2"/>
+      <c r="EY2"/>
+      <c r="EZ2"/>
+      <c r="FA2"/>
+      <c r="FB2"/>
+      <c r="FC2"/>
+      <c r="FD2"/>
+      <c r="FE2"/>
+      <c r="FF2"/>
+      <c r="FG2"/>
+      <c r="FH2"/>
+      <c r="FI2"/>
+      <c r="FJ2"/>
+      <c r="FK2"/>
+      <c r="FL2"/>
+      <c r="FM2"/>
+      <c r="FN2"/>
+      <c r="FO2"/>
+      <c r="FP2"/>
+      <c r="FQ2"/>
+      <c r="FR2"/>
+      <c r="FS2"/>
+      <c r="FT2"/>
+      <c r="FU2"/>
+      <c r="FV2"/>
+      <c r="FW2"/>
+      <c r="FX2"/>
+      <c r="FY2"/>
+      <c r="FZ2"/>
+      <c r="GA2"/>
+      <c r="GB2"/>
+      <c r="GC2"/>
+      <c r="GD2"/>
+      <c r="GE2"/>
+      <c r="GF2"/>
+      <c r="GG2"/>
+      <c r="GH2"/>
+      <c r="GI2"/>
+      <c r="GJ2"/>
+      <c r="GK2"/>
+      <c r="GL2"/>
+      <c r="GM2"/>
+      <c r="GN2"/>
+      <c r="GO2"/>
+      <c r="GP2"/>
+      <c r="GQ2"/>
+      <c r="GR2"/>
+      <c r="GS2"/>
+      <c r="GT2"/>
+      <c r="GU2"/>
+      <c r="GV2"/>
+      <c r="GW2"/>
+      <c r="GX2"/>
+      <c r="GY2"/>
+      <c r="GZ2"/>
+      <c r="HA2"/>
+      <c r="HB2"/>
+      <c r="HC2"/>
+      <c r="HD2"/>
+      <c r="HE2"/>
+      <c r="HF2"/>
+      <c r="HG2"/>
+      <c r="HH2"/>
+      <c r="HI2"/>
+      <c r="HJ2"/>
+      <c r="HK2"/>
+      <c r="HL2"/>
+      <c r="HM2"/>
+      <c r="HN2"/>
+      <c r="HO2"/>
+      <c r="HP2"/>
+      <c r="HQ2"/>
+      <c r="HR2"/>
+      <c r="HS2"/>
+      <c r="HT2"/>
+      <c r="HU2"/>
+    </row>
+    <row r="3" spans="1:229" x14ac:dyDescent="0.35">
+      <c r="A3" s="3" t="s">
+        <v>598</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>599</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>600</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>201</v>
+      </c>
+      <c r="F3" s="3" t="s">
+        <v>202</v>
+      </c>
+      <c r="G3" s="3" t="s">
+        <v>211</v>
+      </c>
+      <c r="H3" s="3" t="s">
+        <v>601</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet37.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{738B4CF9-CA20-4A87-AA62-B89EDC02284E}">
   <dimension ref="A1:HU5"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -21499,25 +21645,25 @@
       </c>
     </row>
     <row r="2" spans="1:229" s="4" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="3" t="s">
+      <c r="A2" s="11" t="s">
         <v>607</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="B2" s="11" t="s">
         <v>608</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="C2" s="11" t="s">
         <v>609</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="D2" s="11" t="s">
         <v>0</v>
       </c>
-      <c r="E2" s="3" t="s">
+      <c r="E2" s="11" t="s">
         <v>201</v>
       </c>
-      <c r="F2" s="3" t="s">
+      <c r="F2" s="11" t="s">
         <v>202</v>
       </c>
-      <c r="G2" s="3" t="s">
+      <c r="G2" s="11" t="s">
         <v>211</v>
       </c>
       <c r="H2" s="11"/>
@@ -21823,6 +21969,377 @@
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet38.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{09B1B3C7-FD6F-4E3B-8CD4-D9B4FAD90EEE}">
+  <dimension ref="A1:HU5"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="50.54296875" customWidth="1"/>
+    <col min="2" max="2" width="52.26953125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="42.453125" customWidth="1"/>
+    <col min="4" max="4" width="33.36328125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="33.08984375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="17.08984375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="40.81640625" customWidth="1"/>
+    <col min="8" max="8" width="65.54296875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:229" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>209</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="2" spans="1:229" s="4" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A2" s="3" t="s">
+        <v>627</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>628</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>629</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>201</v>
+      </c>
+      <c r="F2" s="3" t="s">
+        <v>202</v>
+      </c>
+      <c r="G2" s="3" t="s">
+        <v>211</v>
+      </c>
+      <c r="H2" s="3" t="s">
+        <v>630</v>
+      </c>
+      <c r="I2"/>
+      <c r="J2"/>
+      <c r="K2"/>
+      <c r="L2"/>
+      <c r="M2"/>
+      <c r="N2"/>
+      <c r="O2"/>
+      <c r="P2"/>
+      <c r="Q2"/>
+      <c r="R2"/>
+      <c r="S2"/>
+      <c r="T2"/>
+      <c r="U2"/>
+      <c r="V2"/>
+      <c r="W2"/>
+      <c r="X2"/>
+      <c r="Y2"/>
+      <c r="Z2"/>
+      <c r="AA2"/>
+      <c r="AB2"/>
+      <c r="AC2"/>
+      <c r="AD2"/>
+      <c r="AE2"/>
+      <c r="AF2"/>
+      <c r="AG2"/>
+      <c r="AH2"/>
+      <c r="AI2"/>
+      <c r="AJ2"/>
+      <c r="AK2"/>
+      <c r="AL2"/>
+      <c r="AM2"/>
+      <c r="AN2"/>
+      <c r="AO2"/>
+      <c r="AP2"/>
+      <c r="AQ2"/>
+      <c r="AR2"/>
+      <c r="AS2"/>
+      <c r="AT2"/>
+      <c r="AU2"/>
+      <c r="AV2"/>
+      <c r="AW2"/>
+      <c r="AX2"/>
+      <c r="AY2"/>
+      <c r="AZ2"/>
+      <c r="BA2"/>
+      <c r="BB2"/>
+      <c r="BC2"/>
+      <c r="BD2"/>
+      <c r="BE2"/>
+      <c r="BF2"/>
+      <c r="BG2"/>
+      <c r="BH2"/>
+      <c r="BI2"/>
+      <c r="BJ2"/>
+      <c r="BK2"/>
+      <c r="BL2"/>
+      <c r="BM2"/>
+      <c r="BN2"/>
+      <c r="BO2"/>
+      <c r="BP2"/>
+      <c r="BQ2"/>
+      <c r="BR2"/>
+      <c r="BS2"/>
+      <c r="BT2"/>
+      <c r="BU2"/>
+      <c r="BV2"/>
+      <c r="BW2"/>
+      <c r="BX2"/>
+      <c r="BY2"/>
+      <c r="BZ2"/>
+      <c r="CA2"/>
+      <c r="CB2"/>
+      <c r="CC2"/>
+      <c r="CD2"/>
+      <c r="CE2"/>
+      <c r="CF2"/>
+      <c r="CG2"/>
+      <c r="CH2"/>
+      <c r="CI2"/>
+      <c r="CJ2"/>
+      <c r="CK2"/>
+      <c r="CL2"/>
+      <c r="CM2"/>
+      <c r="CN2"/>
+      <c r="CO2"/>
+      <c r="CP2"/>
+      <c r="CQ2"/>
+      <c r="CR2"/>
+      <c r="CS2"/>
+      <c r="CT2"/>
+      <c r="CU2"/>
+      <c r="CV2"/>
+      <c r="CW2"/>
+      <c r="CX2"/>
+      <c r="CY2"/>
+      <c r="CZ2"/>
+      <c r="DA2"/>
+      <c r="DB2"/>
+      <c r="DC2"/>
+      <c r="DD2"/>
+      <c r="DE2"/>
+      <c r="DF2"/>
+      <c r="DG2"/>
+      <c r="DH2"/>
+      <c r="DI2"/>
+      <c r="DJ2"/>
+      <c r="DK2"/>
+      <c r="DL2"/>
+      <c r="DM2"/>
+      <c r="DN2"/>
+      <c r="DO2"/>
+      <c r="DP2"/>
+      <c r="DQ2"/>
+      <c r="DR2"/>
+      <c r="DS2"/>
+      <c r="DT2"/>
+      <c r="DU2"/>
+      <c r="DV2"/>
+      <c r="DW2"/>
+      <c r="DX2"/>
+      <c r="DY2"/>
+      <c r="DZ2"/>
+      <c r="EA2"/>
+      <c r="EB2"/>
+      <c r="EC2"/>
+      <c r="ED2"/>
+      <c r="EE2"/>
+      <c r="EF2"/>
+      <c r="EG2"/>
+      <c r="EH2"/>
+      <c r="EI2"/>
+      <c r="EJ2"/>
+      <c r="EK2"/>
+      <c r="EL2"/>
+      <c r="EM2"/>
+      <c r="EN2"/>
+      <c r="EO2"/>
+      <c r="EP2"/>
+      <c r="EQ2"/>
+      <c r="ER2"/>
+      <c r="ES2"/>
+      <c r="ET2"/>
+      <c r="EU2"/>
+      <c r="EV2"/>
+      <c r="EW2"/>
+      <c r="EX2"/>
+      <c r="EY2"/>
+      <c r="EZ2"/>
+      <c r="FA2"/>
+      <c r="FB2"/>
+      <c r="FC2"/>
+      <c r="FD2"/>
+      <c r="FE2"/>
+      <c r="FF2"/>
+      <c r="FG2"/>
+      <c r="FH2"/>
+      <c r="FI2"/>
+      <c r="FJ2"/>
+      <c r="FK2"/>
+      <c r="FL2"/>
+      <c r="FM2"/>
+      <c r="FN2"/>
+      <c r="FO2"/>
+      <c r="FP2"/>
+      <c r="FQ2"/>
+      <c r="FR2"/>
+      <c r="FS2"/>
+      <c r="FT2"/>
+      <c r="FU2"/>
+      <c r="FV2"/>
+      <c r="FW2"/>
+      <c r="FX2"/>
+      <c r="FY2"/>
+      <c r="FZ2"/>
+      <c r="GA2"/>
+      <c r="GB2"/>
+      <c r="GC2"/>
+      <c r="GD2"/>
+      <c r="GE2"/>
+      <c r="GF2"/>
+      <c r="GG2"/>
+      <c r="GH2"/>
+      <c r="GI2"/>
+      <c r="GJ2"/>
+      <c r="GK2"/>
+      <c r="GL2"/>
+      <c r="GM2"/>
+      <c r="GN2"/>
+      <c r="GO2"/>
+      <c r="GP2"/>
+      <c r="GQ2"/>
+      <c r="GR2"/>
+      <c r="GS2"/>
+      <c r="GT2"/>
+      <c r="GU2"/>
+      <c r="GV2"/>
+      <c r="GW2"/>
+      <c r="GX2"/>
+      <c r="GY2"/>
+      <c r="GZ2"/>
+      <c r="HA2"/>
+      <c r="HB2"/>
+      <c r="HC2"/>
+      <c r="HD2"/>
+      <c r="HE2"/>
+      <c r="HF2"/>
+      <c r="HG2"/>
+      <c r="HH2"/>
+      <c r="HI2"/>
+      <c r="HJ2"/>
+      <c r="HK2"/>
+      <c r="HL2"/>
+      <c r="HM2"/>
+      <c r="HN2"/>
+      <c r="HO2"/>
+      <c r="HP2"/>
+      <c r="HQ2"/>
+      <c r="HR2"/>
+      <c r="HS2"/>
+      <c r="HT2"/>
+      <c r="HU2"/>
+    </row>
+    <row r="3" spans="1:229" x14ac:dyDescent="0.35">
+      <c r="A3" s="3" t="s">
+        <v>631</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>632</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>633</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>201</v>
+      </c>
+      <c r="F3" s="3" t="s">
+        <v>202</v>
+      </c>
+      <c r="G3" s="3" t="s">
+        <v>211</v>
+      </c>
+      <c r="H3" s="3" t="s">
+        <v>634</v>
+      </c>
+    </row>
+    <row r="4" spans="1:229" x14ac:dyDescent="0.35">
+      <c r="A4" s="3" t="s">
+        <v>636</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>635</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>637</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>201</v>
+      </c>
+      <c r="F4" s="3" t="s">
+        <v>202</v>
+      </c>
+      <c r="G4" s="3" t="s">
+        <v>211</v>
+      </c>
+      <c r="H4" s="3" t="s">
+        <v>638</v>
+      </c>
+    </row>
+    <row r="5" spans="1:229" x14ac:dyDescent="0.35">
+      <c r="A5" s="3" t="s">
+        <v>639</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>640</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>641</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>201</v>
+      </c>
+      <c r="F5" s="3" t="s">
+        <v>202</v>
+      </c>
+      <c r="G5" s="3" t="s">
+        <v>211</v>
+      </c>
+      <c r="H5" s="3" t="s">
+        <v>642</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Added test cases for Subcategory page: SEND Professional US#135
</commit_message>
<xml_diff>
--- a/testdata.xlsx
+++ b/testdata.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29426"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sshiwani\workspace\find-information-products-services-tests\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C3998CDD-2D0D-4FE1-90F0-EC349A662F70}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E6E5EAFA-BB35-47A2-8B35-96DF87C73B5C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="22780" windowHeight="14540" firstSheet="19" activeTab="20" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="22780" windowHeight="14540" firstSheet="38" activeTab="39" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="category_phase" sheetId="1" r:id="rId1"/>
@@ -34,23 +34,25 @@
     <sheet name="UG_EPEYEarlyYearsWorkforce_list" sheetId="35" r:id="rId19"/>
     <sheet name="UG_EPEYFurtherEduWorkforce_list" sheetId="37" r:id="rId20"/>
     <sheet name="UG_EPEYHigherEduWorkforce_list" sheetId="38" r:id="rId21"/>
-    <sheet name="UGSubcategory_AdultLearner" sheetId="16" r:id="rId22"/>
-    <sheet name="UGSubcategory_CareersAdviser" sheetId="17" r:id="rId23"/>
-    <sheet name="UGSubcategory_ChildOrYoungPers" sheetId="18" r:id="rId24"/>
-    <sheet name="UGSubcategory_DfEWorkforce" sheetId="19" r:id="rId25"/>
-    <sheet name="UGSubcategory_Employer" sheetId="20" r:id="rId26"/>
-    <sheet name="UGSubcategory_LAWorkforce" sheetId="21" r:id="rId27"/>
-    <sheet name="UGSubcategory_NEETOrCareerSeek" sheetId="22" r:id="rId28"/>
-    <sheet name="UGSubcategory_ParentOrCarer" sheetId="23" r:id="rId29"/>
-    <sheet name="UGSubcateg_ProfExtUserofDfEData" sheetId="24" r:id="rId30"/>
-    <sheet name="UGSubcategory_SCWorkforce" sheetId="25" r:id="rId31"/>
-    <sheet name="UGSubcategory_SocialWorker" sheetId="27" r:id="rId32"/>
-    <sheet name="UGSubcategory_EPandEYWorkforce" sheetId="29" r:id="rId33"/>
-    <sheet name="EPEYSubcateg_AcademyTWorkforce" sheetId="31" r:id="rId34"/>
-    <sheet name="EPEYSubcateg_AltProSetWorkforce" sheetId="33" r:id="rId35"/>
-    <sheet name="EPEYSubcatg_EarlyYearsWorkforce" sheetId="34" r:id="rId36"/>
-    <sheet name="EPEYSubcatg_FurtherEduWorkforce" sheetId="36" r:id="rId37"/>
-    <sheet name="EPEYSubcatg_HigherEduWorkforce" sheetId="39" r:id="rId38"/>
+    <sheet name="UG_EPEY_SENDProfessional_list" sheetId="40" r:id="rId22"/>
+    <sheet name="UGSubcategory_AdultLearner" sheetId="16" r:id="rId23"/>
+    <sheet name="UGSubcategory_CareersAdviser" sheetId="17" r:id="rId24"/>
+    <sheet name="UGSubcategory_ChildOrYoungPers" sheetId="18" r:id="rId25"/>
+    <sheet name="UGSubcategory_DfEWorkforce" sheetId="19" r:id="rId26"/>
+    <sheet name="UGSubcategory_Employer" sheetId="20" r:id="rId27"/>
+    <sheet name="UGSubcategory_LAWorkforce" sheetId="21" r:id="rId28"/>
+    <sheet name="UGSubcategory_NEETOrCareerSeek" sheetId="22" r:id="rId29"/>
+    <sheet name="UGSubcategory_ParentOrCarer" sheetId="23" r:id="rId30"/>
+    <sheet name="UGSubcateg_ProfExtUserofDfEData" sheetId="24" r:id="rId31"/>
+    <sheet name="UGSubcategory_SCWorkforce" sheetId="25" r:id="rId32"/>
+    <sheet name="UGSubcategory_SocialWorker" sheetId="27" r:id="rId33"/>
+    <sheet name="UGSubcategory_EPandEYWorkforce" sheetId="29" r:id="rId34"/>
+    <sheet name="EPEYSubcateg_AcademyTWorkforce" sheetId="31" r:id="rId35"/>
+    <sheet name="EPEYSubcateg_AltProSetWorkforce" sheetId="33" r:id="rId36"/>
+    <sheet name="EPEYSubcatg_EarlyYearsWorkforce" sheetId="34" r:id="rId37"/>
+    <sheet name="EPEYSubcatg_FurtherEduWorkforce" sheetId="36" r:id="rId38"/>
+    <sheet name="EPEYSubcatg_HigherEduWorkforce" sheetId="39" r:id="rId39"/>
+    <sheet name="EPEYSubcateg_SENDProfessional" sheetId="41" r:id="rId40"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -62,7 +64,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1362" uniqueCount="643">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1434" uniqueCount="674">
   <si>
     <t>Search and filter products and services</t>
   </si>
@@ -1991,6 +1993,99 @@
   </si>
   <si>
     <t>University support staff  (Higher education workforce)</t>
+  </si>
+  <si>
+    <t>categories/user-group/education-provider-and-early-years-workforce/send-professional</t>
+  </si>
+  <si>
+    <t>Browse products in SEND professional</t>
+  </si>
+  <si>
+    <t>ECHP coordinator</t>
+  </si>
+  <si>
+    <t>SEN coordinator</t>
+  </si>
+  <si>
+    <t>SEND speech and language therapist</t>
+  </si>
+  <si>
+    <t>SEND teacher</t>
+  </si>
+  <si>
+    <t>SEND teaching assistant</t>
+  </si>
+  <si>
+    <t>products?userGroup=send-professional</t>
+  </si>
+  <si>
+    <t>ul.moj-filter-tags li a:has-text(' SEND professional ')</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Remove this filter SEND professional </t>
+  </si>
+  <si>
+    <t>SEND professional  (Education provider and early years workforce)</t>
+  </si>
+  <si>
+    <t>ul.moj-filter-tags li a:has-text(' ECHP coordinator ')</t>
+  </si>
+  <si>
+    <t>products?userGroup=echp-coordinator</t>
+  </si>
+  <si>
+    <t>Remove this filter ECHP coordinator</t>
+  </si>
+  <si>
+    <t>ECHP coordinator  (SEND professional)</t>
+  </si>
+  <si>
+    <t>products?userGroup=sen-coordinator</t>
+  </si>
+  <si>
+    <t>ul.moj-filter-tags li a:has-text(' SEN coordinator ')</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Remove this filter SEN coordinator </t>
+  </si>
+  <si>
+    <t>SEN coordinator  (SEND professional)</t>
+  </si>
+  <si>
+    <t>products?userGroup=send-speech-and-language-therapist</t>
+  </si>
+  <si>
+    <t>ul.moj-filter-tags li a:has-text('  SEND speech and language therapist ')</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Remove this filter SEND speech and language therapist </t>
+  </si>
+  <si>
+    <t>SEND speech and language therapist  (SEND professional)</t>
+  </si>
+  <si>
+    <t>products?userGroup=send-teacher</t>
+  </si>
+  <si>
+    <t>ul.moj-filter-tags li a:has-text(' SEND teacher  (SEND professional)')</t>
+  </si>
+  <si>
+    <t>Remove this filter SEND teacher  (SEND professional)</t>
+  </si>
+  <si>
+    <t>SEND teacher  (SEND professional)</t>
+  </si>
+  <si>
+    <t>products?userGroup=send-teaching-assistant</t>
+  </si>
+  <si>
+    <t>ul.moj-filter-tags li a:has-text(' SEND teaching assistant ')</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Remove this filter SEND teaching assistant </t>
+  </si>
+  <si>
+    <t>SEND teaching assistant  (SEND professional)</t>
   </si>
 </sst>
 </file>
@@ -13107,6 +13202,101 @@
 </file>
 
 <file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{85AB9B63-18E3-4595-A79C-C8492E7240D1}">
+  <dimension ref="A1:C10"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="54.1796875" customWidth="1"/>
+    <col min="2" max="2" width="47.453125" customWidth="1"/>
+    <col min="3" max="3" width="50.36328125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A1" s="6" t="s">
+        <v>102</v>
+      </c>
+      <c r="B1" s="6" t="s">
+        <v>103</v>
+      </c>
+      <c r="C1" s="6" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A2" s="3" t="s">
+        <v>643</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>107</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>644</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="B3" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="B4" s="3" t="s">
+        <v>113</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A5" s="3" t="s">
+        <v>147</v>
+      </c>
+      <c r="B5" s="3"/>
+      <c r="C5" s="3"/>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A6" s="3" t="s">
+        <v>645</v>
+      </c>
+      <c r="B6" s="3"/>
+      <c r="C6" s="3"/>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A7" s="3" t="s">
+        <v>646</v>
+      </c>
+      <c r="B7" s="3"/>
+      <c r="C7" s="3"/>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A8" s="3" t="s">
+        <v>647</v>
+      </c>
+      <c r="B8" s="3"/>
+      <c r="C8" s="3"/>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A9" s="3" t="s">
+        <v>648</v>
+      </c>
+      <c r="B9" s="3"/>
+      <c r="C9" s="3"/>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A10" s="3" t="s">
+        <v>649</v>
+      </c>
+      <c r="B10" s="3"/>
+      <c r="C10" s="3"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FB5527F7-85DB-4F8E-B4B3-EC8453E599E1}">
   <dimension ref="A1:HU6"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -13504,7 +13694,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A99CF6C3-F305-48A2-AB80-2C2D7CE6460C}">
   <dimension ref="A1:HU5"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -13875,7 +14065,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5EFF0597-7FD1-4E6A-AA71-DB9F9FAB97A9}">
   <dimension ref="A1:HU7"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -14299,7 +14489,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9F4A57AC-4620-4875-88AE-9F5C739A9042}">
   <dimension ref="A1:HU6"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -14696,7 +14886,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6C1C130F-0899-4810-82F6-950C9CB07234}">
   <dimension ref="A1:HU5"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -15067,7 +15257,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4AB9395B-D522-49AD-B790-5334356249F6}">
   <dimension ref="A1:HU7"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -15490,7 +15680,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet29.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BEE91763-AD0C-4544-A433-3B50C88AEB79}">
   <dimension ref="A1:HU7"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -15909,508 +16099,6 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet29.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{20DD36AA-F163-4AAB-BD30-4AE6290CCAE7}">
-  <dimension ref="A1:HU10"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
-  <cols>
-    <col min="1" max="1" width="50.90625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="52.26953125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="42.453125" customWidth="1"/>
-    <col min="4" max="4" width="33.36328125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="33.08984375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="17.08984375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="40.81640625" customWidth="1"/>
-    <col min="8" max="8" width="62.54296875" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:229" x14ac:dyDescent="0.35">
-      <c r="A1" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="F1" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="G1" s="2" t="s">
-        <v>209</v>
-      </c>
-      <c r="H1" s="2" t="s">
-        <v>210</v>
-      </c>
-    </row>
-    <row r="2" spans="1:229" s="4" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="3" t="s">
-        <v>355</v>
-      </c>
-      <c r="B2" s="3" t="s">
-        <v>356</v>
-      </c>
-      <c r="C2" s="3" t="s">
-        <v>357</v>
-      </c>
-      <c r="D2" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="E2" s="3" t="s">
-        <v>201</v>
-      </c>
-      <c r="F2" s="3" t="s">
-        <v>202</v>
-      </c>
-      <c r="G2" s="3" t="s">
-        <v>211</v>
-      </c>
-      <c r="H2" s="3" t="s">
-        <v>172</v>
-      </c>
-      <c r="I2"/>
-      <c r="J2"/>
-      <c r="K2"/>
-      <c r="L2"/>
-      <c r="M2"/>
-      <c r="N2"/>
-      <c r="O2"/>
-      <c r="P2"/>
-      <c r="Q2"/>
-      <c r="R2"/>
-      <c r="S2"/>
-      <c r="T2"/>
-      <c r="U2"/>
-      <c r="V2"/>
-      <c r="W2"/>
-      <c r="X2"/>
-      <c r="Y2"/>
-      <c r="Z2"/>
-      <c r="AA2"/>
-      <c r="AB2"/>
-      <c r="AC2"/>
-      <c r="AD2"/>
-      <c r="AE2"/>
-      <c r="AF2"/>
-      <c r="AG2"/>
-      <c r="AH2"/>
-      <c r="AI2"/>
-      <c r="AJ2"/>
-      <c r="AK2"/>
-      <c r="AL2"/>
-      <c r="AM2"/>
-      <c r="AN2"/>
-      <c r="AO2"/>
-      <c r="AP2"/>
-      <c r="AQ2"/>
-      <c r="AR2"/>
-      <c r="AS2"/>
-      <c r="AT2"/>
-      <c r="AU2"/>
-      <c r="AV2"/>
-      <c r="AW2"/>
-      <c r="AX2"/>
-      <c r="AY2"/>
-      <c r="AZ2"/>
-      <c r="BA2"/>
-      <c r="BB2"/>
-      <c r="BC2"/>
-      <c r="BD2"/>
-      <c r="BE2"/>
-      <c r="BF2"/>
-      <c r="BG2"/>
-      <c r="BH2"/>
-      <c r="BI2"/>
-      <c r="BJ2"/>
-      <c r="BK2"/>
-      <c r="BL2"/>
-      <c r="BM2"/>
-      <c r="BN2"/>
-      <c r="BO2"/>
-      <c r="BP2"/>
-      <c r="BQ2"/>
-      <c r="BR2"/>
-      <c r="BS2"/>
-      <c r="BT2"/>
-      <c r="BU2"/>
-      <c r="BV2"/>
-      <c r="BW2"/>
-      <c r="BX2"/>
-      <c r="BY2"/>
-      <c r="BZ2"/>
-      <c r="CA2"/>
-      <c r="CB2"/>
-      <c r="CC2"/>
-      <c r="CD2"/>
-      <c r="CE2"/>
-      <c r="CF2"/>
-      <c r="CG2"/>
-      <c r="CH2"/>
-      <c r="CI2"/>
-      <c r="CJ2"/>
-      <c r="CK2"/>
-      <c r="CL2"/>
-      <c r="CM2"/>
-      <c r="CN2"/>
-      <c r="CO2"/>
-      <c r="CP2"/>
-      <c r="CQ2"/>
-      <c r="CR2"/>
-      <c r="CS2"/>
-      <c r="CT2"/>
-      <c r="CU2"/>
-      <c r="CV2"/>
-      <c r="CW2"/>
-      <c r="CX2"/>
-      <c r="CY2"/>
-      <c r="CZ2"/>
-      <c r="DA2"/>
-      <c r="DB2"/>
-      <c r="DC2"/>
-      <c r="DD2"/>
-      <c r="DE2"/>
-      <c r="DF2"/>
-      <c r="DG2"/>
-      <c r="DH2"/>
-      <c r="DI2"/>
-      <c r="DJ2"/>
-      <c r="DK2"/>
-      <c r="DL2"/>
-      <c r="DM2"/>
-      <c r="DN2"/>
-      <c r="DO2"/>
-      <c r="DP2"/>
-      <c r="DQ2"/>
-      <c r="DR2"/>
-      <c r="DS2"/>
-      <c r="DT2"/>
-      <c r="DU2"/>
-      <c r="DV2"/>
-      <c r="DW2"/>
-      <c r="DX2"/>
-      <c r="DY2"/>
-      <c r="DZ2"/>
-      <c r="EA2"/>
-      <c r="EB2"/>
-      <c r="EC2"/>
-      <c r="ED2"/>
-      <c r="EE2"/>
-      <c r="EF2"/>
-      <c r="EG2"/>
-      <c r="EH2"/>
-      <c r="EI2"/>
-      <c r="EJ2"/>
-      <c r="EK2"/>
-      <c r="EL2"/>
-      <c r="EM2"/>
-      <c r="EN2"/>
-      <c r="EO2"/>
-      <c r="EP2"/>
-      <c r="EQ2"/>
-      <c r="ER2"/>
-      <c r="ES2"/>
-      <c r="ET2"/>
-      <c r="EU2"/>
-      <c r="EV2"/>
-      <c r="EW2"/>
-      <c r="EX2"/>
-      <c r="EY2"/>
-      <c r="EZ2"/>
-      <c r="FA2"/>
-      <c r="FB2"/>
-      <c r="FC2"/>
-      <c r="FD2"/>
-      <c r="FE2"/>
-      <c r="FF2"/>
-      <c r="FG2"/>
-      <c r="FH2"/>
-      <c r="FI2"/>
-      <c r="FJ2"/>
-      <c r="FK2"/>
-      <c r="FL2"/>
-      <c r="FM2"/>
-      <c r="FN2"/>
-      <c r="FO2"/>
-      <c r="FP2"/>
-      <c r="FQ2"/>
-      <c r="FR2"/>
-      <c r="FS2"/>
-      <c r="FT2"/>
-      <c r="FU2"/>
-      <c r="FV2"/>
-      <c r="FW2"/>
-      <c r="FX2"/>
-      <c r="FY2"/>
-      <c r="FZ2"/>
-      <c r="GA2"/>
-      <c r="GB2"/>
-      <c r="GC2"/>
-      <c r="GD2"/>
-      <c r="GE2"/>
-      <c r="GF2"/>
-      <c r="GG2"/>
-      <c r="GH2"/>
-      <c r="GI2"/>
-      <c r="GJ2"/>
-      <c r="GK2"/>
-      <c r="GL2"/>
-      <c r="GM2"/>
-      <c r="GN2"/>
-      <c r="GO2"/>
-      <c r="GP2"/>
-      <c r="GQ2"/>
-      <c r="GR2"/>
-      <c r="GS2"/>
-      <c r="GT2"/>
-      <c r="GU2"/>
-      <c r="GV2"/>
-      <c r="GW2"/>
-      <c r="GX2"/>
-      <c r="GY2"/>
-      <c r="GZ2"/>
-      <c r="HA2"/>
-      <c r="HB2"/>
-      <c r="HC2"/>
-      <c r="HD2"/>
-      <c r="HE2"/>
-      <c r="HF2"/>
-      <c r="HG2"/>
-      <c r="HH2"/>
-      <c r="HI2"/>
-      <c r="HJ2"/>
-      <c r="HK2"/>
-      <c r="HL2"/>
-      <c r="HM2"/>
-      <c r="HN2"/>
-      <c r="HO2"/>
-      <c r="HP2"/>
-      <c r="HQ2"/>
-      <c r="HR2"/>
-      <c r="HS2"/>
-      <c r="HT2"/>
-      <c r="HU2"/>
-    </row>
-    <row r="3" spans="1:229" x14ac:dyDescent="0.35">
-      <c r="A3" s="3" t="s">
-        <v>358</v>
-      </c>
-      <c r="B3" s="3" t="s">
-        <v>359</v>
-      </c>
-      <c r="C3" s="3" t="s">
-        <v>360</v>
-      </c>
-      <c r="D3" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="E3" s="3" t="s">
-        <v>201</v>
-      </c>
-      <c r="F3" s="3" t="s">
-        <v>202</v>
-      </c>
-      <c r="G3" s="3" t="s">
-        <v>211</v>
-      </c>
-      <c r="H3" s="3" t="s">
-        <v>361</v>
-      </c>
-    </row>
-    <row r="4" spans="1:229" x14ac:dyDescent="0.35">
-      <c r="A4" s="3" t="s">
-        <v>362</v>
-      </c>
-      <c r="B4" s="3" t="s">
-        <v>363</v>
-      </c>
-      <c r="C4" s="3" t="s">
-        <v>364</v>
-      </c>
-      <c r="D4" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="E4" s="3" t="s">
-        <v>201</v>
-      </c>
-      <c r="F4" s="3" t="s">
-        <v>202</v>
-      </c>
-      <c r="G4" s="3" t="s">
-        <v>211</v>
-      </c>
-      <c r="H4" s="3" t="s">
-        <v>365</v>
-      </c>
-    </row>
-    <row r="5" spans="1:229" x14ac:dyDescent="0.35">
-      <c r="A5" s="8" t="s">
-        <v>366</v>
-      </c>
-      <c r="B5" s="8" t="s">
-        <v>367</v>
-      </c>
-      <c r="C5" s="8" t="s">
-        <v>368</v>
-      </c>
-      <c r="D5" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="E5" s="3" t="s">
-        <v>201</v>
-      </c>
-      <c r="F5" s="3" t="s">
-        <v>202</v>
-      </c>
-      <c r="G5" s="3" t="s">
-        <v>211</v>
-      </c>
-      <c r="H5" s="3" t="s">
-        <v>369</v>
-      </c>
-    </row>
-    <row r="6" spans="1:229" x14ac:dyDescent="0.35">
-      <c r="A6" s="3" t="s">
-        <v>370</v>
-      </c>
-      <c r="B6" s="3" t="s">
-        <v>371</v>
-      </c>
-      <c r="C6" s="3" t="s">
-        <v>372</v>
-      </c>
-      <c r="D6" s="7" t="s">
-        <v>0</v>
-      </c>
-      <c r="E6" s="3" t="s">
-        <v>201</v>
-      </c>
-      <c r="F6" s="3" t="s">
-        <v>202</v>
-      </c>
-      <c r="G6" s="3" t="s">
-        <v>211</v>
-      </c>
-      <c r="H6" s="3" t="s">
-        <v>373</v>
-      </c>
-    </row>
-    <row r="7" spans="1:229" x14ac:dyDescent="0.35">
-      <c r="A7" s="3" t="s">
-        <v>374</v>
-      </c>
-      <c r="B7" s="3" t="s">
-        <v>375</v>
-      </c>
-      <c r="C7" s="3" t="s">
-        <v>376</v>
-      </c>
-      <c r="D7" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="E7" s="3" t="s">
-        <v>201</v>
-      </c>
-      <c r="F7" s="3" t="s">
-        <v>202</v>
-      </c>
-      <c r="G7" s="3" t="s">
-        <v>211</v>
-      </c>
-      <c r="H7" s="3" t="s">
-        <v>377</v>
-      </c>
-    </row>
-    <row r="8" spans="1:229" x14ac:dyDescent="0.35">
-      <c r="A8" s="3" t="s">
-        <v>378</v>
-      </c>
-      <c r="B8" s="3" t="s">
-        <v>379</v>
-      </c>
-      <c r="C8" s="3" t="s">
-        <v>380</v>
-      </c>
-      <c r="D8" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="E8" s="3" t="s">
-        <v>201</v>
-      </c>
-      <c r="F8" s="3" t="s">
-        <v>202</v>
-      </c>
-      <c r="G8" s="3" t="s">
-        <v>211</v>
-      </c>
-      <c r="H8" s="3" t="s">
-        <v>381</v>
-      </c>
-    </row>
-    <row r="9" spans="1:229" x14ac:dyDescent="0.35">
-      <c r="A9" s="3" t="s">
-        <v>382</v>
-      </c>
-      <c r="B9" s="3" t="s">
-        <v>383</v>
-      </c>
-      <c r="C9" s="3" t="s">
-        <v>384</v>
-      </c>
-      <c r="D9" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="E9" s="3" t="s">
-        <v>201</v>
-      </c>
-      <c r="F9" s="3" t="s">
-        <v>202</v>
-      </c>
-      <c r="G9" s="3" t="s">
-        <v>211</v>
-      </c>
-      <c r="H9" s="3" t="s">
-        <v>385</v>
-      </c>
-    </row>
-    <row r="10" spans="1:229" x14ac:dyDescent="0.35">
-      <c r="A10" s="3" t="s">
-        <v>386</v>
-      </c>
-      <c r="B10" s="3" t="s">
-        <v>387</v>
-      </c>
-      <c r="C10" s="3" t="s">
-        <v>388</v>
-      </c>
-      <c r="D10" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="E10" s="3" t="s">
-        <v>201</v>
-      </c>
-      <c r="F10" s="3" t="s">
-        <v>202</v>
-      </c>
-      <c r="G10" s="3" t="s">
-        <v>211</v>
-      </c>
-      <c r="H10" s="3" t="s">
-        <v>389</v>
-      </c>
-    </row>
-  </sheetData>
-  <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -18720,8 +18408,8 @@
 </file>
 
 <file path=xl/worksheets/sheet30.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C6EE6111-FDB3-4B43-8820-BBF68AAFCD6D}">
-  <dimension ref="A1:HU8"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{20DD36AA-F163-4AAB-BD30-4AE6290CCAE7}">
+  <dimension ref="A1:HU10"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="50.90625" bestFit="1" customWidth="1"/>
@@ -18762,13 +18450,13 @@
     </row>
     <row r="2" spans="1:229" s="4" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A2" s="3" t="s">
-        <v>390</v>
+        <v>355</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>391</v>
+        <v>356</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>392</v>
+        <v>357</v>
       </c>
       <c r="D2" s="3" t="s">
         <v>0</v>
@@ -18783,7 +18471,7 @@
         <v>211</v>
       </c>
       <c r="H2" s="3" t="s">
-        <v>183</v>
+        <v>172</v>
       </c>
       <c r="I2"/>
       <c r="J2"/>
@@ -19009,13 +18697,13 @@
     </row>
     <row r="3" spans="1:229" x14ac:dyDescent="0.35">
       <c r="A3" s="3" t="s">
-        <v>393</v>
+        <v>358</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>394</v>
+        <v>359</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>395</v>
+        <v>360</v>
       </c>
       <c r="D3" s="3" t="s">
         <v>0</v>
@@ -19030,18 +18718,18 @@
         <v>211</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>396</v>
+        <v>361</v>
       </c>
     </row>
     <row r="4" spans="1:229" x14ac:dyDescent="0.35">
       <c r="A4" s="3" t="s">
-        <v>397</v>
+        <v>362</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>398</v>
+        <v>363</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>399</v>
+        <v>364</v>
       </c>
       <c r="D4" s="3" t="s">
         <v>0</v>
@@ -19056,18 +18744,18 @@
         <v>211</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>400</v>
+        <v>365</v>
       </c>
     </row>
     <row r="5" spans="1:229" x14ac:dyDescent="0.35">
       <c r="A5" s="8" t="s">
-        <v>401</v>
+        <v>366</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>402</v>
+        <v>367</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>403</v>
+        <v>368</v>
       </c>
       <c r="D5" s="3" t="s">
         <v>0</v>
@@ -19082,18 +18770,18 @@
         <v>211</v>
       </c>
       <c r="H5" s="3" t="s">
-        <v>404</v>
+        <v>369</v>
       </c>
     </row>
     <row r="6" spans="1:229" x14ac:dyDescent="0.35">
       <c r="A6" s="3" t="s">
-        <v>405</v>
+        <v>370</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>406</v>
+        <v>371</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>407</v>
+        <v>372</v>
       </c>
       <c r="D6" s="7" t="s">
         <v>0</v>
@@ -19108,18 +18796,18 @@
         <v>211</v>
       </c>
       <c r="H6" s="3" t="s">
-        <v>408</v>
+        <v>373</v>
       </c>
     </row>
     <row r="7" spans="1:229" x14ac:dyDescent="0.35">
       <c r="A7" s="3" t="s">
-        <v>409</v>
+        <v>374</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>410</v>
+        <v>375</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>411</v>
+        <v>376</v>
       </c>
       <c r="D7" s="3" t="s">
         <v>0</v>
@@ -19134,18 +18822,18 @@
         <v>211</v>
       </c>
       <c r="H7" s="3" t="s">
-        <v>412</v>
+        <v>377</v>
       </c>
     </row>
     <row r="8" spans="1:229" x14ac:dyDescent="0.35">
-      <c r="A8" s="9" t="s">
-        <v>413</v>
-      </c>
-      <c r="B8" s="9" t="s">
-        <v>414</v>
-      </c>
-      <c r="C8" s="9" t="s">
-        <v>415</v>
+      <c r="A8" s="3" t="s">
+        <v>378</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>379</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>380</v>
       </c>
       <c r="D8" s="3" t="s">
         <v>0</v>
@@ -19159,8 +18847,60 @@
       <c r="G8" s="3" t="s">
         <v>211</v>
       </c>
-      <c r="H8" s="9" t="s">
-        <v>416</v>
+      <c r="H8" s="3" t="s">
+        <v>381</v>
+      </c>
+    </row>
+    <row r="9" spans="1:229" x14ac:dyDescent="0.35">
+      <c r="A9" s="3" t="s">
+        <v>382</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>383</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>384</v>
+      </c>
+      <c r="D9" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="E9" s="3" t="s">
+        <v>201</v>
+      </c>
+      <c r="F9" s="3" t="s">
+        <v>202</v>
+      </c>
+      <c r="G9" s="3" t="s">
+        <v>211</v>
+      </c>
+      <c r="H9" s="3" t="s">
+        <v>385</v>
+      </c>
+    </row>
+    <row r="10" spans="1:229" x14ac:dyDescent="0.35">
+      <c r="A10" s="3" t="s">
+        <v>386</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>387</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>388</v>
+      </c>
+      <c r="D10" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="E10" s="3" t="s">
+        <v>201</v>
+      </c>
+      <c r="F10" s="3" t="s">
+        <v>202</v>
+      </c>
+      <c r="G10" s="3" t="s">
+        <v>211</v>
+      </c>
+      <c r="H10" s="3" t="s">
+        <v>389</v>
       </c>
     </row>
   </sheetData>
@@ -19170,8 +18910,8 @@
 </file>
 
 <file path=xl/worksheets/sheet31.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E6428663-7558-48F1-8CD3-947F03FFD4CC}">
-  <dimension ref="A1:HU9"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C6EE6111-FDB3-4B43-8820-BBF68AAFCD6D}">
+  <dimension ref="A1:HU8"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="50.90625" bestFit="1" customWidth="1"/>
@@ -19181,7 +18921,7 @@
     <col min="5" max="5" width="33.08984375" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="17.08984375" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="40.81640625" customWidth="1"/>
-    <col min="8" max="8" width="57.08984375" customWidth="1"/>
+    <col min="8" max="8" width="62.54296875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:229" x14ac:dyDescent="0.35">
@@ -19212,13 +18952,13 @@
     </row>
     <row r="2" spans="1:229" s="4" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A2" s="3" t="s">
-        <v>457</v>
+        <v>390</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>458</v>
+        <v>391</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>459</v>
+        <v>392</v>
       </c>
       <c r="D2" s="3" t="s">
         <v>0</v>
@@ -19233,7 +18973,7 @@
         <v>211</v>
       </c>
       <c r="H2" s="3" t="s">
-        <v>192</v>
+        <v>183</v>
       </c>
       <c r="I2"/>
       <c r="J2"/>
@@ -19459,13 +19199,13 @@
     </row>
     <row r="3" spans="1:229" x14ac:dyDescent="0.35">
       <c r="A3" s="3" t="s">
-        <v>460</v>
+        <v>393</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>461</v>
+        <v>394</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>462</v>
+        <v>395</v>
       </c>
       <c r="D3" s="3" t="s">
         <v>0</v>
@@ -19480,18 +19220,18 @@
         <v>211</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>463</v>
+        <v>396</v>
       </c>
     </row>
     <row r="4" spans="1:229" x14ac:dyDescent="0.35">
       <c r="A4" s="3" t="s">
-        <v>464</v>
+        <v>397</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>467</v>
+        <v>398</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>465</v>
+        <v>399</v>
       </c>
       <c r="D4" s="3" t="s">
         <v>0</v>
@@ -19506,18 +19246,18 @@
         <v>211</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>466</v>
+        <v>400</v>
       </c>
     </row>
     <row r="5" spans="1:229" x14ac:dyDescent="0.35">
       <c r="A5" s="8" t="s">
-        <v>468</v>
+        <v>401</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>469</v>
+        <v>402</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>470</v>
+        <v>403</v>
       </c>
       <c r="D5" s="3" t="s">
         <v>0</v>
@@ -19532,18 +19272,18 @@
         <v>211</v>
       </c>
       <c r="H5" s="3" t="s">
-        <v>471</v>
+        <v>404</v>
       </c>
     </row>
     <row r="6" spans="1:229" x14ac:dyDescent="0.35">
       <c r="A6" s="3" t="s">
-        <v>473</v>
+        <v>405</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>472</v>
+        <v>406</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>474</v>
+        <v>407</v>
       </c>
       <c r="D6" s="7" t="s">
         <v>0</v>
@@ -19558,18 +19298,18 @@
         <v>211</v>
       </c>
       <c r="H6" s="3" t="s">
-        <v>475</v>
+        <v>408</v>
       </c>
     </row>
     <row r="7" spans="1:229" x14ac:dyDescent="0.35">
       <c r="A7" s="3" t="s">
-        <v>476</v>
+        <v>409</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>477</v>
+        <v>410</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>478</v>
+        <v>411</v>
       </c>
       <c r="D7" s="3" t="s">
         <v>0</v>
@@ -19584,18 +19324,18 @@
         <v>211</v>
       </c>
       <c r="H7" s="3" t="s">
-        <v>479</v>
+        <v>412</v>
       </c>
     </row>
     <row r="8" spans="1:229" x14ac:dyDescent="0.35">
-      <c r="A8" s="3" t="s">
-        <v>480</v>
-      </c>
-      <c r="B8" s="3" t="s">
-        <v>481</v>
-      </c>
-      <c r="C8" s="3" t="s">
-        <v>482</v>
+      <c r="A8" s="9" t="s">
+        <v>413</v>
+      </c>
+      <c r="B8" s="9" t="s">
+        <v>414</v>
+      </c>
+      <c r="C8" s="9" t="s">
+        <v>415</v>
       </c>
       <c r="D8" s="3" t="s">
         <v>0</v>
@@ -19609,34 +19349,8 @@
       <c r="G8" s="3" t="s">
         <v>211</v>
       </c>
-      <c r="H8" s="3" t="s">
-        <v>483</v>
-      </c>
-    </row>
-    <row r="9" spans="1:229" x14ac:dyDescent="0.35">
-      <c r="A9" s="3" t="s">
-        <v>484</v>
-      </c>
-      <c r="B9" s="3" t="s">
-        <v>485</v>
-      </c>
-      <c r="C9" s="3" t="s">
-        <v>486</v>
-      </c>
-      <c r="D9" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="E9" s="3" t="s">
-        <v>201</v>
-      </c>
-      <c r="F9" s="3" t="s">
-        <v>202</v>
-      </c>
-      <c r="G9" s="3" t="s">
-        <v>211</v>
-      </c>
-      <c r="H9" s="3" t="s">
-        <v>487</v>
+      <c r="H8" s="9" t="s">
+        <v>416</v>
       </c>
     </row>
   </sheetData>
@@ -19646,8 +19360,8 @@
 </file>
 
 <file path=xl/worksheets/sheet32.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2A4E3580-B709-4E66-9F6E-B7F9948D7FD3}">
-  <dimension ref="A1:HU7"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E6428663-7558-48F1-8CD3-947F03FFD4CC}">
+  <dimension ref="A1:HU9"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="50.90625" bestFit="1" customWidth="1"/>
@@ -19688,13 +19402,13 @@
     </row>
     <row r="2" spans="1:229" s="4" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A2" s="3" t="s">
-        <v>488</v>
+        <v>457</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>489</v>
+        <v>458</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>490</v>
+        <v>459</v>
       </c>
       <c r="D2" s="3" t="s">
         <v>0</v>
@@ -19709,7 +19423,7 @@
         <v>211</v>
       </c>
       <c r="H2" s="3" t="s">
-        <v>491</v>
+        <v>192</v>
       </c>
       <c r="I2"/>
       <c r="J2"/>
@@ -19935,13 +19649,13 @@
     </row>
     <row r="3" spans="1:229" x14ac:dyDescent="0.35">
       <c r="A3" s="3" t="s">
-        <v>492</v>
+        <v>460</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>493</v>
+        <v>461</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>494</v>
+        <v>462</v>
       </c>
       <c r="D3" s="3" t="s">
         <v>0</v>
@@ -19956,18 +19670,18 @@
         <v>211</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>495</v>
+        <v>463</v>
       </c>
     </row>
     <row r="4" spans="1:229" x14ac:dyDescent="0.35">
       <c r="A4" s="3" t="s">
-        <v>496</v>
+        <v>464</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>497</v>
+        <v>467</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>498</v>
+        <v>465</v>
       </c>
       <c r="D4" s="3" t="s">
         <v>0</v>
@@ -19982,18 +19696,18 @@
         <v>211</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>499</v>
+        <v>466</v>
       </c>
     </row>
     <row r="5" spans="1:229" x14ac:dyDescent="0.35">
       <c r="A5" s="8" t="s">
-        <v>500</v>
+        <v>468</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>501</v>
+        <v>469</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>502</v>
+        <v>470</v>
       </c>
       <c r="D5" s="3" t="s">
         <v>0</v>
@@ -20008,18 +19722,18 @@
         <v>211</v>
       </c>
       <c r="H5" s="3" t="s">
-        <v>503</v>
+        <v>471</v>
       </c>
     </row>
     <row r="6" spans="1:229" x14ac:dyDescent="0.35">
       <c r="A6" s="3" t="s">
-        <v>504</v>
+        <v>473</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>505</v>
+        <v>472</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>506</v>
+        <v>474</v>
       </c>
       <c r="D6" s="7" t="s">
         <v>0</v>
@@ -20034,18 +19748,18 @@
         <v>211</v>
       </c>
       <c r="H6" s="3" t="s">
-        <v>507</v>
+        <v>475</v>
       </c>
     </row>
     <row r="7" spans="1:229" x14ac:dyDescent="0.35">
       <c r="A7" s="3" t="s">
-        <v>509</v>
+        <v>476</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>508</v>
+        <v>477</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>510</v>
+        <v>478</v>
       </c>
       <c r="D7" s="3" t="s">
         <v>0</v>
@@ -20060,17 +19774,70 @@
         <v>211</v>
       </c>
       <c r="H7" s="3" t="s">
-        <v>511</v>
+        <v>479</v>
+      </c>
+    </row>
+    <row r="8" spans="1:229" x14ac:dyDescent="0.35">
+      <c r="A8" s="3" t="s">
+        <v>480</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>481</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>482</v>
+      </c>
+      <c r="D8" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="E8" s="3" t="s">
+        <v>201</v>
+      </c>
+      <c r="F8" s="3" t="s">
+        <v>202</v>
+      </c>
+      <c r="G8" s="3" t="s">
+        <v>211</v>
+      </c>
+      <c r="H8" s="3" t="s">
+        <v>483</v>
+      </c>
+    </row>
+    <row r="9" spans="1:229" x14ac:dyDescent="0.35">
+      <c r="A9" s="3" t="s">
+        <v>484</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>485</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>486</v>
+      </c>
+      <c r="D9" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="E9" s="3" t="s">
+        <v>201</v>
+      </c>
+      <c r="F9" s="3" t="s">
+        <v>202</v>
+      </c>
+      <c r="G9" s="3" t="s">
+        <v>211</v>
+      </c>
+      <c r="H9" s="3" t="s">
+        <v>487</v>
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet33.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{95706458-CD50-4C74-87C4-ABAE617927AD}">
-  <dimension ref="A1:HU2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2A4E3580-B709-4E66-9F6E-B7F9948D7FD3}">
+  <dimension ref="A1:HU7"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="50.90625" bestFit="1" customWidth="1"/>
@@ -20111,13 +19878,13 @@
     </row>
     <row r="2" spans="1:229" s="4" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A2" s="3" t="s">
-        <v>512</v>
+        <v>488</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>513</v>
+        <v>489</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>514</v>
+        <v>490</v>
       </c>
       <c r="D2" s="3" t="s">
         <v>0</v>
@@ -20132,7 +19899,7 @@
         <v>211</v>
       </c>
       <c r="H2" s="3" t="s">
-        <v>140</v>
+        <v>491</v>
       </c>
       <c r="I2"/>
       <c r="J2"/>
@@ -20356,14 +20123,144 @@
       <c r="HT2"/>
       <c r="HU2"/>
     </row>
+    <row r="3" spans="1:229" x14ac:dyDescent="0.35">
+      <c r="A3" s="3" t="s">
+        <v>492</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>493</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>494</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>201</v>
+      </c>
+      <c r="F3" s="3" t="s">
+        <v>202</v>
+      </c>
+      <c r="G3" s="3" t="s">
+        <v>211</v>
+      </c>
+      <c r="H3" s="3" t="s">
+        <v>495</v>
+      </c>
+    </row>
+    <row r="4" spans="1:229" x14ac:dyDescent="0.35">
+      <c r="A4" s="3" t="s">
+        <v>496</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>497</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>498</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>201</v>
+      </c>
+      <c r="F4" s="3" t="s">
+        <v>202</v>
+      </c>
+      <c r="G4" s="3" t="s">
+        <v>211</v>
+      </c>
+      <c r="H4" s="3" t="s">
+        <v>499</v>
+      </c>
+    </row>
+    <row r="5" spans="1:229" x14ac:dyDescent="0.35">
+      <c r="A5" s="8" t="s">
+        <v>500</v>
+      </c>
+      <c r="B5" s="8" t="s">
+        <v>501</v>
+      </c>
+      <c r="C5" s="8" t="s">
+        <v>502</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>201</v>
+      </c>
+      <c r="F5" s="3" t="s">
+        <v>202</v>
+      </c>
+      <c r="G5" s="3" t="s">
+        <v>211</v>
+      </c>
+      <c r="H5" s="3" t="s">
+        <v>503</v>
+      </c>
+    </row>
+    <row r="6" spans="1:229" x14ac:dyDescent="0.35">
+      <c r="A6" s="3" t="s">
+        <v>504</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>505</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>506</v>
+      </c>
+      <c r="D6" s="7" t="s">
+        <v>0</v>
+      </c>
+      <c r="E6" s="3" t="s">
+        <v>201</v>
+      </c>
+      <c r="F6" s="3" t="s">
+        <v>202</v>
+      </c>
+      <c r="G6" s="3" t="s">
+        <v>211</v>
+      </c>
+      <c r="H6" s="3" t="s">
+        <v>507</v>
+      </c>
+    </row>
+    <row r="7" spans="1:229" x14ac:dyDescent="0.35">
+      <c r="A7" s="3" t="s">
+        <v>509</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>508</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>510</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="E7" s="3" t="s">
+        <v>201</v>
+      </c>
+      <c r="F7" s="3" t="s">
+        <v>202</v>
+      </c>
+      <c r="G7" s="3" t="s">
+        <v>211</v>
+      </c>
+      <c r="H7" s="3" t="s">
+        <v>511</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet34.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1AD86191-7CFE-4ED9-9129-FF78170AB51E}">
-  <dimension ref="A1:HU12"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{95706458-CD50-4C74-87C4-ABAE617927AD}">
+  <dimension ref="A1:HU2"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="50.90625" bestFit="1" customWidth="1"/>
@@ -20373,7 +20270,7 @@
     <col min="5" max="5" width="33.08984375" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="17.08984375" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="40.81640625" customWidth="1"/>
-    <col min="8" max="8" width="65.54296875" customWidth="1"/>
+    <col min="8" max="8" width="57.08984375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:229" x14ac:dyDescent="0.35">
@@ -20404,13 +20301,13 @@
     </row>
     <row r="2" spans="1:229" s="4" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A2" s="3" t="s">
-        <v>527</v>
+        <v>512</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>528</v>
+        <v>513</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>529</v>
+        <v>514</v>
       </c>
       <c r="D2" s="3" t="s">
         <v>0</v>
@@ -20425,7 +20322,7 @@
         <v>211</v>
       </c>
       <c r="H2" s="3" t="s">
-        <v>530</v>
+        <v>140</v>
       </c>
       <c r="I2"/>
       <c r="J2"/>
@@ -20649,278 +20546,17 @@
       <c r="HT2"/>
       <c r="HU2"/>
     </row>
-    <row r="3" spans="1:229" x14ac:dyDescent="0.35">
-      <c r="A3" s="3" t="s">
-        <v>532</v>
-      </c>
-      <c r="B3" s="3" t="s">
-        <v>531</v>
-      </c>
-      <c r="C3" s="3" t="s">
-        <v>533</v>
-      </c>
-      <c r="D3" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="E3" s="3" t="s">
-        <v>201</v>
-      </c>
-      <c r="F3" s="3" t="s">
-        <v>202</v>
-      </c>
-      <c r="G3" s="3" t="s">
-        <v>211</v>
-      </c>
-      <c r="H3" s="3" t="s">
-        <v>534</v>
-      </c>
-    </row>
-    <row r="4" spans="1:229" x14ac:dyDescent="0.35">
-      <c r="A4" s="3" t="s">
-        <v>535</v>
-      </c>
-      <c r="B4" s="3" t="s">
-        <v>536</v>
-      </c>
-      <c r="C4" s="3" t="s">
-        <v>537</v>
-      </c>
-      <c r="D4" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="E4" s="3" t="s">
-        <v>201</v>
-      </c>
-      <c r="F4" s="3" t="s">
-        <v>202</v>
-      </c>
-      <c r="G4" s="3" t="s">
-        <v>211</v>
-      </c>
-      <c r="H4" s="3" t="s">
-        <v>538</v>
-      </c>
-    </row>
-    <row r="5" spans="1:229" x14ac:dyDescent="0.35">
-      <c r="A5" s="8" t="s">
-        <v>539</v>
-      </c>
-      <c r="B5" s="8" t="s">
-        <v>540</v>
-      </c>
-      <c r="C5" s="8" t="s">
-        <v>541</v>
-      </c>
-      <c r="D5" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="E5" s="3" t="s">
-        <v>201</v>
-      </c>
-      <c r="F5" s="3" t="s">
-        <v>202</v>
-      </c>
-      <c r="G5" s="3" t="s">
-        <v>211</v>
-      </c>
-      <c r="H5" s="3" t="s">
-        <v>542</v>
-      </c>
-    </row>
-    <row r="6" spans="1:229" x14ac:dyDescent="0.35">
-      <c r="A6" s="3" t="s">
-        <v>543</v>
-      </c>
-      <c r="B6" s="3" t="s">
-        <v>544</v>
-      </c>
-      <c r="C6" s="3" t="s">
-        <v>545</v>
-      </c>
-      <c r="D6" s="7" t="s">
-        <v>0</v>
-      </c>
-      <c r="E6" s="3" t="s">
-        <v>201</v>
-      </c>
-      <c r="F6" s="3" t="s">
-        <v>202</v>
-      </c>
-      <c r="G6" s="3" t="s">
-        <v>211</v>
-      </c>
-      <c r="H6" s="3" t="s">
-        <v>546</v>
-      </c>
-    </row>
-    <row r="7" spans="1:229" x14ac:dyDescent="0.35">
-      <c r="A7" s="3" t="s">
-        <v>547</v>
-      </c>
-      <c r="B7" s="3" t="s">
-        <v>548</v>
-      </c>
-      <c r="C7" s="3" t="s">
-        <v>549</v>
-      </c>
-      <c r="D7" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="E7" s="3" t="s">
-        <v>201</v>
-      </c>
-      <c r="F7" s="3" t="s">
-        <v>202</v>
-      </c>
-      <c r="G7" s="3" t="s">
-        <v>211</v>
-      </c>
-      <c r="H7" s="3" t="s">
-        <v>550</v>
-      </c>
-    </row>
-    <row r="8" spans="1:229" x14ac:dyDescent="0.35">
-      <c r="A8" s="3" t="s">
-        <v>551</v>
-      </c>
-      <c r="B8" s="3" t="s">
-        <v>552</v>
-      </c>
-      <c r="C8" s="3" t="s">
-        <v>553</v>
-      </c>
-      <c r="D8" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="E8" s="3" t="s">
-        <v>201</v>
-      </c>
-      <c r="F8" s="3" t="s">
-        <v>202</v>
-      </c>
-      <c r="G8" s="10" t="s">
-        <v>211</v>
-      </c>
-      <c r="H8" s="3" t="s">
-        <v>554</v>
-      </c>
-    </row>
-    <row r="9" spans="1:229" x14ac:dyDescent="0.35">
-      <c r="A9" s="3" t="s">
-        <v>555</v>
-      </c>
-      <c r="B9" s="3" t="s">
-        <v>556</v>
-      </c>
-      <c r="C9" s="3" t="s">
-        <v>558</v>
-      </c>
-      <c r="D9" s="7" t="s">
-        <v>0</v>
-      </c>
-      <c r="E9" s="3" t="s">
-        <v>201</v>
-      </c>
-      <c r="F9" s="3" t="s">
-        <v>202</v>
-      </c>
-      <c r="G9" s="10" t="s">
-        <v>211</v>
-      </c>
-      <c r="H9" s="3" t="s">
-        <v>557</v>
-      </c>
-    </row>
-    <row r="10" spans="1:229" x14ac:dyDescent="0.35">
-      <c r="A10" s="3" t="s">
-        <v>559</v>
-      </c>
-      <c r="B10" s="3" t="s">
-        <v>560</v>
-      </c>
-      <c r="C10" s="3" t="s">
-        <v>561</v>
-      </c>
-      <c r="D10" s="7" t="s">
-        <v>0</v>
-      </c>
-      <c r="E10" s="3" t="s">
-        <v>201</v>
-      </c>
-      <c r="F10" s="3" t="s">
-        <v>202</v>
-      </c>
-      <c r="G10" s="10" t="s">
-        <v>211</v>
-      </c>
-      <c r="H10" s="3" t="s">
-        <v>562</v>
-      </c>
-    </row>
-    <row r="11" spans="1:229" x14ac:dyDescent="0.35">
-      <c r="A11" s="3" t="s">
-        <v>563</v>
-      </c>
-      <c r="B11" s="3" t="s">
-        <v>564</v>
-      </c>
-      <c r="C11" s="3" t="s">
-        <v>565</v>
-      </c>
-      <c r="D11" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="E11" s="3" t="s">
-        <v>201</v>
-      </c>
-      <c r="F11" s="3" t="s">
-        <v>202</v>
-      </c>
-      <c r="G11" s="10" t="s">
-        <v>211</v>
-      </c>
-      <c r="H11" s="3" t="s">
-        <v>566</v>
-      </c>
-    </row>
-    <row r="12" spans="1:229" x14ac:dyDescent="0.35">
-      <c r="A12" s="3" t="s">
-        <v>567</v>
-      </c>
-      <c r="B12" s="3" t="s">
-        <v>568</v>
-      </c>
-      <c r="C12" s="3" t="s">
-        <v>569</v>
-      </c>
-      <c r="D12" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="E12" s="3" t="s">
-        <v>201</v>
-      </c>
-      <c r="F12" s="3" t="s">
-        <v>202</v>
-      </c>
-      <c r="G12" s="10" t="s">
-        <v>211</v>
-      </c>
-      <c r="H12" s="3" t="s">
-        <v>570</v>
-      </c>
-    </row>
   </sheetData>
-  <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet35.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{24EB34D0-BCF8-4F57-88CC-AC842687528F}">
-  <dimension ref="A1:HU5"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1AD86191-7CFE-4ED9-9129-FF78170AB51E}">
+  <dimension ref="A1:HU12"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="52.453125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="50.90625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="52.26953125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="42.453125" customWidth="1"/>
     <col min="4" max="4" width="33.36328125" bestFit="1" customWidth="1"/>
@@ -20958,13 +20594,13 @@
     </row>
     <row r="2" spans="1:229" s="4" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A2" s="3" t="s">
-        <v>576</v>
+        <v>527</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>577</v>
+        <v>528</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>578</v>
+        <v>529</v>
       </c>
       <c r="D2" s="3" t="s">
         <v>0</v>
@@ -20979,7 +20615,7 @@
         <v>211</v>
       </c>
       <c r="H2" s="3" t="s">
-        <v>579</v>
+        <v>530</v>
       </c>
       <c r="I2"/>
       <c r="J2"/>
@@ -21205,13 +20841,13 @@
     </row>
     <row r="3" spans="1:229" x14ac:dyDescent="0.35">
       <c r="A3" s="3" t="s">
-        <v>580</v>
+        <v>532</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>581</v>
+        <v>531</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>582</v>
+        <v>533</v>
       </c>
       <c r="D3" s="3" t="s">
         <v>0</v>
@@ -21226,42 +20862,44 @@
         <v>211</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>583</v>
+        <v>534</v>
       </c>
     </row>
     <row r="4" spans="1:229" x14ac:dyDescent="0.35">
-      <c r="A4" s="11" t="s">
-        <v>584</v>
-      </c>
-      <c r="B4" s="11" t="s">
-        <v>585</v>
-      </c>
-      <c r="C4" s="11" t="s">
-        <v>586</v>
-      </c>
-      <c r="D4" s="11" t="s">
+      <c r="A4" s="3" t="s">
+        <v>535</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>536</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>537</v>
+      </c>
+      <c r="D4" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="E4" s="11" t="s">
+      <c r="E4" s="3" t="s">
         <v>201</v>
       </c>
-      <c r="F4" s="11" t="s">
+      <c r="F4" s="3" t="s">
         <v>202</v>
       </c>
-      <c r="G4" s="11" t="s">
+      <c r="G4" s="3" t="s">
         <v>211</v>
       </c>
-      <c r="H4" s="11"/>
+      <c r="H4" s="3" t="s">
+        <v>538</v>
+      </c>
     </row>
     <row r="5" spans="1:229" x14ac:dyDescent="0.35">
-      <c r="A5" s="3" t="s">
-        <v>587</v>
-      </c>
-      <c r="B5" s="3" t="s">
-        <v>588</v>
-      </c>
-      <c r="C5" s="3" t="s">
-        <v>589</v>
+      <c r="A5" s="8" t="s">
+        <v>539</v>
+      </c>
+      <c r="B5" s="8" t="s">
+        <v>540</v>
+      </c>
+      <c r="C5" s="8" t="s">
+        <v>541</v>
       </c>
       <c r="D5" s="3" t="s">
         <v>0</v>
@@ -21276,17 +20914,200 @@
         <v>211</v>
       </c>
       <c r="H5" s="3" t="s">
-        <v>590</v>
+        <v>542</v>
+      </c>
+    </row>
+    <row r="6" spans="1:229" x14ac:dyDescent="0.35">
+      <c r="A6" s="3" t="s">
+        <v>543</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>544</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>545</v>
+      </c>
+      <c r="D6" s="7" t="s">
+        <v>0</v>
+      </c>
+      <c r="E6" s="3" t="s">
+        <v>201</v>
+      </c>
+      <c r="F6" s="3" t="s">
+        <v>202</v>
+      </c>
+      <c r="G6" s="3" t="s">
+        <v>211</v>
+      </c>
+      <c r="H6" s="3" t="s">
+        <v>546</v>
+      </c>
+    </row>
+    <row r="7" spans="1:229" x14ac:dyDescent="0.35">
+      <c r="A7" s="3" t="s">
+        <v>547</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>548</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>549</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="E7" s="3" t="s">
+        <v>201</v>
+      </c>
+      <c r="F7" s="3" t="s">
+        <v>202</v>
+      </c>
+      <c r="G7" s="3" t="s">
+        <v>211</v>
+      </c>
+      <c r="H7" s="3" t="s">
+        <v>550</v>
+      </c>
+    </row>
+    <row r="8" spans="1:229" x14ac:dyDescent="0.35">
+      <c r="A8" s="3" t="s">
+        <v>551</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>552</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>553</v>
+      </c>
+      <c r="D8" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="E8" s="3" t="s">
+        <v>201</v>
+      </c>
+      <c r="F8" s="3" t="s">
+        <v>202</v>
+      </c>
+      <c r="G8" s="10" t="s">
+        <v>211</v>
+      </c>
+      <c r="H8" s="3" t="s">
+        <v>554</v>
+      </c>
+    </row>
+    <row r="9" spans="1:229" x14ac:dyDescent="0.35">
+      <c r="A9" s="3" t="s">
+        <v>555</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>556</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>558</v>
+      </c>
+      <c r="D9" s="7" t="s">
+        <v>0</v>
+      </c>
+      <c r="E9" s="3" t="s">
+        <v>201</v>
+      </c>
+      <c r="F9" s="3" t="s">
+        <v>202</v>
+      </c>
+      <c r="G9" s="10" t="s">
+        <v>211</v>
+      </c>
+      <c r="H9" s="3" t="s">
+        <v>557</v>
+      </c>
+    </row>
+    <row r="10" spans="1:229" x14ac:dyDescent="0.35">
+      <c r="A10" s="3" t="s">
+        <v>559</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>560</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>561</v>
+      </c>
+      <c r="D10" s="7" t="s">
+        <v>0</v>
+      </c>
+      <c r="E10" s="3" t="s">
+        <v>201</v>
+      </c>
+      <c r="F10" s="3" t="s">
+        <v>202</v>
+      </c>
+      <c r="G10" s="10" t="s">
+        <v>211</v>
+      </c>
+      <c r="H10" s="3" t="s">
+        <v>562</v>
+      </c>
+    </row>
+    <row r="11" spans="1:229" x14ac:dyDescent="0.35">
+      <c r="A11" s="3" t="s">
+        <v>563</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>564</v>
+      </c>
+      <c r="C11" s="3" t="s">
+        <v>565</v>
+      </c>
+      <c r="D11" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="E11" s="3" t="s">
+        <v>201</v>
+      </c>
+      <c r="F11" s="3" t="s">
+        <v>202</v>
+      </c>
+      <c r="G11" s="10" t="s">
+        <v>211</v>
+      </c>
+      <c r="H11" s="3" t="s">
+        <v>566</v>
+      </c>
+    </row>
+    <row r="12" spans="1:229" x14ac:dyDescent="0.35">
+      <c r="A12" s="3" t="s">
+        <v>567</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>568</v>
+      </c>
+      <c r="C12" s="3" t="s">
+        <v>569</v>
+      </c>
+      <c r="D12" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="E12" s="3" t="s">
+        <v>201</v>
+      </c>
+      <c r="F12" s="3" t="s">
+        <v>202</v>
+      </c>
+      <c r="G12" s="10" t="s">
+        <v>211</v>
+      </c>
+      <c r="H12" s="3" t="s">
+        <v>570</v>
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet36.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7271F742-0542-4B33-AEE2-20AE8A69F475}">
-  <dimension ref="A1:HU3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{24EB34D0-BCF8-4F57-88CC-AC842687528F}">
+  <dimension ref="A1:HU5"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="52.453125" bestFit="1" customWidth="1"/>
@@ -21327,13 +21148,13 @@
     </row>
     <row r="2" spans="1:229" s="4" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A2" s="3" t="s">
-        <v>594</v>
+        <v>576</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>595</v>
+        <v>577</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>596</v>
+        <v>578</v>
       </c>
       <c r="D2" s="3" t="s">
         <v>0</v>
@@ -21348,7 +21169,7 @@
         <v>211</v>
       </c>
       <c r="H2" s="3" t="s">
-        <v>597</v>
+        <v>579</v>
       </c>
       <c r="I2"/>
       <c r="J2"/>
@@ -21574,13 +21395,13 @@
     </row>
     <row r="3" spans="1:229" x14ac:dyDescent="0.35">
       <c r="A3" s="3" t="s">
-        <v>598</v>
+        <v>580</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>599</v>
+        <v>581</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>600</v>
+        <v>582</v>
       </c>
       <c r="D3" s="3" t="s">
         <v>0</v>
@@ -21595,7 +21416,57 @@
         <v>211</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>601</v>
+        <v>583</v>
+      </c>
+    </row>
+    <row r="4" spans="1:229" x14ac:dyDescent="0.35">
+      <c r="A4" s="11" t="s">
+        <v>584</v>
+      </c>
+      <c r="B4" s="11" t="s">
+        <v>585</v>
+      </c>
+      <c r="C4" s="11" t="s">
+        <v>586</v>
+      </c>
+      <c r="D4" s="11" t="s">
+        <v>0</v>
+      </c>
+      <c r="E4" s="11" t="s">
+        <v>201</v>
+      </c>
+      <c r="F4" s="11" t="s">
+        <v>202</v>
+      </c>
+      <c r="G4" s="11" t="s">
+        <v>211</v>
+      </c>
+      <c r="H4" s="11"/>
+    </row>
+    <row r="5" spans="1:229" x14ac:dyDescent="0.35">
+      <c r="A5" s="3" t="s">
+        <v>587</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>588</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>589</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>201</v>
+      </c>
+      <c r="F5" s="3" t="s">
+        <v>202</v>
+      </c>
+      <c r="G5" s="3" t="s">
+        <v>211</v>
+      </c>
+      <c r="H5" s="3" t="s">
+        <v>590</v>
       </c>
     </row>
   </sheetData>
@@ -21604,6 +21475,325 @@
 </file>
 
 <file path=xl/worksheets/sheet37.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7271F742-0542-4B33-AEE2-20AE8A69F475}">
+  <dimension ref="A1:HU3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="52.453125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="52.26953125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="42.453125" customWidth="1"/>
+    <col min="4" max="4" width="33.36328125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="33.08984375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="17.08984375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="40.81640625" customWidth="1"/>
+    <col min="8" max="8" width="65.54296875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:229" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>209</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="2" spans="1:229" s="4" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A2" s="3" t="s">
+        <v>594</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>595</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>596</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>201</v>
+      </c>
+      <c r="F2" s="3" t="s">
+        <v>202</v>
+      </c>
+      <c r="G2" s="3" t="s">
+        <v>211</v>
+      </c>
+      <c r="H2" s="3" t="s">
+        <v>597</v>
+      </c>
+      <c r="I2"/>
+      <c r="J2"/>
+      <c r="K2"/>
+      <c r="L2"/>
+      <c r="M2"/>
+      <c r="N2"/>
+      <c r="O2"/>
+      <c r="P2"/>
+      <c r="Q2"/>
+      <c r="R2"/>
+      <c r="S2"/>
+      <c r="T2"/>
+      <c r="U2"/>
+      <c r="V2"/>
+      <c r="W2"/>
+      <c r="X2"/>
+      <c r="Y2"/>
+      <c r="Z2"/>
+      <c r="AA2"/>
+      <c r="AB2"/>
+      <c r="AC2"/>
+      <c r="AD2"/>
+      <c r="AE2"/>
+      <c r="AF2"/>
+      <c r="AG2"/>
+      <c r="AH2"/>
+      <c r="AI2"/>
+      <c r="AJ2"/>
+      <c r="AK2"/>
+      <c r="AL2"/>
+      <c r="AM2"/>
+      <c r="AN2"/>
+      <c r="AO2"/>
+      <c r="AP2"/>
+      <c r="AQ2"/>
+      <c r="AR2"/>
+      <c r="AS2"/>
+      <c r="AT2"/>
+      <c r="AU2"/>
+      <c r="AV2"/>
+      <c r="AW2"/>
+      <c r="AX2"/>
+      <c r="AY2"/>
+      <c r="AZ2"/>
+      <c r="BA2"/>
+      <c r="BB2"/>
+      <c r="BC2"/>
+      <c r="BD2"/>
+      <c r="BE2"/>
+      <c r="BF2"/>
+      <c r="BG2"/>
+      <c r="BH2"/>
+      <c r="BI2"/>
+      <c r="BJ2"/>
+      <c r="BK2"/>
+      <c r="BL2"/>
+      <c r="BM2"/>
+      <c r="BN2"/>
+      <c r="BO2"/>
+      <c r="BP2"/>
+      <c r="BQ2"/>
+      <c r="BR2"/>
+      <c r="BS2"/>
+      <c r="BT2"/>
+      <c r="BU2"/>
+      <c r="BV2"/>
+      <c r="BW2"/>
+      <c r="BX2"/>
+      <c r="BY2"/>
+      <c r="BZ2"/>
+      <c r="CA2"/>
+      <c r="CB2"/>
+      <c r="CC2"/>
+      <c r="CD2"/>
+      <c r="CE2"/>
+      <c r="CF2"/>
+      <c r="CG2"/>
+      <c r="CH2"/>
+      <c r="CI2"/>
+      <c r="CJ2"/>
+      <c r="CK2"/>
+      <c r="CL2"/>
+      <c r="CM2"/>
+      <c r="CN2"/>
+      <c r="CO2"/>
+      <c r="CP2"/>
+      <c r="CQ2"/>
+      <c r="CR2"/>
+      <c r="CS2"/>
+      <c r="CT2"/>
+      <c r="CU2"/>
+      <c r="CV2"/>
+      <c r="CW2"/>
+      <c r="CX2"/>
+      <c r="CY2"/>
+      <c r="CZ2"/>
+      <c r="DA2"/>
+      <c r="DB2"/>
+      <c r="DC2"/>
+      <c r="DD2"/>
+      <c r="DE2"/>
+      <c r="DF2"/>
+      <c r="DG2"/>
+      <c r="DH2"/>
+      <c r="DI2"/>
+      <c r="DJ2"/>
+      <c r="DK2"/>
+      <c r="DL2"/>
+      <c r="DM2"/>
+      <c r="DN2"/>
+      <c r="DO2"/>
+      <c r="DP2"/>
+      <c r="DQ2"/>
+      <c r="DR2"/>
+      <c r="DS2"/>
+      <c r="DT2"/>
+      <c r="DU2"/>
+      <c r="DV2"/>
+      <c r="DW2"/>
+      <c r="DX2"/>
+      <c r="DY2"/>
+      <c r="DZ2"/>
+      <c r="EA2"/>
+      <c r="EB2"/>
+      <c r="EC2"/>
+      <c r="ED2"/>
+      <c r="EE2"/>
+      <c r="EF2"/>
+      <c r="EG2"/>
+      <c r="EH2"/>
+      <c r="EI2"/>
+      <c r="EJ2"/>
+      <c r="EK2"/>
+      <c r="EL2"/>
+      <c r="EM2"/>
+      <c r="EN2"/>
+      <c r="EO2"/>
+      <c r="EP2"/>
+      <c r="EQ2"/>
+      <c r="ER2"/>
+      <c r="ES2"/>
+      <c r="ET2"/>
+      <c r="EU2"/>
+      <c r="EV2"/>
+      <c r="EW2"/>
+      <c r="EX2"/>
+      <c r="EY2"/>
+      <c r="EZ2"/>
+      <c r="FA2"/>
+      <c r="FB2"/>
+      <c r="FC2"/>
+      <c r="FD2"/>
+      <c r="FE2"/>
+      <c r="FF2"/>
+      <c r="FG2"/>
+      <c r="FH2"/>
+      <c r="FI2"/>
+      <c r="FJ2"/>
+      <c r="FK2"/>
+      <c r="FL2"/>
+      <c r="FM2"/>
+      <c r="FN2"/>
+      <c r="FO2"/>
+      <c r="FP2"/>
+      <c r="FQ2"/>
+      <c r="FR2"/>
+      <c r="FS2"/>
+      <c r="FT2"/>
+      <c r="FU2"/>
+      <c r="FV2"/>
+      <c r="FW2"/>
+      <c r="FX2"/>
+      <c r="FY2"/>
+      <c r="FZ2"/>
+      <c r="GA2"/>
+      <c r="GB2"/>
+      <c r="GC2"/>
+      <c r="GD2"/>
+      <c r="GE2"/>
+      <c r="GF2"/>
+      <c r="GG2"/>
+      <c r="GH2"/>
+      <c r="GI2"/>
+      <c r="GJ2"/>
+      <c r="GK2"/>
+      <c r="GL2"/>
+      <c r="GM2"/>
+      <c r="GN2"/>
+      <c r="GO2"/>
+      <c r="GP2"/>
+      <c r="GQ2"/>
+      <c r="GR2"/>
+      <c r="GS2"/>
+      <c r="GT2"/>
+      <c r="GU2"/>
+      <c r="GV2"/>
+      <c r="GW2"/>
+      <c r="GX2"/>
+      <c r="GY2"/>
+      <c r="GZ2"/>
+      <c r="HA2"/>
+      <c r="HB2"/>
+      <c r="HC2"/>
+      <c r="HD2"/>
+      <c r="HE2"/>
+      <c r="HF2"/>
+      <c r="HG2"/>
+      <c r="HH2"/>
+      <c r="HI2"/>
+      <c r="HJ2"/>
+      <c r="HK2"/>
+      <c r="HL2"/>
+      <c r="HM2"/>
+      <c r="HN2"/>
+      <c r="HO2"/>
+      <c r="HP2"/>
+      <c r="HQ2"/>
+      <c r="HR2"/>
+      <c r="HS2"/>
+      <c r="HT2"/>
+      <c r="HU2"/>
+    </row>
+    <row r="3" spans="1:229" x14ac:dyDescent="0.35">
+      <c r="A3" s="3" t="s">
+        <v>598</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>599</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>600</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>201</v>
+      </c>
+      <c r="F3" s="3" t="s">
+        <v>202</v>
+      </c>
+      <c r="G3" s="3" t="s">
+        <v>211</v>
+      </c>
+      <c r="H3" s="3" t="s">
+        <v>601</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet38.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{738B4CF9-CA20-4A87-AA62-B89EDC02284E}">
   <dimension ref="A1:HU5"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -21973,7 +22163,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet38.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet39.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{09B1B3C7-FD6F-4E3B-8CD4-D9B4FAD90EEE}">
   <dimension ref="A1:HU5"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -23151,6 +23341,430 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet40.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{23CC273B-FFDA-44C0-9F09-DBCCADFC6C49}">
+  <dimension ref="A1:HU7"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="50.54296875" customWidth="1"/>
+    <col min="2" max="2" width="52.26953125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="42.453125" customWidth="1"/>
+    <col min="4" max="4" width="33.36328125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="33.08984375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="17.08984375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="40.81640625" customWidth="1"/>
+    <col min="8" max="8" width="65.54296875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:229" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>209</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="2" spans="1:229" s="4" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A2" s="3" t="s">
+        <v>650</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>651</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>652</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>201</v>
+      </c>
+      <c r="F2" s="3" t="s">
+        <v>202</v>
+      </c>
+      <c r="G2" s="3" t="s">
+        <v>211</v>
+      </c>
+      <c r="H2" s="3" t="s">
+        <v>653</v>
+      </c>
+      <c r="I2"/>
+      <c r="J2"/>
+      <c r="K2"/>
+      <c r="L2"/>
+      <c r="M2"/>
+      <c r="N2"/>
+      <c r="O2"/>
+      <c r="P2"/>
+      <c r="Q2"/>
+      <c r="R2"/>
+      <c r="S2"/>
+      <c r="T2"/>
+      <c r="U2"/>
+      <c r="V2"/>
+      <c r="W2"/>
+      <c r="X2"/>
+      <c r="Y2"/>
+      <c r="Z2"/>
+      <c r="AA2"/>
+      <c r="AB2"/>
+      <c r="AC2"/>
+      <c r="AD2"/>
+      <c r="AE2"/>
+      <c r="AF2"/>
+      <c r="AG2"/>
+      <c r="AH2"/>
+      <c r="AI2"/>
+      <c r="AJ2"/>
+      <c r="AK2"/>
+      <c r="AL2"/>
+      <c r="AM2"/>
+      <c r="AN2"/>
+      <c r="AO2"/>
+      <c r="AP2"/>
+      <c r="AQ2"/>
+      <c r="AR2"/>
+      <c r="AS2"/>
+      <c r="AT2"/>
+      <c r="AU2"/>
+      <c r="AV2"/>
+      <c r="AW2"/>
+      <c r="AX2"/>
+      <c r="AY2"/>
+      <c r="AZ2"/>
+      <c r="BA2"/>
+      <c r="BB2"/>
+      <c r="BC2"/>
+      <c r="BD2"/>
+      <c r="BE2"/>
+      <c r="BF2"/>
+      <c r="BG2"/>
+      <c r="BH2"/>
+      <c r="BI2"/>
+      <c r="BJ2"/>
+      <c r="BK2"/>
+      <c r="BL2"/>
+      <c r="BM2"/>
+      <c r="BN2"/>
+      <c r="BO2"/>
+      <c r="BP2"/>
+      <c r="BQ2"/>
+      <c r="BR2"/>
+      <c r="BS2"/>
+      <c r="BT2"/>
+      <c r="BU2"/>
+      <c r="BV2"/>
+      <c r="BW2"/>
+      <c r="BX2"/>
+      <c r="BY2"/>
+      <c r="BZ2"/>
+      <c r="CA2"/>
+      <c r="CB2"/>
+      <c r="CC2"/>
+      <c r="CD2"/>
+      <c r="CE2"/>
+      <c r="CF2"/>
+      <c r="CG2"/>
+      <c r="CH2"/>
+      <c r="CI2"/>
+      <c r="CJ2"/>
+      <c r="CK2"/>
+      <c r="CL2"/>
+      <c r="CM2"/>
+      <c r="CN2"/>
+      <c r="CO2"/>
+      <c r="CP2"/>
+      <c r="CQ2"/>
+      <c r="CR2"/>
+      <c r="CS2"/>
+      <c r="CT2"/>
+      <c r="CU2"/>
+      <c r="CV2"/>
+      <c r="CW2"/>
+      <c r="CX2"/>
+      <c r="CY2"/>
+      <c r="CZ2"/>
+      <c r="DA2"/>
+      <c r="DB2"/>
+      <c r="DC2"/>
+      <c r="DD2"/>
+      <c r="DE2"/>
+      <c r="DF2"/>
+      <c r="DG2"/>
+      <c r="DH2"/>
+      <c r="DI2"/>
+      <c r="DJ2"/>
+      <c r="DK2"/>
+      <c r="DL2"/>
+      <c r="DM2"/>
+      <c r="DN2"/>
+      <c r="DO2"/>
+      <c r="DP2"/>
+      <c r="DQ2"/>
+      <c r="DR2"/>
+      <c r="DS2"/>
+      <c r="DT2"/>
+      <c r="DU2"/>
+      <c r="DV2"/>
+      <c r="DW2"/>
+      <c r="DX2"/>
+      <c r="DY2"/>
+      <c r="DZ2"/>
+      <c r="EA2"/>
+      <c r="EB2"/>
+      <c r="EC2"/>
+      <c r="ED2"/>
+      <c r="EE2"/>
+      <c r="EF2"/>
+      <c r="EG2"/>
+      <c r="EH2"/>
+      <c r="EI2"/>
+      <c r="EJ2"/>
+      <c r="EK2"/>
+      <c r="EL2"/>
+      <c r="EM2"/>
+      <c r="EN2"/>
+      <c r="EO2"/>
+      <c r="EP2"/>
+      <c r="EQ2"/>
+      <c r="ER2"/>
+      <c r="ES2"/>
+      <c r="ET2"/>
+      <c r="EU2"/>
+      <c r="EV2"/>
+      <c r="EW2"/>
+      <c r="EX2"/>
+      <c r="EY2"/>
+      <c r="EZ2"/>
+      <c r="FA2"/>
+      <c r="FB2"/>
+      <c r="FC2"/>
+      <c r="FD2"/>
+      <c r="FE2"/>
+      <c r="FF2"/>
+      <c r="FG2"/>
+      <c r="FH2"/>
+      <c r="FI2"/>
+      <c r="FJ2"/>
+      <c r="FK2"/>
+      <c r="FL2"/>
+      <c r="FM2"/>
+      <c r="FN2"/>
+      <c r="FO2"/>
+      <c r="FP2"/>
+      <c r="FQ2"/>
+      <c r="FR2"/>
+      <c r="FS2"/>
+      <c r="FT2"/>
+      <c r="FU2"/>
+      <c r="FV2"/>
+      <c r="FW2"/>
+      <c r="FX2"/>
+      <c r="FY2"/>
+      <c r="FZ2"/>
+      <c r="GA2"/>
+      <c r="GB2"/>
+      <c r="GC2"/>
+      <c r="GD2"/>
+      <c r="GE2"/>
+      <c r="GF2"/>
+      <c r="GG2"/>
+      <c r="GH2"/>
+      <c r="GI2"/>
+      <c r="GJ2"/>
+      <c r="GK2"/>
+      <c r="GL2"/>
+      <c r="GM2"/>
+      <c r="GN2"/>
+      <c r="GO2"/>
+      <c r="GP2"/>
+      <c r="GQ2"/>
+      <c r="GR2"/>
+      <c r="GS2"/>
+      <c r="GT2"/>
+      <c r="GU2"/>
+      <c r="GV2"/>
+      <c r="GW2"/>
+      <c r="GX2"/>
+      <c r="GY2"/>
+      <c r="GZ2"/>
+      <c r="HA2"/>
+      <c r="HB2"/>
+      <c r="HC2"/>
+      <c r="HD2"/>
+      <c r="HE2"/>
+      <c r="HF2"/>
+      <c r="HG2"/>
+      <c r="HH2"/>
+      <c r="HI2"/>
+      <c r="HJ2"/>
+      <c r="HK2"/>
+      <c r="HL2"/>
+      <c r="HM2"/>
+      <c r="HN2"/>
+      <c r="HO2"/>
+      <c r="HP2"/>
+      <c r="HQ2"/>
+      <c r="HR2"/>
+      <c r="HS2"/>
+      <c r="HT2"/>
+      <c r="HU2"/>
+    </row>
+    <row r="3" spans="1:229" x14ac:dyDescent="0.35">
+      <c r="A3" s="3" t="s">
+        <v>655</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>654</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>656</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>201</v>
+      </c>
+      <c r="F3" s="3" t="s">
+        <v>202</v>
+      </c>
+      <c r="G3" s="3" t="s">
+        <v>211</v>
+      </c>
+      <c r="H3" s="3" t="s">
+        <v>657</v>
+      </c>
+    </row>
+    <row r="4" spans="1:229" x14ac:dyDescent="0.35">
+      <c r="A4" s="3" t="s">
+        <v>658</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>659</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>660</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>201</v>
+      </c>
+      <c r="F4" s="3" t="s">
+        <v>202</v>
+      </c>
+      <c r="G4" s="3" t="s">
+        <v>211</v>
+      </c>
+      <c r="H4" s="3" t="s">
+        <v>661</v>
+      </c>
+    </row>
+    <row r="5" spans="1:229" x14ac:dyDescent="0.35">
+      <c r="A5" s="3" t="s">
+        <v>662</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>663</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>664</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>201</v>
+      </c>
+      <c r="F5" s="3" t="s">
+        <v>202</v>
+      </c>
+      <c r="G5" s="3" t="s">
+        <v>211</v>
+      </c>
+      <c r="H5" s="3" t="s">
+        <v>665</v>
+      </c>
+    </row>
+    <row r="6" spans="1:229" x14ac:dyDescent="0.35">
+      <c r="A6" s="3" t="s">
+        <v>666</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>667</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>668</v>
+      </c>
+      <c r="D6" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="E6" s="3" t="s">
+        <v>201</v>
+      </c>
+      <c r="F6" s="3" t="s">
+        <v>202</v>
+      </c>
+      <c r="G6" s="3" t="s">
+        <v>211</v>
+      </c>
+      <c r="H6" s="3" t="s">
+        <v>669</v>
+      </c>
+    </row>
+    <row r="7" spans="1:229" x14ac:dyDescent="0.35">
+      <c r="A7" s="3" t="s">
+        <v>670</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>671</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>672</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="E7" s="3" t="s">
+        <v>201</v>
+      </c>
+      <c r="F7" s="3" t="s">
+        <v>202</v>
+      </c>
+      <c r="G7" s="3" t="s">
+        <v>211</v>
+      </c>
+      <c r="H7" s="3" t="s">
+        <v>673</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F0334D8A-9DDC-4B51-9686-8ED497406295}">
   <dimension ref="A1:C9"/>

</xml_diff>